<commit_message>
Fix normalized naming and created graphs and update the columns parameter
</commit_message>
<xml_diff>
--- a/BioSensorAnalysisSrcCode/EIS_Analysis/Austin_EIS/MegaExcel/Processed Chips for PCAI1ia/Chip 21.xlsx
+++ b/BioSensorAnalysisSrcCode/EIS_Analysis/Austin_EIS/MegaExcel/Processed Chips for PCAI1ia/Chip 21.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB1"/>
+  <dimension ref="A1:AB11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -528,12 +528,12 @@
       </c>
       <c r="W1" t="inlineStr">
         <is>
-          <t>Cycle</t>
+          <t>Model</t>
         </is>
       </c>
       <c r="X1" t="inlineStr">
         <is>
-          <t>Model</t>
+          <t>b</t>
         </is>
       </c>
       <c r="Y1" t="inlineStr">
@@ -543,7 +543,7 @@
       </c>
       <c r="Z1" t="inlineStr">
         <is>
-          <t>Rp</t>
+          <t>delta Rct-i</t>
         </is>
       </c>
       <c r="AA1" t="inlineStr">
@@ -555,6 +555,526 @@
         <is>
           <t>n</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B2" t="n">
+        <v>-604.1999999999998</v>
+      </c>
+      <c r="D2" t="n">
+        <v>1.84241e-07</v>
+      </c>
+      <c r="E2" t="n">
+        <v>-48.485</v>
+      </c>
+      <c r="F2" t="n">
+        <v/>
+      </c>
+      <c r="G2" t="n">
+        <v/>
+      </c>
+      <c r="H2" t="n">
+        <v/>
+      </c>
+      <c r="I2" t="n">
+        <v/>
+      </c>
+      <c r="J2" t="n">
+        <v>9.644800140610634</v>
+      </c>
+      <c r="K2" t="n">
+        <v>81.93371453681854</v>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>y = 7.056x + -25925.977</t>
+        </is>
+      </c>
+      <c r="X2" t="n">
+        <v>-25925.97725441957</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>3.973360418002409e-09</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>604.1999999999998</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>1.000000000002033e-08</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>0.8190105121528939</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B3" t="n">
+        <v>-559.77</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1.89606e-07</v>
+      </c>
+      <c r="E3" t="n">
+        <v>-49.79</v>
+      </c>
+      <c r="F3" t="n">
+        <v/>
+      </c>
+      <c r="G3" t="n">
+        <v/>
+      </c>
+      <c r="H3" t="n">
+        <v/>
+      </c>
+      <c r="I3" t="n">
+        <v/>
+      </c>
+      <c r="J3" t="n">
+        <v>10.7497149678286</v>
+      </c>
+      <c r="K3" t="n">
+        <v>82.56790490797303</v>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>y = 7.666x + -27402.847</t>
+        </is>
+      </c>
+      <c r="X3" t="n">
+        <v>-27402.84736786969</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>1.897271783591817e-18</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>559.77</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>1e-08</v>
+      </c>
+      <c r="AB3" t="n">
+        <v>0.8192380225601228</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B4" t="n">
+        <v>-540.23</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1.92888e-07</v>
+      </c>
+      <c r="E4" t="n">
+        <v>-50.599</v>
+      </c>
+      <c r="F4" t="n">
+        <v/>
+      </c>
+      <c r="G4" t="n">
+        <v/>
+      </c>
+      <c r="H4" t="n">
+        <v/>
+      </c>
+      <c r="I4" t="n">
+        <v/>
+      </c>
+      <c r="J4" t="n">
+        <v>11.24861645299463</v>
+      </c>
+      <c r="K4" t="n">
+        <v>82.86147480804301</v>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>y = 7.985x + -27984.201</t>
+        </is>
+      </c>
+      <c r="X4" t="n">
+        <v>-27984.20086789379</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>1.274334709434572e-10</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>540.23</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>1.000000000000405e-08</v>
+      </c>
+      <c r="AB4" t="n">
+        <v>0.8194306751329862</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>12</v>
+      </c>
+      <c r="B5" t="n">
+        <v>-512.1300000000001</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1.96208e-07</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-51.329</v>
+      </c>
+      <c r="F5" t="n">
+        <v/>
+      </c>
+      <c r="G5" t="n">
+        <v/>
+      </c>
+      <c r="H5" t="n">
+        <v/>
+      </c>
+      <c r="I5" t="n">
+        <v/>
+      </c>
+      <c r="J5" t="n">
+        <v>12.13290401259441</v>
+      </c>
+      <c r="K5" t="n">
+        <v>83.23250269088234</v>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>y = 8.427x + -29046.995</t>
+        </is>
+      </c>
+      <c r="X5" t="n">
+        <v>-29046.99463667542</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>1.579012405788227e-10</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>512.1300000000001</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>1.00000000000001e-08</v>
+      </c>
+      <c r="AB5" t="n">
+        <v>0.8196603524056216</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>15</v>
+      </c>
+      <c r="B6" t="n">
+        <v>-504.75</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1.98503e-07</v>
+      </c>
+      <c r="E6" t="n">
+        <v>-51.875</v>
+      </c>
+      <c r="F6" t="n">
+        <v/>
+      </c>
+      <c r="G6" t="n">
+        <v/>
+      </c>
+      <c r="H6" t="n">
+        <v/>
+      </c>
+      <c r="I6" t="n">
+        <v/>
+      </c>
+      <c r="J6" t="n">
+        <v>12.38093257540135</v>
+      </c>
+      <c r="K6" t="n">
+        <v>83.34227232969749</v>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>y = 8.567x + -29058.639</t>
+        </is>
+      </c>
+      <c r="X6" t="n">
+        <v>-29058.63871125671</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>4.911906337866607e-10</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>504.75</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>1.000000000000073e-08</v>
+      </c>
+      <c r="AB6" t="n">
+        <v>0.8198786462700921</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>18</v>
+      </c>
+      <c r="B7" t="n">
+        <v>-493.4400000000001</v>
+      </c>
+      <c r="D7" t="n">
+        <v>2.00804e-07</v>
+      </c>
+      <c r="E7" t="n">
+        <v>-52.396</v>
+      </c>
+      <c r="F7" t="n">
+        <v/>
+      </c>
+      <c r="G7" t="n">
+        <v/>
+      </c>
+      <c r="H7" t="n">
+        <v/>
+      </c>
+      <c r="I7" t="n">
+        <v/>
+      </c>
+      <c r="J7" t="n">
+        <v>12.87957765198097</v>
+      </c>
+      <c r="K7" t="n">
+        <v>83.48385721504475</v>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>y = 8.755x + -29264.941</t>
+        </is>
+      </c>
+      <c r="X7" t="n">
+        <v>-29264.9409855333</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>1.123012009317532e-16</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>493.4400000000001</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>1e-08</v>
+      </c>
+      <c r="AB7" t="n">
+        <v>0.8201164885884019</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>21</v>
+      </c>
+      <c r="B8" t="n">
+        <v>-496.9099999999999</v>
+      </c>
+      <c r="D8" t="n">
+        <v>2.02918e-07</v>
+      </c>
+      <c r="E8" t="n">
+        <v>-52.821</v>
+      </c>
+      <c r="F8" t="n">
+        <v/>
+      </c>
+      <c r="G8" t="n">
+        <v/>
+      </c>
+      <c r="H8" t="n">
+        <v/>
+      </c>
+      <c r="I8" t="n">
+        <v/>
+      </c>
+      <c r="J8" t="n">
+        <v>11.49941191698496</v>
+      </c>
+      <c r="K8" t="n">
+        <v>83.2328377728806</v>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>y = 8.427x + -27659.995</t>
+        </is>
+      </c>
+      <c r="X8" t="n">
+        <v>-27659.99456902865</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>5.529700177760481e-12</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>496.9099999999999</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>1.000000000000038e-08</v>
+      </c>
+      <c r="AB8" t="n">
+        <v>0.8203440186358629</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>24</v>
+      </c>
+      <c r="B9" t="n">
+        <v>-489.0599999999999</v>
+      </c>
+      <c r="D9" t="n">
+        <v>2.04758e-07</v>
+      </c>
+      <c r="E9" t="n">
+        <v>-53.283</v>
+      </c>
+      <c r="F9" t="n">
+        <v/>
+      </c>
+      <c r="G9" t="n">
+        <v/>
+      </c>
+      <c r="H9" t="n">
+        <v/>
+      </c>
+      <c r="I9" t="n">
+        <v/>
+      </c>
+      <c r="J9" t="n">
+        <v>11.84341408076169</v>
+      </c>
+      <c r="K9" t="n">
+        <v>83.38119694298761</v>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>y = 8.618x + -27949.070</t>
+        </is>
+      </c>
+      <c r="X9" t="n">
+        <v>-27949.07001255509</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>3.952318134702614e-09</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>489.0599999999999</v>
+      </c>
+      <c r="AA9" t="n">
+        <v>1.000000000014565e-08</v>
+      </c>
+      <c r="AB9" t="n">
+        <v>0.8205870384037237</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>27</v>
+      </c>
+      <c r="B10" t="n">
+        <v>-477.1399999999999</v>
+      </c>
+      <c r="D10" t="n">
+        <v>2.06513e-07</v>
+      </c>
+      <c r="E10" t="n">
+        <v>-53.649</v>
+      </c>
+      <c r="F10" t="n">
+        <v/>
+      </c>
+      <c r="G10" t="n">
+        <v/>
+      </c>
+      <c r="H10" t="n">
+        <v/>
+      </c>
+      <c r="I10" t="n">
+        <v/>
+      </c>
+      <c r="J10" t="n">
+        <v>12.13603096097347</v>
+      </c>
+      <c r="K10" t="n">
+        <v>83.54601674051274</v>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>y = 8.840x + -28364.159</t>
+        </is>
+      </c>
+      <c r="X10" t="n">
+        <v>-28364.1585730412</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>8.695782116767691e-09</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>477.1399999999999</v>
+      </c>
+      <c r="AA10" t="n">
+        <v>1.000000000000013e-08</v>
+      </c>
+      <c r="AB10" t="n">
+        <v>0.8208473253213493</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>30</v>
+      </c>
+      <c r="B11" t="n">
+        <v>-455.8200000000002</v>
+      </c>
+      <c r="D11" t="n">
+        <v>2.08089e-07</v>
+      </c>
+      <c r="E11" t="n">
+        <v>-53.984</v>
+      </c>
+      <c r="F11" t="n">
+        <v/>
+      </c>
+      <c r="G11" t="n">
+        <v/>
+      </c>
+      <c r="H11" t="n">
+        <v/>
+      </c>
+      <c r="I11" t="n">
+        <v/>
+      </c>
+      <c r="J11" t="n">
+        <v>14.47057370159176</v>
+      </c>
+      <c r="K11" t="n">
+        <v>83.98408608789487</v>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>y = 9.489x + -30286.635</t>
+        </is>
+      </c>
+      <c r="X11" t="n">
+        <v>-30286.63477810142</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>7.399923275621092e-09</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>455.8200000000002</v>
+      </c>
+      <c r="AA11" t="n">
+        <v>1.000000000000328e-08</v>
+      </c>
+      <c r="AB11" t="n">
+        <v>0.8211046539370254</v>
       </c>
     </row>
   </sheetData>
@@ -674,12 +1194,12 @@
       </c>
       <c r="W1" t="inlineStr">
         <is>
-          <t>Cycle</t>
+          <t>Model</t>
         </is>
       </c>
       <c r="X1" t="inlineStr">
         <is>
-          <t>Model</t>
+          <t>b</t>
         </is>
       </c>
       <c r="Y1" t="inlineStr">
@@ -689,7 +1209,7 @@
       </c>
       <c r="Z1" t="inlineStr">
         <is>
-          <t>Rp</t>
+          <t>delta Rct-i</t>
         </is>
       </c>
       <c r="AA1" t="inlineStr">
@@ -734,19 +1254,19 @@
       <c r="K2" t="n">
         <v>83.03716034820951</v>
       </c>
-      <c r="W2" t="n">
-        <v>1</v>
-      </c>
-      <c r="X2" t="inlineStr">
+      <c r="W2" t="inlineStr">
         <is>
           <t>y = 8.188x + -28805.250</t>
         </is>
+      </c>
+      <c r="X2" t="n">
+        <v>-28805.24954287466</v>
       </c>
       <c r="Y2" t="n">
         <v>3.461751648758845e-09</v>
       </c>
       <c r="Z2" t="n">
-        <v>4126.568694892875</v>
+        <v>570.52</v>
       </c>
       <c r="AA2" t="n">
         <v>1.000000000000682e-08</v>
@@ -786,19 +1306,19 @@
       <c r="K3" t="n">
         <v>82.77928794294931</v>
       </c>
-      <c r="W3" t="n">
-        <v>2</v>
-      </c>
-      <c r="X3" t="inlineStr">
+      <c r="W3" t="inlineStr">
         <is>
           <t>y = 7.893x + -26594.526</t>
         </is>
+      </c>
+      <c r="X3" t="n">
+        <v>-26594.52615563833</v>
       </c>
       <c r="Y3" t="n">
         <v>1.945267163618647e-08</v>
       </c>
       <c r="Z3" t="n">
-        <v>3984.43311368162</v>
+        <v>576.1600000000003</v>
       </c>
       <c r="AA3" t="n">
         <v>1.000000000000073e-08</v>
@@ -838,19 +1358,19 @@
       <c r="K4" t="n">
         <v>83.15696832756892</v>
       </c>
-      <c r="W4" t="n">
-        <v>3</v>
-      </c>
-      <c r="X4" t="inlineStr">
+      <c r="W4" t="inlineStr">
         <is>
           <t>y = 8.333x + -27815.874</t>
         </is>
+      </c>
+      <c r="X4" t="n">
+        <v>-27815.87381972411</v>
       </c>
       <c r="Y4" t="n">
         <v>9.744149832265997e-15</v>
       </c>
       <c r="Z4" t="n">
-        <v>3924.695747861717</v>
+        <v>551.21</v>
       </c>
       <c r="AA4" t="n">
         <v>1.000000000000394e-08</v>
@@ -890,19 +1410,19 @@
       <c r="K5" t="n">
         <v>82.85600964996303</v>
       </c>
-      <c r="W5" t="n">
-        <v>4</v>
-      </c>
-      <c r="X5" t="inlineStr">
+      <c r="W5" t="inlineStr">
         <is>
           <t>y = 7.979x + -26194.989</t>
         </is>
+      </c>
+      <c r="X5" t="n">
+        <v>-26194.98924499944</v>
       </c>
       <c r="Y5" t="n">
         <v>2.041724315974994e-15</v>
       </c>
       <c r="Z5" t="n">
-        <v>3877.998216129423</v>
+        <v>560.8499999999999</v>
       </c>
       <c r="AA5" t="n">
         <v>1e-08</v>
@@ -942,19 +1462,19 @@
       <c r="K6" t="n">
         <v>82.54954797767374</v>
       </c>
-      <c r="W6" t="n">
-        <v>5</v>
-      </c>
-      <c r="X6" t="inlineStr">
+      <c r="W6" t="inlineStr">
         <is>
           <t>y = 7.647x + -24734.360</t>
         </is>
+      </c>
+      <c r="X6" t="n">
+        <v>-24734.36023161278</v>
       </c>
       <c r="Y6" t="n">
         <v>2.64856299099321e-10</v>
       </c>
       <c r="Z6" t="n">
-        <v>3835.907573896849</v>
+        <v>574.8999999999996</v>
       </c>
       <c r="AA6" t="n">
         <v>1.000000000000014e-08</v>
@@ -994,19 +1514,19 @@
       <c r="K7" t="n">
         <v>82.98278493842304</v>
       </c>
-      <c r="W7" t="n">
-        <v>6</v>
-      </c>
-      <c r="X7" t="inlineStr">
+      <c r="W7" t="inlineStr">
         <is>
           <t>y = 8.124x + -26162.317</t>
         </is>
+      </c>
+      <c r="X7" t="n">
+        <v>-26162.31709657338</v>
       </c>
       <c r="Y7" t="n">
         <v>3.845840421510457e-10</v>
       </c>
       <c r="Z7" t="n">
-        <v>3796.855465673337</v>
+        <v>546.5799999999999</v>
       </c>
       <c r="AA7" t="n">
         <v>1.000000000000006e-08</v>
@@ -1046,19 +1566,19 @@
       <c r="K8" t="n">
         <v>83.04933641167069</v>
       </c>
-      <c r="W8" t="n">
-        <v>7</v>
-      </c>
-      <c r="X8" t="inlineStr">
+      <c r="W8" t="inlineStr">
         <is>
           <t>y = 8.203x + -26167.616</t>
         </is>
+      </c>
+      <c r="X8" t="n">
+        <v>-26167.61583122996</v>
       </c>
       <c r="Y8" t="n">
         <v>9.518381345387516e-11</v>
       </c>
       <c r="Z8" t="n">
-        <v>3757.938164876658</v>
+        <v>542.5900000000001</v>
       </c>
       <c r="AA8" t="n">
         <v>1.000000000000125e-08</v>
@@ -1098,19 +1618,19 @@
       <c r="K9" t="n">
         <v>83.06972347938839</v>
       </c>
-      <c r="W9" t="n">
-        <v>8</v>
-      </c>
-      <c r="X9" t="inlineStr">
+      <c r="W9" t="inlineStr">
         <is>
           <t>y = 8.227x + -26000.871</t>
         </is>
+      </c>
+      <c r="X9" t="n">
+        <v>-26000.87059454789</v>
       </c>
       <c r="Y9" t="n">
         <v>8.962322664060081e-11</v>
       </c>
       <c r="Z9" t="n">
-        <v>3720.957971118632</v>
+        <v>538.27</v>
       </c>
       <c r="AA9" t="n">
         <v>1e-08</v>
@@ -1150,19 +1670,19 @@
       <c r="K10" t="n">
         <v>83.17228099437796</v>
       </c>
-      <c r="W10" t="n">
-        <v>9</v>
-      </c>
-      <c r="X10" t="inlineStr">
+      <c r="W10" t="inlineStr">
         <is>
           <t>y = 8.352x + -26168.492</t>
         </is>
+      </c>
+      <c r="X10" t="n">
+        <v>-26168.49190365453</v>
       </c>
       <c r="Y10" t="n">
         <v>1.490559670089616e-10</v>
       </c>
       <c r="Z10" t="n">
-        <v>3684.621667345081</v>
+        <v>529.23</v>
       </c>
       <c r="AA10" t="n">
         <v>1.000000000003612e-08</v>
@@ -1202,19 +1722,19 @@
       <c r="K11" t="n">
         <v>83.25738709885832</v>
       </c>
-      <c r="W11" t="n">
-        <v>10</v>
-      </c>
-      <c r="X11" t="inlineStr">
+      <c r="W11" t="inlineStr">
         <is>
           <t>y = 8.458x + -26289.539</t>
         </is>
+      </c>
+      <c r="X11" t="n">
+        <v>-26289.53935116196</v>
       </c>
       <c r="Y11" t="n">
         <v>4.437929537938406e-09</v>
       </c>
       <c r="Z11" t="n">
-        <v>3650.464634807239</v>
+        <v>519.21</v>
       </c>
       <c r="AA11" t="n">
         <v>1.000000000000007e-08</v>
@@ -1254,19 +1774,19 @@
       <c r="K12" t="n">
         <v>83.3041612171084</v>
       </c>
-      <c r="W12" t="n">
-        <v>11</v>
-      </c>
-      <c r="X12" t="inlineStr">
+      <c r="W12" t="inlineStr">
         <is>
           <t>y = 8.518x + -26240.547</t>
         </is>
+      </c>
+      <c r="X12" t="n">
+        <v>-26240.54747800111</v>
       </c>
       <c r="Y12" t="n">
         <v>2.383232571510424e-10</v>
       </c>
       <c r="Z12" t="n">
-        <v>3617.155723543447</v>
+        <v>516.1799999999998</v>
       </c>
       <c r="AA12" t="n">
         <v>1.000000000001773e-08</v>
@@ -1306,19 +1826,19 @@
       <c r="K13" t="n">
         <v>83.33122177428928</v>
       </c>
-      <c r="W13" t="n">
-        <v>12</v>
-      </c>
-      <c r="X13" t="inlineStr">
+      <c r="W13" t="inlineStr">
         <is>
           <t>y = 8.553x + -26122.057</t>
         </is>
+      </c>
+      <c r="X13" t="n">
+        <v>-26122.0567214235</v>
       </c>
       <c r="Y13" t="n">
         <v>4.014741715271358e-13</v>
       </c>
       <c r="Z13" t="n">
-        <v>3582.32258116732</v>
+        <v>513.4200000000001</v>
       </c>
       <c r="AA13" t="n">
         <v>1.000000000000027e-08</v>
@@ -1358,19 +1878,19 @@
       <c r="K14" t="n">
         <v>83.41799697640784</v>
       </c>
-      <c r="W14" t="n">
-        <v>13</v>
-      </c>
-      <c r="X14" t="inlineStr">
+      <c r="W14" t="inlineStr">
         <is>
           <t>y = 8.667x + -26249.616</t>
         </is>
+      </c>
+      <c r="X14" t="n">
+        <v>-26249.61645178953</v>
       </c>
       <c r="Y14" t="n">
         <v>1.888537158384933e-12</v>
       </c>
       <c r="Z14" t="n">
-        <v>3549.319981128023</v>
+        <v>502.8000000000002</v>
       </c>
       <c r="AA14" t="n">
         <v>1.000000000000761e-08</v>
@@ -1410,19 +1930,19 @@
       <c r="K15" t="n">
         <v>83.49762236962256</v>
       </c>
-      <c r="W15" t="n">
-        <v>14</v>
-      </c>
-      <c r="X15" t="inlineStr">
+      <c r="W15" t="inlineStr">
         <is>
           <t>y = 8.774x + -26350.972</t>
         </is>
+      </c>
+      <c r="X15" t="n">
+        <v>-26350.97202279682</v>
       </c>
       <c r="Y15" t="n">
         <v>1.326908466148628e-09</v>
       </c>
       <c r="Z15" t="n">
-        <v>3516.682615553374</v>
+        <v>497.02</v>
       </c>
       <c r="AA15" t="n">
         <v>1.000000000015281e-08</v>
@@ -1462,19 +1982,19 @@
       <c r="K16" t="n">
         <v>83.58986217207287</v>
       </c>
-      <c r="W16" t="n">
-        <v>15</v>
-      </c>
-      <c r="X16" t="inlineStr">
+      <c r="W16" t="inlineStr">
         <is>
           <t>y = 8.901x + -26514.200</t>
         </is>
+      </c>
+      <c r="X16" t="n">
+        <v>-26514.20003327129</v>
       </c>
       <c r="Y16" t="n">
         <v>2.361418140254665e-09</v>
       </c>
       <c r="Z16" t="n">
-        <v>3483.903390530033</v>
+        <v>488.79</v>
       </c>
       <c r="AA16" t="n">
         <v>1.000000000023654e-08</v>
@@ -1514,19 +2034,19 @@
       <c r="K17" t="n">
         <v>83.65675633393472</v>
       </c>
-      <c r="W17" t="n">
-        <v>16</v>
-      </c>
-      <c r="X17" t="inlineStr">
+      <c r="W17" t="inlineStr">
         <is>
           <t>y = 8.996x + -26560.827</t>
         </is>
+      </c>
+      <c r="X17" t="n">
+        <v>-26560.82693334683</v>
       </c>
       <c r="Y17" t="n">
         <v>2.435386738540102e-09</v>
       </c>
       <c r="Z17" t="n">
-        <v>3450.868737054808</v>
+        <v>484.3299999999999</v>
       </c>
       <c r="AA17" t="n">
         <v>1.000000000015642e-08</v>
@@ -1566,19 +2086,19 @@
       <c r="K18" t="n">
         <v>83.71418135828506</v>
       </c>
-      <c r="W18" t="n">
-        <v>17</v>
-      </c>
-      <c r="X18" t="inlineStr">
+      <c r="W18" t="inlineStr">
         <is>
           <t>y = 9.078x + -26574.965</t>
         </is>
+      </c>
+      <c r="X18" t="n">
+        <v>-26574.96493488604</v>
       </c>
       <c r="Y18" t="n">
         <v>2.737982188141498e-09</v>
       </c>
       <c r="Z18" t="n">
-        <v>3418.952274950283</v>
+        <v>476.6399999999999</v>
       </c>
       <c r="AA18" t="n">
         <v>1.000000000016111e-08</v>
@@ -1618,19 +2138,19 @@
       <c r="K19" t="n">
         <v>83.4745844242114</v>
       </c>
-      <c r="W19" t="n">
-        <v>18</v>
-      </c>
-      <c r="X19" t="inlineStr">
+      <c r="W19" t="inlineStr">
         <is>
           <t>y = 8.742x + -25251.260</t>
         </is>
+      </c>
+      <c r="X19" t="n">
+        <v>-25251.2601737917</v>
       </c>
       <c r="Y19" t="n">
         <v>1.084371702312922e-10</v>
       </c>
       <c r="Z19" t="n">
-        <v>3386.141736488252</v>
+        <v>486.1899999999996</v>
       </c>
       <c r="AA19" t="n">
         <v>1.000000000001499e-08</v>
@@ -1670,19 +2190,19 @@
       <c r="K20" t="n">
         <v>83.84403438060421</v>
       </c>
-      <c r="W20" t="n">
-        <v>19</v>
-      </c>
-      <c r="X20" t="inlineStr">
+      <c r="W20" t="inlineStr">
         <is>
           <t>y = 9.272x + -26666.734</t>
         </is>
+      </c>
+      <c r="X20" t="n">
+        <v>-26666.73359235622</v>
       </c>
       <c r="Y20" t="n">
         <v>2.691471049114605e-10</v>
       </c>
       <c r="Z20" t="n">
-        <v>3353.553789033743</v>
+        <v>464.6700000000001</v>
       </c>
       <c r="AA20" t="n">
         <v>1.000000000000395e-08</v>
@@ -1722,19 +2242,19 @@
       <c r="K21" t="n">
         <v>83.89368881574332</v>
       </c>
-      <c r="W21" t="n">
-        <v>20</v>
-      </c>
-      <c r="X21" t="inlineStr">
+      <c r="W21" t="inlineStr">
         <is>
           <t>y = 9.347x + -26660.418</t>
         </is>
+      </c>
+      <c r="X21" t="n">
+        <v>-26660.41809050335</v>
       </c>
       <c r="Y21" t="n">
         <v>2.87682995133163e-09</v>
       </c>
       <c r="Z21" t="n">
-        <v>3321.892580425197</v>
+        <v>461.3199999999997</v>
       </c>
       <c r="AA21" t="n">
         <v>1.000000000063688e-08</v>
@@ -1774,19 +2294,19 @@
       <c r="K22" t="n">
         <v>83.73274450889936</v>
       </c>
-      <c r="W22" t="n">
-        <v>21</v>
-      </c>
-      <c r="X22" t="inlineStr">
+      <c r="W22" t="inlineStr">
         <is>
           <t>y = 9.106x + -25628.790</t>
         </is>
+      </c>
+      <c r="X22" t="n">
+        <v>-25628.79036655436</v>
       </c>
       <c r="Y22" t="n">
         <v>1.176717711878263e-10</v>
       </c>
       <c r="Z22" t="n">
-        <v>3290.260175203482</v>
+        <v>463.2199999999998</v>
       </c>
       <c r="AA22" t="n">
         <v>1.000000000002077e-08</v>
@@ -1806,7 +2326,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB1"/>
+  <dimension ref="A1:AB22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1912,12 +2432,12 @@
       </c>
       <c r="W1" t="inlineStr">
         <is>
-          <t>Cycle</t>
+          <t>Model</t>
         </is>
       </c>
       <c r="X1" t="inlineStr">
         <is>
-          <t>Model</t>
+          <t>b</t>
         </is>
       </c>
       <c r="Y1" t="inlineStr">
@@ -1927,7 +2447,7 @@
       </c>
       <c r="Z1" t="inlineStr">
         <is>
-          <t>Rp</t>
+          <t>delta Rct-i</t>
         </is>
       </c>
       <c r="AA1" t="inlineStr">
@@ -1939,6 +2459,1098 @@
         <is>
           <t>n</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1.428571428571429</v>
+      </c>
+      <c r="B2" t="n">
+        <v>-621.8600000000006</v>
+      </c>
+      <c r="D2" t="n">
+        <v>1.87206e-07</v>
+      </c>
+      <c r="E2" t="n">
+        <v>-49.827</v>
+      </c>
+      <c r="F2" t="n">
+        <v/>
+      </c>
+      <c r="G2" t="n">
+        <v/>
+      </c>
+      <c r="H2" t="n">
+        <v/>
+      </c>
+      <c r="I2" t="n">
+        <v/>
+      </c>
+      <c r="J2" t="n">
+        <v>8.971279781828869</v>
+      </c>
+      <c r="K2" t="n">
+        <v>81.72770232173299</v>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>y = 6.878x + -24495.060</t>
+        </is>
+      </c>
+      <c r="X2" t="n">
+        <v>-24495.06033497604</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>9.372481880738808e-09</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>621.8600000000006</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>1.000000000000242e-08</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>0.8215088365301008</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2.857142857142857</v>
+      </c>
+      <c r="B3" t="n">
+        <v>-541.2000000000003</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1.97114e-07</v>
+      </c>
+      <c r="E3" t="n">
+        <v>-51.566</v>
+      </c>
+      <c r="F3" t="n">
+        <v/>
+      </c>
+      <c r="G3" t="n">
+        <v/>
+      </c>
+      <c r="H3" t="n">
+        <v/>
+      </c>
+      <c r="I3" t="n">
+        <v/>
+      </c>
+      <c r="J3" t="n">
+        <v>10.48545068401926</v>
+      </c>
+      <c r="K3" t="n">
+        <v>82.69512048064934</v>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>y = 7.801x + -26459.890</t>
+        </is>
+      </c>
+      <c r="X3" t="n">
+        <v>-26459.89008797356</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>1.008242152951607e-09</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>541.2000000000003</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>1e-08</v>
+      </c>
+      <c r="AB3" t="n">
+        <v>0.8216535762943605</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>4.285714285714286</v>
+      </c>
+      <c r="B4" t="n">
+        <v>-523.04</v>
+      </c>
+      <c r="D4" t="n">
+        <v>2.00293e-07</v>
+      </c>
+      <c r="E4" t="n">
+        <v>-52.188</v>
+      </c>
+      <c r="F4" t="n">
+        <v/>
+      </c>
+      <c r="G4" t="n">
+        <v/>
+      </c>
+      <c r="H4" t="n">
+        <v/>
+      </c>
+      <c r="I4" t="n">
+        <v/>
+      </c>
+      <c r="J4" t="n">
+        <v>11.00178176254374</v>
+      </c>
+      <c r="K4" t="n">
+        <v>82.94486466278292</v>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>y = 8.080x + -26910.568</t>
+        </is>
+      </c>
+      <c r="X4" t="n">
+        <v>-26910.56761976944</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>1.569572573701757e-10</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>523.04</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>1.000000000000016e-08</v>
+      </c>
+      <c r="AB4" t="n">
+        <v>0.821813012113298</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>5.714285714285714</v>
+      </c>
+      <c r="B5" t="n">
+        <v>-488.54</v>
+      </c>
+      <c r="D5" t="n">
+        <v>2.02227e-07</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-52.642</v>
+      </c>
+      <c r="F5" t="n">
+        <v/>
+      </c>
+      <c r="G5" t="n">
+        <v/>
+      </c>
+      <c r="H5" t="n">
+        <v/>
+      </c>
+      <c r="I5" t="n">
+        <v/>
+      </c>
+      <c r="J5" t="n">
+        <v>12.93401924215682</v>
+      </c>
+      <c r="K5" t="n">
+        <v>83.53065245071322</v>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>y = 8.819x + -29195.631</t>
+        </is>
+      </c>
+      <c r="X5" t="n">
+        <v>-29195.63144525173</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>5.336967142759836e-10</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>488.54</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>1.000000000000285e-08</v>
+      </c>
+      <c r="AB5" t="n">
+        <v>0.8219961851990103</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>7.142857142857143</v>
+      </c>
+      <c r="B6" t="n">
+        <v>-501.6999999999998</v>
+      </c>
+      <c r="D6" t="n">
+        <v>2.03998e-07</v>
+      </c>
+      <c r="E6" t="n">
+        <v>-52.988</v>
+      </c>
+      <c r="F6" t="n">
+        <v/>
+      </c>
+      <c r="G6" t="n">
+        <v/>
+      </c>
+      <c r="H6" t="n">
+        <v/>
+      </c>
+      <c r="I6" t="n">
+        <v/>
+      </c>
+      <c r="J6" t="n">
+        <v>11.47089912342078</v>
+      </c>
+      <c r="K6" t="n">
+        <v>83.24190023170245</v>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>y = 8.439x + -27475.483</t>
+        </is>
+      </c>
+      <c r="X6" t="n">
+        <v>-27475.48268528328</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>5.254567269568468e-09</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>501.6999999999998</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>1.000000000000448e-08</v>
+      </c>
+      <c r="AB6" t="n">
+        <v>0.8222059667745614</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>8.571428571428571</v>
+      </c>
+      <c r="B7" t="n">
+        <v>-471.4399999999996</v>
+      </c>
+      <c r="D7" t="n">
+        <v>2.05772e-07</v>
+      </c>
+      <c r="E7" t="n">
+        <v>-53.367</v>
+      </c>
+      <c r="F7" t="n">
+        <v/>
+      </c>
+      <c r="G7" t="n">
+        <v/>
+      </c>
+      <c r="H7" t="n">
+        <v/>
+      </c>
+      <c r="I7" t="n">
+        <v/>
+      </c>
+      <c r="J7" t="n">
+        <v>13.65657237747221</v>
+      </c>
+      <c r="K7" t="n">
+        <v>83.74787270538825</v>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>y = 9.128x + -29552.577</t>
+        </is>
+      </c>
+      <c r="X7" t="n">
+        <v>-29552.57746903169</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>5.172261010524144e-18</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>471.4399999999996</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>1e-08</v>
+      </c>
+      <c r="AB7" t="n">
+        <v>0.8223993915203321</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>10</v>
+      </c>
+      <c r="B8" t="n">
+        <v>-498.8800000000001</v>
+      </c>
+      <c r="D8" t="n">
+        <v>2.07111e-07</v>
+      </c>
+      <c r="E8" t="n">
+        <v>-53.677</v>
+      </c>
+      <c r="F8" t="n">
+        <v/>
+      </c>
+      <c r="G8" t="n">
+        <v/>
+      </c>
+      <c r="H8" t="n">
+        <v/>
+      </c>
+      <c r="I8" t="n">
+        <v/>
+      </c>
+      <c r="J8" t="n">
+        <v>10.81835284157761</v>
+      </c>
+      <c r="K8" t="n">
+        <v>83.0780307273682</v>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>y = 8.237x + -26156.503</t>
+        </is>
+      </c>
+      <c r="X8" t="n">
+        <v>-26156.50274033273</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>1.199142879722051e-08</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>498.8800000000001</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>1.000000000000031e-08</v>
+      </c>
+      <c r="AB8" t="n">
+        <v>0.8224917489242677</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>11.42857142857143</v>
+      </c>
+      <c r="B9" t="n">
+        <v>-472.9899999999998</v>
+      </c>
+      <c r="D9" t="n">
+        <v>2.08269e-07</v>
+      </c>
+      <c r="E9" t="n">
+        <v>-53.972</v>
+      </c>
+      <c r="F9" t="n">
+        <v/>
+      </c>
+      <c r="G9" t="n">
+        <v/>
+      </c>
+      <c r="H9" t="n">
+        <v/>
+      </c>
+      <c r="I9" t="n">
+        <v/>
+      </c>
+      <c r="J9" t="n">
+        <v>12.1932321892061</v>
+      </c>
+      <c r="K9" t="n">
+        <v>83.57504379592744</v>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>y = 8.880x + -28122.514</t>
+        </is>
+      </c>
+      <c r="X9" t="n">
+        <v>-28122.51402882813</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>1.637636171640223e-10</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>472.9899999999998</v>
+      </c>
+      <c r="AA9" t="n">
+        <v>1.000000000000328e-08</v>
+      </c>
+      <c r="AB9" t="n">
+        <v>0.8226360180207569</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>12.85714285714286</v>
+      </c>
+      <c r="B10" t="n">
+        <v>-469.02</v>
+      </c>
+      <c r="D10" t="n">
+        <v>2.09535e-07</v>
+      </c>
+      <c r="E10" t="n">
+        <v>-54.226</v>
+      </c>
+      <c r="F10" t="n">
+        <v/>
+      </c>
+      <c r="G10" t="n">
+        <v/>
+      </c>
+      <c r="H10" t="n">
+        <v/>
+      </c>
+      <c r="I10" t="n">
+        <v/>
+      </c>
+      <c r="J10" t="n">
+        <v>12.40674030947839</v>
+      </c>
+      <c r="K10" t="n">
+        <v>83.62302121797003</v>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>y = 8.948x + -28110.581</t>
+        </is>
+      </c>
+      <c r="X10" t="n">
+        <v>-28110.58107177476</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>3.136585321634133e-10</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>469.02</v>
+      </c>
+      <c r="AA10" t="n">
+        <v>1.000000000002126e-08</v>
+      </c>
+      <c r="AB10" t="n">
+        <v>0.8228078231698415</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>14.28571428571429</v>
+      </c>
+      <c r="B11" t="n">
+        <v>-476.0100000000002</v>
+      </c>
+      <c r="D11" t="n">
+        <v>2.10802e-07</v>
+      </c>
+      <c r="E11" t="n">
+        <v>-54.511</v>
+      </c>
+      <c r="F11" t="n">
+        <v/>
+      </c>
+      <c r="G11" t="n">
+        <v/>
+      </c>
+      <c r="H11" t="n">
+        <v/>
+      </c>
+      <c r="I11" t="n">
+        <v/>
+      </c>
+      <c r="J11" t="n">
+        <v>11.38292210211237</v>
+      </c>
+      <c r="K11" t="n">
+        <v>83.38207143142075</v>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>y = 8.619x + -26730.662</t>
+        </is>
+      </c>
+      <c r="X11" t="n">
+        <v>-26730.66167624396</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>5.822225911921077e-10</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>476.0100000000002</v>
+      </c>
+      <c r="AA11" t="n">
+        <v>1.000000000000367e-08</v>
+      </c>
+      <c r="AB11" t="n">
+        <v>0.8230241303461643</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>15.71428571428572</v>
+      </c>
+      <c r="B12" t="n">
+        <v>-458.4400000000001</v>
+      </c>
+      <c r="D12" t="n">
+        <v>2.11994e-07</v>
+      </c>
+      <c r="E12" t="n">
+        <v>-54.782</v>
+      </c>
+      <c r="F12" t="n">
+        <v/>
+      </c>
+      <c r="G12" t="n">
+        <v/>
+      </c>
+      <c r="H12" t="n">
+        <v/>
+      </c>
+      <c r="I12" t="n">
+        <v/>
+      </c>
+      <c r="J12" t="n">
+        <v>12.88592392067534</v>
+      </c>
+      <c r="K12" t="n">
+        <v>83.76091421806797</v>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>y = 9.147x + -28254.609</t>
+        </is>
+      </c>
+      <c r="X12" t="n">
+        <v>-28254.60890465227</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>2.341753663240482e-10</v>
+      </c>
+      <c r="Z12" t="n">
+        <v>458.4400000000001</v>
+      </c>
+      <c r="AA12" t="n">
+        <v>1.000000000000736e-08</v>
+      </c>
+      <c r="AB12" t="n">
+        <v>0.8232926077894073</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>17.14285714285714</v>
+      </c>
+      <c r="B13" t="n">
+        <v>-463.9000000000001</v>
+      </c>
+      <c r="D13" t="n">
+        <v>2.13431e-07</v>
+      </c>
+      <c r="E13" t="n">
+        <v>-55.077</v>
+      </c>
+      <c r="F13" t="n">
+        <v/>
+      </c>
+      <c r="G13" t="n">
+        <v/>
+      </c>
+      <c r="H13" t="n">
+        <v/>
+      </c>
+      <c r="I13" t="n">
+        <v/>
+      </c>
+      <c r="J13" t="n">
+        <v>11.74876553682504</v>
+      </c>
+      <c r="K13" t="n">
+        <v>83.53051278117373</v>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>y = 8.819x + -26870.432</t>
+        </is>
+      </c>
+      <c r="X13" t="n">
+        <v>-26870.43207501114</v>
+      </c>
+      <c r="Y13" t="n">
+        <v>9.977220009734805e-09</v>
+      </c>
+      <c r="Z13" t="n">
+        <v>463.9000000000001</v>
+      </c>
+      <c r="AA13" t="n">
+        <v>1.000000000006445e-08</v>
+      </c>
+      <c r="AB13" t="n">
+        <v>0.8235980887516039</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>18.57142857142857</v>
+      </c>
+      <c r="B14" t="n">
+        <v>-438.6100000000001</v>
+      </c>
+      <c r="D14" t="n">
+        <v>2.14758e-07</v>
+      </c>
+      <c r="E14" t="n">
+        <v>-55.381</v>
+      </c>
+      <c r="F14" t="n">
+        <v/>
+      </c>
+      <c r="G14" t="n">
+        <v/>
+      </c>
+      <c r="H14" t="n">
+        <v/>
+      </c>
+      <c r="I14" t="n">
+        <v/>
+      </c>
+      <c r="J14" t="n">
+        <v>13.43942880447634</v>
+      </c>
+      <c r="K14" t="n">
+        <v>83.99752230931105</v>
+      </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>y = 9.510x + -28865.086</t>
+        </is>
+      </c>
+      <c r="X14" t="n">
+        <v>-28865.08604200661</v>
+      </c>
+      <c r="Y14" t="n">
+        <v>1.846181921349008e-10</v>
+      </c>
+      <c r="Z14" t="n">
+        <v>438.6100000000001</v>
+      </c>
+      <c r="AA14" t="n">
+        <v>1.000000000002417e-08</v>
+      </c>
+      <c r="AB14" t="n">
+        <v>0.8239263039008332</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>20</v>
+      </c>
+      <c r="B15" t="n">
+        <v>-434.0499999999997</v>
+      </c>
+      <c r="D15" t="n">
+        <v>2.15967e-07</v>
+      </c>
+      <c r="E15" t="n">
+        <v>-55.647</v>
+      </c>
+      <c r="F15" t="n">
+        <v/>
+      </c>
+      <c r="G15" t="n">
+        <v/>
+      </c>
+      <c r="H15" t="n">
+        <v/>
+      </c>
+      <c r="I15" t="n">
+        <v/>
+      </c>
+      <c r="J15" t="n">
+        <v>13.58324764400449</v>
+      </c>
+      <c r="K15" t="n">
+        <v>84.07801630969796</v>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>y = 9.641x + -28999.210</t>
+        </is>
+      </c>
+      <c r="X15" t="n">
+        <v>-28999.21012447367</v>
+      </c>
+      <c r="Y15" t="n">
+        <v>7.274745846453659e-17</v>
+      </c>
+      <c r="Z15" t="n">
+        <v>434.0499999999997</v>
+      </c>
+      <c r="AA15" t="n">
+        <v>1e-08</v>
+      </c>
+      <c r="AB15" t="n">
+        <v>0.8242877132069509</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>21.42857142857143</v>
+      </c>
+      <c r="B16" t="n">
+        <v>-409.9300000000003</v>
+      </c>
+      <c r="D16" t="n">
+        <v>2.17439e-07</v>
+      </c>
+      <c r="E16" t="n">
+        <v>-55.948</v>
+      </c>
+      <c r="F16" t="n">
+        <v/>
+      </c>
+      <c r="G16" t="n">
+        <v/>
+      </c>
+      <c r="H16" t="n">
+        <v/>
+      </c>
+      <c r="I16" t="n">
+        <v/>
+      </c>
+      <c r="J16" t="n">
+        <v>16.26868729934995</v>
+      </c>
+      <c r="K16" t="n">
+        <v>84.53943587335078</v>
+      </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>y = 10.461x + -31332.519</t>
+        </is>
+      </c>
+      <c r="X16" t="n">
+        <v>-31332.51856013672</v>
+      </c>
+      <c r="Y16" t="n">
+        <v>6.987080395847131e-11</v>
+      </c>
+      <c r="Z16" t="n">
+        <v>409.9300000000003</v>
+      </c>
+      <c r="AA16" t="n">
+        <v>1.000000000000087e-08</v>
+      </c>
+      <c r="AB16" t="n">
+        <v>0.8246312406385589</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>22.85714285714286</v>
+      </c>
+      <c r="B17" t="n">
+        <v>-435.7400000000002</v>
+      </c>
+      <c r="D17" t="n">
+        <v>2.18927e-07</v>
+      </c>
+      <c r="E17" t="n">
+        <v>-56.241</v>
+      </c>
+      <c r="F17" t="n">
+        <v/>
+      </c>
+      <c r="G17" t="n">
+        <v/>
+      </c>
+      <c r="H17" t="n">
+        <v/>
+      </c>
+      <c r="I17" t="n">
+        <v/>
+      </c>
+      <c r="J17" t="n">
+        <v>12.60844112304573</v>
+      </c>
+      <c r="K17" t="n">
+        <v>83.90205459380411</v>
+      </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>y = 9.360x + -27488.920</t>
+        </is>
+      </c>
+      <c r="X17" t="n">
+        <v>-27488.91959558622</v>
+      </c>
+      <c r="Y17" t="n">
+        <v>3.287138289903484e-11</v>
+      </c>
+      <c r="Z17" t="n">
+        <v>435.7400000000002</v>
+      </c>
+      <c r="AA17" t="n">
+        <v>1.000000000001291e-08</v>
+      </c>
+      <c r="AB17" t="n">
+        <v>0.8249915339153899</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>24.28571428571428</v>
+      </c>
+      <c r="B18" t="n">
+        <v>-415.1600000000003</v>
+      </c>
+      <c r="D18" t="n">
+        <v>2.20174e-07</v>
+      </c>
+      <c r="E18" t="n">
+        <v>-56.525</v>
+      </c>
+      <c r="F18" t="n">
+        <v/>
+      </c>
+      <c r="G18" t="n">
+        <v/>
+      </c>
+      <c r="H18" t="n">
+        <v/>
+      </c>
+      <c r="I18" t="n">
+        <v/>
+      </c>
+      <c r="J18" t="n">
+        <v>14.41395902063149</v>
+      </c>
+      <c r="K18" t="n">
+        <v>84.29987466413274</v>
+      </c>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>y = 10.018x + -29291.809</t>
+        </is>
+      </c>
+      <c r="X18" t="n">
+        <v>-29291.80914406236</v>
+      </c>
+      <c r="Y18" t="n">
+        <v>2.418275026610593e-10</v>
+      </c>
+      <c r="Z18" t="n">
+        <v>415.1600000000003</v>
+      </c>
+      <c r="AA18" t="n">
+        <v>1.00000000000023e-08</v>
+      </c>
+      <c r="AB18" t="n">
+        <v>0.8253601593971416</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>25.71428571428572</v>
+      </c>
+      <c r="B19" t="n">
+        <v>-414.77</v>
+      </c>
+      <c r="D19" t="n">
+        <v>2.21328e-07</v>
+      </c>
+      <c r="E19" t="n">
+        <v>-56.726</v>
+      </c>
+      <c r="F19" t="n">
+        <v/>
+      </c>
+      <c r="G19" t="n">
+        <v/>
+      </c>
+      <c r="H19" t="n">
+        <v/>
+      </c>
+      <c r="I19" t="n">
+        <v/>
+      </c>
+      <c r="J19" t="n">
+        <v>14.4982036260707</v>
+      </c>
+      <c r="K19" t="n">
+        <v>84.32844899281338</v>
+      </c>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>y = 10.069x + -29172.394</t>
+        </is>
+      </c>
+      <c r="X19" t="n">
+        <v>-29172.39393842236</v>
+      </c>
+      <c r="Y19" t="n">
+        <v>2.771806947516841e-10</v>
+      </c>
+      <c r="Z19" t="n">
+        <v>414.77</v>
+      </c>
+      <c r="AA19" t="n">
+        <v>1.000000000000171e-08</v>
+      </c>
+      <c r="AB19" t="n">
+        <v>0.8257193254943649</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>27.14285714285714</v>
+      </c>
+      <c r="B20" t="n">
+        <v>-403.4700000000003</v>
+      </c>
+      <c r="D20" t="n">
+        <v>2.22747e-07</v>
+      </c>
+      <c r="E20" t="n">
+        <v>-57.082</v>
+      </c>
+      <c r="F20" t="n">
+        <v/>
+      </c>
+      <c r="G20" t="n">
+        <v/>
+      </c>
+      <c r="H20" t="n">
+        <v/>
+      </c>
+      <c r="I20" t="n">
+        <v/>
+      </c>
+      <c r="J20" t="n">
+        <v>14.89435706182895</v>
+      </c>
+      <c r="K20" t="n">
+        <v>84.4302627780539</v>
+      </c>
+      <c r="W20" t="inlineStr">
+        <is>
+          <t>y = 10.255x + -29428.389</t>
+        </is>
+      </c>
+      <c r="X20" t="n">
+        <v>-29428.38938475875</v>
+      </c>
+      <c r="Y20" t="n">
+        <v>2.072852205262699e-10</v>
+      </c>
+      <c r="Z20" t="n">
+        <v>403.4700000000003</v>
+      </c>
+      <c r="AA20" t="n">
+        <v>1.000000000000288e-08</v>
+      </c>
+      <c r="AB20" t="n">
+        <v>0.8260818835119356</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>28.57142857142857</v>
+      </c>
+      <c r="B21" t="n">
+        <v>-397.8999999999996</v>
+      </c>
+      <c r="D21" t="n">
+        <v>2.24003e-07</v>
+      </c>
+      <c r="E21" t="n">
+        <v>-57.337</v>
+      </c>
+      <c r="F21" t="n">
+        <v/>
+      </c>
+      <c r="G21" t="n">
+        <v/>
+      </c>
+      <c r="H21" t="n">
+        <v/>
+      </c>
+      <c r="I21" t="n">
+        <v/>
+      </c>
+      <c r="J21" t="n">
+        <v>15.0791072111039</v>
+      </c>
+      <c r="K21" t="n">
+        <v>84.50920830985854</v>
+      </c>
+      <c r="W21" t="inlineStr">
+        <is>
+          <t>y = 10.403x + -29591.879</t>
+        </is>
+      </c>
+      <c r="X21" t="n">
+        <v>-29591.87863106111</v>
+      </c>
+      <c r="Y21" t="n">
+        <v>2.092233388533273e-10</v>
+      </c>
+      <c r="Z21" t="n">
+        <v>397.8999999999996</v>
+      </c>
+      <c r="AA21" t="n">
+        <v>1.000000000000298e-08</v>
+      </c>
+      <c r="AB21" t="n">
+        <v>0.8264371626841915</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>30</v>
+      </c>
+      <c r="B22" t="n">
+        <v>-399.04</v>
+      </c>
+      <c r="D22" t="n">
+        <v>2.24989e-07</v>
+      </c>
+      <c r="E22" t="n">
+        <v>-57.543</v>
+      </c>
+      <c r="F22" t="n">
+        <v/>
+      </c>
+      <c r="G22" t="n">
+        <v/>
+      </c>
+      <c r="H22" t="n">
+        <v/>
+      </c>
+      <c r="I22" t="n">
+        <v/>
+      </c>
+      <c r="J22" t="n">
+        <v>14.96843484024677</v>
+      </c>
+      <c r="K22" t="n">
+        <v>84.50080576692156</v>
+      </c>
+      <c r="W22" t="inlineStr">
+        <is>
+          <t>y = 10.387x + -29268.610</t>
+        </is>
+      </c>
+      <c r="X22" t="n">
+        <v>-29268.61044251429</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>3.390292703957733e-10</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>399.04</v>
+      </c>
+      <c r="AA22" t="n">
+        <v>1.00000000000001e-08</v>
+      </c>
+      <c r="AB22" t="n">
+        <v>0.8267985441944087</v>
       </c>
     </row>
   </sheetData>
@@ -2058,12 +3670,12 @@
       </c>
       <c r="W1" t="inlineStr">
         <is>
-          <t>Cycle</t>
+          <t>Model</t>
         </is>
       </c>
       <c r="X1" t="inlineStr">
         <is>
-          <t>Model</t>
+          <t>b</t>
         </is>
       </c>
       <c r="Y1" t="inlineStr">
@@ -2073,7 +3685,7 @@
       </c>
       <c r="Z1" t="inlineStr">
         <is>
-          <t>Rp</t>
+          <t>delta Rct-i</t>
         </is>
       </c>
       <c r="AA1" t="inlineStr">
@@ -2118,19 +3730,19 @@
       <c r="K2" t="n">
         <v>55.50366380056415</v>
       </c>
-      <c r="W2" t="n">
-        <v>1</v>
-      </c>
-      <c r="X2" t="inlineStr">
+      <c r="W2" t="inlineStr">
         <is>
           <t>y = 1.455x + -43677.779</t>
         </is>
+      </c>
+      <c r="X2" t="n">
+        <v>-43677.778780635</v>
       </c>
       <c r="Y2" t="n">
         <v>2883.489211920488</v>
       </c>
       <c r="Z2" t="n">
-        <v>2080.703758691029</v>
+        <v>2982.699999999997</v>
       </c>
       <c r="AA2" t="n">
         <v>2.191155442269083e-06</v>
@@ -2170,19 +3782,19 @@
       <c r="K3" t="n">
         <v>60.779374732112</v>
       </c>
-      <c r="W3" t="n">
-        <v>2</v>
-      </c>
-      <c r="X3" t="inlineStr">
+      <c r="W3" t="inlineStr">
         <is>
           <t>y = 1.788x + -46447.827</t>
         </is>
+      </c>
+      <c r="X3" t="n">
+        <v>-46447.82712472187</v>
       </c>
       <c r="Y3" t="n">
         <v>1950.814450412289</v>
       </c>
       <c r="Z3" t="n">
-        <v>1764.10020359153</v>
+        <v>2560.099999999999</v>
       </c>
       <c r="AA3" t="n">
         <v>1.764139868533671e-06</v>
@@ -2222,19 +3834,19 @@
       <c r="K4" t="n">
         <v>62.09075804055832</v>
       </c>
-      <c r="W4" t="n">
-        <v>3</v>
-      </c>
-      <c r="X4" t="inlineStr">
+      <c r="W4" t="inlineStr">
         <is>
           <t>y = 1.888x + -47352.154</t>
         </is>
+      </c>
+      <c r="X4" t="n">
+        <v>-47352.15425404939</v>
       </c>
       <c r="Y4" t="n">
         <v>2015.383294903022</v>
       </c>
       <c r="Z4" t="n">
-        <v>1825.196364559226</v>
+        <v>2463.299999999999</v>
       </c>
       <c r="AA4" t="n">
         <v>1.414664423208874e-06</v>
@@ -2274,19 +3886,19 @@
       <c r="K5" t="n">
         <v>62.82142842637428</v>
       </c>
-      <c r="W5" t="n">
-        <v>4</v>
-      </c>
-      <c r="X5" t="inlineStr">
+      <c r="W5" t="inlineStr">
         <is>
           <t>y = 1.948x + -48044.553</t>
         </is>
+      </c>
+      <c r="X5" t="n">
+        <v>-48044.55278719714</v>
       </c>
       <c r="Y5" t="n">
         <v>2019.360931709148</v>
       </c>
       <c r="Z5" t="n">
-        <v>1829.841161391234</v>
+        <v>2418.199999999997</v>
       </c>
       <c r="AA5" t="n">
         <v>1.405679274327418e-06</v>
@@ -2326,19 +3938,19 @@
       <c r="K6" t="n">
         <v>63.26015544520055</v>
       </c>
-      <c r="W6" t="n">
-        <v>5</v>
-      </c>
-      <c r="X6" t="inlineStr">
+      <c r="W6" t="inlineStr">
         <is>
           <t>y = 1.985x + -48301.493</t>
         </is>
+      </c>
+      <c r="X6" t="n">
+        <v>-48301.49317769516</v>
       </c>
       <c r="Y6" t="n">
         <v>2013.376304596488</v>
       </c>
       <c r="Z6" t="n">
-        <v>1825.085703212622</v>
+        <v>2392.299999999999</v>
       </c>
       <c r="AA6" t="n">
         <v>1.661507495215767e-06</v>
@@ -2378,19 +3990,19 @@
       <c r="K7" t="n">
         <v>63.66654811532521</v>
       </c>
-      <c r="W7" t="n">
-        <v>6</v>
-      </c>
-      <c r="X7" t="inlineStr">
+      <c r="W7" t="inlineStr">
         <is>
           <t>y = 2.020x + -48536.451</t>
         </is>
+      </c>
+      <c r="X7" t="n">
+        <v>-48536.4509105106</v>
       </c>
       <c r="Y7" t="n">
         <v>2010.272054506718</v>
       </c>
       <c r="Z7" t="n">
-        <v>1822.911231973246</v>
+        <v>2369</v>
       </c>
       <c r="AA7" t="n">
         <v>1.654722408470943e-06</v>
@@ -2430,19 +4042,19 @@
       <c r="K8" t="n">
         <v>63.99325261592055</v>
       </c>
-      <c r="W8" t="n">
-        <v>7</v>
-      </c>
-      <c r="X8" t="inlineStr">
+      <c r="W8" t="inlineStr">
         <is>
           <t>y = 2.050x + -48625.749</t>
         </is>
+      </c>
+      <c r="X8" t="n">
+        <v>-48625.74946949843</v>
       </c>
       <c r="Y8" t="n">
         <v>2006.865871564456</v>
       </c>
       <c r="Z8" t="n">
-        <v>1820.427341985811</v>
+        <v>2363.799999999999</v>
       </c>
       <c r="AA8" t="n">
         <v>1.652679632918364e-06</v>
@@ -2482,19 +4094,19 @@
       <c r="K9" t="n">
         <v>64.23105464881762</v>
       </c>
-      <c r="W9" t="n">
-        <v>8</v>
-      </c>
-      <c r="X9" t="inlineStr">
+      <c r="W9" t="inlineStr">
         <is>
           <t>y = 2.071x + -48529.138</t>
         </is>
+      </c>
+      <c r="X9" t="n">
+        <v>-48529.13810753277</v>
       </c>
       <c r="Y9" t="n">
         <v>2048.121562254793</v>
       </c>
       <c r="Z9" t="n">
-        <v>1859.966738194793</v>
+        <v>2347.199999999997</v>
       </c>
       <c r="AA9" t="n">
         <v>1.610289555534342e-06</v>
@@ -2534,19 +4146,19 @@
       <c r="K10" t="n">
         <v>64.48284246075836</v>
       </c>
-      <c r="W10" t="n">
-        <v>9</v>
-      </c>
-      <c r="X10" t="inlineStr">
+      <c r="W10" t="inlineStr">
         <is>
           <t>y = 2.095x + -48484.064</t>
         </is>
+      </c>
+      <c r="X10" t="n">
+        <v>-48484.0635360629</v>
       </c>
       <c r="Y10" t="n">
         <v>2056.781931524606</v>
       </c>
       <c r="Z10" t="n">
-        <v>1868.963630238603</v>
+        <v>2334.799999999999</v>
       </c>
       <c r="AA10" t="n">
         <v>1.596751668275329e-06</v>
@@ -2586,19 +4198,19 @@
       <c r="K11" t="n">
         <v>64.66816861197613</v>
       </c>
-      <c r="W11" t="n">
-        <v>10</v>
-      </c>
-      <c r="X11" t="inlineStr">
+      <c r="W11" t="inlineStr">
         <is>
           <t>y = 2.112x + -48283.050</t>
         </is>
+      </c>
+      <c r="X11" t="n">
+        <v>-48283.0499287217</v>
       </c>
       <c r="Y11" t="n">
         <v>2014.642061059314</v>
       </c>
       <c r="Z11" t="n">
-        <v>1829.866113799269</v>
+        <v>2328.900000000001</v>
       </c>
       <c r="AA11" t="n">
         <v>1.626963053200119e-06</v>
@@ -2724,12 +4336,12 @@
       </c>
       <c r="W1" t="inlineStr">
         <is>
-          <t>Cycle</t>
+          <t>Model</t>
         </is>
       </c>
       <c r="X1" t="inlineStr">
         <is>
-          <t>Model</t>
+          <t>b</t>
         </is>
       </c>
       <c r="Y1" t="inlineStr">
@@ -2739,7 +4351,7 @@
       </c>
       <c r="Z1" t="inlineStr">
         <is>
-          <t>Rp</t>
+          <t>delta Rct-i</t>
         </is>
       </c>
       <c r="AA1" t="inlineStr">
@@ -2784,19 +4396,19 @@
       <c r="K2" t="n">
         <v>81.58370115852892</v>
       </c>
-      <c r="W2" t="n">
-        <v>1</v>
-      </c>
-      <c r="X2" t="inlineStr">
+      <c r="W2" t="inlineStr">
         <is>
           <t>y = 6.759x + -24183.133</t>
         </is>
+      </c>
+      <c r="X2" t="n">
+        <v>-24183.13325951939</v>
       </c>
       <c r="Y2" t="n">
         <v>8.18558636998039e-09</v>
       </c>
       <c r="Z2" t="n">
-        <v>4197.135296207487</v>
+        <v>643.6899999999996</v>
       </c>
       <c r="AA2" t="n">
         <v>1.000000000003627e-08</v>
@@ -2836,19 +4448,19 @@
       <c r="K3" t="n">
         <v>82.35250125129245</v>
       </c>
-      <c r="W3" t="n">
-        <v>2</v>
-      </c>
-      <c r="X3" t="inlineStr">
+      <c r="W3" t="inlineStr">
         <is>
           <t>y = 7.448x + -25132.257</t>
         </is>
+      </c>
+      <c r="X3" t="n">
+        <v>-25132.25704839991</v>
       </c>
       <c r="Y3" t="n">
         <v>2.855706839303508e-09</v>
       </c>
       <c r="Z3" t="n">
-        <v>3982.710374021114</v>
+        <v>562.5099999999998</v>
       </c>
       <c r="AA3" t="n">
         <v>1.000000000000005e-08</v>
@@ -2888,19 +4500,19 @@
       <c r="K4" t="n">
         <v>82.71503741314046</v>
       </c>
-      <c r="W4" t="n">
-        <v>3</v>
-      </c>
-      <c r="X4" t="inlineStr">
+      <c r="W4" t="inlineStr">
         <is>
           <t>y = 7.823x + -25921.327</t>
         </is>
+      </c>
+      <c r="X4" t="n">
+        <v>-25921.32667909566</v>
       </c>
       <c r="Y4" t="n">
         <v>1.061910452679619e-11</v>
       </c>
       <c r="Z4" t="n">
-        <v>3908.154320430063</v>
+        <v>531.9699999999998</v>
       </c>
       <c r="AA4" t="n">
         <v>1e-08</v>
@@ -2940,19 +4552,19 @@
       <c r="K5" t="n">
         <v>83.35054759925181</v>
       </c>
-      <c r="W5" t="n">
-        <v>4</v>
-      </c>
-      <c r="X5" t="inlineStr">
+      <c r="W5" t="inlineStr">
         <is>
           <t>y = 8.578x + -28240.688</t>
         </is>
+      </c>
+      <c r="X5" t="n">
+        <v>-28240.68808179591</v>
       </c>
       <c r="Y5" t="n">
         <v>2.392805453571923e-09</v>
       </c>
       <c r="Z5" t="n">
-        <v>3856.895157992336</v>
+        <v>495.4700000000003</v>
       </c>
       <c r="AA5" t="n">
         <v>1.000000000000218e-08</v>
@@ -2992,19 +4604,19 @@
       <c r="K6" t="n">
         <v>83.09810507894832</v>
       </c>
-      <c r="W6" t="n">
-        <v>5</v>
-      </c>
-      <c r="X6" t="inlineStr">
+      <c r="W6" t="inlineStr">
         <is>
           <t>y = 8.261x + -26753.213</t>
         </is>
+      </c>
+      <c r="X6" t="n">
+        <v>-26753.21345103956</v>
       </c>
       <c r="Y6" t="n">
         <v>9.456756740009373e-11</v>
       </c>
       <c r="Z6" t="n">
-        <v>3811.837128442961</v>
+        <v>502.3099999999999</v>
       </c>
       <c r="AA6" t="n">
         <v>1.000000000000069e-08</v>
@@ -3044,19 +4656,19 @@
       <c r="K7" t="n">
         <v>83.68321242761351</v>
       </c>
-      <c r="W7" t="n">
-        <v>6</v>
-      </c>
-      <c r="X7" t="inlineStr">
+      <c r="W7" t="inlineStr">
         <is>
           <t>y = 9.034x + -29115.473</t>
         </is>
+      </c>
+      <c r="X7" t="n">
+        <v>-29115.47264585606</v>
       </c>
       <c r="Y7" t="n">
         <v>125.0389400380478</v>
       </c>
       <c r="Z7" t="n">
-        <v>4016.786618265003</v>
+        <v>468.73</v>
       </c>
       <c r="AA7" t="n">
         <v>1.911798595083981e-08</v>
@@ -3096,19 +4708,19 @@
       <c r="K8" t="n">
         <v>83.61406326098518</v>
       </c>
-      <c r="W8" t="n">
-        <v>7</v>
-      </c>
-      <c r="X8" t="inlineStr">
+      <c r="W8" t="inlineStr">
         <is>
           <t>y = 8.935x + -28394.391</t>
         </is>
+      </c>
+      <c r="X8" t="n">
+        <v>-28394.39105021164</v>
       </c>
       <c r="Y8" t="n">
         <v>2.063089794802132e-08</v>
       </c>
       <c r="Z8" t="n">
-        <v>3730.626176126394</v>
+        <v>449.2600000000002</v>
       </c>
       <c r="AA8" t="n">
         <v>1.000000000000704e-08</v>
@@ -3148,19 +4760,19 @@
       <c r="K9" t="n">
         <v>83.70529570207415</v>
       </c>
-      <c r="W9" t="n">
-        <v>8</v>
-      </c>
-      <c r="X9" t="inlineStr">
+      <c r="W9" t="inlineStr">
         <is>
           <t>y = 9.066x + -28548.425</t>
         </is>
+      </c>
+      <c r="X9" t="n">
+        <v>-28548.42548320814</v>
       </c>
       <c r="Y9" t="n">
         <v>1.630872492385224e-10</v>
       </c>
       <c r="Z9" t="n">
-        <v>3694.783648524833</v>
+        <v>438.2799999999997</v>
       </c>
       <c r="AA9" t="n">
         <v>1.00000000000811e-08</v>
@@ -3200,19 +4812,19 @@
       <c r="K10" t="n">
         <v>83.78413149258013</v>
       </c>
-      <c r="W10" t="n">
-        <v>9</v>
-      </c>
-      <c r="X10" t="inlineStr">
+      <c r="W10" t="inlineStr">
         <is>
           <t>y = 9.181x + -28674.715</t>
         </is>
+      </c>
+      <c r="X10" t="n">
+        <v>-28674.71482569155</v>
       </c>
       <c r="Y10" t="n">
         <v>3.259689340340592e-10</v>
       </c>
       <c r="Z10" t="n">
-        <v>3661.15466635551</v>
+        <v>438.5299999999997</v>
       </c>
       <c r="AA10" t="n">
         <v>1.000000000000035e-08</v>
@@ -3252,19 +4864,19 @@
       <c r="K11" t="n">
         <v>83.88371344689703</v>
       </c>
-      <c r="W11" t="n">
-        <v>10</v>
-      </c>
-      <c r="X11" t="inlineStr">
+      <c r="W11" t="inlineStr">
         <is>
           <t>y = 9.332x + -28898.503</t>
         </is>
+      </c>
+      <c r="X11" t="n">
+        <v>-28898.50286554719</v>
       </c>
       <c r="Y11" t="n">
         <v>2.584869732792946e-10</v>
       </c>
       <c r="Z11" t="n">
-        <v>3628.426219168407</v>
+        <v>425.21</v>
       </c>
       <c r="AA11" t="n">
         <v>1.000000000000108e-08</v>
@@ -3304,19 +4916,19 @@
       <c r="K12" t="n">
         <v>84.01179981942853</v>
       </c>
-      <c r="W12" t="n">
-        <v>11</v>
-      </c>
-      <c r="X12" t="inlineStr">
+      <c r="W12" t="inlineStr">
         <is>
           <t>y = 9.533x + -29319.538</t>
         </is>
+      </c>
+      <c r="X12" t="n">
+        <v>-29319.53796829532</v>
       </c>
       <c r="Y12" t="n">
         <v>1.514289416406875e-10</v>
       </c>
       <c r="Z12" t="n">
-        <v>3596.877893152952</v>
+        <v>419.1199999999999</v>
       </c>
       <c r="AA12" t="n">
         <v>1.00000000000106e-08</v>
@@ -3356,19 +4968,19 @@
       <c r="K13" t="n">
         <v>84.07878823873421</v>
       </c>
-      <c r="W13" t="n">
-        <v>12</v>
-      </c>
-      <c r="X13" t="inlineStr">
+      <c r="W13" t="inlineStr">
         <is>
           <t>y = 9.642x + -29404.166</t>
         </is>
+      </c>
+      <c r="X13" t="n">
+        <v>-29404.16599194265</v>
       </c>
       <c r="Y13" t="n">
         <v>1.120530536052821e-08</v>
       </c>
       <c r="Z13" t="n">
-        <v>3565.168694081408</v>
+        <v>411.21</v>
       </c>
       <c r="AA13" t="n">
         <v>1.000000000000027e-08</v>
@@ -3408,19 +5020,19 @@
       <c r="K14" t="n">
         <v>84.18596511964131</v>
       </c>
-      <c r="W14" t="n">
-        <v>13</v>
-      </c>
-      <c r="X14" t="inlineStr">
+      <c r="W14" t="inlineStr">
         <is>
           <t>y = 9.821x + -29709.095</t>
         </is>
+      </c>
+      <c r="X14" t="n">
+        <v>-29709.0951033068</v>
       </c>
       <c r="Y14" t="n">
         <v>9.505757559990949e-09</v>
       </c>
       <c r="Z14" t="n">
-        <v>3534.132273106329</v>
+        <v>400.27</v>
       </c>
       <c r="AA14" t="n">
         <v>1.000000000000331e-08</v>
@@ -3460,19 +5072,19 @@
       <c r="K15" t="n">
         <v>84.20713005907987</v>
       </c>
-      <c r="W15" t="n">
-        <v>14</v>
-      </c>
-      <c r="X15" t="inlineStr">
+      <c r="W15" t="inlineStr">
         <is>
           <t>y = 9.857x + -29577.413</t>
         </is>
+      </c>
+      <c r="X15" t="n">
+        <v>-29577.41319756097</v>
       </c>
       <c r="Y15" t="n">
         <v>4.405966353261179e-12</v>
       </c>
       <c r="Z15" t="n">
-        <v>3503.030557362109</v>
+        <v>400.6700000000001</v>
       </c>
       <c r="AA15" t="n">
         <v>1.000000000005382e-08</v>
@@ -3512,19 +5124,19 @@
       <c r="K16" t="n">
         <v>84.26304068018455</v>
       </c>
-      <c r="W16" t="n">
-        <v>15</v>
-      </c>
-      <c r="X16" t="inlineStr">
+      <c r="W16" t="inlineStr">
         <is>
           <t>y = 9.954x + -29628.455</t>
         </is>
+      </c>
+      <c r="X16" t="n">
+        <v>-29628.45510555273</v>
       </c>
       <c r="Y16" t="n">
         <v>8.707214415280754e-10</v>
       </c>
       <c r="Z16" t="n">
-        <v>3472.204119141927</v>
+        <v>396.9400000000001</v>
       </c>
       <c r="AA16" t="n">
         <v>1e-08</v>
@@ -3564,19 +5176,19 @@
       <c r="K17" t="n">
         <v>84.38437580484043</v>
       </c>
-      <c r="W17" t="n">
-        <v>16</v>
-      </c>
-      <c r="X17" t="inlineStr">
+      <c r="W17" t="inlineStr">
         <is>
           <t>y = 10.170x + -30028.579</t>
         </is>
+      </c>
+      <c r="X17" t="n">
+        <v>-30028.57892337986</v>
       </c>
       <c r="Y17" t="n">
         <v>1.390207030577781e-09</v>
       </c>
       <c r="Z17" t="n">
-        <v>3441.373366417077</v>
+        <v>386.3600000000001</v>
       </c>
       <c r="AA17" t="n">
         <v>1.00000000001704e-08</v>
@@ -3616,19 +5228,19 @@
       <c r="K18" t="n">
         <v>84.46375950983405</v>
       </c>
-      <c r="W18" t="n">
-        <v>17</v>
-      </c>
-      <c r="X18" t="inlineStr">
+      <c r="W18" t="inlineStr">
         <is>
           <t>y = 10.317x + -30211.572</t>
         </is>
+      </c>
+      <c r="X18" t="n">
+        <v>-30211.57208073499</v>
       </c>
       <c r="Y18" t="n">
         <v>1.154298452146454e-11</v>
       </c>
       <c r="Z18" t="n">
-        <v>3410.426010644573</v>
+        <v>379.3499999999999</v>
       </c>
       <c r="AA18" t="n">
         <v>1.000000000000535e-08</v>
@@ -3668,19 +5280,19 @@
       <c r="K19" t="n">
         <v>84.19032214251865</v>
       </c>
-      <c r="W19" t="n">
-        <v>18</v>
-      </c>
-      <c r="X19" t="inlineStr">
+      <c r="W19" t="inlineStr">
         <is>
           <t>y = 9.828x + -28412.792</t>
         </is>
+      </c>
+      <c r="X19" t="n">
+        <v>-28412.79198105791</v>
       </c>
       <c r="Y19" t="n">
         <v>2.517315629913945e-09</v>
       </c>
       <c r="Z19" t="n">
-        <v>3380.128435820616</v>
+        <v>390.4100000000003</v>
       </c>
       <c r="AA19" t="n">
         <v>1.000000000089883e-08</v>
@@ -3720,19 +5332,19 @@
       <c r="K20" t="n">
         <v>84.60014254065234</v>
       </c>
-      <c r="W20" t="n">
-        <v>19</v>
-      </c>
-      <c r="X20" t="inlineStr">
+      <c r="W20" t="inlineStr">
         <is>
           <t>y = 10.579x + -30467.949</t>
         </is>
+      </c>
+      <c r="X20" t="n">
+        <v>-30467.94887651073</v>
       </c>
       <c r="Y20" t="n">
         <v>2.5093519068961e-11</v>
       </c>
       <c r="Z20" t="n">
-        <v>3348.381877410202</v>
+        <v>368.52</v>
       </c>
       <c r="AA20" t="n">
         <v>1.00000000000073e-08</v>
@@ -3772,19 +5384,19 @@
       <c r="K21" t="n">
         <v>84.31946038118039</v>
       </c>
-      <c r="W21" t="n">
-        <v>20</v>
-      </c>
-      <c r="X21" t="inlineStr">
+      <c r="W21" t="inlineStr">
         <is>
           <t>y = 10.053x + -28565.884</t>
         </is>
+      </c>
+      <c r="X21" t="n">
+        <v>-28565.88371232273</v>
       </c>
       <c r="Y21" t="n">
         <v>1.449632556628533e-11</v>
       </c>
       <c r="Z21" t="n">
-        <v>3316.26452106183</v>
+        <v>379.8200000000002</v>
       </c>
       <c r="AA21" t="n">
         <v>1.000000000000639e-08</v>
@@ -3824,19 +5436,19 @@
       <c r="K22" t="n">
         <v>84.78441736683563</v>
       </c>
-      <c r="W22" t="n">
-        <v>21</v>
-      </c>
-      <c r="X22" t="inlineStr">
+      <c r="W22" t="inlineStr">
         <is>
           <t>y = 10.955x + -31006.395</t>
         </is>
+      </c>
+      <c r="X22" t="n">
+        <v>-31006.39486152134</v>
       </c>
       <c r="Y22" t="n">
         <v>1.409007508995995e-11</v>
       </c>
       <c r="Z22" t="n">
-        <v>3284.11934365875</v>
+        <v>353.6400000000003</v>
       </c>
       <c r="AA22" t="n">
         <v>1.000000000000556e-08</v>
@@ -3962,12 +5574,12 @@
       </c>
       <c r="W1" t="inlineStr">
         <is>
-          <t>Cycle</t>
+          <t>Model</t>
         </is>
       </c>
       <c r="X1" t="inlineStr">
         <is>
-          <t>Model</t>
+          <t>b</t>
         </is>
       </c>
       <c r="Y1" t="inlineStr">
@@ -3977,7 +5589,7 @@
       </c>
       <c r="Z1" t="inlineStr">
         <is>
-          <t>Rp</t>
+          <t>delta Rct-i</t>
         </is>
       </c>
       <c r="AA1" t="inlineStr">
@@ -4022,19 +5634,19 @@
       <c r="K2" t="n">
         <v>59.13296351765025</v>
       </c>
-      <c r="W2" t="n">
-        <v>1</v>
-      </c>
-      <c r="X2" t="inlineStr">
+      <c r="W2" t="inlineStr">
         <is>
           <t>y = 1.673x + -45240.389</t>
         </is>
+      </c>
+      <c r="X2" t="n">
+        <v>-45240.3889864725</v>
       </c>
       <c r="Y2" t="n">
         <v>1956.981062621956</v>
       </c>
       <c r="Z2" t="n">
-        <v>1768.128452230034</v>
+        <v>2912.600000000002</v>
       </c>
       <c r="AA2" t="n">
         <v>1.571690957730544e-06</v>
@@ -4074,19 +5686,19 @@
       <c r="K3" t="n">
         <v>61.82421419133203</v>
       </c>
-      <c r="W3" t="n">
-        <v>2</v>
-      </c>
-      <c r="X3" t="inlineStr">
+      <c r="W3" t="inlineStr">
         <is>
           <t>y = 1.867x + -45857.046</t>
         </is>
+      </c>
+      <c r="X3" t="n">
+        <v>-45857.04613273493</v>
       </c>
       <c r="Y3" t="n">
         <v>1979.249072103158</v>
       </c>
       <c r="Z3" t="n">
-        <v>1792.33888738741</v>
+        <v>2718.200000000001</v>
       </c>
       <c r="AA3" t="n">
         <v>1.450875310280992e-06</v>
@@ -4126,19 +5738,19 @@
       <c r="K4" t="n">
         <v>62.58370357284059</v>
       </c>
-      <c r="W4" t="n">
-        <v>3</v>
-      </c>
-      <c r="X4" t="inlineStr">
+      <c r="W4" t="inlineStr">
         <is>
           <t>y = 1.928x + -45986.207</t>
         </is>
+      </c>
+      <c r="X4" t="n">
+        <v>-45986.20733642069</v>
       </c>
       <c r="Y4" t="n">
         <v>2019.450788730009</v>
       </c>
       <c r="Z4" t="n">
-        <v>1831.238120154344</v>
+        <v>2677.599999999999</v>
       </c>
       <c r="AA4" t="n">
         <v>1.408136428363595e-06</v>
@@ -4178,19 +5790,19 @@
       <c r="K5" t="n">
         <v>63.00392211446661</v>
       </c>
-      <c r="W5" t="n">
-        <v>4</v>
-      </c>
-      <c r="X5" t="inlineStr">
+      <c r="W5" t="inlineStr">
         <is>
           <t>y = 1.963x + -46019.634</t>
         </is>
+      </c>
+      <c r="X5" t="n">
+        <v>-46019.63413940557</v>
       </c>
       <c r="Y5" t="n">
         <v>2032.692439338152</v>
       </c>
       <c r="Z5" t="n">
-        <v>1844.767937746745</v>
+        <v>2665.600000000002</v>
       </c>
       <c r="AA5" t="n">
         <v>1.642772286163007e-06</v>
@@ -4230,19 +5842,19 @@
       <c r="K6" t="n">
         <v>63.07764854462515</v>
       </c>
-      <c r="W6" t="n">
-        <v>5</v>
-      </c>
-      <c r="X6" t="inlineStr">
+      <c r="W6" t="inlineStr">
         <is>
           <t>y = 1.969x + -45443.822</t>
         </is>
+      </c>
+      <c r="X6" t="n">
+        <v>-45443.82219027122</v>
       </c>
       <c r="Y6" t="n">
         <v>2037.839430945596</v>
       </c>
       <c r="Z6" t="n">
-        <v>1850.520666925785</v>
+        <v>2695.099999999999</v>
       </c>
       <c r="AA6" t="n">
         <v>1.631187797574851e-06</v>
@@ -4282,19 +5894,19 @@
       <c r="K7" t="n">
         <v>63.26747318032066</v>
       </c>
-      <c r="W7" t="n">
-        <v>6</v>
-      </c>
-      <c r="X7" t="inlineStr">
+      <c r="W7" t="inlineStr">
         <is>
           <t>y = 1.985x + -45181.243</t>
         </is>
+      </c>
+      <c r="X7" t="n">
+        <v>-45181.24346535742</v>
       </c>
       <c r="Y7" t="n">
         <v>2089.150040683206</v>
       </c>
       <c r="Z7" t="n">
-        <v>1900.018103241254</v>
+        <v>2688.900000000001</v>
       </c>
       <c r="AA7" t="n">
         <v>1.324157460973251e-06</v>
@@ -4334,19 +5946,19 @@
       <c r="K8" t="n">
         <v>63.32971181267361</v>
       </c>
-      <c r="W8" t="n">
-        <v>7</v>
-      </c>
-      <c r="X8" t="inlineStr">
+      <c r="W8" t="inlineStr">
         <is>
           <t>y = 1.991x + -44667.205</t>
         </is>
+      </c>
+      <c r="X8" t="n">
+        <v>-44667.20504721891</v>
       </c>
       <c r="Y8" t="n">
         <v>2055.020950709662</v>
       </c>
       <c r="Z8" t="n">
-        <v>1868.58676095677</v>
+        <v>2689.600000000002</v>
       </c>
       <c r="AA8" t="n">
         <v>1.60057361096518e-06</v>
@@ -4386,19 +5998,19 @@
       <c r="K9" t="n">
         <v>63.64317165555217</v>
       </c>
-      <c r="W9" t="n">
-        <v>8</v>
-      </c>
-      <c r="X9" t="inlineStr">
+      <c r="W9" t="inlineStr">
         <is>
           <t>y = 2.018x + -44748.728</t>
         </is>
+      </c>
+      <c r="X9" t="n">
+        <v>-44748.72817072683</v>
       </c>
       <c r="Y9" t="n">
         <v>2053.697762144098</v>
       </c>
       <c r="Z9" t="n">
-        <v>1868.2901992821</v>
+        <v>2663.900000000001</v>
       </c>
       <c r="AA9" t="n">
         <v>1.595567646677031e-06</v>
@@ -4438,19 +6050,19 @@
       <c r="K10" t="n">
         <v>63.57617945324454</v>
       </c>
-      <c r="W10" t="n">
-        <v>9</v>
-      </c>
-      <c r="X10" t="inlineStr">
+      <c r="W10" t="inlineStr">
         <is>
           <t>y = 2.012x + -44007.994</t>
         </is>
+      </c>
+      <c r="X10" t="n">
+        <v>-44007.99359489807</v>
       </c>
       <c r="Y10" t="n">
         <v>2069.231919864614</v>
       </c>
       <c r="Z10" t="n">
-        <v>1884.084555784315</v>
+        <v>2681.299999999999</v>
       </c>
       <c r="AA10" t="n">
         <v>1.574361891415273e-06</v>
@@ -4490,19 +6102,19 @@
       <c r="K11" t="n">
         <v>63.75561889004117</v>
       </c>
-      <c r="W11" t="n">
-        <v>10</v>
-      </c>
-      <c r="X11" t="inlineStr">
+      <c r="W11" t="inlineStr">
         <is>
           <t>y = 2.028x + -43836.838</t>
         </is>
+      </c>
+      <c r="X11" t="n">
+        <v>-43836.83812154708</v>
       </c>
       <c r="Y11" t="n">
         <v>2065.449527872279</v>
       </c>
       <c r="Z11" t="n">
-        <v>1881.401289827784</v>
+        <v>2660.700000000001</v>
       </c>
       <c r="AA11" t="n">
         <v>1.571495531452732e-06</v>
@@ -4628,12 +6240,12 @@
       </c>
       <c r="W1" t="inlineStr">
         <is>
-          <t>Cycle</t>
+          <t>Model</t>
         </is>
       </c>
       <c r="X1" t="inlineStr">
         <is>
-          <t>Model</t>
+          <t>b</t>
         </is>
       </c>
       <c r="Y1" t="inlineStr">
@@ -4643,7 +6255,7 @@
       </c>
       <c r="Z1" t="inlineStr">
         <is>
-          <t>Rp</t>
+          <t>delta Rct-i</t>
         </is>
       </c>
       <c r="AA1" t="inlineStr">
@@ -4688,19 +6300,19 @@
       <c r="K2" t="n">
         <v>81.21776653976325</v>
       </c>
-      <c r="W2" t="n">
-        <v>1</v>
-      </c>
-      <c r="X2" t="inlineStr">
+      <c r="W2" t="inlineStr">
         <is>
           <t>y = 6.473x + -23177.174</t>
         </is>
+      </c>
+      <c r="X2" t="n">
+        <v>-23177.17443704293</v>
       </c>
       <c r="Y2" t="n">
         <v>8.893462476884348e-10</v>
       </c>
       <c r="Z2" t="n">
-        <v>4228.089117988718</v>
+        <v>758.0999999999999</v>
       </c>
       <c r="AA2" t="n">
         <v>1.000000000000006e-08</v>
@@ -4740,19 +6352,19 @@
       <c r="K3" t="n">
         <v>81.52623268285021</v>
       </c>
-      <c r="W3" t="n">
-        <v>2</v>
-      </c>
-      <c r="X3" t="inlineStr">
+      <c r="W3" t="inlineStr">
         <is>
           <t>y = 6.712x + -22620.911</t>
         </is>
+      </c>
+      <c r="X3" t="n">
+        <v>-22620.91124627536</v>
       </c>
       <c r="Y3" t="n">
         <v>3.064630490463671e-09</v>
       </c>
       <c r="Z3" t="n">
-        <v>3995.00470750756</v>
+        <v>712.6700000000001</v>
       </c>
       <c r="AA3" t="n">
         <v>1.000000000000431e-08</v>
@@ -4792,19 +6404,19 @@
       <c r="K4" t="n">
         <v>81.58447887943476</v>
       </c>
-      <c r="W4" t="n">
-        <v>3</v>
-      </c>
-      <c r="X4" t="inlineStr">
+      <c r="W4" t="inlineStr">
         <is>
           <t>y = 6.759x + -22344.308</t>
         </is>
+      </c>
+      <c r="X4" t="n">
+        <v>-22344.30760975299</v>
       </c>
       <c r="Y4" t="n">
         <v>1.437133177459935e-09</v>
       </c>
       <c r="Z4" t="n">
-        <v>3919.7152960145</v>
+        <v>702.6100000000001</v>
       </c>
       <c r="AA4" t="n">
         <v>1.000000000000007e-08</v>
@@ -4844,19 +6456,19 @@
       <c r="K5" t="n">
         <v>81.67211594857707</v>
       </c>
-      <c r="W5" t="n">
-        <v>4</v>
-      </c>
-      <c r="X5" t="inlineStr">
+      <c r="W5" t="inlineStr">
         <is>
           <t>y = 6.831x + -22318.030</t>
         </is>
+      </c>
+      <c r="X5" t="n">
+        <v>-22318.02970931322</v>
       </c>
       <c r="Y5" t="n">
         <v>8.525199959196454e-09</v>
       </c>
       <c r="Z5" t="n">
-        <v>3869.999130203362</v>
+        <v>688.3299999999999</v>
       </c>
       <c r="AA5" t="n">
         <v>1.000000000000002e-08</v>
@@ -4896,19 +6508,19 @@
       <c r="K6" t="n">
         <v>81.73150307854043</v>
       </c>
-      <c r="W6" t="n">
-        <v>5</v>
-      </c>
-      <c r="X6" t="inlineStr">
+      <c r="W6" t="inlineStr">
         <is>
           <t>y = 6.881x + -22244.566</t>
         </is>
+      </c>
+      <c r="X6" t="n">
+        <v>-22244.56552976538</v>
       </c>
       <c r="Y6" t="n">
         <v>108.5492817197652</v>
       </c>
       <c r="Z6" t="n">
-        <v>4157.638945999423</v>
+        <v>682.8699999999999</v>
       </c>
       <c r="AA6" t="n">
         <v>1.540680380679318e-08</v>
@@ -4948,19 +6560,19 @@
       <c r="K7" t="n">
         <v>81.85659717212884</v>
       </c>
-      <c r="W7" t="n">
-        <v>6</v>
-      </c>
-      <c r="X7" t="inlineStr">
+      <c r="W7" t="inlineStr">
         <is>
           <t>y = 6.988x + -22361.418</t>
         </is>
+      </c>
+      <c r="X7" t="n">
+        <v>-22361.41772853267</v>
       </c>
       <c r="Y7" t="n">
         <v>3.161141659038213e-10</v>
       </c>
       <c r="Z7" t="n">
-        <v>3783.196584692455</v>
+        <v>669.9400000000001</v>
       </c>
       <c r="AA7" t="n">
         <v>1.000000000002135e-08</v>
@@ -5000,19 +6612,19 @@
       <c r="K8" t="n">
         <v>81.89930620615482</v>
       </c>
-      <c r="W8" t="n">
-        <v>7</v>
-      </c>
-      <c r="X8" t="inlineStr">
+      <c r="W8" t="inlineStr">
         <is>
           <t>y = 7.026x + -22260.468</t>
         </is>
+      </c>
+      <c r="X8" t="n">
+        <v>-22260.46846365806</v>
       </c>
       <c r="Y8" t="n">
         <v>7.603127593450079e-10</v>
       </c>
       <c r="Z8" t="n">
-        <v>3742.39318797351</v>
+        <v>664.0700000000002</v>
       </c>
       <c r="AA8" t="n">
         <v>1.000000000000009e-08</v>
@@ -5052,19 +6664,19 @@
       <c r="K9" t="n">
         <v>81.96286628218232</v>
       </c>
-      <c r="W9" t="n">
-        <v>8</v>
-      </c>
-      <c r="X9" t="inlineStr">
+      <c r="W9" t="inlineStr">
         <is>
           <t>y = 7.082x + -22222.796</t>
         </is>
+      </c>
+      <c r="X9" t="n">
+        <v>-22222.79574531389</v>
       </c>
       <c r="Y9" t="n">
         <v>1.521868844776335e-10</v>
       </c>
       <c r="Z9" t="n">
-        <v>3703.725698002615</v>
+        <v>657.4099999999999</v>
       </c>
       <c r="AA9" t="n">
         <v>1.000000000000382e-08</v>
@@ -5104,19 +6716,19 @@
       <c r="K10" t="n">
         <v>82.06739887001213</v>
       </c>
-      <c r="W10" t="n">
-        <v>9</v>
-      </c>
-      <c r="X10" t="inlineStr">
+      <c r="W10" t="inlineStr">
         <is>
           <t>y = 7.177x + -22321.139</t>
         </is>
+      </c>
+      <c r="X10" t="n">
+        <v>-22321.13870224415</v>
       </c>
       <c r="Y10" t="n">
         <v>1.914373975216812e-11</v>
       </c>
       <c r="Z10" t="n">
-        <v>3666.83455351343</v>
+        <v>647.9000000000001</v>
       </c>
       <c r="AA10" t="n">
         <v>1e-08</v>
@@ -5156,19 +6768,19 @@
       <c r="K11" t="n">
         <v>82.10739524777436</v>
       </c>
-      <c r="W11" t="n">
-        <v>10</v>
-      </c>
-      <c r="X11" t="inlineStr">
+      <c r="W11" t="inlineStr">
         <is>
           <t>y = 7.213x + -22237.743</t>
         </is>
+      </c>
+      <c r="X11" t="n">
+        <v>-22237.74262316509</v>
       </c>
       <c r="Y11" t="n">
         <v>1.537612853485187e-09</v>
       </c>
       <c r="Z11" t="n">
-        <v>3631.830470287303</v>
+        <v>643.7400000000002</v>
       </c>
       <c r="AA11" t="n">
         <v>1e-08</v>
@@ -5208,19 +6820,19 @@
       <c r="K12" t="n">
         <v>81.93366593735455</v>
       </c>
-      <c r="W12" t="n">
-        <v>11</v>
-      </c>
-      <c r="X12" t="inlineStr">
+      <c r="W12" t="inlineStr">
         <is>
           <t>y = 7.056x + -21469.974</t>
         </is>
+      </c>
+      <c r="X12" t="n">
+        <v>-21469.97362443178</v>
       </c>
       <c r="Y12" t="n">
         <v>2.59594962930328e-10</v>
       </c>
       <c r="Z12" t="n">
-        <v>3597.710134803611</v>
+        <v>646.8200000000002</v>
       </c>
       <c r="AA12" t="n">
         <v>1.000000000000025e-08</v>
@@ -5260,19 +6872,19 @@
       <c r="K13" t="n">
         <v>81.95928549382815</v>
       </c>
-      <c r="W13" t="n">
-        <v>12</v>
-      </c>
-      <c r="X13" t="inlineStr">
+      <c r="W13" t="inlineStr">
         <is>
           <t>y = 7.079x + -21355.930</t>
         </is>
+      </c>
+      <c r="X13" t="n">
+        <v>-21355.93043890158</v>
       </c>
       <c r="Y13" t="n">
         <v>2.201600607771591e-09</v>
       </c>
       <c r="Z13" t="n">
-        <v>3565.162528323268</v>
+        <v>643.23</v>
       </c>
       <c r="AA13" t="n">
         <v>1.000000000004395e-08</v>
@@ -5312,19 +6924,19 @@
       <c r="K14" t="n">
         <v>82.31012372062959</v>
       </c>
-      <c r="W14" t="n">
-        <v>13</v>
-      </c>
-      <c r="X14" t="inlineStr">
+      <c r="W14" t="inlineStr">
         <is>
           <t>y = 7.406x + -22274.287</t>
         </is>
+      </c>
+      <c r="X14" t="n">
+        <v>-22274.28733436464</v>
       </c>
       <c r="Y14" t="n">
         <v>9.726162347189987e-10</v>
       </c>
       <c r="Z14" t="n">
-        <v>3533.235419048723</v>
+        <v>623.8000000000002</v>
       </c>
       <c r="AA14" t="n">
         <v>1.000000000000054e-08</v>
@@ -5364,19 +6976,19 @@
       <c r="K15" t="n">
         <v>82.38273360514714</v>
       </c>
-      <c r="W15" t="n">
-        <v>14</v>
-      </c>
-      <c r="X15" t="inlineStr">
+      <c r="W15" t="inlineStr">
         <is>
           <t>y = 7.477x + -22305.630</t>
         </is>
+      </c>
+      <c r="X15" t="n">
+        <v>-22305.63043253864</v>
       </c>
       <c r="Y15" t="n">
         <v>2.388420229840544e-13</v>
       </c>
       <c r="Z15" t="n">
-        <v>3502.544657250044</v>
+        <v>618.7000000000003</v>
       </c>
       <c r="AA15" t="n">
         <v>1.00000000000016e-08</v>
@@ -5416,19 +7028,19 @@
       <c r="K16" t="n">
         <v>82.49166770061491</v>
       </c>
-      <c r="W16" t="n">
-        <v>15</v>
-      </c>
-      <c r="X16" t="inlineStr">
+      <c r="W16" t="inlineStr">
         <is>
           <t>y = 7.587x + -22446.190</t>
         </is>
+      </c>
+      <c r="X16" t="n">
+        <v>-22446.19013596027</v>
       </c>
       <c r="Y16" t="n">
         <v>2.934456815630635e-13</v>
       </c>
       <c r="Z16" t="n">
-        <v>3470.791470776857</v>
+        <v>610.1700000000001</v>
       </c>
       <c r="AA16" t="n">
         <v>1e-08</v>
@@ -5468,19 +7080,19 @@
       <c r="K17" t="n">
         <v>82.59867494685955</v>
       </c>
-      <c r="W17" t="n">
-        <v>16</v>
-      </c>
-      <c r="X17" t="inlineStr">
+      <c r="W17" t="inlineStr">
         <is>
           <t>y = 7.698x + -22596.090</t>
         </is>
+      </c>
+      <c r="X17" t="n">
+        <v>-22596.09049655399</v>
       </c>
       <c r="Y17" t="n">
         <v>4.093997846238827e-11</v>
       </c>
       <c r="Z17" t="n">
-        <v>3439.868900978634</v>
+        <v>598.5599999999999</v>
       </c>
       <c r="AA17" t="n">
         <v>1.000000000000001e-08</v>
@@ -5520,19 +7132,19 @@
       <c r="K18" t="n">
         <v>82.3239304054328</v>
       </c>
-      <c r="W18" t="n">
-        <v>17</v>
-      </c>
-      <c r="X18" t="inlineStr">
+      <c r="W18" t="inlineStr">
         <is>
           <t>y = 7.419x + -21479.229</t>
         </is>
+      </c>
+      <c r="X18" t="n">
+        <v>-21479.22854676919</v>
       </c>
       <c r="Y18" t="n">
         <v>3.318572629114995e-10</v>
       </c>
       <c r="Z18" t="n">
-        <v>3407.362653459402</v>
+        <v>613.0899999999997</v>
       </c>
       <c r="AA18" t="n">
         <v>1.000000000000108e-08</v>
@@ -5572,19 +7184,19 @@
       <c r="K19" t="n">
         <v>82.67180465252127</v>
       </c>
-      <c r="W19" t="n">
-        <v>18</v>
-      </c>
-      <c r="X19" t="inlineStr">
+      <c r="W19" t="inlineStr">
         <is>
           <t>y = 7.776x + -22439.000</t>
         </is>
+      </c>
+      <c r="X19" t="n">
+        <v>-22438.99957906457</v>
       </c>
       <c r="Y19" t="n">
         <v>3.254157878042292e-10</v>
       </c>
       <c r="Z19" t="n">
-        <v>3376.308599464076</v>
+        <v>594.2599999999998</v>
       </c>
       <c r="AA19" t="n">
         <v>1.000000000000126e-08</v>
@@ -5624,19 +7236,19 @@
       <c r="K20" t="n">
         <v>82.78546780548824</v>
       </c>
-      <c r="W20" t="n">
-        <v>19</v>
-      </c>
-      <c r="X20" t="inlineStr">
+      <c r="W20" t="inlineStr">
         <is>
           <t>y = 7.900x + -22600.622</t>
         </is>
+      </c>
+      <c r="X20" t="n">
+        <v>-22600.62203483048</v>
       </c>
       <c r="Y20" t="n">
         <v>4.211313836099983e-10</v>
       </c>
       <c r="Z20" t="n">
-        <v>3343.295576878203</v>
+        <v>582.8000000000002</v>
       </c>
       <c r="AA20" t="n">
         <v>1.000000000000235e-08</v>
@@ -5676,19 +7288,19 @@
       <c r="K21" t="n">
         <v>82.84831353049789</v>
       </c>
-      <c r="W21" t="n">
-        <v>20</v>
-      </c>
-      <c r="X21" t="inlineStr">
+      <c r="W21" t="inlineStr">
         <is>
           <t>y = 7.970x + -22600.837</t>
         </is>
+      </c>
+      <c r="X21" t="n">
+        <v>-22600.83675982003</v>
       </c>
       <c r="Y21" t="n">
         <v>4.352747599166061e-10</v>
       </c>
       <c r="Z21" t="n">
-        <v>3311.167146405325</v>
+        <v>577.4700000000003</v>
       </c>
       <c r="AA21" t="n">
         <v>1.000000000000249e-08</v>
@@ -5728,19 +7340,19 @@
       <c r="K22" t="n">
         <v>82.9000537171266</v>
       </c>
-      <c r="W22" t="n">
-        <v>21</v>
-      </c>
-      <c r="X22" t="inlineStr">
+      <c r="W22" t="inlineStr">
         <is>
           <t>y = 8.029x + -22571.668</t>
         </is>
+      </c>
+      <c r="X22" t="n">
+        <v>-22571.66848477024</v>
       </c>
       <c r="Y22" t="n">
         <v>5.382503022771223e-10</v>
       </c>
       <c r="Z22" t="n">
-        <v>3279.976366698247</v>
+        <v>572.5799999999999</v>
       </c>
       <c r="AA22" t="n">
         <v>1.000000000000328e-08</v>
@@ -5866,12 +7478,12 @@
       </c>
       <c r="W1" t="inlineStr">
         <is>
-          <t>Cycle</t>
+          <t>Model</t>
         </is>
       </c>
       <c r="X1" t="inlineStr">
         <is>
-          <t>Model</t>
+          <t>b</t>
         </is>
       </c>
       <c r="Y1" t="inlineStr">
@@ -5881,7 +7493,7 @@
       </c>
       <c r="Z1" t="inlineStr">
         <is>
-          <t>Rp</t>
+          <t>delta Rct-i</t>
         </is>
       </c>
       <c r="AA1" t="inlineStr">
@@ -5926,19 +7538,19 @@
       <c r="K2" t="n">
         <v>67.8967954848812</v>
       </c>
-      <c r="W2" t="n">
-        <v>1</v>
-      </c>
-      <c r="X2" t="inlineStr">
+      <c r="W2" t="inlineStr">
         <is>
           <t>y = 2.462x + -49517.091</t>
         </is>
+      </c>
+      <c r="X2" t="n">
+        <v>-49517.09064727029</v>
       </c>
       <c r="Y2" t="n">
         <v>2129.258059778241</v>
       </c>
       <c r="Z2" t="n">
-        <v>1951.723150083427</v>
+        <v>2141.299999999999</v>
       </c>
       <c r="AA2" t="n">
         <v>1.331561679608598e-06</v>
@@ -5978,19 +7590,19 @@
       <c r="K3" t="n">
         <v>68.40828343426492</v>
       </c>
-      <c r="W3" t="n">
-        <v>2</v>
-      </c>
-      <c r="X3" t="inlineStr">
+      <c r="W3" t="inlineStr">
         <is>
           <t>y = 2.527x + -47690.154</t>
         </is>
+      </c>
+      <c r="X3" t="n">
+        <v>-47690.15351683742</v>
       </c>
       <c r="Y3" t="n">
         <v>1024.357689096387</v>
       </c>
       <c r="Z3" t="n">
-        <v>805.7256111545275</v>
+        <v>2049</v>
       </c>
       <c r="AA3" t="n">
         <v>5.084512325403472e-06</v>
@@ -6030,19 +7642,19 @@
       <c r="K4" t="n">
         <v>68.7005504568087</v>
       </c>
-      <c r="W4" t="n">
-        <v>3</v>
-      </c>
-      <c r="X4" t="inlineStr">
+      <c r="W4" t="inlineStr">
         <is>
           <t>y = 2.565x + -47355.050</t>
         </is>
+      </c>
+      <c r="X4" t="n">
+        <v>-47355.04958175466</v>
       </c>
       <c r="Y4" t="n">
         <v>1024.280845988597</v>
       </c>
       <c r="Z4" t="n">
-        <v>805.6647883388291</v>
+        <v>2006</v>
       </c>
       <c r="AA4" t="n">
         <v>5.758943613172105e-07</v>
@@ -6082,19 +7694,19 @@
       <c r="K5" t="n">
         <v>68.69624047288853</v>
       </c>
-      <c r="W5" t="n">
-        <v>4</v>
-      </c>
-      <c r="X5" t="inlineStr">
+      <c r="W5" t="inlineStr">
         <is>
           <t>y = 2.564x + -46602.830</t>
         </is>
+      </c>
+      <c r="X5" t="n">
+        <v>-46602.83010421869</v>
       </c>
       <c r="Y5" t="n">
         <v>1020.435705028042</v>
       </c>
       <c r="Z5" t="n">
-        <v>802.6869968887955</v>
+        <v>1995.799999999999</v>
       </c>
       <c r="AA5" t="n">
         <v>5.815535215137008e-07</v>
@@ -6134,19 +7746,19 @@
       <c r="K6" t="n">
         <v>68.72210006186269</v>
       </c>
-      <c r="W6" t="n">
-        <v>5</v>
-      </c>
-      <c r="X6" t="inlineStr">
+      <c r="W6" t="inlineStr">
         <is>
           <t>y = 2.568x + -46037.558</t>
         </is>
+      </c>
+      <c r="X6" t="n">
+        <v>-46037.55812443314</v>
       </c>
       <c r="Y6" t="n">
         <v>1018.750217461095</v>
       </c>
       <c r="Z6" t="n">
-        <v>801.3644191667836</v>
+        <v>1985</v>
       </c>
       <c r="AA6" t="n">
         <v>5.873364916621856e-07</v>
@@ -6186,19 +7798,19 @@
       <c r="K7" t="n">
         <v>68.83956829932609</v>
       </c>
-      <c r="W7" t="n">
-        <v>6</v>
-      </c>
-      <c r="X7" t="inlineStr">
+      <c r="W7" t="inlineStr">
         <is>
           <t>y = 2.583x + -45732.522</t>
         </is>
+      </c>
+      <c r="X7" t="n">
+        <v>-45732.5218983997</v>
       </c>
       <c r="Y7" t="n">
         <v>1050.278977589443</v>
       </c>
       <c r="Z7" t="n">
-        <v>825.9004722203405</v>
+        <v>1968.5</v>
       </c>
       <c r="AA7" t="n">
         <v>6.083861780229042e-07</v>
@@ -6238,19 +7850,19 @@
       <c r="K8" t="n">
         <v>68.86571051610399</v>
       </c>
-      <c r="W8" t="n">
-        <v>7</v>
-      </c>
-      <c r="X8" t="inlineStr">
+      <c r="W8" t="inlineStr">
         <is>
           <t>y = 2.587x + -45235.986</t>
         </is>
+      </c>
+      <c r="X8" t="n">
+        <v>-45235.98649035033</v>
       </c>
       <c r="Y8" t="n">
         <v>1034.012317430827</v>
       </c>
       <c r="Z8" t="n">
-        <v>813.2709220478805</v>
+        <v>1958.599999999999</v>
       </c>
       <c r="AA8" t="n">
         <v>6.070105779354064e-07</v>
@@ -6290,19 +7902,19 @@
       <c r="K9" t="n">
         <v>69.12960456163179</v>
       </c>
-      <c r="W9" t="n">
-        <v>8</v>
-      </c>
-      <c r="X9" t="inlineStr">
+      <c r="W9" t="inlineStr">
         <is>
           <t>y = 2.623x + -45376.592</t>
         </is>
+      </c>
+      <c r="X9" t="n">
+        <v>-45376.59162594052</v>
       </c>
       <c r="Y9" t="n">
         <v>1032.644189121561</v>
       </c>
       <c r="Z9" t="n">
-        <v>812.2355099879258</v>
+        <v>1927.5</v>
       </c>
       <c r="AA9" t="n">
         <v>6.128409756477646e-07</v>
@@ -6342,19 +7954,19 @@
       <c r="K10" t="n">
         <v>69.22144833149954</v>
       </c>
-      <c r="W10" t="n">
-        <v>9</v>
-      </c>
-      <c r="X10" t="inlineStr">
+      <c r="W10" t="inlineStr">
         <is>
           <t>y = 2.635x + -45061.159</t>
         </is>
+      </c>
+      <c r="X10" t="n">
+        <v>-45061.15871900824</v>
       </c>
       <c r="Y10" t="n">
         <v>1054.766489828831</v>
       </c>
       <c r="Z10" t="n">
-        <v>829.4637197581885</v>
+        <v>1911.800000000003</v>
       </c>
       <c r="AA10" t="n">
         <v>6.296471027099854e-07</v>
@@ -6394,19 +8006,19 @@
       <c r="K11" t="n">
         <v>69.27583805023222</v>
       </c>
-      <c r="W11" t="n">
-        <v>10</v>
-      </c>
-      <c r="X11" t="inlineStr">
+      <c r="W11" t="inlineStr">
         <is>
           <t>y = 2.643x + -44681.577</t>
         </is>
+      </c>
+      <c r="X11" t="n">
+        <v>-44681.57681083908</v>
       </c>
       <c r="Y11" t="n">
         <v>1039.18120141719</v>
       </c>
       <c r="Z11" t="n">
-        <v>817.3672774843495</v>
+        <v>1900.5</v>
       </c>
       <c r="AA11" t="n">
         <v>6.282777388457208e-07</v>
@@ -6532,12 +8144,12 @@
       </c>
       <c r="W1" t="inlineStr">
         <is>
-          <t>Cycle</t>
+          <t>Model</t>
         </is>
       </c>
       <c r="X1" t="inlineStr">
         <is>
-          <t>Model</t>
+          <t>b</t>
         </is>
       </c>
       <c r="Y1" t="inlineStr">
@@ -6547,7 +8159,7 @@
       </c>
       <c r="Z1" t="inlineStr">
         <is>
-          <t>Rp</t>
+          <t>delta Rct-i</t>
         </is>
       </c>
       <c r="AA1" t="inlineStr">
@@ -6592,19 +8204,19 @@
       <c r="K2" t="n">
         <v>81.92598843870702</v>
       </c>
-      <c r="W2" t="n">
-        <v>1</v>
-      </c>
-      <c r="X2" t="inlineStr">
+      <c r="W2" t="inlineStr">
         <is>
           <t>y = 7.049x + -25240.866</t>
         </is>
+      </c>
+      <c r="X2" t="n">
+        <v>-25240.86560628705</v>
       </c>
       <c r="Y2" t="n">
         <v>6.270757693317334e-11</v>
       </c>
       <c r="Z2" t="n">
-        <v>4205.884890064634</v>
+        <v>689.3400000000001</v>
       </c>
       <c r="AA2" t="n">
         <v>1.000000000000227e-08</v>
@@ -6644,19 +8256,19 @@
       <c r="K3" t="n">
         <v>82.52186782671926</v>
       </c>
-      <c r="W3" t="n">
-        <v>2</v>
-      </c>
-      <c r="X3" t="inlineStr">
+      <c r="W3" t="inlineStr">
         <is>
           <t>y = 7.618x + -25918.451</t>
         </is>
+      </c>
+      <c r="X3" t="n">
+        <v>-25918.45067978542</v>
       </c>
       <c r="Y3" t="n">
         <v>1.366125040588221e-09</v>
       </c>
       <c r="Z3" t="n">
-        <v>4006.036155422891</v>
+        <v>622.9000000000001</v>
       </c>
       <c r="AA3" t="n">
         <v>1.000000000001866e-08</v>
@@ -6696,19 +8308,19 @@
       <c r="K4" t="n">
         <v>82.19585679206008</v>
       </c>
-      <c r="W4" t="n">
-        <v>3</v>
-      </c>
-      <c r="X4" t="inlineStr">
+      <c r="W4" t="inlineStr">
         <is>
           <t>y = 7.296x + -24256.194</t>
         </is>
+      </c>
+      <c r="X4" t="n">
+        <v>-24256.1941018422</v>
       </c>
       <c r="Y4" t="n">
         <v>1.090156318120623e-10</v>
       </c>
       <c r="Z4" t="n">
-        <v>3935.821912233584</v>
+        <v>637.5699999999997</v>
       </c>
       <c r="AA4" t="n">
         <v>1.00000000000013e-08</v>
@@ -6748,19 +8360,19 @@
       <c r="K5" t="n">
         <v>82.58540269535408</v>
       </c>
-      <c r="W5" t="n">
-        <v>4</v>
-      </c>
-      <c r="X5" t="inlineStr">
+      <c r="W5" t="inlineStr">
         <is>
           <t>y = 7.684x + -25357.761</t>
         </is>
+      </c>
+      <c r="X5" t="n">
+        <v>-25357.76128331328</v>
       </c>
       <c r="Y5" t="n">
         <v>1.062312420446039e-09</v>
       </c>
       <c r="Z5" t="n">
-        <v>3883.031795920439</v>
+        <v>610.0599999999999</v>
       </c>
       <c r="AA5" t="n">
         <v>1.000000000003094e-08</v>
@@ -6800,19 +8412,19 @@
       <c r="K6" t="n">
         <v>82.33371852200311</v>
       </c>
-      <c r="W6" t="n">
-        <v>5</v>
-      </c>
-      <c r="X6" t="inlineStr">
+      <c r="W6" t="inlineStr">
         <is>
           <t>y = 7.429x + -24112.986</t>
         </is>
+      </c>
+      <c r="X6" t="n">
+        <v>-24112.9860223846</v>
       </c>
       <c r="Y6" t="n">
         <v>8.118152899628944e-10</v>
       </c>
       <c r="Z6" t="n">
-        <v>3835.022553553898</v>
+        <v>620.27</v>
       </c>
       <c r="AA6" t="n">
         <v>1.000000000085918e-08</v>
@@ -6852,19 +8464,19 @@
       <c r="K7" t="n">
         <v>82.34583155799149</v>
       </c>
-      <c r="W7" t="n">
-        <v>6</v>
-      </c>
-      <c r="X7" t="inlineStr">
+      <c r="W7" t="inlineStr">
         <is>
           <t>y = 7.441x + -23880.978</t>
         </is>
+      </c>
+      <c r="X7" t="n">
+        <v>-23880.97846679137</v>
       </c>
       <c r="Y7" t="n">
         <v>5.527629492869572e-09</v>
       </c>
       <c r="Z7" t="n">
-        <v>3789.242727888626</v>
+        <v>617.1799999999998</v>
       </c>
       <c r="AA7" t="n">
         <v>1.000000000001076e-08</v>
@@ -6904,19 +8516,19 @@
       <c r="K8" t="n">
         <v>82.44111830493971</v>
       </c>
-      <c r="W8" t="n">
-        <v>7</v>
-      </c>
-      <c r="X8" t="inlineStr">
+      <c r="W8" t="inlineStr">
         <is>
           <t>y = 7.536x + -23942.900</t>
         </is>
+      </c>
+      <c r="X8" t="n">
+        <v>-23942.89984628868</v>
       </c>
       <c r="Y8" t="n">
         <v>1.841086815799093e-18</v>
       </c>
       <c r="Z8" t="n">
-        <v>3746.924357180184</v>
+        <v>605.4100000000003</v>
       </c>
       <c r="AA8" t="n">
         <v>1e-08</v>
@@ -6956,19 +8568,19 @@
       <c r="K9" t="n">
         <v>82.11554340852989</v>
       </c>
-      <c r="W9" t="n">
-        <v>8</v>
-      </c>
-      <c r="X9" t="inlineStr">
+      <c r="W9" t="inlineStr">
         <is>
           <t>y = 7.221x + -22608.239</t>
         </is>
+      </c>
+      <c r="X9" t="n">
+        <v>-22608.23938092466</v>
       </c>
       <c r="Y9" t="n">
         <v>5.253107119837181e-09</v>
       </c>
       <c r="Z9" t="n">
-        <v>3707.706541242992</v>
+        <v>625.48</v>
       </c>
       <c r="AA9" t="n">
         <v>1.000000000000546e-08</v>
@@ -7008,19 +8620,19 @@
       <c r="K10" t="n">
         <v>82.46241860074358</v>
       </c>
-      <c r="W10" t="n">
-        <v>9</v>
-      </c>
-      <c r="X10" t="inlineStr">
+      <c r="W10" t="inlineStr">
         <is>
           <t>y = 7.557x + -23554.239</t>
         </is>
+      </c>
+      <c r="X10" t="n">
+        <v>-23554.23940132603</v>
       </c>
       <c r="Y10" t="n">
         <v>1.065173126294553e-09</v>
       </c>
       <c r="Z10" t="n">
-        <v>3671.700118648755</v>
+        <v>607.4200000000001</v>
       </c>
       <c r="AA10" t="n">
         <v>1.000000000003668e-08</v>
@@ -7060,19 +8672,19 @@
       <c r="K11" t="n">
         <v>82.25373176874217</v>
       </c>
-      <c r="W11" t="n">
-        <v>10</v>
-      </c>
-      <c r="X11" t="inlineStr">
+      <c r="W11" t="inlineStr">
         <is>
           <t>y = 7.351x + -22608.792</t>
         </is>
+      </c>
+      <c r="X11" t="n">
+        <v>-22608.79222095496</v>
       </c>
       <c r="Y11" t="n">
         <v>1.443028795686406e-11</v>
       </c>
       <c r="Z11" t="n">
-        <v>3636.999587679381</v>
+        <v>607.5099999999998</v>
       </c>
       <c r="AA11" t="n">
         <v>1e-08</v>
@@ -7112,19 +8724,19 @@
       <c r="K12" t="n">
         <v>82.70205581033102</v>
       </c>
-      <c r="W12" t="n">
-        <v>11</v>
-      </c>
-      <c r="X12" t="inlineStr">
+      <c r="W12" t="inlineStr">
         <is>
           <t>y = 7.808x + -23927.933</t>
         </is>
+      </c>
+      <c r="X12" t="n">
+        <v>-23927.93281765433</v>
       </c>
       <c r="Y12" t="n">
         <v>6.340449691658653e-09</v>
       </c>
       <c r="Z12" t="n">
-        <v>3601.486744222801</v>
+        <v>580.0799999999999</v>
       </c>
       <c r="AA12" t="n">
         <v>1.000000000000003e-08</v>
@@ -7164,19 +8776,19 @@
       <c r="K13" t="n">
         <v>82.74905240944111</v>
       </c>
-      <c r="W13" t="n">
-        <v>12</v>
-      </c>
-      <c r="X13" t="inlineStr">
+      <c r="W13" t="inlineStr">
         <is>
           <t>y = 7.860x + -23877.651</t>
         </is>
+      </c>
+      <c r="X13" t="n">
+        <v>-23877.65084057717</v>
       </c>
       <c r="Y13" t="n">
         <v>2.483823806000081e-09</v>
       </c>
       <c r="Z13" t="n">
-        <v>3567.391755983299</v>
+        <v>573.3999999999996</v>
       </c>
       <c r="AA13" t="n">
         <v>1.00000000000465e-08</v>
@@ -7216,19 +8828,19 @@
       <c r="K14" t="n">
         <v>82.86281829493637</v>
       </c>
-      <c r="W14" t="n">
-        <v>13</v>
-      </c>
-      <c r="X14" t="inlineStr">
+      <c r="W14" t="inlineStr">
         <is>
           <t>y = 7.986x + -24035.146</t>
         </is>
+      </c>
+      <c r="X14" t="n">
+        <v>-24035.14571194406</v>
       </c>
       <c r="Y14" t="n">
         <v>8.260371997464482e-10</v>
       </c>
       <c r="Z14" t="n">
-        <v>3530.136990515655</v>
+        <v>562.2199999999998</v>
       </c>
       <c r="AA14" t="n">
         <v>1.00000000000052e-08</v>
@@ -7268,19 +8880,19 @@
       <c r="K15" t="n">
         <v>82.94103451587154</v>
       </c>
-      <c r="W15" t="n">
-        <v>14</v>
-      </c>
-      <c r="X15" t="inlineStr">
+      <c r="W15" t="inlineStr">
         <is>
           <t>y = 8.076x + -24077.967</t>
         </is>
+      </c>
+      <c r="X15" t="n">
+        <v>-24077.96734353064</v>
       </c>
       <c r="Y15" t="n">
         <v>1.045967857513008e-08</v>
       </c>
       <c r="Z15" t="n">
-        <v>3494.753960988774</v>
+        <v>555.21</v>
       </c>
       <c r="AA15" t="n">
         <v>1.000000000000096e-08</v>
@@ -7320,19 +8932,19 @@
       <c r="K16" t="n">
         <v>83.0375652473957</v>
       </c>
-      <c r="W16" t="n">
-        <v>15</v>
-      </c>
-      <c r="X16" t="inlineStr">
+      <c r="W16" t="inlineStr">
         <is>
           <t>y = 8.189x + -24198.237</t>
         </is>
+      </c>
+      <c r="X16" t="n">
+        <v>-24198.23749121563</v>
       </c>
       <c r="Y16" t="n">
         <v>1.948108843070904e-11</v>
       </c>
       <c r="Z16" t="n">
-        <v>3458.818557263857</v>
+        <v>546.6100000000001</v>
       </c>
       <c r="AA16" t="n">
         <v>1e-08</v>
@@ -7372,19 +8984,19 @@
       <c r="K17" t="n">
         <v>82.79544935182111</v>
       </c>
-      <c r="W17" t="n">
-        <v>16</v>
-      </c>
-      <c r="X17" t="inlineStr">
+      <c r="W17" t="inlineStr">
         <is>
           <t>y = 7.911x + -23037.618</t>
         </is>
+      </c>
+      <c r="X17" t="n">
+        <v>-23037.61815999198</v>
       </c>
       <c r="Y17" t="n">
         <v>1.043567252003006e-10</v>
       </c>
       <c r="Z17" t="n">
-        <v>3422.892343149957</v>
+        <v>557.5999999999999</v>
       </c>
       <c r="AA17" t="n">
         <v>1.000000000000179e-08</v>
@@ -7424,19 +9036,19 @@
       <c r="K18" t="n">
         <v>83.14318054784211</v>
       </c>
-      <c r="W18" t="n">
-        <v>17</v>
-      </c>
-      <c r="X18" t="inlineStr">
+      <c r="W18" t="inlineStr">
         <is>
           <t>y = 8.316x + -24101.993</t>
         </is>
+      </c>
+      <c r="X18" t="n">
+        <v>-24101.99252541294</v>
       </c>
       <c r="Y18" t="n">
         <v>9.423737355848379e-10</v>
       </c>
       <c r="Z18" t="n">
-        <v>3386.592759906148</v>
+        <v>540.46</v>
       </c>
       <c r="AA18" t="n">
         <v>1.000000000013627e-08</v>
@@ -7476,19 +9088,19 @@
       <c r="K19" t="n">
         <v>83.23921478381426</v>
       </c>
-      <c r="W19" t="n">
-        <v>18</v>
-      </c>
-      <c r="X19" t="inlineStr">
+      <c r="W19" t="inlineStr">
         <is>
           <t>y = 8.435x + -24210.426</t>
         </is>
+      </c>
+      <c r="X19" t="n">
+        <v>-24210.42648286345</v>
       </c>
       <c r="Y19" t="n">
         <v>7.560569546736046e-10</v>
       </c>
       <c r="Z19" t="n">
-        <v>3350.73296563084</v>
+        <v>529.46</v>
       </c>
       <c r="AA19" t="n">
         <v>1.000000000000281e-08</v>
@@ -7528,19 +9140,19 @@
       <c r="K20" t="n">
         <v>83.08193209915974</v>
       </c>
-      <c r="W20" t="n">
-        <v>19</v>
-      </c>
-      <c r="X20" t="inlineStr">
+      <c r="W20" t="inlineStr">
         <is>
           <t>y = 8.242x + -23325.088</t>
         </is>
+      </c>
+      <c r="X20" t="n">
+        <v>-23325.0883676794</v>
       </c>
       <c r="Y20" t="n">
         <v>8.443247870371154e-10</v>
       </c>
       <c r="Z20" t="n">
-        <v>3315.237452897345</v>
+        <v>533.9000000000001</v>
       </c>
       <c r="AA20" t="n">
         <v>1.00000000000028e-08</v>
@@ -7580,19 +9192,19 @@
       <c r="K21" t="n">
         <v>83.46426574963074</v>
       </c>
-      <c r="W21" t="n">
-        <v>20</v>
-      </c>
-      <c r="X21" t="inlineStr">
+      <c r="W21" t="inlineStr">
         <is>
           <t>y = 8.728x + -24580.988</t>
         </is>
+      </c>
+      <c r="X21" t="n">
+        <v>-24580.98805300962</v>
       </c>
       <c r="Y21" t="n">
         <v>1.059451165241389e-09</v>
       </c>
       <c r="Z21" t="n">
-        <v>3280.066896952231</v>
+        <v>510.9400000000001</v>
       </c>
       <c r="AA21" t="n">
         <v>1.000000000000019e-08</v>
@@ -7632,19 +9244,19 @@
       <c r="K22" t="n">
         <v>83.20923398910719</v>
       </c>
-      <c r="W22" t="n">
-        <v>21</v>
-      </c>
-      <c r="X22" t="inlineStr">
+      <c r="W22" t="inlineStr">
         <is>
           <t>y = 8.398x + -23311.864</t>
         </is>
+      </c>
+      <c r="X22" t="n">
+        <v>-23311.86417902619</v>
       </c>
       <c r="Y22" t="n">
         <v>5.943266053885061e-11</v>
       </c>
       <c r="Z22" t="n">
-        <v>3244.75084351878</v>
+        <v>520.3700000000003</v>
       </c>
       <c r="AA22" t="n">
         <v>1.000000000000284e-08</v>
@@ -7770,12 +9382,12 @@
       </c>
       <c r="W1" t="inlineStr">
         <is>
-          <t>Cycle</t>
+          <t>Model</t>
         </is>
       </c>
       <c r="X1" t="inlineStr">
         <is>
-          <t>Model</t>
+          <t>b</t>
         </is>
       </c>
       <c r="Y1" t="inlineStr">
@@ -7785,7 +9397,7 @@
       </c>
       <c r="Z1" t="inlineStr">
         <is>
-          <t>Rp</t>
+          <t>delta Rct-i</t>
         </is>
       </c>
       <c r="AA1" t="inlineStr">
@@ -7830,19 +9442,19 @@
       <c r="K2" t="n">
         <v>14.04836917377372</v>
       </c>
-      <c r="W2" t="n">
-        <v>1</v>
-      </c>
-      <c r="X2" t="inlineStr">
+      <c r="W2" t="inlineStr">
         <is>
           <t>y = 0.250x + 1473.925</t>
         </is>
+      </c>
+      <c r="X2" t="n">
+        <v>1473.924585948794</v>
       </c>
       <c r="Y2" t="n">
         <v>1401.196004579856</v>
       </c>
       <c r="Z2" t="n">
-        <v>1631.18191604417</v>
+        <v>7685.355</v>
       </c>
       <c r="AA2" t="n">
         <v>1.051011123548062e-06</v>
@@ -7882,19 +9494,19 @@
       <c r="K3" t="n">
         <v>12.42863116636923</v>
       </c>
-      <c r="W3" t="n">
-        <v>2</v>
-      </c>
-      <c r="X3" t="inlineStr">
+      <c r="W3" t="inlineStr">
         <is>
           <t>y = 0.220x + 1422.857</t>
         </is>
+      </c>
+      <c r="X3" t="n">
+        <v>1422.856753080394</v>
       </c>
       <c r="Y3" t="n">
         <v>1347.116838125768</v>
       </c>
       <c r="Z3" t="n">
-        <v>1908.251136774144</v>
+        <v>6655.179999999999</v>
       </c>
       <c r="AA3" t="n">
         <v>1.08770333002106e-06</v>
@@ -7934,19 +9546,19 @@
       <c r="K4" t="n">
         <v>11.98989350002953</v>
       </c>
-      <c r="W4" t="n">
-        <v>3</v>
-      </c>
-      <c r="X4" t="inlineStr">
+      <c r="W4" t="inlineStr">
         <is>
           <t>y = 0.212x + 1403.473</t>
         </is>
+      </c>
+      <c r="X4" t="n">
+        <v>1403.472960239763</v>
       </c>
       <c r="Y4" t="n">
         <v>1332.669021893373</v>
       </c>
       <c r="Z4" t="n">
-        <v>1978.149661239184</v>
+        <v>6413.009999999999</v>
       </c>
       <c r="AA4" t="n">
         <v>4.270518337465608e-07</v>
@@ -7986,19 +9598,19 @@
       <c r="K5" t="n">
         <v>80.32331536215419</v>
       </c>
-      <c r="W5" t="n">
-        <v>4</v>
-      </c>
-      <c r="X5" t="inlineStr">
+      <c r="W5" t="inlineStr">
         <is>
           <t>y = 5.865x + -32709.549</t>
         </is>
+      </c>
+      <c r="X5" t="n">
+        <v>-32709.54889527945</v>
       </c>
       <c r="Y5" t="n">
         <v>1326.417365955968</v>
       </c>
       <c r="Z5" t="n">
-        <v>1998.175729126543</v>
+        <v>870.4200000000001</v>
       </c>
       <c r="AA5" t="n">
         <v>6.826957621136403e-07</v>
@@ -8038,19 +9650,19 @@
       <c r="K6" t="n">
         <v>80.35829297873626</v>
       </c>
-      <c r="W6" t="n">
-        <v>5</v>
-      </c>
-      <c r="X6" t="inlineStr">
+      <c r="W6" t="inlineStr">
         <is>
           <t>y = 5.886x + -32337.579</t>
         </is>
+      </c>
+      <c r="X6" t="n">
+        <v>-32337.57892839805</v>
       </c>
       <c r="Y6" t="n">
         <v>1320.827331146576</v>
       </c>
       <c r="Z6" t="n">
-        <v>2033.248541069018</v>
+        <v>864.4000000000005</v>
       </c>
       <c r="AA6" t="n">
         <v>7.760050573478072e-07</v>
@@ -8090,19 +9702,19 @@
       <c r="K7" t="n">
         <v>80.39969583627452</v>
       </c>
-      <c r="W7" t="n">
-        <v>6</v>
-      </c>
-      <c r="X7" t="inlineStr">
+      <c r="W7" t="inlineStr">
         <is>
           <t>y = 5.912x + -32085.271</t>
         </is>
+      </c>
+      <c r="X7" t="n">
+        <v>-32085.27061135535</v>
       </c>
       <c r="Y7" t="n">
         <v>1315.908761296211</v>
       </c>
       <c r="Z7" t="n">
-        <v>2022.189329838532</v>
+        <v>858.6799999999994</v>
       </c>
       <c r="AA7" t="n">
         <v>7.749964132148386e-07</v>
@@ -8142,19 +9754,19 @@
       <c r="K8" t="n">
         <v>80.53824382515876</v>
       </c>
-      <c r="W8" t="n">
-        <v>7</v>
-      </c>
-      <c r="X8" t="inlineStr">
+      <c r="W8" t="inlineStr">
         <is>
           <t>y = 6.000x + -32163.559</t>
         </is>
+      </c>
+      <c r="X8" t="n">
+        <v>-32163.55918792906</v>
       </c>
       <c r="Y8" t="n">
         <v>1307.59177113655</v>
       </c>
       <c r="Z8" t="n">
-        <v>2080.286576406515</v>
+        <v>839.7600000000002</v>
       </c>
       <c r="AA8" t="n">
         <v>6.154688151701993e-07</v>
@@ -8194,19 +9806,19 @@
       <c r="K9" t="n">
         <v>80.6858002155312</v>
       </c>
-      <c r="W9" t="n">
-        <v>8</v>
-      </c>
-      <c r="X9" t="inlineStr">
+      <c r="W9" t="inlineStr">
         <is>
           <t>y = 6.097x + -32317.318</t>
         </is>
+      </c>
+      <c r="X9" t="n">
+        <v>-32317.31811041562</v>
       </c>
       <c r="Y9" t="n">
         <v>1280.492410046041</v>
       </c>
       <c r="Z9" t="n">
-        <v>2085.27265334374</v>
+        <v>828.3000000000002</v>
       </c>
       <c r="AA9" t="n">
         <v>3.492951438614063e-07</v>
@@ -8246,19 +9858,19 @@
       <c r="K10" t="n">
         <v>80.56235710207405</v>
       </c>
-      <c r="W10" t="n">
-        <v>9</v>
-      </c>
-      <c r="X10" t="inlineStr">
+      <c r="W10" t="inlineStr">
         <is>
           <t>y = 6.016x + -31493.670</t>
         </is>
+      </c>
+      <c r="X10" t="n">
+        <v>-31493.67015169379</v>
       </c>
       <c r="Y10" t="n">
         <v>1274.975530408735</v>
       </c>
       <c r="Z10" t="n">
-        <v>2094.781360184912</v>
+        <v>834.3899999999994</v>
       </c>
       <c r="AA10" t="n">
         <v>3.42099152654186e-07</v>
@@ -8298,19 +9910,19 @@
       <c r="K11" t="n">
         <v>80.67249240768061</v>
       </c>
-      <c r="W11" t="n">
-        <v>10</v>
-      </c>
-      <c r="X11" t="inlineStr">
+      <c r="W11" t="inlineStr">
         <is>
           <t>y = 6.088x + -31522.520</t>
         </is>
+      </c>
+      <c r="X11" t="n">
+        <v>-31522.51990936588</v>
       </c>
       <c r="Y11" t="n">
         <v>1268.580589533905</v>
       </c>
       <c r="Z11" t="n">
-        <v>2113.911687240773</v>
+        <v>823.4700000000003</v>
       </c>
       <c r="AA11" t="n">
         <v>3.320901754157028e-07</v>

</xml_diff>

<commit_message>
added the time vs slope and Rct graphs for each concentration
</commit_message>
<xml_diff>
--- a/BioSensorAnalysisSrcCode/EIS_Analysis/Austin_EIS/MegaExcel/Processed Chips for PCAI1ia/Chip 21.xlsx
+++ b/BioSensorAnalysisSrcCode/EIS_Analysis/Austin_EIS/MegaExcel/Processed Chips for PCAI1ia/Chip 21.xlsx
@@ -528,12 +528,12 @@
       </c>
       <c r="W1" t="inlineStr">
         <is>
-          <t>Model</t>
+          <t>linear_eq_m</t>
         </is>
       </c>
       <c r="X1" t="inlineStr">
         <is>
-          <t>b</t>
+          <t>linear_eq_b</t>
         </is>
       </c>
       <c r="Y1" t="inlineStr">
@@ -588,10 +588,8 @@
       <c r="K2" t="n">
         <v>81.93371453681854</v>
       </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>y = 7.056x + -25925.977</t>
-        </is>
+      <c r="W2" t="n">
+        <v>7.056128382896103</v>
       </c>
       <c r="X2" t="n">
         <v>-25925.97725441957</v>
@@ -600,7 +598,7 @@
         <v>3.973360418002409e-09</v>
       </c>
       <c r="Z2" t="n">
-        <v>604.1999999999998</v>
+        <v>4338.281983477777</v>
       </c>
       <c r="AA2" t="n">
         <v>1.000000000002033e-08</v>
@@ -640,10 +638,8 @@
       <c r="K3" t="n">
         <v>82.56790490797303</v>
       </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>y = 7.666x + -27402.847</t>
-        </is>
+      <c r="W3" t="n">
+        <v>7.665949846301568</v>
       </c>
       <c r="X3" t="n">
         <v>-27402.84736786969</v>
@@ -652,7 +648,7 @@
         <v>1.897271783591817e-18</v>
       </c>
       <c r="Z3" t="n">
-        <v>559.77</v>
+        <v>4211.914002274965</v>
       </c>
       <c r="AA3" t="n">
         <v>1e-08</v>
@@ -692,10 +688,8 @@
       <c r="K4" t="n">
         <v>82.86147480804301</v>
       </c>
-      <c r="W4" t="inlineStr">
-        <is>
-          <t>y = 7.985x + -27984.201</t>
-        </is>
+      <c r="W4" t="n">
+        <v>7.984703555408088</v>
       </c>
       <c r="X4" t="n">
         <v>-27984.20086789379</v>
@@ -704,7 +698,7 @@
         <v>1.274334709434572e-10</v>
       </c>
       <c r="Z4" t="n">
-        <v>540.23</v>
+        <v>4123.658205090058</v>
       </c>
       <c r="AA4" t="n">
         <v>1.000000000000405e-08</v>
@@ -744,10 +738,8 @@
       <c r="K5" t="n">
         <v>83.23250269088234</v>
       </c>
-      <c r="W5" t="inlineStr">
-        <is>
-          <t>y = 8.427x + -29046.995</t>
-        </is>
+      <c r="W5" t="n">
+        <v>8.426908924262568</v>
       </c>
       <c r="X5" t="n">
         <v>-29046.99463667542</v>
@@ -756,7 +748,7 @@
         <v>1.579012405788227e-10</v>
       </c>
       <c r="Z5" t="n">
-        <v>512.1300000000001</v>
+        <v>4045.209555784623</v>
       </c>
       <c r="AA5" t="n">
         <v>1.00000000000001e-08</v>
@@ -796,10 +788,8 @@
       <c r="K6" t="n">
         <v>83.34227232969749</v>
       </c>
-      <c r="W6" t="inlineStr">
-        <is>
-          <t>y = 8.567x + -29058.639</t>
-        </is>
+      <c r="W6" t="n">
+        <v>8.567138151478588</v>
       </c>
       <c r="X6" t="n">
         <v>-29058.63871125671</v>
@@ -808,7 +798,7 @@
         <v>4.911906337866607e-10</v>
       </c>
       <c r="Z6" t="n">
-        <v>504.75</v>
+        <v>3976.629059890452</v>
       </c>
       <c r="AA6" t="n">
         <v>1.000000000000073e-08</v>
@@ -848,10 +838,8 @@
       <c r="K7" t="n">
         <v>83.48385721504475</v>
       </c>
-      <c r="W7" t="inlineStr">
-        <is>
-          <t>y = 8.755x + -29264.941</t>
-        </is>
+      <c r="W7" t="n">
+        <v>8.754955989400166</v>
       </c>
       <c r="X7" t="n">
         <v>-29264.9409855333</v>
@@ -860,7 +848,7 @@
         <v>1.123012009317532e-16</v>
       </c>
       <c r="Z7" t="n">
-        <v>493.4400000000001</v>
+        <v>3915.936364038092</v>
       </c>
       <c r="AA7" t="n">
         <v>1e-08</v>
@@ -900,10 +888,8 @@
       <c r="K8" t="n">
         <v>83.2328377728806</v>
       </c>
-      <c r="W8" t="inlineStr">
-        <is>
-          <t>y = 8.427x + -27659.995</t>
-        </is>
+      <c r="W8" t="n">
+        <v>8.427330096299851</v>
       </c>
       <c r="X8" t="n">
         <v>-27659.99456902865</v>
@@ -912,7 +898,7 @@
         <v>5.529700177760481e-12</v>
       </c>
       <c r="Z8" t="n">
-        <v>496.9099999999999</v>
+        <v>3860.964985101534</v>
       </c>
       <c r="AA8" t="n">
         <v>1.000000000000038e-08</v>
@@ -952,10 +938,8 @@
       <c r="K9" t="n">
         <v>83.38119694298761</v>
       </c>
-      <c r="W9" t="inlineStr">
-        <is>
-          <t>y = 8.618x + -27949.070</t>
-        </is>
+      <c r="W9" t="n">
+        <v>8.617975811175112</v>
       </c>
       <c r="X9" t="n">
         <v>-27949.07001255509</v>
@@ -964,7 +948,7 @@
         <v>3.952318134702614e-09</v>
       </c>
       <c r="Z9" t="n">
-        <v>489.0599999999999</v>
+        <v>3810.555620282222</v>
       </c>
       <c r="AA9" t="n">
         <v>1.000000000014565e-08</v>
@@ -1004,10 +988,8 @@
       <c r="K10" t="n">
         <v>83.54601674051274</v>
       </c>
-      <c r="W10" t="inlineStr">
-        <is>
-          <t>y = 8.840x + -28364.159</t>
-        </is>
+      <c r="W10" t="n">
+        <v>8.840004601098626</v>
       </c>
       <c r="X10" t="n">
         <v>-28364.1585730412</v>
@@ -1016,7 +998,7 @@
         <v>8.695782116767691e-09</v>
       </c>
       <c r="Z10" t="n">
-        <v>477.1399999999999</v>
+        <v>3764.259433155244</v>
       </c>
       <c r="AA10" t="n">
         <v>1.000000000000013e-08</v>
@@ -1056,10 +1038,8 @@
       <c r="K11" t="n">
         <v>83.98408608789487</v>
       </c>
-      <c r="W11" t="inlineStr">
-        <is>
-          <t>y = 9.489x + -30286.635</t>
-        </is>
+      <c r="W11" t="n">
+        <v>9.489010888761005</v>
       </c>
       <c r="X11" t="n">
         <v>-30286.63477810142</v>
@@ -1068,7 +1048,7 @@
         <v>7.399923275621092e-09</v>
       </c>
       <c r="Z11" t="n">
-        <v>455.8200000000002</v>
+        <v>3722.293840317449</v>
       </c>
       <c r="AA11" t="n">
         <v>1.000000000000328e-08</v>
@@ -1194,12 +1174,12 @@
       </c>
       <c r="W1" t="inlineStr">
         <is>
-          <t>Model</t>
+          <t>linear_eq_m</t>
         </is>
       </c>
       <c r="X1" t="inlineStr">
         <is>
-          <t>b</t>
+          <t>linear_eq_b</t>
         </is>
       </c>
       <c r="Y1" t="inlineStr">
@@ -1254,10 +1234,8 @@
       <c r="K2" t="n">
         <v>83.03716034820951</v>
       </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>y = 8.188x + -28805.250</t>
-        </is>
+      <c r="W2" t="n">
+        <v>8.188246816501445</v>
       </c>
       <c r="X2" t="n">
         <v>-28805.24954287466</v>
@@ -1266,7 +1244,7 @@
         <v>3.461751648758845e-09</v>
       </c>
       <c r="Z2" t="n">
-        <v>570.52</v>
+        <v>4126.568694892875</v>
       </c>
       <c r="AA2" t="n">
         <v>1.000000000000682e-08</v>
@@ -1306,10 +1284,8 @@
       <c r="K3" t="n">
         <v>82.77928794294931</v>
       </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>y = 7.893x + -26594.526</t>
-        </is>
+      <c r="W3" t="n">
+        <v>7.892868022291462</v>
       </c>
       <c r="X3" t="n">
         <v>-26594.52615563833</v>
@@ -1318,7 +1294,7 @@
         <v>1.945267163618647e-08</v>
       </c>
       <c r="Z3" t="n">
-        <v>576.1600000000003</v>
+        <v>3984.43311368162</v>
       </c>
       <c r="AA3" t="n">
         <v>1.000000000000073e-08</v>
@@ -1358,10 +1334,8 @@
       <c r="K4" t="n">
         <v>83.15696832756892</v>
       </c>
-      <c r="W4" t="inlineStr">
-        <is>
-          <t>y = 8.333x + -27815.874</t>
-        </is>
+      <c r="W4" t="n">
+        <v>8.333015818065139</v>
       </c>
       <c r="X4" t="n">
         <v>-27815.87381972411</v>
@@ -1370,7 +1344,7 @@
         <v>9.744149832265997e-15</v>
       </c>
       <c r="Z4" t="n">
-        <v>551.21</v>
+        <v>3924.695747861717</v>
       </c>
       <c r="AA4" t="n">
         <v>1.000000000000394e-08</v>
@@ -1410,10 +1384,8 @@
       <c r="K5" t="n">
         <v>82.85600964996303</v>
       </c>
-      <c r="W5" t="inlineStr">
-        <is>
-          <t>y = 7.979x + -26194.989</t>
-        </is>
+      <c r="W5" t="n">
+        <v>7.978531553448255</v>
       </c>
       <c r="X5" t="n">
         <v>-26194.98924499944</v>
@@ -1422,7 +1394,7 @@
         <v>2.041724315974994e-15</v>
       </c>
       <c r="Z5" t="n">
-        <v>560.8499999999999</v>
+        <v>3877.998216129423</v>
       </c>
       <c r="AA5" t="n">
         <v>1e-08</v>
@@ -1462,10 +1434,8 @@
       <c r="K6" t="n">
         <v>82.54954797767374</v>
       </c>
-      <c r="W6" t="inlineStr">
-        <is>
-          <t>y = 7.647x + -24734.360</t>
-        </is>
+      <c r="W6" t="n">
+        <v>7.646848147423739</v>
       </c>
       <c r="X6" t="n">
         <v>-24734.36023161278</v>
@@ -1474,7 +1444,7 @@
         <v>2.64856299099321e-10</v>
       </c>
       <c r="Z6" t="n">
-        <v>574.8999999999996</v>
+        <v>3835.907573896849</v>
       </c>
       <c r="AA6" t="n">
         <v>1.000000000000014e-08</v>
@@ -1514,10 +1484,8 @@
       <c r="K7" t="n">
         <v>82.98278493842304</v>
       </c>
-      <c r="W7" t="inlineStr">
-        <is>
-          <t>y = 8.124x + -26162.317</t>
-        </is>
+      <c r="W7" t="n">
+        <v>8.124165758103105</v>
       </c>
       <c r="X7" t="n">
         <v>-26162.31709657338</v>
@@ -1526,7 +1494,7 @@
         <v>3.845840421510457e-10</v>
       </c>
       <c r="Z7" t="n">
-        <v>546.5799999999999</v>
+        <v>3796.855465673337</v>
       </c>
       <c r="AA7" t="n">
         <v>1.000000000000006e-08</v>
@@ -1566,10 +1534,8 @@
       <c r="K8" t="n">
         <v>83.04933641167069</v>
       </c>
-      <c r="W8" t="inlineStr">
-        <is>
-          <t>y = 8.203x + -26167.616</t>
-        </is>
+      <c r="W8" t="n">
+        <v>8.202732937191056</v>
       </c>
       <c r="X8" t="n">
         <v>-26167.61583122996</v>
@@ -1578,7 +1544,7 @@
         <v>9.518381345387516e-11</v>
       </c>
       <c r="Z8" t="n">
-        <v>542.5900000000001</v>
+        <v>3757.938164876658</v>
       </c>
       <c r="AA8" t="n">
         <v>1.000000000000125e-08</v>
@@ -1618,10 +1584,8 @@
       <c r="K9" t="n">
         <v>83.06972347938839</v>
       </c>
-      <c r="W9" t="inlineStr">
-        <is>
-          <t>y = 8.227x + -26000.871</t>
-        </is>
+      <c r="W9" t="n">
+        <v>8.22710126910142</v>
       </c>
       <c r="X9" t="n">
         <v>-26000.87059454789</v>
@@ -1630,7 +1594,7 @@
         <v>8.962322664060081e-11</v>
       </c>
       <c r="Z9" t="n">
-        <v>538.27</v>
+        <v>3720.957971118632</v>
       </c>
       <c r="AA9" t="n">
         <v>1e-08</v>
@@ -1670,10 +1634,8 @@
       <c r="K10" t="n">
         <v>83.17228099437796</v>
       </c>
-      <c r="W10" t="inlineStr">
-        <is>
-          <t>y = 8.352x + -26168.492</t>
-        </is>
+      <c r="W10" t="n">
+        <v>8.351883155148055</v>
       </c>
       <c r="X10" t="n">
         <v>-26168.49190365453</v>
@@ -1682,7 +1644,7 @@
         <v>1.490559670089616e-10</v>
       </c>
       <c r="Z10" t="n">
-        <v>529.23</v>
+        <v>3684.621667345081</v>
       </c>
       <c r="AA10" t="n">
         <v>1.000000000003612e-08</v>
@@ -1722,10 +1684,8 @@
       <c r="K11" t="n">
         <v>83.25738709885832</v>
       </c>
-      <c r="W11" t="inlineStr">
-        <is>
-          <t>y = 8.458x + -26289.539</t>
-        </is>
+      <c r="W11" t="n">
+        <v>8.458300041527908</v>
       </c>
       <c r="X11" t="n">
         <v>-26289.53935116196</v>
@@ -1734,7 +1694,7 @@
         <v>4.437929537938406e-09</v>
       </c>
       <c r="Z11" t="n">
-        <v>519.21</v>
+        <v>3650.464634807239</v>
       </c>
       <c r="AA11" t="n">
         <v>1.000000000000007e-08</v>
@@ -1774,10 +1734,8 @@
       <c r="K12" t="n">
         <v>83.3041612171084</v>
       </c>
-      <c r="W12" t="inlineStr">
-        <is>
-          <t>y = 8.518x + -26240.547</t>
-        </is>
+      <c r="W12" t="n">
+        <v>8.517933067400584</v>
       </c>
       <c r="X12" t="n">
         <v>-26240.54747800111</v>
@@ -1786,7 +1744,7 @@
         <v>2.383232571510424e-10</v>
       </c>
       <c r="Z12" t="n">
-        <v>516.1799999999998</v>
+        <v>3617.155723543447</v>
       </c>
       <c r="AA12" t="n">
         <v>1.000000000001773e-08</v>
@@ -1826,10 +1784,8 @@
       <c r="K13" t="n">
         <v>83.33122177428928</v>
       </c>
-      <c r="W13" t="inlineStr">
-        <is>
-          <t>y = 8.553x + -26122.057</t>
-        </is>
+      <c r="W13" t="n">
+        <v>8.552813198045033</v>
       </c>
       <c r="X13" t="n">
         <v>-26122.0567214235</v>
@@ -1838,7 +1794,7 @@
         <v>4.014741715271358e-13</v>
       </c>
       <c r="Z13" t="n">
-        <v>513.4200000000001</v>
+        <v>3582.32258116732</v>
       </c>
       <c r="AA13" t="n">
         <v>1.000000000000027e-08</v>
@@ -1878,10 +1834,8 @@
       <c r="K14" t="n">
         <v>83.41799697640784</v>
       </c>
-      <c r="W14" t="inlineStr">
-        <is>
-          <t>y = 8.667x + -26249.616</t>
-        </is>
+      <c r="W14" t="n">
+        <v>8.66658913136353</v>
       </c>
       <c r="X14" t="n">
         <v>-26249.61645178953</v>
@@ -1890,7 +1844,7 @@
         <v>1.888537158384933e-12</v>
       </c>
       <c r="Z14" t="n">
-        <v>502.8000000000002</v>
+        <v>3549.319981128023</v>
       </c>
       <c r="AA14" t="n">
         <v>1.000000000000761e-08</v>
@@ -1930,10 +1884,8 @@
       <c r="K15" t="n">
         <v>83.49762236962256</v>
       </c>
-      <c r="W15" t="inlineStr">
-        <is>
-          <t>y = 8.774x + -26350.972</t>
-        </is>
+      <c r="W15" t="n">
+        <v>8.7736503319221</v>
       </c>
       <c r="X15" t="n">
         <v>-26350.97202279682</v>
@@ -1942,7 +1894,7 @@
         <v>1.326908466148628e-09</v>
       </c>
       <c r="Z15" t="n">
-        <v>497.02</v>
+        <v>3516.682615553374</v>
       </c>
       <c r="AA15" t="n">
         <v>1.000000000015281e-08</v>
@@ -1982,10 +1934,8 @@
       <c r="K16" t="n">
         <v>83.58986217207287</v>
       </c>
-      <c r="W16" t="inlineStr">
-        <is>
-          <t>y = 8.901x + -26514.200</t>
-        </is>
+      <c r="W16" t="n">
+        <v>8.90098312632013</v>
       </c>
       <c r="X16" t="n">
         <v>-26514.20003327129</v>
@@ -1994,7 +1944,7 @@
         <v>2.361418140254665e-09</v>
       </c>
       <c r="Z16" t="n">
-        <v>488.79</v>
+        <v>3483.903390530033</v>
       </c>
       <c r="AA16" t="n">
         <v>1.000000000023654e-08</v>
@@ -2034,10 +1984,8 @@
       <c r="K17" t="n">
         <v>83.65675633393472</v>
       </c>
-      <c r="W17" t="inlineStr">
-        <is>
-          <t>y = 8.996x + -26560.827</t>
-        </is>
+      <c r="W17" t="n">
+        <v>8.995634276371785</v>
       </c>
       <c r="X17" t="n">
         <v>-26560.82693334683</v>
@@ -2046,7 +1994,7 @@
         <v>2.435386738540102e-09</v>
       </c>
       <c r="Z17" t="n">
-        <v>484.3299999999999</v>
+        <v>3450.868737054808</v>
       </c>
       <c r="AA17" t="n">
         <v>1.000000000015642e-08</v>
@@ -2086,10 +2034,8 @@
       <c r="K18" t="n">
         <v>83.71418135828506</v>
       </c>
-      <c r="W18" t="inlineStr">
-        <is>
-          <t>y = 9.078x + -26574.965</t>
-        </is>
+      <c r="W18" t="n">
+        <v>9.07848753310482</v>
       </c>
       <c r="X18" t="n">
         <v>-26574.96493488604</v>
@@ -2098,7 +2044,7 @@
         <v>2.737982188141498e-09</v>
       </c>
       <c r="Z18" t="n">
-        <v>476.6399999999999</v>
+        <v>3418.952274950283</v>
       </c>
       <c r="AA18" t="n">
         <v>1.000000000016111e-08</v>
@@ -2138,10 +2084,8 @@
       <c r="K19" t="n">
         <v>83.4745844242114</v>
       </c>
-      <c r="W19" t="inlineStr">
-        <is>
-          <t>y = 8.742x + -25251.260</t>
-        </is>
+      <c r="W19" t="n">
+        <v>8.742406958038117</v>
       </c>
       <c r="X19" t="n">
         <v>-25251.2601737917</v>
@@ -2150,7 +2094,7 @@
         <v>1.084371702312922e-10</v>
       </c>
       <c r="Z19" t="n">
-        <v>486.1899999999996</v>
+        <v>3386.141736488252</v>
       </c>
       <c r="AA19" t="n">
         <v>1.000000000001499e-08</v>
@@ -2190,10 +2134,8 @@
       <c r="K20" t="n">
         <v>83.84403438060421</v>
       </c>
-      <c r="W20" t="inlineStr">
-        <is>
-          <t>y = 9.272x + -26666.734</t>
-        </is>
+      <c r="W20" t="n">
+        <v>9.271517045761952</v>
       </c>
       <c r="X20" t="n">
         <v>-26666.73359235622</v>
@@ -2202,7 +2144,7 @@
         <v>2.691471049114605e-10</v>
       </c>
       <c r="Z20" t="n">
-        <v>464.6700000000001</v>
+        <v>3353.553789033743</v>
       </c>
       <c r="AA20" t="n">
         <v>1.000000000000395e-08</v>
@@ -2242,10 +2184,8 @@
       <c r="K21" t="n">
         <v>83.89368881574332</v>
       </c>
-      <c r="W21" t="inlineStr">
-        <is>
-          <t>y = 9.347x + -26660.418</t>
-        </is>
+      <c r="W21" t="n">
+        <v>9.347490844756734</v>
       </c>
       <c r="X21" t="n">
         <v>-26660.41809050335</v>
@@ -2254,7 +2194,7 @@
         <v>2.87682995133163e-09</v>
       </c>
       <c r="Z21" t="n">
-        <v>461.3199999999997</v>
+        <v>3321.892580425197</v>
       </c>
       <c r="AA21" t="n">
         <v>1.000000000063688e-08</v>
@@ -2294,10 +2234,8 @@
       <c r="K22" t="n">
         <v>83.73274450889936</v>
       </c>
-      <c r="W22" t="inlineStr">
-        <is>
-          <t>y = 9.106x + -25628.790</t>
-        </is>
+      <c r="W22" t="n">
+        <v>9.105594005269653</v>
       </c>
       <c r="X22" t="n">
         <v>-25628.79036655436</v>
@@ -2306,7 +2244,7 @@
         <v>1.176717711878263e-10</v>
       </c>
       <c r="Z22" t="n">
-        <v>463.2199999999998</v>
+        <v>3290.260175203482</v>
       </c>
       <c r="AA22" t="n">
         <v>1.000000000002077e-08</v>
@@ -2432,12 +2370,12 @@
       </c>
       <c r="W1" t="inlineStr">
         <is>
-          <t>Model</t>
+          <t>linear_eq_m</t>
         </is>
       </c>
       <c r="X1" t="inlineStr">
         <is>
-          <t>b</t>
+          <t>linear_eq_b</t>
         </is>
       </c>
       <c r="Y1" t="inlineStr">
@@ -2492,10 +2430,8 @@
       <c r="K2" t="n">
         <v>81.72770232173299</v>
       </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>y = 6.878x + -24495.060</t>
-        </is>
+      <c r="W2" t="n">
+        <v>6.878029839080033</v>
       </c>
       <c r="X2" t="n">
         <v>-24495.06033497604</v>
@@ -2504,7 +2440,7 @@
         <v>9.372481880738808e-09</v>
       </c>
       <c r="Z2" t="n">
-        <v>621.8600000000006</v>
+        <v>4196.134374984057</v>
       </c>
       <c r="AA2" t="n">
         <v>1.000000000000242e-08</v>
@@ -2544,10 +2480,8 @@
       <c r="K3" t="n">
         <v>82.69512048064934</v>
       </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>y = 7.801x + -26459.890</t>
-        </is>
+      <c r="W3" t="n">
+        <v>7.800949923085768</v>
       </c>
       <c r="X3" t="n">
         <v>-26459.89008797356</v>
@@ -2556,7 +2490,7 @@
         <v>1.008242152951607e-09</v>
       </c>
       <c r="Z3" t="n">
-        <v>541.2000000000003</v>
+        <v>4001.223256966525</v>
       </c>
       <c r="AA3" t="n">
         <v>1e-08</v>
@@ -2596,10 +2530,8 @@
       <c r="K4" t="n">
         <v>82.94486466278292</v>
       </c>
-      <c r="W4" t="inlineStr">
-        <is>
-          <t>y = 8.080x + -26910.568</t>
-        </is>
+      <c r="W4" t="n">
+        <v>8.080058683684083</v>
       </c>
       <c r="X4" t="n">
         <v>-26910.56761976944</v>
@@ -2608,7 +2540,7 @@
         <v>1.569572573701757e-10</v>
       </c>
       <c r="Z4" t="n">
-        <v>523.04</v>
+        <v>3927.541019956939</v>
       </c>
       <c r="AA4" t="n">
         <v>1.000000000000016e-08</v>
@@ -2648,10 +2580,8 @@
       <c r="K5" t="n">
         <v>83.53065245071322</v>
       </c>
-      <c r="W5" t="inlineStr">
-        <is>
-          <t>y = 8.819x + -29195.631</t>
-        </is>
+      <c r="W5" t="n">
+        <v>8.818831288572417</v>
       </c>
       <c r="X5" t="n">
         <v>-29195.63144525173</v>
@@ -2660,7 +2590,7 @@
         <v>5.336967142759836e-10</v>
       </c>
       <c r="Z5" t="n">
-        <v>488.54</v>
+        <v>3877.104852299329</v>
       </c>
       <c r="AA5" t="n">
         <v>1.000000000000285e-08</v>
@@ -2700,10 +2630,8 @@
       <c r="K6" t="n">
         <v>83.24190023170245</v>
       </c>
-      <c r="W6" t="inlineStr">
-        <is>
-          <t>y = 8.439x + -27475.483</t>
-        </is>
+      <c r="W6" t="n">
+        <v>8.438736668793522</v>
       </c>
       <c r="X6" t="n">
         <v>-27475.48268528328</v>
@@ -2712,7 +2640,7 @@
         <v>5.254567269568468e-09</v>
       </c>
       <c r="Z6" t="n">
-        <v>501.6999999999998</v>
+        <v>3829.970003896831</v>
       </c>
       <c r="AA6" t="n">
         <v>1.000000000000448e-08</v>
@@ -2752,10 +2680,8 @@
       <c r="K7" t="n">
         <v>83.74787270538825</v>
       </c>
-      <c r="W7" t="inlineStr">
-        <is>
-          <t>y = 9.128x + -29552.577</t>
-        </is>
+      <c r="W7" t="n">
+        <v>9.127803218983839</v>
       </c>
       <c r="X7" t="n">
         <v>-29552.57746903169</v>
@@ -2764,7 +2690,7 @@
         <v>5.172261010524144e-18</v>
       </c>
       <c r="Z7" t="n">
-        <v>471.4399999999996</v>
+        <v>3785.515982341406</v>
       </c>
       <c r="AA7" t="n">
         <v>1e-08</v>
@@ -2804,10 +2730,8 @@
       <c r="K8" t="n">
         <v>83.0780307273682</v>
       </c>
-      <c r="W8" t="inlineStr">
-        <is>
-          <t>y = 8.237x + -26156.503</t>
-        </is>
+      <c r="W8" t="n">
+        <v>8.237071748372559</v>
       </c>
       <c r="X8" t="n">
         <v>-26156.50274033273</v>
@@ -2816,7 +2740,7 @@
         <v>1.199142879722051e-08</v>
       </c>
       <c r="Z8" t="n">
-        <v>498.8800000000001</v>
+        <v>3748.021297279653</v>
       </c>
       <c r="AA8" t="n">
         <v>1.000000000000031e-08</v>
@@ -2856,10 +2780,8 @@
       <c r="K9" t="n">
         <v>83.57504379592744</v>
       </c>
-      <c r="W9" t="inlineStr">
-        <is>
-          <t>y = 8.880x + -28122.514</t>
-        </is>
+      <c r="W9" t="n">
+        <v>8.880281587326241</v>
       </c>
       <c r="X9" t="n">
         <v>-28122.51402882813</v>
@@ -2868,7 +2790,7 @@
         <v>1.637636171640223e-10</v>
       </c>
       <c r="Z9" t="n">
-        <v>472.9899999999998</v>
+        <v>3715.869776117712</v>
       </c>
       <c r="AA9" t="n">
         <v>1.000000000000328e-08</v>
@@ -2908,10 +2830,8 @@
       <c r="K10" t="n">
         <v>83.62302121797003</v>
       </c>
-      <c r="W10" t="inlineStr">
-        <is>
-          <t>y = 8.948x + -28110.581</t>
-        </is>
+      <c r="W10" t="n">
+        <v>8.947653972029627</v>
       </c>
       <c r="X10" t="n">
         <v>-28110.58107177476</v>
@@ -2920,7 +2840,7 @@
         <v>3.136585321634133e-10</v>
       </c>
       <c r="Z10" t="n">
-        <v>469.02</v>
+        <v>3684.196568731055</v>
       </c>
       <c r="AA10" t="n">
         <v>1.000000000002126e-08</v>
@@ -2960,10 +2880,8 @@
       <c r="K11" t="n">
         <v>83.38207143142075</v>
       </c>
-      <c r="W11" t="inlineStr">
-        <is>
-          <t>y = 8.619x + -26730.662</t>
-        </is>
+      <c r="W11" t="n">
+        <v>8.619124778391566</v>
       </c>
       <c r="X11" t="n">
         <v>-26730.66167624396</v>
@@ -2972,7 +2890,7 @@
         <v>5.822225911921077e-10</v>
       </c>
       <c r="Z11" t="n">
-        <v>476.0100000000002</v>
+        <v>3651.20362987053</v>
       </c>
       <c r="AA11" t="n">
         <v>1.000000000000367e-08</v>
@@ -3012,10 +2930,8 @@
       <c r="K12" t="n">
         <v>83.76091421806797</v>
       </c>
-      <c r="W12" t="inlineStr">
-        <is>
-          <t>y = 9.147x + -28254.609</t>
-        </is>
+      <c r="W12" t="n">
+        <v>9.147035139904293</v>
       </c>
       <c r="X12" t="n">
         <v>-28254.60890465227</v>
@@ -3024,7 +2940,7 @@
         <v>2.341753663240482e-10</v>
       </c>
       <c r="Z12" t="n">
-        <v>458.4400000000001</v>
+        <v>3616.918719992228</v>
       </c>
       <c r="AA12" t="n">
         <v>1.000000000000736e-08</v>
@@ -3064,10 +2980,8 @@
       <c r="K13" t="n">
         <v>83.53051278117373</v>
       </c>
-      <c r="W13" t="inlineStr">
-        <is>
-          <t>y = 8.819x + -26870.432</t>
-        </is>
+      <c r="W13" t="n">
+        <v>8.818639271244814</v>
       </c>
       <c r="X13" t="n">
         <v>-26870.43207501114</v>
@@ -3076,7 +2990,7 @@
         <v>9.977220009734805e-09</v>
       </c>
       <c r="Z13" t="n">
-        <v>463.9000000000001</v>
+        <v>3581.519667313898</v>
       </c>
       <c r="AA13" t="n">
         <v>1.000000000006445e-08</v>
@@ -3116,10 +3030,8 @@
       <c r="K14" t="n">
         <v>83.99752230931105</v>
       </c>
-      <c r="W14" t="inlineStr">
-        <is>
-          <t>y = 9.510x + -28865.086</t>
-        </is>
+      <c r="W14" t="n">
+        <v>9.510408268448648</v>
       </c>
       <c r="X14" t="n">
         <v>-28865.08604200661</v>
@@ -3128,7 +3040,7 @@
         <v>1.846181921349008e-10</v>
       </c>
       <c r="Z14" t="n">
-        <v>438.6100000000001</v>
+        <v>3545.4081768414</v>
       </c>
       <c r="AA14" t="n">
         <v>1.000000000002417e-08</v>
@@ -3168,10 +3080,8 @@
       <c r="K15" t="n">
         <v>84.07801630969796</v>
       </c>
-      <c r="W15" t="inlineStr">
-        <is>
-          <t>y = 9.641x + -28999.210</t>
-        </is>
+      <c r="W15" t="n">
+        <v>9.640621907913772</v>
       </c>
       <c r="X15" t="n">
         <v>-28999.21012447367</v>
@@ -3180,7 +3090,7 @@
         <v>7.274745846453659e-17</v>
       </c>
       <c r="Z15" t="n">
-        <v>434.0499999999997</v>
+        <v>3509.33830096486</v>
       </c>
       <c r="AA15" t="n">
         <v>1e-08</v>
@@ -3220,10 +3130,8 @@
       <c r="K16" t="n">
         <v>84.53943587335078</v>
       </c>
-      <c r="W16" t="inlineStr">
-        <is>
-          <t>y = 10.461x + -31332.519</t>
-        </is>
+      <c r="W16" t="n">
+        <v>10.46086088441136</v>
       </c>
       <c r="X16" t="n">
         <v>-31332.51856013672</v>
@@ -3232,7 +3140,7 @@
         <v>6.987080395847131e-11</v>
       </c>
       <c r="Z16" t="n">
-        <v>409.9300000000003</v>
+        <v>3473.240372442296</v>
       </c>
       <c r="AA16" t="n">
         <v>1.000000000000087e-08</v>
@@ -3272,10 +3180,8 @@
       <c r="K17" t="n">
         <v>83.90205459380411</v>
       </c>
-      <c r="W17" t="inlineStr">
-        <is>
-          <t>y = 9.360x + -27488.920</t>
-        </is>
+      <c r="W17" t="n">
+        <v>9.3604122323783</v>
       </c>
       <c r="X17" t="n">
         <v>-27488.91959558622</v>
@@ -3284,7 +3190,7 @@
         <v>3.287138289903484e-11</v>
       </c>
       <c r="Z17" t="n">
-        <v>435.7400000000002</v>
+        <v>3437.571463798545</v>
       </c>
       <c r="AA17" t="n">
         <v>1.000000000001291e-08</v>
@@ -3324,10 +3230,8 @@
       <c r="K18" t="n">
         <v>84.29987466413274</v>
       </c>
-      <c r="W18" t="inlineStr">
-        <is>
-          <t>y = 10.018x + -29291.809</t>
-        </is>
+      <c r="W18" t="n">
+        <v>10.0184862321058</v>
       </c>
       <c r="X18" t="n">
         <v>-29291.80914406236</v>
@@ -3336,7 +3240,7 @@
         <v>2.418275026610593e-10</v>
       </c>
       <c r="Z18" t="n">
-        <v>415.1600000000003</v>
+        <v>3402.6790027316</v>
       </c>
       <c r="AA18" t="n">
         <v>1.00000000000023e-08</v>
@@ -3376,10 +3280,8 @@
       <c r="K19" t="n">
         <v>84.32844899281338</v>
       </c>
-      <c r="W19" t="inlineStr">
-        <is>
-          <t>y = 10.069x + -29172.394</t>
-        </is>
+      <c r="W19" t="n">
+        <v>10.06929498205723</v>
       </c>
       <c r="X19" t="n">
         <v>-29172.39393842236</v>
@@ -3388,7 +3290,7 @@
         <v>2.771806947516841e-10</v>
       </c>
       <c r="Z19" t="n">
-        <v>414.77</v>
+        <v>3368.694983689623</v>
       </c>
       <c r="AA19" t="n">
         <v>1.000000000000171e-08</v>
@@ -3428,10 +3330,8 @@
       <c r="K20" t="n">
         <v>84.4302627780539</v>
       </c>
-      <c r="W20" t="inlineStr">
-        <is>
-          <t>y = 10.255x + -29428.389</t>
-        </is>
+      <c r="W20" t="n">
+        <v>10.25455688729133</v>
       </c>
       <c r="X20" t="n">
         <v>-29428.38938475875</v>
@@ -3440,7 +3340,7 @@
         <v>2.072852205262699e-10</v>
       </c>
       <c r="Z20" t="n">
-        <v>403.4700000000003</v>
+        <v>3335.453195006065</v>
       </c>
       <c r="AA20" t="n">
         <v>1.000000000000288e-08</v>
@@ -3480,10 +3380,8 @@
       <c r="K21" t="n">
         <v>84.50920830985854</v>
       </c>
-      <c r="W21" t="inlineStr">
-        <is>
-          <t>y = 10.403x + -29591.879</t>
-        </is>
+      <c r="W21" t="n">
+        <v>10.40292123314168</v>
       </c>
       <c r="X21" t="n">
         <v>-29591.87863106111</v>
@@ -3492,7 +3390,7 @@
         <v>2.092233388533273e-10</v>
       </c>
       <c r="Z21" t="n">
-        <v>397.8999999999996</v>
+        <v>3302.771891228992</v>
       </c>
       <c r="AA21" t="n">
         <v>1.000000000000298e-08</v>
@@ -3532,10 +3430,8 @@
       <c r="K22" t="n">
         <v>84.50080576692156</v>
       </c>
-      <c r="W22" t="inlineStr">
-        <is>
-          <t>y = 10.387x + -29268.610</t>
-        </is>
+      <c r="W22" t="n">
+        <v>10.38692818344269</v>
       </c>
       <c r="X22" t="n">
         <v>-29268.61044251429</v>
@@ -3544,7 +3440,7 @@
         <v>3.390292703957733e-10</v>
       </c>
       <c r="Z22" t="n">
-        <v>399.04</v>
+        <v>3271.052418534506</v>
       </c>
       <c r="AA22" t="n">
         <v>1.00000000000001e-08</v>
@@ -3670,12 +3566,12 @@
       </c>
       <c r="W1" t="inlineStr">
         <is>
-          <t>Model</t>
+          <t>linear_eq_m</t>
         </is>
       </c>
       <c r="X1" t="inlineStr">
         <is>
-          <t>b</t>
+          <t>linear_eq_b</t>
         </is>
       </c>
       <c r="Y1" t="inlineStr">
@@ -3730,10 +3626,8 @@
       <c r="K2" t="n">
         <v>55.50366380056415</v>
       </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>y = 1.455x + -43677.779</t>
-        </is>
+      <c r="W2" t="n">
+        <v>1.455208368256948</v>
       </c>
       <c r="X2" t="n">
         <v>-43677.778780635</v>
@@ -3742,7 +3636,7 @@
         <v>2883.489211920488</v>
       </c>
       <c r="Z2" t="n">
-        <v>2982.699999999997</v>
+        <v>2080.703758691029</v>
       </c>
       <c r="AA2" t="n">
         <v>2.191155442269083e-06</v>
@@ -3782,10 +3676,8 @@
       <c r="K3" t="n">
         <v>60.779374732112</v>
       </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>y = 1.788x + -46447.827</t>
-        </is>
+      <c r="W3" t="n">
+        <v>1.787777821178867</v>
       </c>
       <c r="X3" t="n">
         <v>-46447.82712472187</v>
@@ -3794,7 +3686,7 @@
         <v>1950.814450412289</v>
       </c>
       <c r="Z3" t="n">
-        <v>2560.099999999999</v>
+        <v>1764.10020359153</v>
       </c>
       <c r="AA3" t="n">
         <v>1.764139868533671e-06</v>
@@ -3834,10 +3726,8 @@
       <c r="K4" t="n">
         <v>62.09075804055832</v>
       </c>
-      <c r="W4" t="inlineStr">
-        <is>
-          <t>y = 1.888x + -47352.154</t>
-        </is>
+      <c r="W4" t="n">
+        <v>1.887934884098565</v>
       </c>
       <c r="X4" t="n">
         <v>-47352.15425404939</v>
@@ -3846,7 +3736,7 @@
         <v>2015.383294903022</v>
       </c>
       <c r="Z4" t="n">
-        <v>2463.299999999999</v>
+        <v>1825.196364559226</v>
       </c>
       <c r="AA4" t="n">
         <v>1.414664423208874e-06</v>
@@ -3886,10 +3776,8 @@
       <c r="K5" t="n">
         <v>62.82142842637428</v>
       </c>
-      <c r="W5" t="inlineStr">
-        <is>
-          <t>y = 1.948x + -48044.553</t>
-        </is>
+      <c r="W5" t="n">
+        <v>1.947580845256805</v>
       </c>
       <c r="X5" t="n">
         <v>-48044.55278719714</v>
@@ -3898,7 +3786,7 @@
         <v>2019.360931709148</v>
       </c>
       <c r="Z5" t="n">
-        <v>2418.199999999997</v>
+        <v>1829.841161391234</v>
       </c>
       <c r="AA5" t="n">
         <v>1.405679274327418e-06</v>
@@ -3938,10 +3826,8 @@
       <c r="K6" t="n">
         <v>63.26015544520055</v>
       </c>
-      <c r="W6" t="inlineStr">
-        <is>
-          <t>y = 1.985x + -48301.493</t>
-        </is>
+      <c r="W6" t="n">
+        <v>1.984838858002761</v>
       </c>
       <c r="X6" t="n">
         <v>-48301.49317769516</v>
@@ -3950,7 +3836,7 @@
         <v>2013.376304596488</v>
       </c>
       <c r="Z6" t="n">
-        <v>2392.299999999999</v>
+        <v>1825.085703212622</v>
       </c>
       <c r="AA6" t="n">
         <v>1.661507495215767e-06</v>
@@ -3990,10 +3876,8 @@
       <c r="K7" t="n">
         <v>63.66654811532521</v>
       </c>
-      <c r="W7" t="inlineStr">
-        <is>
-          <t>y = 2.020x + -48536.451</t>
-        </is>
+      <c r="W7" t="n">
+        <v>2.020375685943431</v>
       </c>
       <c r="X7" t="n">
         <v>-48536.4509105106</v>
@@ -4002,7 +3886,7 @@
         <v>2010.272054506718</v>
       </c>
       <c r="Z7" t="n">
-        <v>2369</v>
+        <v>1822.911231973246</v>
       </c>
       <c r="AA7" t="n">
         <v>1.654722408470943e-06</v>
@@ -4042,10 +3926,8 @@
       <c r="K8" t="n">
         <v>63.99325261592055</v>
       </c>
-      <c r="W8" t="inlineStr">
-        <is>
-          <t>y = 2.050x + -48625.749</t>
-        </is>
+      <c r="W8" t="n">
+        <v>2.049691175226336</v>
       </c>
       <c r="X8" t="n">
         <v>-48625.74946949843</v>
@@ -4054,7 +3936,7 @@
         <v>2006.865871564456</v>
       </c>
       <c r="Z8" t="n">
-        <v>2363.799999999999</v>
+        <v>1820.427341985811</v>
       </c>
       <c r="AA8" t="n">
         <v>1.652679632918364e-06</v>
@@ -4094,10 +3976,8 @@
       <c r="K9" t="n">
         <v>64.23105464881762</v>
       </c>
-      <c r="W9" t="inlineStr">
-        <is>
-          <t>y = 2.071x + -48529.138</t>
-        </is>
+      <c r="W9" t="n">
+        <v>2.071463871847322</v>
       </c>
       <c r="X9" t="n">
         <v>-48529.13810753277</v>
@@ -4106,7 +3986,7 @@
         <v>2048.121562254793</v>
       </c>
       <c r="Z9" t="n">
-        <v>2347.199999999997</v>
+        <v>1859.966738194793</v>
       </c>
       <c r="AA9" t="n">
         <v>1.610289555534342e-06</v>
@@ -4146,10 +4026,8 @@
       <c r="K10" t="n">
         <v>64.48284246075836</v>
       </c>
-      <c r="W10" t="inlineStr">
-        <is>
-          <t>y = 2.095x + -48484.064</t>
-        </is>
+      <c r="W10" t="n">
+        <v>2.094928901833129</v>
       </c>
       <c r="X10" t="n">
         <v>-48484.0635360629</v>
@@ -4158,7 +4036,7 @@
         <v>2056.781931524606</v>
       </c>
       <c r="Z10" t="n">
-        <v>2334.799999999999</v>
+        <v>1868.963630238603</v>
       </c>
       <c r="AA10" t="n">
         <v>1.596751668275329e-06</v>
@@ -4198,10 +4076,8 @@
       <c r="K11" t="n">
         <v>64.66816861197613</v>
       </c>
-      <c r="W11" t="inlineStr">
-        <is>
-          <t>y = 2.112x + -48283.050</t>
-        </is>
+      <c r="W11" t="n">
+        <v>2.1124779939027</v>
       </c>
       <c r="X11" t="n">
         <v>-48283.0499287217</v>
@@ -4210,7 +4086,7 @@
         <v>2014.642061059314</v>
       </c>
       <c r="Z11" t="n">
-        <v>2328.900000000001</v>
+        <v>1829.866113799269</v>
       </c>
       <c r="AA11" t="n">
         <v>1.626963053200119e-06</v>
@@ -4336,12 +4212,12 @@
       </c>
       <c r="W1" t="inlineStr">
         <is>
-          <t>Model</t>
+          <t>linear_eq_m</t>
         </is>
       </c>
       <c r="X1" t="inlineStr">
         <is>
-          <t>b</t>
+          <t>linear_eq_b</t>
         </is>
       </c>
       <c r="Y1" t="inlineStr">
@@ -4396,10 +4272,8 @@
       <c r="K2" t="n">
         <v>81.58370115852892</v>
       </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>y = 6.759x + -24183.133</t>
-        </is>
+      <c r="W2" t="n">
+        <v>6.758682237918834</v>
       </c>
       <c r="X2" t="n">
         <v>-24183.13325951939</v>
@@ -4408,7 +4282,7 @@
         <v>8.18558636998039e-09</v>
       </c>
       <c r="Z2" t="n">
-        <v>643.6899999999996</v>
+        <v>4197.135296207487</v>
       </c>
       <c r="AA2" t="n">
         <v>1.000000000003627e-08</v>
@@ -4448,10 +4322,8 @@
       <c r="K3" t="n">
         <v>82.35250125129245</v>
       </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>y = 7.448x + -25132.257</t>
-        </is>
+      <c r="W3" t="n">
+        <v>7.447549727111983</v>
       </c>
       <c r="X3" t="n">
         <v>-25132.25704839991</v>
@@ -4460,7 +4332,7 @@
         <v>2.855706839303508e-09</v>
       </c>
       <c r="Z3" t="n">
-        <v>562.5099999999998</v>
+        <v>3982.710374021114</v>
       </c>
       <c r="AA3" t="n">
         <v>1.000000000000005e-08</v>
@@ -4500,10 +4372,8 @@
       <c r="K4" t="n">
         <v>82.71503741314046</v>
       </c>
-      <c r="W4" t="inlineStr">
-        <is>
-          <t>y = 7.823x + -25921.327</t>
-        </is>
+      <c r="W4" t="n">
+        <v>7.822510117524848</v>
       </c>
       <c r="X4" t="n">
         <v>-25921.32667909566</v>
@@ -4512,7 +4382,7 @@
         <v>1.061910452679619e-11</v>
       </c>
       <c r="Z4" t="n">
-        <v>531.9699999999998</v>
+        <v>3908.154320430063</v>
       </c>
       <c r="AA4" t="n">
         <v>1e-08</v>
@@ -4552,10 +4422,8 @@
       <c r="K5" t="n">
         <v>83.35054759925181</v>
       </c>
-      <c r="W5" t="inlineStr">
-        <is>
-          <t>y = 8.578x + -28240.688</t>
-        </is>
+      <c r="W5" t="n">
+        <v>8.577896509081079</v>
       </c>
       <c r="X5" t="n">
         <v>-28240.68808179591</v>
@@ -4564,7 +4432,7 @@
         <v>2.392805453571923e-09</v>
       </c>
       <c r="Z5" t="n">
-        <v>495.4700000000003</v>
+        <v>3856.895157992336</v>
       </c>
       <c r="AA5" t="n">
         <v>1.000000000000218e-08</v>
@@ -4604,10 +4472,8 @@
       <c r="K6" t="n">
         <v>83.09810507894832</v>
       </c>
-      <c r="W6" t="inlineStr">
-        <is>
-          <t>y = 8.261x + -26753.213</t>
-        </is>
+      <c r="W6" t="n">
+        <v>8.261263868754211</v>
       </c>
       <c r="X6" t="n">
         <v>-26753.21345103956</v>
@@ -4616,7 +4482,7 @@
         <v>9.456756740009373e-11</v>
       </c>
       <c r="Z6" t="n">
-        <v>502.3099999999999</v>
+        <v>3811.837128442961</v>
       </c>
       <c r="AA6" t="n">
         <v>1.000000000000069e-08</v>
@@ -4656,10 +4522,8 @@
       <c r="K7" t="n">
         <v>83.68321242761351</v>
       </c>
-      <c r="W7" t="inlineStr">
-        <is>
-          <t>y = 9.034x + -29115.473</t>
-        </is>
+      <c r="W7" t="n">
+        <v>9.033618946549847</v>
       </c>
       <c r="X7" t="n">
         <v>-29115.47264585606</v>
@@ -4668,7 +4532,7 @@
         <v>125.0389400380478</v>
       </c>
       <c r="Z7" t="n">
-        <v>468.73</v>
+        <v>4016.786618265003</v>
       </c>
       <c r="AA7" t="n">
         <v>1.911798595083981e-08</v>
@@ -4708,10 +4572,8 @@
       <c r="K8" t="n">
         <v>83.61406326098518</v>
       </c>
-      <c r="W8" t="inlineStr">
-        <is>
-          <t>y = 8.935x + -28394.391</t>
-        </is>
+      <c r="W8" t="n">
+        <v>8.934998202371187</v>
       </c>
       <c r="X8" t="n">
         <v>-28394.39105021164</v>
@@ -4720,7 +4582,7 @@
         <v>2.063089794802132e-08</v>
       </c>
       <c r="Z8" t="n">
-        <v>449.2600000000002</v>
+        <v>3730.626176126394</v>
       </c>
       <c r="AA8" t="n">
         <v>1.000000000000704e-08</v>
@@ -4760,10 +4622,8 @@
       <c r="K9" t="n">
         <v>83.70529570207415</v>
       </c>
-      <c r="W9" t="inlineStr">
-        <is>
-          <t>y = 9.066x + -28548.425</t>
-        </is>
+      <c r="W9" t="n">
+        <v>9.065568782995225</v>
       </c>
       <c r="X9" t="n">
         <v>-28548.42548320814</v>
@@ -4772,7 +4632,7 @@
         <v>1.630872492385224e-10</v>
       </c>
       <c r="Z9" t="n">
-        <v>438.2799999999997</v>
+        <v>3694.783648524833</v>
       </c>
       <c r="AA9" t="n">
         <v>1.00000000000811e-08</v>
@@ -4812,10 +4672,8 @@
       <c r="K10" t="n">
         <v>83.78413149258013</v>
       </c>
-      <c r="W10" t="inlineStr">
-        <is>
-          <t>y = 9.181x + -28674.715</t>
-        </is>
+      <c r="W10" t="n">
+        <v>9.181471872814651</v>
       </c>
       <c r="X10" t="n">
         <v>-28674.71482569155</v>
@@ -4824,7 +4682,7 @@
         <v>3.259689340340592e-10</v>
       </c>
       <c r="Z10" t="n">
-        <v>438.5299999999997</v>
+        <v>3661.15466635551</v>
       </c>
       <c r="AA10" t="n">
         <v>1.000000000000035e-08</v>
@@ -4864,10 +4722,8 @@
       <c r="K11" t="n">
         <v>83.88371344689703</v>
       </c>
-      <c r="W11" t="inlineStr">
-        <is>
-          <t>y = 9.332x + -28898.503</t>
-        </is>
+      <c r="W11" t="n">
+        <v>9.332129387060517</v>
       </c>
       <c r="X11" t="n">
         <v>-28898.50286554719</v>
@@ -4876,7 +4732,7 @@
         <v>2.584869732792946e-10</v>
       </c>
       <c r="Z11" t="n">
-        <v>425.21</v>
+        <v>3628.426219168407</v>
       </c>
       <c r="AA11" t="n">
         <v>1.000000000000108e-08</v>
@@ -4916,10 +4772,8 @@
       <c r="K12" t="n">
         <v>84.01179981942853</v>
       </c>
-      <c r="W12" t="inlineStr">
-        <is>
-          <t>y = 9.533x + -29319.538</t>
-        </is>
+      <c r="W12" t="n">
+        <v>9.533250255418919</v>
       </c>
       <c r="X12" t="n">
         <v>-29319.53796829532</v>
@@ -4928,7 +4782,7 @@
         <v>1.514289416406875e-10</v>
       </c>
       <c r="Z12" t="n">
-        <v>419.1199999999999</v>
+        <v>3596.877893152952</v>
       </c>
       <c r="AA12" t="n">
         <v>1.00000000000106e-08</v>
@@ -4968,10 +4822,8 @@
       <c r="K13" t="n">
         <v>84.07878823873421</v>
       </c>
-      <c r="W13" t="inlineStr">
-        <is>
-          <t>y = 9.642x + -29404.166</t>
-        </is>
+      <c r="W13" t="n">
+        <v>9.641887719501662</v>
       </c>
       <c r="X13" t="n">
         <v>-29404.16599194265</v>
@@ -4980,7 +4832,7 @@
         <v>1.120530536052821e-08</v>
       </c>
       <c r="Z13" t="n">
-        <v>411.21</v>
+        <v>3565.168694081408</v>
       </c>
       <c r="AA13" t="n">
         <v>1.000000000000027e-08</v>
@@ -5020,10 +4872,8 @@
       <c r="K14" t="n">
         <v>84.18596511964131</v>
       </c>
-      <c r="W14" t="inlineStr">
-        <is>
-          <t>y = 9.821x + -29709.095</t>
-        </is>
+      <c r="W14" t="n">
+        <v>9.82088818954032</v>
       </c>
       <c r="X14" t="n">
         <v>-29709.0951033068</v>
@@ -5032,7 +4882,7 @@
         <v>9.505757559990949e-09</v>
       </c>
       <c r="Z14" t="n">
-        <v>400.27</v>
+        <v>3534.132273106329</v>
       </c>
       <c r="AA14" t="n">
         <v>1.000000000000331e-08</v>
@@ -5072,10 +4922,8 @@
       <c r="K15" t="n">
         <v>84.20713005907987</v>
       </c>
-      <c r="W15" t="inlineStr">
-        <is>
-          <t>y = 9.857x + -29577.413</t>
-        </is>
+      <c r="W15" t="n">
+        <v>9.857017025935924</v>
       </c>
       <c r="X15" t="n">
         <v>-29577.41319756097</v>
@@ -5084,7 +4932,7 @@
         <v>4.405966353261179e-12</v>
       </c>
       <c r="Z15" t="n">
-        <v>400.6700000000001</v>
+        <v>3503.030557362109</v>
       </c>
       <c r="AA15" t="n">
         <v>1.000000000005382e-08</v>
@@ -5124,10 +4972,8 @@
       <c r="K16" t="n">
         <v>84.26304068018455</v>
       </c>
-      <c r="W16" t="inlineStr">
-        <is>
-          <t>y = 9.954x + -29628.455</t>
-        </is>
+      <c r="W16" t="n">
+        <v>9.953735051293265</v>
       </c>
       <c r="X16" t="n">
         <v>-29628.45510555273</v>
@@ -5136,7 +4982,7 @@
         <v>8.707214415280754e-10</v>
       </c>
       <c r="Z16" t="n">
-        <v>396.9400000000001</v>
+        <v>3472.204119141927</v>
       </c>
       <c r="AA16" t="n">
         <v>1e-08</v>
@@ -5176,10 +5022,8 @@
       <c r="K17" t="n">
         <v>84.38437580484043</v>
       </c>
-      <c r="W17" t="inlineStr">
-        <is>
-          <t>y = 10.170x + -30028.579</t>
-        </is>
+      <c r="W17" t="n">
+        <v>10.17023136997246</v>
       </c>
       <c r="X17" t="n">
         <v>-30028.57892337986</v>
@@ -5188,7 +5032,7 @@
         <v>1.390207030577781e-09</v>
       </c>
       <c r="Z17" t="n">
-        <v>386.3600000000001</v>
+        <v>3441.373366417077</v>
       </c>
       <c r="AA17" t="n">
         <v>1.00000000001704e-08</v>
@@ -5228,10 +5072,8 @@
       <c r="K18" t="n">
         <v>84.46375950983405</v>
       </c>
-      <c r="W18" t="inlineStr">
-        <is>
-          <t>y = 10.317x + -30211.572</t>
-        </is>
+      <c r="W18" t="n">
+        <v>10.31699296569295</v>
       </c>
       <c r="X18" t="n">
         <v>-30211.57208073499</v>
@@ -5240,7 +5082,7 @@
         <v>1.154298452146454e-11</v>
       </c>
       <c r="Z18" t="n">
-        <v>379.3499999999999</v>
+        <v>3410.426010644573</v>
       </c>
       <c r="AA18" t="n">
         <v>1.000000000000535e-08</v>
@@ -5280,10 +5122,8 @@
       <c r="K19" t="n">
         <v>84.19032214251865</v>
       </c>
-      <c r="W19" t="inlineStr">
-        <is>
-          <t>y = 9.828x + -28412.792</t>
-        </is>
+      <c r="W19" t="n">
+        <v>9.828304242510258</v>
       </c>
       <c r="X19" t="n">
         <v>-28412.79198105791</v>
@@ -5292,7 +5132,7 @@
         <v>2.517315629913945e-09</v>
       </c>
       <c r="Z19" t="n">
-        <v>390.4100000000003</v>
+        <v>3380.128435820616</v>
       </c>
       <c r="AA19" t="n">
         <v>1.000000000089883e-08</v>
@@ -5332,10 +5172,8 @@
       <c r="K20" t="n">
         <v>84.60014254065234</v>
       </c>
-      <c r="W20" t="inlineStr">
-        <is>
-          <t>y = 10.579x + -30467.949</t>
-        </is>
+      <c r="W20" t="n">
+        <v>10.57917590622605</v>
       </c>
       <c r="X20" t="n">
         <v>-30467.94887651073</v>
@@ -5344,7 +5182,7 @@
         <v>2.5093519068961e-11</v>
       </c>
       <c r="Z20" t="n">
-        <v>368.52</v>
+        <v>3348.381877410202</v>
       </c>
       <c r="AA20" t="n">
         <v>1.00000000000073e-08</v>
@@ -5384,10 +5222,8 @@
       <c r="K21" t="n">
         <v>84.31946038118039</v>
       </c>
-      <c r="W21" t="inlineStr">
-        <is>
-          <t>y = 10.053x + -28565.884</t>
-        </is>
+      <c r="W21" t="n">
+        <v>10.05325717439083</v>
       </c>
       <c r="X21" t="n">
         <v>-28565.88371232273</v>
@@ -5396,7 +5232,7 @@
         <v>1.449632556628533e-11</v>
       </c>
       <c r="Z21" t="n">
-        <v>379.8200000000002</v>
+        <v>3316.26452106183</v>
       </c>
       <c r="AA21" t="n">
         <v>1.000000000000639e-08</v>
@@ -5436,10 +5272,8 @@
       <c r="K22" t="n">
         <v>84.78441736683563</v>
       </c>
-      <c r="W22" t="inlineStr">
-        <is>
-          <t>y = 10.955x + -31006.395</t>
-        </is>
+      <c r="W22" t="n">
+        <v>10.95513952314243</v>
       </c>
       <c r="X22" t="n">
         <v>-31006.39486152134</v>
@@ -5448,7 +5282,7 @@
         <v>1.409007508995995e-11</v>
       </c>
       <c r="Z22" t="n">
-        <v>353.6400000000003</v>
+        <v>3284.11934365875</v>
       </c>
       <c r="AA22" t="n">
         <v>1.000000000000556e-08</v>
@@ -5574,12 +5408,12 @@
       </c>
       <c r="W1" t="inlineStr">
         <is>
-          <t>Model</t>
+          <t>linear_eq_m</t>
         </is>
       </c>
       <c r="X1" t="inlineStr">
         <is>
-          <t>b</t>
+          <t>linear_eq_b</t>
         </is>
       </c>
       <c r="Y1" t="inlineStr">
@@ -5634,10 +5468,8 @@
       <c r="K2" t="n">
         <v>59.13296351765025</v>
       </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>y = 1.673x + -45240.389</t>
-        </is>
+      <c r="W2" t="n">
+        <v>1.673061869120372</v>
       </c>
       <c r="X2" t="n">
         <v>-45240.3889864725</v>
@@ -5646,7 +5478,7 @@
         <v>1956.981062621956</v>
       </c>
       <c r="Z2" t="n">
-        <v>2912.600000000002</v>
+        <v>1768.128452230034</v>
       </c>
       <c r="AA2" t="n">
         <v>1.571690957730544e-06</v>
@@ -5686,10 +5518,8 @@
       <c r="K3" t="n">
         <v>61.82421419133203</v>
       </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>y = 1.867x + -45857.046</t>
-        </is>
+      <c r="W3" t="n">
+        <v>1.866886174674419</v>
       </c>
       <c r="X3" t="n">
         <v>-45857.04613273493</v>
@@ -5698,7 +5528,7 @@
         <v>1979.249072103158</v>
       </c>
       <c r="Z3" t="n">
-        <v>2718.200000000001</v>
+        <v>1792.33888738741</v>
       </c>
       <c r="AA3" t="n">
         <v>1.450875310280992e-06</v>
@@ -5738,10 +5568,8 @@
       <c r="K4" t="n">
         <v>62.58370357284059</v>
       </c>
-      <c r="W4" t="inlineStr">
-        <is>
-          <t>y = 1.928x + -45986.207</t>
-        </is>
+      <c r="W4" t="n">
+        <v>1.927853301463998</v>
       </c>
       <c r="X4" t="n">
         <v>-45986.20733642069</v>
@@ -5750,7 +5578,7 @@
         <v>2019.450788730009</v>
       </c>
       <c r="Z4" t="n">
-        <v>2677.599999999999</v>
+        <v>1831.238120154344</v>
       </c>
       <c r="AA4" t="n">
         <v>1.408136428363595e-06</v>
@@ -5790,10 +5618,8 @@
       <c r="K5" t="n">
         <v>63.00392211446661</v>
       </c>
-      <c r="W5" t="inlineStr">
-        <is>
-          <t>y = 1.963x + -46019.634</t>
-        </is>
+      <c r="W5" t="n">
+        <v>1.962942677070821</v>
       </c>
       <c r="X5" t="n">
         <v>-46019.63413940557</v>
@@ -5802,7 +5628,7 @@
         <v>2032.692439338152</v>
       </c>
       <c r="Z5" t="n">
-        <v>2665.600000000002</v>
+        <v>1844.767937746745</v>
       </c>
       <c r="AA5" t="n">
         <v>1.642772286163007e-06</v>
@@ -5842,10 +5668,8 @@
       <c r="K6" t="n">
         <v>63.07764854462515</v>
       </c>
-      <c r="W6" t="inlineStr">
-        <is>
-          <t>y = 1.969x + -45443.822</t>
-        </is>
+      <c r="W6" t="n">
+        <v>1.969203369077214</v>
       </c>
       <c r="X6" t="n">
         <v>-45443.82219027122</v>
@@ -5854,7 +5678,7 @@
         <v>2037.839430945596</v>
       </c>
       <c r="Z6" t="n">
-        <v>2695.099999999999</v>
+        <v>1850.520666925785</v>
       </c>
       <c r="AA6" t="n">
         <v>1.631187797574851e-06</v>
@@ -5894,10 +5718,8 @@
       <c r="K7" t="n">
         <v>63.26747318032066</v>
       </c>
-      <c r="W7" t="inlineStr">
-        <is>
-          <t>y = 1.985x + -45181.243</t>
-        </is>
+      <c r="W7" t="n">
+        <v>1.985469894752495</v>
       </c>
       <c r="X7" t="n">
         <v>-45181.24346535742</v>
@@ -5906,7 +5728,7 @@
         <v>2089.150040683206</v>
       </c>
       <c r="Z7" t="n">
-        <v>2688.900000000001</v>
+        <v>1900.018103241254</v>
       </c>
       <c r="AA7" t="n">
         <v>1.324157460973251e-06</v>
@@ -5946,10 +5768,8 @@
       <c r="K8" t="n">
         <v>63.32971181267361</v>
       </c>
-      <c r="W8" t="inlineStr">
-        <is>
-          <t>y = 1.991x + -44667.205</t>
-        </is>
+      <c r="W8" t="n">
+        <v>1.9908499405116</v>
       </c>
       <c r="X8" t="n">
         <v>-44667.20504721891</v>
@@ -5958,7 +5778,7 @@
         <v>2055.020950709662</v>
       </c>
       <c r="Z8" t="n">
-        <v>2689.600000000002</v>
+        <v>1868.58676095677</v>
       </c>
       <c r="AA8" t="n">
         <v>1.60057361096518e-06</v>
@@ -5998,10 +5818,8 @@
       <c r="K9" t="n">
         <v>63.64317165555217</v>
       </c>
-      <c r="W9" t="inlineStr">
-        <is>
-          <t>y = 2.018x + -44748.728</t>
-        </is>
+      <c r="W9" t="n">
+        <v>2.018303990390019</v>
       </c>
       <c r="X9" t="n">
         <v>-44748.72817072683</v>
@@ -6010,7 +5828,7 @@
         <v>2053.697762144098</v>
       </c>
       <c r="Z9" t="n">
-        <v>2663.900000000001</v>
+        <v>1868.2901992821</v>
       </c>
       <c r="AA9" t="n">
         <v>1.595567646677031e-06</v>
@@ -6050,10 +5868,8 @@
       <c r="K10" t="n">
         <v>63.57617945324454</v>
       </c>
-      <c r="W10" t="inlineStr">
-        <is>
-          <t>y = 2.012x + -44007.994</t>
-        </is>
+      <c r="W10" t="n">
+        <v>2.012385783015704</v>
       </c>
       <c r="X10" t="n">
         <v>-44007.99359489807</v>
@@ -6062,7 +5878,7 @@
         <v>2069.231919864614</v>
       </c>
       <c r="Z10" t="n">
-        <v>2681.299999999999</v>
+        <v>1884.084555784315</v>
       </c>
       <c r="AA10" t="n">
         <v>1.574361891415273e-06</v>
@@ -6102,10 +5918,8 @@
       <c r="K11" t="n">
         <v>63.75561889004117</v>
       </c>
-      <c r="W11" t="inlineStr">
-        <is>
-          <t>y = 2.028x + -43836.838</t>
-        </is>
+      <c r="W11" t="n">
+        <v>2.028300823091671</v>
       </c>
       <c r="X11" t="n">
         <v>-43836.83812154708</v>
@@ -6114,7 +5928,7 @@
         <v>2065.449527872279</v>
       </c>
       <c r="Z11" t="n">
-        <v>2660.700000000001</v>
+        <v>1881.401289827784</v>
       </c>
       <c r="AA11" t="n">
         <v>1.571495531452732e-06</v>
@@ -6240,12 +6054,12 @@
       </c>
       <c r="W1" t="inlineStr">
         <is>
-          <t>Model</t>
+          <t>linear_eq_m</t>
         </is>
       </c>
       <c r="X1" t="inlineStr">
         <is>
-          <t>b</t>
+          <t>linear_eq_b</t>
         </is>
       </c>
       <c r="Y1" t="inlineStr">
@@ -6300,10 +6114,8 @@
       <c r="K2" t="n">
         <v>81.21776653976325</v>
       </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>y = 6.473x + -23177.174</t>
-        </is>
+      <c r="W2" t="n">
+        <v>6.472882445081373</v>
       </c>
       <c r="X2" t="n">
         <v>-23177.17443704293</v>
@@ -6312,7 +6124,7 @@
         <v>8.893462476884348e-10</v>
       </c>
       <c r="Z2" t="n">
-        <v>758.0999999999999</v>
+        <v>4228.089117988718</v>
       </c>
       <c r="AA2" t="n">
         <v>1.000000000000006e-08</v>
@@ -6352,10 +6164,8 @@
       <c r="K3" t="n">
         <v>81.52623268285021</v>
       </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>y = 6.712x + -22620.911</t>
-        </is>
+      <c r="W3" t="n">
+        <v>6.712176999914741</v>
       </c>
       <c r="X3" t="n">
         <v>-22620.91124627536</v>
@@ -6364,7 +6174,7 @@
         <v>3.064630490463671e-09</v>
       </c>
       <c r="Z3" t="n">
-        <v>712.6700000000001</v>
+        <v>3995.00470750756</v>
       </c>
       <c r="AA3" t="n">
         <v>1.000000000000431e-08</v>
@@ -6404,10 +6214,8 @@
       <c r="K4" t="n">
         <v>81.58447887943476</v>
       </c>
-      <c r="W4" t="inlineStr">
-        <is>
-          <t>y = 6.759x + -22344.308</t>
-        </is>
+      <c r="W4" t="n">
+        <v>6.759315917681994</v>
       </c>
       <c r="X4" t="n">
         <v>-22344.30760975299</v>
@@ -6416,7 +6224,7 @@
         <v>1.437133177459935e-09</v>
       </c>
       <c r="Z4" t="n">
-        <v>702.6100000000001</v>
+        <v>3919.7152960145</v>
       </c>
       <c r="AA4" t="n">
         <v>1.000000000000007e-08</v>
@@ -6456,10 +6264,8 @@
       <c r="K5" t="n">
         <v>81.67211594857707</v>
       </c>
-      <c r="W5" t="inlineStr">
-        <is>
-          <t>y = 6.831x + -22318.030</t>
-        </is>
+      <c r="W5" t="n">
+        <v>6.831474423149162</v>
       </c>
       <c r="X5" t="n">
         <v>-22318.02970931322</v>
@@ -6468,7 +6274,7 @@
         <v>8.525199959196454e-09</v>
       </c>
       <c r="Z5" t="n">
-        <v>688.3299999999999</v>
+        <v>3869.999130203362</v>
       </c>
       <c r="AA5" t="n">
         <v>1.000000000000002e-08</v>
@@ -6508,10 +6314,8 @@
       <c r="K6" t="n">
         <v>81.73150307854043</v>
       </c>
-      <c r="W6" t="inlineStr">
-        <is>
-          <t>y = 6.881x + -22244.566</t>
-        </is>
+      <c r="W6" t="n">
+        <v>6.881235801010916</v>
       </c>
       <c r="X6" t="n">
         <v>-22244.56552976538</v>
@@ -6520,7 +6324,7 @@
         <v>108.5492817197652</v>
       </c>
       <c r="Z6" t="n">
-        <v>682.8699999999999</v>
+        <v>4157.638945999423</v>
       </c>
       <c r="AA6" t="n">
         <v>1.540680380679318e-08</v>
@@ -6560,10 +6364,8 @@
       <c r="K7" t="n">
         <v>81.85659717212884</v>
       </c>
-      <c r="W7" t="inlineStr">
-        <is>
-          <t>y = 6.988x + -22361.418</t>
-        </is>
+      <c r="W7" t="n">
+        <v>6.988411976938719</v>
       </c>
       <c r="X7" t="n">
         <v>-22361.41772853267</v>
@@ -6572,7 +6374,7 @@
         <v>3.161141659038213e-10</v>
       </c>
       <c r="Z7" t="n">
-        <v>669.9400000000001</v>
+        <v>3783.196584692455</v>
       </c>
       <c r="AA7" t="n">
         <v>1.000000000002135e-08</v>
@@ -6612,10 +6414,8 @@
       <c r="K8" t="n">
         <v>81.89930620615482</v>
       </c>
-      <c r="W8" t="inlineStr">
-        <is>
-          <t>y = 7.026x + -22260.468</t>
-        </is>
+      <c r="W8" t="n">
+        <v>7.02575635341005</v>
       </c>
       <c r="X8" t="n">
         <v>-22260.46846365806</v>
@@ -6624,7 +6424,7 @@
         <v>7.603127593450079e-10</v>
       </c>
       <c r="Z8" t="n">
-        <v>664.0700000000002</v>
+        <v>3742.39318797351</v>
       </c>
       <c r="AA8" t="n">
         <v>1.000000000000009e-08</v>
@@ -6664,10 +6464,8 @@
       <c r="K9" t="n">
         <v>81.96286628218232</v>
       </c>
-      <c r="W9" t="inlineStr">
-        <is>
-          <t>y = 7.082x + -22222.796</t>
-        </is>
+      <c r="W9" t="n">
+        <v>7.082062600769506</v>
       </c>
       <c r="X9" t="n">
         <v>-22222.79574531389</v>
@@ -6676,7 +6474,7 @@
         <v>1.521868844776335e-10</v>
       </c>
       <c r="Z9" t="n">
-        <v>657.4099999999999</v>
+        <v>3703.725698002615</v>
       </c>
       <c r="AA9" t="n">
         <v>1.000000000000382e-08</v>
@@ -6716,10 +6514,8 @@
       <c r="K10" t="n">
         <v>82.06739887001213</v>
       </c>
-      <c r="W10" t="inlineStr">
-        <is>
-          <t>y = 7.177x + -22321.139</t>
-        </is>
+      <c r="W10" t="n">
+        <v>7.176614623348527</v>
       </c>
       <c r="X10" t="n">
         <v>-22321.13870224415</v>
@@ -6728,7 +6524,7 @@
         <v>1.914373975216812e-11</v>
       </c>
       <c r="Z10" t="n">
-        <v>647.9000000000001</v>
+        <v>3666.83455351343</v>
       </c>
       <c r="AA10" t="n">
         <v>1e-08</v>
@@ -6768,10 +6564,8 @@
       <c r="K11" t="n">
         <v>82.10739524777436</v>
       </c>
-      <c r="W11" t="inlineStr">
-        <is>
-          <t>y = 7.213x + -22237.743</t>
-        </is>
+      <c r="W11" t="n">
+        <v>7.213450414240349</v>
       </c>
       <c r="X11" t="n">
         <v>-22237.74262316509</v>
@@ -6780,7 +6574,7 @@
         <v>1.537612853485187e-09</v>
       </c>
       <c r="Z11" t="n">
-        <v>643.7400000000002</v>
+        <v>3631.830470287303</v>
       </c>
       <c r="AA11" t="n">
         <v>1e-08</v>
@@ -6820,10 +6614,8 @@
       <c r="K12" t="n">
         <v>81.93366593735455</v>
       </c>
-      <c r="W12" t="inlineStr">
-        <is>
-          <t>y = 7.056x + -21469.974</t>
-        </is>
+      <c r="W12" t="n">
+        <v>7.056085302919087</v>
       </c>
       <c r="X12" t="n">
         <v>-21469.97362443178</v>
@@ -6832,7 +6624,7 @@
         <v>2.59594962930328e-10</v>
       </c>
       <c r="Z12" t="n">
-        <v>646.8200000000002</v>
+        <v>3597.710134803611</v>
       </c>
       <c r="AA12" t="n">
         <v>1.000000000000025e-08</v>
@@ -6872,10 +6664,8 @@
       <c r="K13" t="n">
         <v>81.95928549382815</v>
       </c>
-      <c r="W13" t="inlineStr">
-        <is>
-          <t>y = 7.079x + -21355.930</t>
-        </is>
+      <c r="W13" t="n">
+        <v>7.078866966160795</v>
       </c>
       <c r="X13" t="n">
         <v>-21355.93043890158</v>
@@ -6884,7 +6674,7 @@
         <v>2.201600607771591e-09</v>
       </c>
       <c r="Z13" t="n">
-        <v>643.23</v>
+        <v>3565.162528323268</v>
       </c>
       <c r="AA13" t="n">
         <v>1.000000000004395e-08</v>
@@ -6924,10 +6714,8 @@
       <c r="K14" t="n">
         <v>82.31012372062959</v>
       </c>
-      <c r="W14" t="inlineStr">
-        <is>
-          <t>y = 7.406x + -22274.287</t>
-        </is>
+      <c r="W14" t="n">
+        <v>7.40601471082383</v>
       </c>
       <c r="X14" t="n">
         <v>-22274.28733436464</v>
@@ -6936,7 +6724,7 @@
         <v>9.726162347189987e-10</v>
       </c>
       <c r="Z14" t="n">
-        <v>623.8000000000002</v>
+        <v>3533.235419048723</v>
       </c>
       <c r="AA14" t="n">
         <v>1.000000000000054e-08</v>
@@ -6976,10 +6764,8 @@
       <c r="K15" t="n">
         <v>82.38273360514714</v>
       </c>
-      <c r="W15" t="inlineStr">
-        <is>
-          <t>y = 7.477x + -22305.630</t>
-        </is>
+      <c r="W15" t="n">
+        <v>7.477461791898191</v>
       </c>
       <c r="X15" t="n">
         <v>-22305.63043253864</v>
@@ -6988,7 +6774,7 @@
         <v>2.388420229840544e-13</v>
       </c>
       <c r="Z15" t="n">
-        <v>618.7000000000003</v>
+        <v>3502.544657250044</v>
       </c>
       <c r="AA15" t="n">
         <v>1.00000000000016e-08</v>
@@ -7028,10 +6814,8 @@
       <c r="K16" t="n">
         <v>82.49166770061491</v>
       </c>
-      <c r="W16" t="inlineStr">
-        <is>
-          <t>y = 7.587x + -22446.190</t>
-        </is>
+      <c r="W16" t="n">
+        <v>7.587227678750804</v>
       </c>
       <c r="X16" t="n">
         <v>-22446.19013596027</v>
@@ -7040,7 +6824,7 @@
         <v>2.934456815630635e-13</v>
       </c>
       <c r="Z16" t="n">
-        <v>610.1700000000001</v>
+        <v>3470.791470776857</v>
       </c>
       <c r="AA16" t="n">
         <v>1e-08</v>
@@ -7080,10 +6864,8 @@
       <c r="K17" t="n">
         <v>82.59867494685955</v>
       </c>
-      <c r="W17" t="inlineStr">
-        <is>
-          <t>y = 7.698x + -22596.090</t>
-        </is>
+      <c r="W17" t="n">
+        <v>7.698179601444978</v>
       </c>
       <c r="X17" t="n">
         <v>-22596.09049655399</v>
@@ -7092,7 +6874,7 @@
         <v>4.093997846238827e-11</v>
       </c>
       <c r="Z17" t="n">
-        <v>598.5599999999999</v>
+        <v>3439.868900978634</v>
       </c>
       <c r="AA17" t="n">
         <v>1.000000000000001e-08</v>
@@ -7132,10 +6914,8 @@
       <c r="K18" t="n">
         <v>82.3239304054328</v>
       </c>
-      <c r="W18" t="inlineStr">
-        <is>
-          <t>y = 7.419x + -21479.229</t>
-        </is>
+      <c r="W18" t="n">
+        <v>7.419496836146045</v>
       </c>
       <c r="X18" t="n">
         <v>-21479.22854676919</v>
@@ -7144,7 +6924,7 @@
         <v>3.318572629114995e-10</v>
       </c>
       <c r="Z18" t="n">
-        <v>613.0899999999997</v>
+        <v>3407.362653459402</v>
       </c>
       <c r="AA18" t="n">
         <v>1.000000000000108e-08</v>
@@ -7184,10 +6964,8 @@
       <c r="K19" t="n">
         <v>82.67180465252127</v>
       </c>
-      <c r="W19" t="inlineStr">
-        <is>
-          <t>y = 7.776x + -22439.000</t>
-        </is>
+      <c r="W19" t="n">
+        <v>7.775858499810237</v>
       </c>
       <c r="X19" t="n">
         <v>-22438.99957906457</v>
@@ -7196,7 +6974,7 @@
         <v>3.254157878042292e-10</v>
       </c>
       <c r="Z19" t="n">
-        <v>594.2599999999998</v>
+        <v>3376.308599464076</v>
       </c>
       <c r="AA19" t="n">
         <v>1.000000000000126e-08</v>
@@ -7236,10 +7014,8 @@
       <c r="K20" t="n">
         <v>82.78546780548824</v>
       </c>
-      <c r="W20" t="inlineStr">
-        <is>
-          <t>y = 7.900x + -22600.622</t>
-        </is>
+      <c r="W20" t="n">
+        <v>7.899701026673189</v>
       </c>
       <c r="X20" t="n">
         <v>-22600.62203483048</v>
@@ -7248,7 +7024,7 @@
         <v>4.211313836099983e-10</v>
       </c>
       <c r="Z20" t="n">
-        <v>582.8000000000002</v>
+        <v>3343.295576878203</v>
       </c>
       <c r="AA20" t="n">
         <v>1.000000000000235e-08</v>
@@ -7288,10 +7064,8 @@
       <c r="K21" t="n">
         <v>82.84831353049789</v>
       </c>
-      <c r="W21" t="inlineStr">
-        <is>
-          <t>y = 7.970x + -22600.837</t>
-        </is>
+      <c r="W21" t="n">
+        <v>7.969855957690283</v>
       </c>
       <c r="X21" t="n">
         <v>-22600.83675982003</v>
@@ -7300,7 +7074,7 @@
         <v>4.352747599166061e-10</v>
       </c>
       <c r="Z21" t="n">
-        <v>577.4700000000003</v>
+        <v>3311.167146405325</v>
       </c>
       <c r="AA21" t="n">
         <v>1.000000000000249e-08</v>
@@ -7340,10 +7114,8 @@
       <c r="K22" t="n">
         <v>82.9000537171266</v>
       </c>
-      <c r="W22" t="inlineStr">
-        <is>
-          <t>y = 8.029x + -22571.668</t>
-        </is>
+      <c r="W22" t="n">
+        <v>8.02854099564165</v>
       </c>
       <c r="X22" t="n">
         <v>-22571.66848477024</v>
@@ -7352,7 +7124,7 @@
         <v>5.382503022771223e-10</v>
       </c>
       <c r="Z22" t="n">
-        <v>572.5799999999999</v>
+        <v>3279.976366698247</v>
       </c>
       <c r="AA22" t="n">
         <v>1.000000000000328e-08</v>
@@ -7478,12 +7250,12 @@
       </c>
       <c r="W1" t="inlineStr">
         <is>
-          <t>Model</t>
+          <t>linear_eq_m</t>
         </is>
       </c>
       <c r="X1" t="inlineStr">
         <is>
-          <t>b</t>
+          <t>linear_eq_b</t>
         </is>
       </c>
       <c r="Y1" t="inlineStr">
@@ -7538,10 +7310,8 @@
       <c r="K2" t="n">
         <v>67.8967954848812</v>
       </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>y = 2.462x + -49517.091</t>
-        </is>
+      <c r="W2" t="n">
+        <v>2.462307943772473</v>
       </c>
       <c r="X2" t="n">
         <v>-49517.09064727029</v>
@@ -7550,7 +7320,7 @@
         <v>2129.258059778241</v>
       </c>
       <c r="Z2" t="n">
-        <v>2141.299999999999</v>
+        <v>1951.723150083427</v>
       </c>
       <c r="AA2" t="n">
         <v>1.331561679608598e-06</v>
@@ -7590,10 +7360,8 @@
       <c r="K3" t="n">
         <v>68.40828343426492</v>
       </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>y = 2.527x + -47690.154</t>
-        </is>
+      <c r="W3" t="n">
+        <v>2.526778916544654</v>
       </c>
       <c r="X3" t="n">
         <v>-47690.15351683742</v>
@@ -7602,7 +7370,7 @@
         <v>1024.357689096387</v>
       </c>
       <c r="Z3" t="n">
-        <v>2049</v>
+        <v>805.7256111545275</v>
       </c>
       <c r="AA3" t="n">
         <v>5.084512325403472e-06</v>
@@ -7642,10 +7410,8 @@
       <c r="K4" t="n">
         <v>68.7005504568087</v>
       </c>
-      <c r="W4" t="inlineStr">
-        <is>
-          <t>y = 2.565x + -47355.050</t>
-        </is>
+      <c r="W4" t="n">
+        <v>2.564940179461613</v>
       </c>
       <c r="X4" t="n">
         <v>-47355.04958175466</v>
@@ -7654,7 +7420,7 @@
         <v>1024.280845988597</v>
       </c>
       <c r="Z4" t="n">
-        <v>2006</v>
+        <v>805.6647883388291</v>
       </c>
       <c r="AA4" t="n">
         <v>5.758943613172105e-07</v>
@@ -7694,10 +7460,8 @@
       <c r="K5" t="n">
         <v>68.69624047288853</v>
       </c>
-      <c r="W5" t="inlineStr">
-        <is>
-          <t>y = 2.564x + -46602.830</t>
-        </is>
+      <c r="W5" t="n">
+        <v>2.564370177372474</v>
       </c>
       <c r="X5" t="n">
         <v>-46602.83010421869</v>
@@ -7706,7 +7470,7 @@
         <v>1020.435705028042</v>
       </c>
       <c r="Z5" t="n">
-        <v>1995.799999999999</v>
+        <v>802.6869968887955</v>
       </c>
       <c r="AA5" t="n">
         <v>5.815535215137008e-07</v>
@@ -7746,10 +7510,8 @@
       <c r="K6" t="n">
         <v>68.72210006186269</v>
       </c>
-      <c r="W6" t="inlineStr">
-        <is>
-          <t>y = 2.568x + -46037.558</t>
-        </is>
+      <c r="W6" t="n">
+        <v>2.567793450881607</v>
       </c>
       <c r="X6" t="n">
         <v>-46037.55812443314</v>
@@ -7758,7 +7520,7 @@
         <v>1018.750217461095</v>
       </c>
       <c r="Z6" t="n">
-        <v>1985</v>
+        <v>801.3644191667836</v>
       </c>
       <c r="AA6" t="n">
         <v>5.873364916621856e-07</v>
@@ -7798,10 +7560,8 @@
       <c r="K7" t="n">
         <v>68.83956829932609</v>
       </c>
-      <c r="W7" t="inlineStr">
-        <is>
-          <t>y = 2.583x + -45732.522</t>
-        </is>
+      <c r="W7" t="n">
+        <v>2.583444246888489</v>
       </c>
       <c r="X7" t="n">
         <v>-45732.5218983997</v>
@@ -7810,7 +7570,7 @@
         <v>1050.278977589443</v>
       </c>
       <c r="Z7" t="n">
-        <v>1968.5</v>
+        <v>825.9004722203405</v>
       </c>
       <c r="AA7" t="n">
         <v>6.083861780229042e-07</v>
@@ -7850,10 +7610,8 @@
       <c r="K8" t="n">
         <v>68.86571051610399</v>
       </c>
-      <c r="W8" t="inlineStr">
-        <is>
-          <t>y = 2.587x + -45235.986</t>
-        </is>
+      <c r="W8" t="n">
+        <v>2.586949862146434</v>
       </c>
       <c r="X8" t="n">
         <v>-45235.98649035033</v>
@@ -7862,7 +7620,7 @@
         <v>1034.012317430827</v>
       </c>
       <c r="Z8" t="n">
-        <v>1958.599999999999</v>
+        <v>813.2709220478805</v>
       </c>
       <c r="AA8" t="n">
         <v>6.070105779354064e-07</v>
@@ -7902,10 +7660,8 @@
       <c r="K9" t="n">
         <v>69.12960456163179</v>
       </c>
-      <c r="W9" t="inlineStr">
-        <is>
-          <t>y = 2.623x + -45376.592</t>
-        </is>
+      <c r="W9" t="n">
+        <v>2.622806744487687</v>
       </c>
       <c r="X9" t="n">
         <v>-45376.59162594052</v>
@@ -7914,7 +7670,7 @@
         <v>1032.644189121561</v>
       </c>
       <c r="Z9" t="n">
-        <v>1927.5</v>
+        <v>812.2355099879258</v>
       </c>
       <c r="AA9" t="n">
         <v>6.128409756477646e-07</v>
@@ -7954,10 +7710,8 @@
       <c r="K10" t="n">
         <v>69.22144833149954</v>
       </c>
-      <c r="W10" t="inlineStr">
-        <is>
-          <t>y = 2.635x + -45061.159</t>
-        </is>
+      <c r="W10" t="n">
+        <v>2.635490114028662</v>
       </c>
       <c r="X10" t="n">
         <v>-45061.15871900824</v>
@@ -7966,7 +7720,7 @@
         <v>1054.766489828831</v>
       </c>
       <c r="Z10" t="n">
-        <v>1911.800000000003</v>
+        <v>829.4637197581885</v>
       </c>
       <c r="AA10" t="n">
         <v>6.296471027099854e-07</v>
@@ -8006,10 +7760,8 @@
       <c r="K11" t="n">
         <v>69.27583805023222</v>
       </c>
-      <c r="W11" t="inlineStr">
-        <is>
-          <t>y = 2.643x + -44681.577</t>
-        </is>
+      <c r="W11" t="n">
+        <v>2.643051828466184</v>
       </c>
       <c r="X11" t="n">
         <v>-44681.57681083908</v>
@@ -8018,7 +7770,7 @@
         <v>1039.18120141719</v>
       </c>
       <c r="Z11" t="n">
-        <v>1900.5</v>
+        <v>817.3672774843495</v>
       </c>
       <c r="AA11" t="n">
         <v>6.282777388457208e-07</v>
@@ -8144,12 +7896,12 @@
       </c>
       <c r="W1" t="inlineStr">
         <is>
-          <t>Model</t>
+          <t>linear_eq_m</t>
         </is>
       </c>
       <c r="X1" t="inlineStr">
         <is>
-          <t>b</t>
+          <t>linear_eq_b</t>
         </is>
       </c>
       <c r="Y1" t="inlineStr">
@@ -8204,10 +7956,8 @@
       <c r="K2" t="n">
         <v>81.92598843870702</v>
       </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>y = 7.049x + -25240.866</t>
-        </is>
+      <c r="W2" t="n">
+        <v>7.049286214257195</v>
       </c>
       <c r="X2" t="n">
         <v>-25240.86560628705</v>
@@ -8216,7 +7966,7 @@
         <v>6.270757693317334e-11</v>
       </c>
       <c r="Z2" t="n">
-        <v>689.3400000000001</v>
+        <v>4205.884890064634</v>
       </c>
       <c r="AA2" t="n">
         <v>1.000000000000227e-08</v>
@@ -8256,10 +8006,8 @@
       <c r="K3" t="n">
         <v>82.52186782671926</v>
       </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>y = 7.618x + -25918.451</t>
-        </is>
+      <c r="W3" t="n">
+        <v>7.618221291437048</v>
       </c>
       <c r="X3" t="n">
         <v>-25918.45067978542</v>
@@ -8268,7 +8016,7 @@
         <v>1.366125040588221e-09</v>
       </c>
       <c r="Z3" t="n">
-        <v>622.9000000000001</v>
+        <v>4006.036155422891</v>
       </c>
       <c r="AA3" t="n">
         <v>1.000000000001866e-08</v>
@@ -8308,10 +8056,8 @@
       <c r="K4" t="n">
         <v>82.19585679206008</v>
       </c>
-      <c r="W4" t="inlineStr">
-        <is>
-          <t>y = 7.296x + -24256.194</t>
-        </is>
+      <c r="W4" t="n">
+        <v>7.29625406322539</v>
       </c>
       <c r="X4" t="n">
         <v>-24256.1941018422</v>
@@ -8320,7 +8066,7 @@
         <v>1.090156318120623e-10</v>
       </c>
       <c r="Z4" t="n">
-        <v>637.5699999999997</v>
+        <v>3935.821912233584</v>
       </c>
       <c r="AA4" t="n">
         <v>1.00000000000013e-08</v>
@@ -8360,10 +8106,8 @@
       <c r="K5" t="n">
         <v>82.58540269535408</v>
       </c>
-      <c r="W5" t="inlineStr">
-        <is>
-          <t>y = 7.684x + -25357.761</t>
-        </is>
+      <c r="W5" t="n">
+        <v>7.684245096782929</v>
       </c>
       <c r="X5" t="n">
         <v>-25357.76128331328</v>
@@ -8372,7 +8116,7 @@
         <v>1.062312420446039e-09</v>
       </c>
       <c r="Z5" t="n">
-        <v>610.0599999999999</v>
+        <v>3883.031795920439</v>
       </c>
       <c r="AA5" t="n">
         <v>1.000000000003094e-08</v>
@@ -8412,10 +8156,8 @@
       <c r="K6" t="n">
         <v>82.33371852200311</v>
       </c>
-      <c r="W6" t="inlineStr">
-        <is>
-          <t>y = 7.429x + -24112.986</t>
-        </is>
+      <c r="W6" t="n">
+        <v>7.429084099949907</v>
       </c>
       <c r="X6" t="n">
         <v>-24112.9860223846</v>
@@ -8424,7 +8166,7 @@
         <v>8.118152899628944e-10</v>
       </c>
       <c r="Z6" t="n">
-        <v>620.27</v>
+        <v>3835.022553553898</v>
       </c>
       <c r="AA6" t="n">
         <v>1.000000000085918e-08</v>
@@ -8464,10 +8206,8 @@
       <c r="K7" t="n">
         <v>82.34583155799149</v>
       </c>
-      <c r="W7" t="inlineStr">
-        <is>
-          <t>y = 7.441x + -23880.978</t>
-        </is>
+      <c r="W7" t="n">
+        <v>7.44098232084799</v>
       </c>
       <c r="X7" t="n">
         <v>-23880.97846679137</v>
@@ -8476,7 +8216,7 @@
         <v>5.527629492869572e-09</v>
       </c>
       <c r="Z7" t="n">
-        <v>617.1799999999998</v>
+        <v>3789.242727888626</v>
       </c>
       <c r="AA7" t="n">
         <v>1.000000000001076e-08</v>
@@ -8516,10 +8256,8 @@
       <c r="K8" t="n">
         <v>82.44111830493971</v>
       </c>
-      <c r="W8" t="inlineStr">
-        <is>
-          <t>y = 7.536x + -23942.900</t>
-        </is>
+      <c r="W8" t="n">
+        <v>7.535901164749899</v>
       </c>
       <c r="X8" t="n">
         <v>-23942.89984628868</v>
@@ -8528,7 +8266,7 @@
         <v>1.841086815799093e-18</v>
       </c>
       <c r="Z8" t="n">
-        <v>605.4100000000003</v>
+        <v>3746.924357180184</v>
       </c>
       <c r="AA8" t="n">
         <v>1e-08</v>
@@ -8568,10 +8306,8 @@
       <c r="K9" t="n">
         <v>82.11554340852989</v>
       </c>
-      <c r="W9" t="inlineStr">
-        <is>
-          <t>y = 7.221x + -22608.239</t>
-        </is>
+      <c r="W9" t="n">
+        <v>7.221000223836894</v>
       </c>
       <c r="X9" t="n">
         <v>-22608.23938092466</v>
@@ -8580,7 +8316,7 @@
         <v>5.253107119837181e-09</v>
       </c>
       <c r="Z9" t="n">
-        <v>625.48</v>
+        <v>3707.706541242992</v>
       </c>
       <c r="AA9" t="n">
         <v>1.000000000000546e-08</v>
@@ -8620,10 +8356,8 @@
       <c r="K10" t="n">
         <v>82.46241860074358</v>
       </c>
-      <c r="W10" t="inlineStr">
-        <is>
-          <t>y = 7.557x + -23554.239</t>
-        </is>
+      <c r="W10" t="n">
+        <v>7.557445478560795</v>
       </c>
       <c r="X10" t="n">
         <v>-23554.23940132603</v>
@@ -8632,7 +8366,7 @@
         <v>1.065173126294553e-09</v>
       </c>
       <c r="Z10" t="n">
-        <v>607.4200000000001</v>
+        <v>3671.700118648755</v>
       </c>
       <c r="AA10" t="n">
         <v>1.000000000003668e-08</v>
@@ -8672,10 +8406,8 @@
       <c r="K11" t="n">
         <v>82.25373176874217</v>
       </c>
-      <c r="W11" t="inlineStr">
-        <is>
-          <t>y = 7.351x + -22608.792</t>
-        </is>
+      <c r="W11" t="n">
+        <v>7.351444418213736</v>
       </c>
       <c r="X11" t="n">
         <v>-22608.79222095496</v>
@@ -8684,7 +8416,7 @@
         <v>1.443028795686406e-11</v>
       </c>
       <c r="Z11" t="n">
-        <v>607.5099999999998</v>
+        <v>3636.999587679381</v>
       </c>
       <c r="AA11" t="n">
         <v>1e-08</v>
@@ -8724,10 +8456,8 @@
       <c r="K12" t="n">
         <v>82.70205581033102</v>
       </c>
-      <c r="W12" t="inlineStr">
-        <is>
-          <t>y = 7.808x + -23927.933</t>
-        </is>
+      <c r="W12" t="n">
+        <v>7.80844417533286</v>
       </c>
       <c r="X12" t="n">
         <v>-23927.93281765433</v>
@@ -8736,7 +8466,7 @@
         <v>6.340449691658653e-09</v>
       </c>
       <c r="Z12" t="n">
-        <v>580.0799999999999</v>
+        <v>3601.486744222801</v>
       </c>
       <c r="AA12" t="n">
         <v>1.000000000000003e-08</v>
@@ -8776,10 +8506,8 @@
       <c r="K13" t="n">
         <v>82.74905240944111</v>
       </c>
-      <c r="W13" t="inlineStr">
-        <is>
-          <t>y = 7.860x + -23877.651</t>
-        </is>
+      <c r="W13" t="n">
+        <v>7.859603940662041</v>
       </c>
       <c r="X13" t="n">
         <v>-23877.65084057717</v>
@@ -8788,7 +8516,7 @@
         <v>2.483823806000081e-09</v>
       </c>
       <c r="Z13" t="n">
-        <v>573.3999999999996</v>
+        <v>3567.391755983299</v>
       </c>
       <c r="AA13" t="n">
         <v>1.00000000000465e-08</v>
@@ -8828,10 +8556,8 @@
       <c r="K14" t="n">
         <v>82.86281829493637</v>
       </c>
-      <c r="W14" t="inlineStr">
-        <is>
-          <t>y = 7.986x + -24035.146</t>
-        </is>
+      <c r="W14" t="n">
+        <v>7.986222243966027</v>
       </c>
       <c r="X14" t="n">
         <v>-24035.14571194406</v>
@@ -8840,7 +8566,7 @@
         <v>8.260371997464482e-10</v>
       </c>
       <c r="Z14" t="n">
-        <v>562.2199999999998</v>
+        <v>3530.136990515655</v>
       </c>
       <c r="AA14" t="n">
         <v>1.00000000000052e-08</v>
@@ -8880,10 +8606,8 @@
       <c r="K15" t="n">
         <v>82.94103451587154</v>
       </c>
-      <c r="W15" t="inlineStr">
-        <is>
-          <t>y = 8.076x + -24077.967</t>
-        </is>
+      <c r="W15" t="n">
+        <v>8.07562985450261</v>
       </c>
       <c r="X15" t="n">
         <v>-24077.96734353064</v>
@@ -8892,7 +8616,7 @@
         <v>1.045967857513008e-08</v>
       </c>
       <c r="Z15" t="n">
-        <v>555.21</v>
+        <v>3494.753960988774</v>
       </c>
       <c r="AA15" t="n">
         <v>1.000000000000096e-08</v>
@@ -8932,10 +8656,8 @@
       <c r="K16" t="n">
         <v>83.0375652473957</v>
       </c>
-      <c r="W16" t="inlineStr">
-        <is>
-          <t>y = 8.189x + -24198.237</t>
-        </is>
+      <c r="W16" t="n">
+        <v>8.188727723224851</v>
       </c>
       <c r="X16" t="n">
         <v>-24198.23749121563</v>
@@ -8944,7 +8666,7 @@
         <v>1.948108843070904e-11</v>
       </c>
       <c r="Z16" t="n">
-        <v>546.6100000000001</v>
+        <v>3458.818557263857</v>
       </c>
       <c r="AA16" t="n">
         <v>1e-08</v>
@@ -8984,10 +8706,8 @@
       <c r="K17" t="n">
         <v>82.79544935182111</v>
       </c>
-      <c r="W17" t="inlineStr">
-        <is>
-          <t>y = 7.911x + -23037.618</t>
-        </is>
+      <c r="W17" t="n">
+        <v>7.910762136185138</v>
       </c>
       <c r="X17" t="n">
         <v>-23037.61815999198</v>
@@ -8996,7 +8716,7 @@
         <v>1.043567252003006e-10</v>
       </c>
       <c r="Z17" t="n">
-        <v>557.5999999999999</v>
+        <v>3422.892343149957</v>
       </c>
       <c r="AA17" t="n">
         <v>1.000000000000179e-08</v>
@@ -9036,10 +8756,8 @@
       <c r="K18" t="n">
         <v>83.14318054784211</v>
       </c>
-      <c r="W18" t="inlineStr">
-        <is>
-          <t>y = 8.316x + -24101.993</t>
-        </is>
+      <c r="W18" t="n">
+        <v>8.316099111059023</v>
       </c>
       <c r="X18" t="n">
         <v>-24101.99252541294</v>
@@ -9048,7 +8766,7 @@
         <v>9.423737355848379e-10</v>
       </c>
       <c r="Z18" t="n">
-        <v>540.46</v>
+        <v>3386.592759906148</v>
       </c>
       <c r="AA18" t="n">
         <v>1.000000000013627e-08</v>
@@ -9088,10 +8806,8 @@
       <c r="K19" t="n">
         <v>83.23921478381426</v>
       </c>
-      <c r="W19" t="inlineStr">
-        <is>
-          <t>y = 8.435x + -24210.426</t>
-        </is>
+      <c r="W19" t="n">
+        <v>8.435353424215609</v>
       </c>
       <c r="X19" t="n">
         <v>-24210.42648286345</v>
@@ -9100,7 +8816,7 @@
         <v>7.560569546736046e-10</v>
       </c>
       <c r="Z19" t="n">
-        <v>529.46</v>
+        <v>3350.73296563084</v>
       </c>
       <c r="AA19" t="n">
         <v>1.000000000000281e-08</v>
@@ -9140,10 +8856,8 @@
       <c r="K20" t="n">
         <v>83.08193209915974</v>
       </c>
-      <c r="W20" t="inlineStr">
-        <is>
-          <t>y = 8.242x + -23325.088</t>
-        </is>
+      <c r="W20" t="n">
+        <v>8.241762454362968</v>
       </c>
       <c r="X20" t="n">
         <v>-23325.0883676794</v>
@@ -9152,7 +8866,7 @@
         <v>8.443247870371154e-10</v>
       </c>
       <c r="Z20" t="n">
-        <v>533.9000000000001</v>
+        <v>3315.237452897345</v>
       </c>
       <c r="AA20" t="n">
         <v>1.00000000000028e-08</v>
@@ -9192,10 +8906,8 @@
       <c r="K21" t="n">
         <v>83.46426574963074</v>
       </c>
-      <c r="W21" t="inlineStr">
-        <is>
-          <t>y = 8.728x + -24580.988</t>
-        </is>
+      <c r="W21" t="n">
+        <v>8.728484192577547</v>
       </c>
       <c r="X21" t="n">
         <v>-24580.98805300962</v>
@@ -9204,7 +8916,7 @@
         <v>1.059451165241389e-09</v>
       </c>
       <c r="Z21" t="n">
-        <v>510.9400000000001</v>
+        <v>3280.066896952231</v>
       </c>
       <c r="AA21" t="n">
         <v>1.000000000000019e-08</v>
@@ -9244,10 +8956,8 @@
       <c r="K22" t="n">
         <v>83.20923398910719</v>
       </c>
-      <c r="W22" t="inlineStr">
-        <is>
-          <t>y = 8.398x + -23311.864</t>
-        </is>
+      <c r="W22" t="n">
+        <v>8.397763159282347</v>
       </c>
       <c r="X22" t="n">
         <v>-23311.86417902619</v>
@@ -9256,7 +8966,7 @@
         <v>5.943266053885061e-11</v>
       </c>
       <c r="Z22" t="n">
-        <v>520.3700000000003</v>
+        <v>3244.75084351878</v>
       </c>
       <c r="AA22" t="n">
         <v>1.000000000000284e-08</v>
@@ -9382,12 +9092,12 @@
       </c>
       <c r="W1" t="inlineStr">
         <is>
-          <t>Model</t>
+          <t>linear_eq_m</t>
         </is>
       </c>
       <c r="X1" t="inlineStr">
         <is>
-          <t>b</t>
+          <t>linear_eq_b</t>
         </is>
       </c>
       <c r="Y1" t="inlineStr">
@@ -9442,10 +9152,8 @@
       <c r="K2" t="n">
         <v>14.04836917377372</v>
       </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>y = 0.250x + 1473.925</t>
-        </is>
+      <c r="W2" t="n">
+        <v>0.250224872485355</v>
       </c>
       <c r="X2" t="n">
         <v>1473.924585948794</v>
@@ -9454,7 +9162,7 @@
         <v>1401.196004579856</v>
       </c>
       <c r="Z2" t="n">
-        <v>7685.355</v>
+        <v>1631.18191604417</v>
       </c>
       <c r="AA2" t="n">
         <v>1.051011123548062e-06</v>
@@ -9494,10 +9202,8 @@
       <c r="K3" t="n">
         <v>12.42863116636923</v>
       </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>y = 0.220x + 1422.857</t>
-        </is>
+      <c r="W3" t="n">
+        <v>0.2203881811794194</v>
       </c>
       <c r="X3" t="n">
         <v>1422.856753080394</v>
@@ -9506,7 +9212,7 @@
         <v>1347.116838125768</v>
       </c>
       <c r="Z3" t="n">
-        <v>6655.179999999999</v>
+        <v>1908.251136774144</v>
       </c>
       <c r="AA3" t="n">
         <v>1.08770333002106e-06</v>
@@ -9546,10 +9252,8 @@
       <c r="K4" t="n">
         <v>11.98989350002953</v>
       </c>
-      <c r="W4" t="inlineStr">
-        <is>
-          <t>y = 0.212x + 1403.473</t>
-        </is>
+      <c r="W4" t="n">
+        <v>0.2123722074512932</v>
       </c>
       <c r="X4" t="n">
         <v>1403.472960239763</v>
@@ -9558,7 +9262,7 @@
         <v>1332.669021893373</v>
       </c>
       <c r="Z4" t="n">
-        <v>6413.009999999999</v>
+        <v>1978.149661239184</v>
       </c>
       <c r="AA4" t="n">
         <v>4.270518337465608e-07</v>
@@ -9598,10 +9302,8 @@
       <c r="K5" t="n">
         <v>80.32331536215419</v>
       </c>
-      <c r="W5" t="inlineStr">
-        <is>
-          <t>y = 5.865x + -32709.549</t>
-        </is>
+      <c r="W5" t="n">
+        <v>5.864609396856677</v>
       </c>
       <c r="X5" t="n">
         <v>-32709.54889527945</v>
@@ -9610,7 +9312,7 @@
         <v>1326.417365955968</v>
       </c>
       <c r="Z5" t="n">
-        <v>870.4200000000001</v>
+        <v>1998.175729126543</v>
       </c>
       <c r="AA5" t="n">
         <v>6.826957621136403e-07</v>
@@ -9650,10 +9352,8 @@
       <c r="K6" t="n">
         <v>80.35829297873626</v>
       </c>
-      <c r="W6" t="inlineStr">
-        <is>
-          <t>y = 5.886x + -32337.579</t>
-        </is>
+      <c r="W6" t="n">
+        <v>5.886293953849571</v>
       </c>
       <c r="X6" t="n">
         <v>-32337.57892839805</v>
@@ -9662,7 +9362,7 @@
         <v>1320.827331146576</v>
       </c>
       <c r="Z6" t="n">
-        <v>864.4000000000005</v>
+        <v>2033.248541069018</v>
       </c>
       <c r="AA6" t="n">
         <v>7.760050573478072e-07</v>
@@ -9702,10 +9402,8 @@
       <c r="K7" t="n">
         <v>80.39969583627452</v>
       </c>
-      <c r="W7" t="inlineStr">
-        <is>
-          <t>y = 5.912x + -32085.271</t>
-        </is>
+      <c r="W7" t="n">
+        <v>5.912164149640939</v>
       </c>
       <c r="X7" t="n">
         <v>-32085.27061135535</v>
@@ -9714,7 +9412,7 @@
         <v>1315.908761296211</v>
       </c>
       <c r="Z7" t="n">
-        <v>858.6799999999994</v>
+        <v>2022.189329838532</v>
       </c>
       <c r="AA7" t="n">
         <v>7.749964132148386e-07</v>
@@ -9754,10 +9452,8 @@
       <c r="K8" t="n">
         <v>80.53824382515876</v>
       </c>
-      <c r="W8" t="inlineStr">
-        <is>
-          <t>y = 6.000x + -32163.559</t>
-        </is>
+      <c r="W8" t="n">
+        <v>6.000365549949415</v>
       </c>
       <c r="X8" t="n">
         <v>-32163.55918792906</v>
@@ -9766,7 +9462,7 @@
         <v>1307.59177113655</v>
       </c>
       <c r="Z8" t="n">
-        <v>839.7600000000002</v>
+        <v>2080.286576406515</v>
       </c>
       <c r="AA8" t="n">
         <v>6.154688151701993e-07</v>
@@ -9806,10 +9502,8 @@
       <c r="K9" t="n">
         <v>80.6858002155312</v>
       </c>
-      <c r="W9" t="inlineStr">
-        <is>
-          <t>y = 6.097x + -32317.318</t>
-        </is>
+      <c r="W9" t="n">
+        <v>6.097160595387405</v>
       </c>
       <c r="X9" t="n">
         <v>-32317.31811041562</v>
@@ -9818,7 +9512,7 @@
         <v>1280.492410046041</v>
       </c>
       <c r="Z9" t="n">
-        <v>828.3000000000002</v>
+        <v>2085.27265334374</v>
       </c>
       <c r="AA9" t="n">
         <v>3.492951438614063e-07</v>
@@ -9858,10 +9552,8 @@
       <c r="K10" t="n">
         <v>80.56235710207405</v>
       </c>
-      <c r="W10" t="inlineStr">
-        <is>
-          <t>y = 6.016x + -31493.670</t>
-        </is>
+      <c r="W10" t="n">
+        <v>6.015978499081236</v>
       </c>
       <c r="X10" t="n">
         <v>-31493.67015169379</v>
@@ -9870,7 +9562,7 @@
         <v>1274.975530408735</v>
       </c>
       <c r="Z10" t="n">
-        <v>834.3899999999994</v>
+        <v>2094.781360184912</v>
       </c>
       <c r="AA10" t="n">
         <v>3.42099152654186e-07</v>
@@ -9910,10 +9602,8 @@
       <c r="K11" t="n">
         <v>80.67249240768061</v>
       </c>
-      <c r="W11" t="inlineStr">
-        <is>
-          <t>y = 6.088x + -31522.520</t>
-        </is>
+      <c r="W11" t="n">
+        <v>6.088306330156096</v>
       </c>
       <c r="X11" t="n">
         <v>-31522.51990936588</v>
@@ -9922,7 +9612,7 @@
         <v>1268.580589533905</v>
       </c>
       <c r="Z11" t="n">
-        <v>823.4700000000003</v>
+        <v>2113.911687240773</v>
       </c>
       <c r="AA11" t="n">
         <v>3.320901754157028e-07</v>

</xml_diff>

<commit_message>
updated how the time is calcauted
</commit_message>
<xml_diff>
--- a/BioSensorAnalysisSrcCode/EIS_Analysis/Austin_EIS/MegaExcel/Processed Chips for PCAI1ia/Chip 21.xlsx
+++ b/BioSensorAnalysisSrcCode/EIS_Analysis/Austin_EIS/MegaExcel/Processed Chips for PCAI1ia/Chip 21.xlsx
@@ -428,7 +428,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>time(s)</t>
+          <t>time(mins)</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -559,7 +559,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>3</v>
+        <v>1.5</v>
       </c>
       <c r="B2" t="n">
         <v>-604.1999999999998</v>
@@ -609,7 +609,7 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="B3" t="n">
         <v>-559.77</v>
@@ -659,7 +659,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>9</v>
+        <v>4.5</v>
       </c>
       <c r="B4" t="n">
         <v>-540.23</v>
@@ -709,7 +709,7 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="B5" t="n">
         <v>-512.1300000000001</v>
@@ -759,7 +759,7 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>15</v>
+        <v>7.5</v>
       </c>
       <c r="B6" t="n">
         <v>-504.75</v>
@@ -809,7 +809,7 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="B7" t="n">
         <v>-493.4400000000001</v>
@@ -859,7 +859,7 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>21</v>
+        <v>10.5</v>
       </c>
       <c r="B8" t="n">
         <v>-496.9099999999999</v>
@@ -909,7 +909,7 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="B9" t="n">
         <v>-489.0599999999999</v>
@@ -959,7 +959,7 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>27</v>
+        <v>13.5</v>
       </c>
       <c r="B10" t="n">
         <v>-477.1399999999999</v>
@@ -1009,7 +1009,7 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="B11" t="n">
         <v>-455.8200000000002</v>
@@ -1074,7 +1074,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>time(s)</t>
+          <t>time(mins)</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -2270,7 +2270,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>time(s)</t>
+          <t>time(mins)</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -3466,7 +3466,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>time(s)</t>
+          <t>time(mins)</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -3597,7 +3597,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>3</v>
+        <v>1.5</v>
       </c>
       <c r="B2" t="n">
         <v>-2982.699999999997</v>
@@ -3647,7 +3647,7 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="B3" t="n">
         <v>-2560.099999999999</v>
@@ -3697,7 +3697,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>9</v>
+        <v>4.5</v>
       </c>
       <c r="B4" t="n">
         <v>-2463.299999999999</v>
@@ -3747,7 +3747,7 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="B5" t="n">
         <v>-2418.199999999997</v>
@@ -3797,7 +3797,7 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>15</v>
+        <v>7.5</v>
       </c>
       <c r="B6" t="n">
         <v>-2392.299999999999</v>
@@ -3847,7 +3847,7 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="B7" t="n">
         <v>-2369</v>
@@ -3897,7 +3897,7 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>21</v>
+        <v>10.5</v>
       </c>
       <c r="B8" t="n">
         <v>-2363.799999999999</v>
@@ -3947,7 +3947,7 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="B9" t="n">
         <v>-2347.199999999997</v>
@@ -3997,7 +3997,7 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>27</v>
+        <v>13.5</v>
       </c>
       <c r="B10" t="n">
         <v>-2334.799999999999</v>
@@ -4047,7 +4047,7 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="B11" t="n">
         <v>-2328.900000000001</v>
@@ -4112,7 +4112,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>time(s)</t>
+          <t>time(mins)</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -5308,7 +5308,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>time(s)</t>
+          <t>time(mins)</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -5439,7 +5439,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>3</v>
+        <v>1.5</v>
       </c>
       <c r="B2" t="n">
         <v>-2912.600000000002</v>
@@ -5489,7 +5489,7 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="B3" t="n">
         <v>-2718.200000000001</v>
@@ -5539,7 +5539,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>9</v>
+        <v>4.5</v>
       </c>
       <c r="B4" t="n">
         <v>-2677.599999999999</v>
@@ -5589,7 +5589,7 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="B5" t="n">
         <v>-2665.600000000002</v>
@@ -5639,7 +5639,7 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>15</v>
+        <v>7.5</v>
       </c>
       <c r="B6" t="n">
         <v>-2695.099999999999</v>
@@ -5689,7 +5689,7 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="B7" t="n">
         <v>-2688.900000000001</v>
@@ -5739,7 +5739,7 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>21</v>
+        <v>10.5</v>
       </c>
       <c r="B8" t="n">
         <v>-2689.600000000002</v>
@@ -5789,7 +5789,7 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="B9" t="n">
         <v>-2663.900000000001</v>
@@ -5839,7 +5839,7 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>27</v>
+        <v>13.5</v>
       </c>
       <c r="B10" t="n">
         <v>-2681.299999999999</v>
@@ -5889,7 +5889,7 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="B11" t="n">
         <v>-2660.700000000001</v>
@@ -5954,7 +5954,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>time(s)</t>
+          <t>time(mins)</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -7150,7 +7150,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>time(s)</t>
+          <t>time(mins)</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -7281,7 +7281,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>3</v>
+        <v>1.5</v>
       </c>
       <c r="B2" t="n">
         <v>-2141.299999999999</v>
@@ -7331,7 +7331,7 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="B3" t="n">
         <v>-2049</v>
@@ -7381,7 +7381,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>9</v>
+        <v>4.5</v>
       </c>
       <c r="B4" t="n">
         <v>-2006</v>
@@ -7431,7 +7431,7 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="B5" t="n">
         <v>-1995.799999999999</v>
@@ -7481,7 +7481,7 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>15</v>
+        <v>7.5</v>
       </c>
       <c r="B6" t="n">
         <v>-1985</v>
@@ -7531,7 +7531,7 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="B7" t="n">
         <v>-1968.5</v>
@@ -7581,7 +7581,7 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>21</v>
+        <v>10.5</v>
       </c>
       <c r="B8" t="n">
         <v>-1958.599999999999</v>
@@ -7631,7 +7631,7 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="B9" t="n">
         <v>-1927.5</v>
@@ -7681,7 +7681,7 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>27</v>
+        <v>13.5</v>
       </c>
       <c r="B10" t="n">
         <v>-1911.800000000003</v>
@@ -7731,7 +7731,7 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="B11" t="n">
         <v>-1900.5</v>
@@ -7796,7 +7796,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>time(s)</t>
+          <t>time(mins)</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -8992,7 +8992,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>time(s)</t>
+          <t>time(mins)</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -9123,7 +9123,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>3</v>
+        <v>1.5</v>
       </c>
       <c r="B2" t="n">
         <v>-7685.355</v>
@@ -9173,7 +9173,7 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="B3" t="n">
         <v>-6655.179999999999</v>
@@ -9223,7 +9223,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>9</v>
+        <v>4.5</v>
       </c>
       <c r="B4" t="n">
         <v>-6413.009999999999</v>
@@ -9273,7 +9273,7 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="B5" t="n">
         <v>-870.4200000000001</v>
@@ -9323,7 +9323,7 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>15</v>
+        <v>7.5</v>
       </c>
       <c r="B6" t="n">
         <v>-864.4000000000005</v>
@@ -9373,7 +9373,7 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="B7" t="n">
         <v>-858.6799999999994</v>
@@ -9423,7 +9423,7 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>21</v>
+        <v>10.5</v>
       </c>
       <c r="B8" t="n">
         <v>-839.7600000000002</v>
@@ -9473,7 +9473,7 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="B9" t="n">
         <v>-828.3000000000002</v>
@@ -9523,7 +9523,7 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>27</v>
+        <v>13.5</v>
       </c>
       <c r="B10" t="n">
         <v>-834.3899999999994</v>
@@ -9573,7 +9573,7 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="B11" t="n">
         <v>-823.4700000000003</v>

</xml_diff>

<commit_message>
changed code b/c found error with negative resistance
</commit_message>
<xml_diff>
--- a/BioSensorAnalysisSrcCode/EIS_Analysis/Austin_EIS/MegaExcel/Processed Chips for PCAI1ia/Chip 21.xlsx
+++ b/BioSensorAnalysisSrcCode/EIS_Analysis/Austin_EIS/MegaExcel/Processed Chips for PCAI1ia/Chip 21.xlsx
@@ -562,7 +562,7 @@
         <v>1.5</v>
       </c>
       <c r="B2" t="n">
-        <v>-604.1999999999998</v>
+        <v>3413.305</v>
       </c>
       <c r="D2" t="n">
         <v>1.84241e-07</v>
@@ -612,7 +612,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="n">
-        <v>-559.77</v>
+        <v>3306.557</v>
       </c>
       <c r="D3" t="n">
         <v>1.89606e-07</v>
@@ -662,7 +662,7 @@
         <v>4.5</v>
       </c>
       <c r="B4" t="n">
-        <v>-540.23</v>
+        <v>3231.904</v>
       </c>
       <c r="D4" t="n">
         <v>1.92888e-07</v>
@@ -712,7 +712,7 @@
         <v>6</v>
       </c>
       <c r="B5" t="n">
-        <v>-512.1300000000001</v>
+        <v>3169.252</v>
       </c>
       <c r="D5" t="n">
         <v>1.96208e-07</v>
@@ -762,7 +762,7 @@
         <v>7.5</v>
       </c>
       <c r="B6" t="n">
-        <v>-504.75</v>
+        <v>3112.06</v>
       </c>
       <c r="D6" t="n">
         <v>1.98503e-07</v>
@@ -812,7 +812,7 @@
         <v>9</v>
       </c>
       <c r="B7" t="n">
-        <v>-493.4400000000001</v>
+        <v>3058.458</v>
       </c>
       <c r="D7" t="n">
         <v>2.00804e-07</v>
@@ -862,7 +862,7 @@
         <v>10.5</v>
       </c>
       <c r="B8" t="n">
-        <v>-496.9099999999999</v>
+        <v>3000.47</v>
       </c>
       <c r="D8" t="n">
         <v>2.02918e-07</v>
@@ -912,7 +912,7 @@
         <v>12</v>
       </c>
       <c r="B9" t="n">
-        <v>-489.0599999999999</v>
+        <v>2954.274</v>
       </c>
       <c r="D9" t="n">
         <v>2.04758e-07</v>
@@ -962,7 +962,7 @@
         <v>13.5</v>
       </c>
       <c r="B10" t="n">
-        <v>-477.1399999999999</v>
+        <v>2919.242</v>
       </c>
       <c r="D10" t="n">
         <v>2.06513e-07</v>
@@ -1012,7 +1012,7 @@
         <v>15</v>
       </c>
       <c r="B11" t="n">
-        <v>-455.8200000000002</v>
+        <v>2899.646</v>
       </c>
       <c r="D11" t="n">
         <v>2.08089e-07</v>
@@ -1208,7 +1208,7 @@
         <v>1.428571428571429</v>
       </c>
       <c r="B2" t="n">
-        <v>-570.52</v>
+        <v>3248.999</v>
       </c>
       <c r="D2" t="n">
         <v>1.88742e-07</v>
@@ -1258,7 +1258,7 @@
         <v>2.857142857142857</v>
       </c>
       <c r="B3" t="n">
-        <v>-576.1600000000003</v>
+        <v>3097.392</v>
       </c>
       <c r="D3" t="n">
         <v>1.94412e-07</v>
@@ -1308,7 +1308,7 @@
         <v>4.285714285714286</v>
       </c>
       <c r="B4" t="n">
-        <v>-551.21</v>
+        <v>3064.714</v>
       </c>
       <c r="D4" t="n">
         <v>1.96919e-07</v>
@@ -1358,7 +1358,7 @@
         <v>5.714285714285714</v>
       </c>
       <c r="B5" t="n">
-        <v>-560.8499999999999</v>
+        <v>3009.657</v>
       </c>
       <c r="D5" t="n">
         <v>1.98783e-07</v>
@@ -1408,7 +1408,7 @@
         <v>7.142857142857143</v>
       </c>
       <c r="B6" t="n">
-        <v>-574.8999999999996</v>
+        <v>2957.534</v>
       </c>
       <c r="D6" t="n">
         <v>2.0035e-07</v>
@@ -1458,7 +1458,7 @@
         <v>8.571428571428571</v>
       </c>
       <c r="B7" t="n">
-        <v>-546.5799999999999</v>
+        <v>2943.712</v>
       </c>
       <c r="D7" t="n">
         <v>2.02176e-07</v>
@@ -1508,7 +1508,7 @@
         <v>10</v>
       </c>
       <c r="B8" t="n">
-        <v>-542.5900000000001</v>
+        <v>2911.219</v>
       </c>
       <c r="D8" t="n">
         <v>2.03803e-07</v>
@@ -1558,7 +1558,7 @@
         <v>11.42857142857143</v>
       </c>
       <c r="B9" t="n">
-        <v>-538.27</v>
+        <v>2880.446</v>
       </c>
       <c r="D9" t="n">
         <v>2.05322e-07</v>
@@ -1608,7 +1608,7 @@
         <v>12.85714285714286</v>
       </c>
       <c r="B10" t="n">
-        <v>-529.23</v>
+        <v>2852.948</v>
       </c>
       <c r="D10" t="n">
         <v>2.07006e-07</v>
@@ -1658,7 +1658,7 @@
         <v>14.28571428571429</v>
       </c>
       <c r="B11" t="n">
-        <v>-519.21</v>
+        <v>2828.632</v>
       </c>
       <c r="D11" t="n">
         <v>2.08414e-07</v>
@@ -1708,7 +1708,7 @@
         <v>15.71428571428572</v>
       </c>
       <c r="B12" t="n">
-        <v>-516.1799999999998</v>
+        <v>2797.849</v>
       </c>
       <c r="D12" t="n">
         <v>2.09889e-07</v>
@@ -1758,7 +1758,7 @@
         <v>17.14285714285714</v>
       </c>
       <c r="B13" t="n">
-        <v>-513.4200000000001</v>
+        <v>2771.233</v>
       </c>
       <c r="D13" t="n">
         <v>2.11233e-07</v>
@@ -1808,7 +1808,7 @@
         <v>18.57142857142857</v>
       </c>
       <c r="B14" t="n">
-        <v>-502.8000000000002</v>
+        <v>2747.889</v>
       </c>
       <c r="D14" t="n">
         <v>2.12644e-07</v>
@@ -1858,7 +1858,7 @@
         <v>20</v>
       </c>
       <c r="B15" t="n">
-        <v>-497.02</v>
+        <v>2720.894</v>
       </c>
       <c r="D15" t="n">
         <v>2.14135e-07</v>
@@ -1908,7 +1908,7 @@
         <v>21.42857142857143</v>
       </c>
       <c r="B16" t="n">
-        <v>-488.79</v>
+        <v>2697.365</v>
       </c>
       <c r="D16" t="n">
         <v>2.15492e-07</v>
@@ -1958,7 +1958,7 @@
         <v>22.85714285714286</v>
       </c>
       <c r="B17" t="n">
-        <v>-484.3299999999999</v>
+        <v>2668.899</v>
       </c>
       <c r="D17" t="n">
         <v>2.16987e-07</v>
@@ -2008,7 +2008,7 @@
         <v>24.28571428571428</v>
       </c>
       <c r="B18" t="n">
-        <v>-476.6399999999999</v>
+        <v>2644.901</v>
       </c>
       <c r="D18" t="n">
         <v>2.18403e-07</v>
@@ -2058,7 +2058,7 @@
         <v>25.71428571428572</v>
       </c>
       <c r="B19" t="n">
-        <v>-486.1899999999996</v>
+        <v>2603.785</v>
       </c>
       <c r="D19" t="n">
         <v>2.19807e-07</v>
@@ -2108,7 +2108,7 @@
         <v>27.14285714285714</v>
       </c>
       <c r="B20" t="n">
-        <v>-464.6700000000001</v>
+        <v>2591.371</v>
       </c>
       <c r="D20" t="n">
         <v>2.21247e-07</v>
@@ -2158,7 +2158,7 @@
         <v>28.57142857142857</v>
       </c>
       <c r="B21" t="n">
-        <v>-461.3199999999997</v>
+        <v>2569.274</v>
       </c>
       <c r="D21" t="n">
         <v>2.22464e-07</v>
@@ -2208,7 +2208,7 @@
         <v>30</v>
       </c>
       <c r="B22" t="n">
-        <v>-463.2199999999998</v>
+        <v>2529.954</v>
       </c>
       <c r="D22" t="n">
         <v>2.24132e-07</v>
@@ -2404,7 +2404,7 @@
         <v>1.428571428571429</v>
       </c>
       <c r="B2" t="n">
-        <v>-621.8600000000006</v>
+        <v>3304.173</v>
       </c>
       <c r="D2" t="n">
         <v>1.87206e-07</v>
@@ -2454,7 +2454,7 @@
         <v>2.857142857142857</v>
       </c>
       <c r="B3" t="n">
-        <v>-541.2000000000003</v>
+        <v>3121.984</v>
       </c>
       <c r="D3" t="n">
         <v>1.97114e-07</v>
@@ -2504,7 +2504,7 @@
         <v>4.285714285714286</v>
       </c>
       <c r="B4" t="n">
-        <v>-523.04</v>
+        <v>3056.405</v>
       </c>
       <c r="D4" t="n">
         <v>2.00293e-07</v>
@@ -2554,7 +2554,7 @@
         <v>5.714285714285714</v>
       </c>
       <c r="B5" t="n">
-        <v>-488.54</v>
+        <v>3037.554</v>
       </c>
       <c r="D5" t="n">
         <v>2.02227e-07</v>
@@ -2604,7 +2604,7 @@
         <v>7.142857142857143</v>
       </c>
       <c r="B6" t="n">
-        <v>-501.6999999999998</v>
+        <v>2978.261</v>
       </c>
       <c r="D6" t="n">
         <v>2.03998e-07</v>
@@ -2654,7 +2654,7 @@
         <v>8.571428571428571</v>
       </c>
       <c r="B7" t="n">
-        <v>-471.4399999999996</v>
+        <v>2959.788</v>
       </c>
       <c r="D7" t="n">
         <v>2.05772e-07</v>
@@ -2704,7 +2704,7 @@
         <v>10</v>
       </c>
       <c r="B8" t="n">
-        <v>-498.8800000000001</v>
+        <v>2896.144</v>
       </c>
       <c r="D8" t="n">
         <v>2.07111e-07</v>
@@ -2754,7 +2754,7 @@
         <v>11.42857142857143</v>
       </c>
       <c r="B9" t="n">
-        <v>-472.9899999999998</v>
+        <v>2888.916</v>
       </c>
       <c r="D9" t="n">
         <v>2.08269e-07</v>
@@ -2804,7 +2804,7 @@
         <v>12.85714285714286</v>
       </c>
       <c r="B10" t="n">
-        <v>-469.02</v>
+        <v>2858.486</v>
       </c>
       <c r="D10" t="n">
         <v>2.09535e-07</v>
@@ -2854,7 +2854,7 @@
         <v>14.28571428571429</v>
       </c>
       <c r="B11" t="n">
-        <v>-476.0100000000002</v>
+        <v>2818.328</v>
       </c>
       <c r="D11" t="n">
         <v>2.10802e-07</v>
@@ -2904,7 +2904,7 @@
         <v>15.71428571428572</v>
       </c>
       <c r="B12" t="n">
-        <v>-458.4400000000001</v>
+        <v>2803.71</v>
       </c>
       <c r="D12" t="n">
         <v>2.11994e-07</v>
@@ -2954,7 +2954,7 @@
         <v>17.14285714285714</v>
       </c>
       <c r="B13" t="n">
-        <v>-463.9000000000001</v>
+        <v>2761.828</v>
       </c>
       <c r="D13" t="n">
         <v>2.13431e-07</v>
@@ -3004,7 +3004,7 @@
         <v>18.57142857142857</v>
       </c>
       <c r="B14" t="n">
-        <v>-438.6100000000001</v>
+        <v>2751.992</v>
       </c>
       <c r="D14" t="n">
         <v>2.14758e-07</v>
@@ -3054,7 +3054,7 @@
         <v>20</v>
       </c>
       <c r="B15" t="n">
-        <v>-434.0499999999997</v>
+        <v>2724.057</v>
       </c>
       <c r="D15" t="n">
         <v>2.15967e-07</v>
@@ -3104,7 +3104,7 @@
         <v>21.42857142857143</v>
       </c>
       <c r="B16" t="n">
-        <v>-409.9300000000003</v>
+        <v>2712.438</v>
       </c>
       <c r="D16" t="n">
         <v>2.17439e-07</v>
@@ -3154,7 +3154,7 @@
         <v>22.85714285714286</v>
       </c>
       <c r="B17" t="n">
-        <v>-435.7400000000002</v>
+        <v>2648.633</v>
       </c>
       <c r="D17" t="n">
         <v>2.18927e-07</v>
@@ -3204,7 +3204,7 @@
         <v>24.28571428571428</v>
       </c>
       <c r="B18" t="n">
-        <v>-415.1600000000003</v>
+        <v>2635.999</v>
       </c>
       <c r="D18" t="n">
         <v>2.20174e-07</v>
@@ -3254,7 +3254,7 @@
         <v>25.71428571428572</v>
       </c>
       <c r="B19" t="n">
-        <v>-414.77</v>
+        <v>2609.567</v>
       </c>
       <c r="D19" t="n">
         <v>2.21328e-07</v>
@@ -3304,7 +3304,7 @@
         <v>27.14285714285714</v>
       </c>
       <c r="B20" t="n">
-        <v>-403.4700000000003</v>
+        <v>2582.512</v>
       </c>
       <c r="D20" t="n">
         <v>2.22747e-07</v>
@@ -3354,7 +3354,7 @@
         <v>28.57142857142857</v>
       </c>
       <c r="B21" t="n">
-        <v>-397.8999999999996</v>
+        <v>2556.327</v>
       </c>
       <c r="D21" t="n">
         <v>2.24003e-07</v>
@@ -3404,7 +3404,7 @@
         <v>30</v>
       </c>
       <c r="B22" t="n">
-        <v>-399.04</v>
+        <v>2533.141</v>
       </c>
       <c r="D22" t="n">
         <v>2.24989e-07</v>
@@ -3600,7 +3600,7 @@
         <v>1.5</v>
       </c>
       <c r="B2" t="n">
-        <v>-2982.699999999997</v>
+        <v>33526.17</v>
       </c>
       <c r="D2" t="n">
         <v>1.07149e-08</v>
@@ -3650,7 +3650,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="n">
-        <v>-2560.099999999999</v>
+        <v>28322.376</v>
       </c>
       <c r="D3" t="n">
         <v>1.37638e-08</v>
@@ -3700,7 +3700,7 @@
         <v>4.5</v>
       </c>
       <c r="B4" t="n">
-        <v>-2463.299999999999</v>
+        <v>27190.091</v>
       </c>
       <c r="D4" t="n">
         <v>1.46789e-08</v>
@@ -3750,7 +3750,7 @@
         <v>6</v>
       </c>
       <c r="B5" t="n">
-        <v>-2418.199999999997</v>
+        <v>26657.818</v>
       </c>
       <c r="D5" t="n">
         <v>1.51748e-08</v>
@@ -3800,7 +3800,7 @@
         <v>7.5</v>
       </c>
       <c r="B6" t="n">
-        <v>-2392.299999999999</v>
+        <v>26254.083</v>
       </c>
       <c r="D6" t="n">
         <v>1.5568e-08</v>
@@ -3850,7 +3850,7 @@
         <v>9</v>
       </c>
       <c r="B7" t="n">
-        <v>-2369</v>
+        <v>25885.734</v>
       </c>
       <c r="D7" t="n">
         <v>1.59554e-08</v>
@@ -3900,7 +3900,7 @@
         <v>10.5</v>
       </c>
       <c r="B8" t="n">
-        <v>-2363.799999999999</v>
+        <v>25521.475</v>
       </c>
       <c r="D8" t="n">
         <v>1.6328e-08</v>
@@ -3950,7 +3950,7 @@
         <v>12</v>
       </c>
       <c r="B9" t="n">
-        <v>-2347.199999999997</v>
+        <v>25183.032</v>
       </c>
       <c r="D9" t="n">
         <v>1.66744e-08</v>
@@ -4000,7 +4000,7 @@
         <v>13.5</v>
       </c>
       <c r="B10" t="n">
-        <v>-2334.799999999999</v>
+        <v>24857.975</v>
       </c>
       <c r="D10" t="n">
         <v>1.70294e-08</v>
@@ -4050,7 +4050,7 @@
         <v>15</v>
       </c>
       <c r="B11" t="n">
-        <v>-2328.900000000001</v>
+        <v>24538.509</v>
       </c>
       <c r="D11" t="n">
         <v>1.73844e-08</v>
@@ -4246,7 +4246,7 @@
         <v>1.428571428571429</v>
       </c>
       <c r="B2" t="n">
-        <v>-643.6899999999996</v>
+        <v>3321.554</v>
       </c>
       <c r="D2" t="n">
         <v>1.86118e-07</v>
@@ -4296,7 +4296,7 @@
         <v>2.857142857142857</v>
       </c>
       <c r="B3" t="n">
-        <v>-562.5099999999998</v>
+        <v>3106.75</v>
       </c>
       <c r="D3" t="n">
         <v>1.97542e-07</v>
@@ -4346,7 +4346,7 @@
         <v>4.285714285714286</v>
       </c>
       <c r="B4" t="n">
-        <v>-531.9699999999998</v>
+        <v>3042.389</v>
       </c>
       <c r="D4" t="n">
         <v>2.01286e-07</v>
@@ -4396,7 +4396,7 @@
         <v>5.714285714285714</v>
       </c>
       <c r="B5" t="n">
-        <v>-495.4700000000003</v>
+        <v>3019.559</v>
       </c>
       <c r="D5" t="n">
         <v>2.036e-07</v>
@@ -4446,7 +4446,7 @@
         <v>7.142857142857143</v>
       </c>
       <c r="B6" t="n">
-        <v>-502.3099999999999</v>
+        <v>2961.543</v>
       </c>
       <c r="D6" t="n">
         <v>2.05551e-07</v>
@@ -4496,7 +4496,7 @@
         <v>8.571428571428571</v>
       </c>
       <c r="B7" t="n">
-        <v>-468.73</v>
+        <v>2942.584</v>
       </c>
       <c r="D7" t="n">
         <v>2.07554e-07</v>
@@ -4546,7 +4546,7 @@
         <v>10</v>
       </c>
       <c r="B8" t="n">
-        <v>-449.2600000000002</v>
+        <v>2896.458</v>
       </c>
       <c r="D8" t="n">
         <v>2.10392e-07</v>
@@ -4596,7 +4596,7 @@
         <v>11.42857142857143</v>
       </c>
       <c r="B9" t="n">
-        <v>-438.2799999999997</v>
+        <v>2867.432</v>
       </c>
       <c r="D9" t="n">
         <v>2.11914e-07</v>
@@ -4646,7 +4646,7 @@
         <v>12.85714285714286</v>
       </c>
       <c r="B10" t="n">
-        <v>-438.5299999999997</v>
+        <v>2837.095</v>
       </c>
       <c r="D10" t="n">
         <v>2.13002e-07</v>
@@ -4696,7 +4696,7 @@
         <v>14.28571428571429</v>
       </c>
       <c r="B11" t="n">
-        <v>-425.21</v>
+        <v>2812.008</v>
       </c>
       <c r="D11" t="n">
         <v>2.14599e-07</v>
@@ -4746,7 +4746,7 @@
         <v>15.71428571428572</v>
       </c>
       <c r="B12" t="n">
-        <v>-419.1199999999999</v>
+        <v>2790.329</v>
       </c>
       <c r="D12" t="n">
         <v>2.15609e-07</v>
@@ -4796,7 +4796,7 @@
         <v>17.14285714285714</v>
       </c>
       <c r="B13" t="n">
-        <v>-411.21</v>
+        <v>2766.869</v>
       </c>
       <c r="D13" t="n">
         <v>2.16844e-07</v>
@@ -4846,7 +4846,7 @@
         <v>18.57142857142857</v>
       </c>
       <c r="B14" t="n">
-        <v>-400.27</v>
+        <v>2739.898</v>
       </c>
       <c r="D14" t="n">
         <v>2.18279e-07</v>
@@ -4896,7 +4896,7 @@
         <v>20</v>
       </c>
       <c r="B15" t="n">
-        <v>-400.6700000000001</v>
+        <v>2715.872</v>
       </c>
       <c r="D15" t="n">
         <v>2.19196e-07</v>
@@ -4946,7 +4946,7 @@
         <v>21.42857142857143</v>
       </c>
       <c r="B16" t="n">
-        <v>-396.9400000000001</v>
+        <v>2690.1</v>
       </c>
       <c r="D16" t="n">
         <v>2.20409e-07</v>
@@ -4996,7 +4996,7 @@
         <v>22.85714285714286</v>
       </c>
       <c r="B17" t="n">
-        <v>-386.3600000000001</v>
+        <v>2669.379</v>
       </c>
       <c r="D17" t="n">
         <v>2.21682e-07</v>
@@ -5046,7 +5046,7 @@
         <v>24.28571428571428</v>
       </c>
       <c r="B18" t="n">
-        <v>-379.3499999999999</v>
+        <v>2641.589</v>
       </c>
       <c r="D18" t="n">
         <v>2.22962e-07</v>
@@ -5096,7 +5096,7 @@
         <v>25.71428571428572</v>
       </c>
       <c r="B19" t="n">
-        <v>-390.4100000000003</v>
+        <v>2606.438</v>
       </c>
       <c r="D19" t="n">
         <v>2.23933e-07</v>
@@ -5146,7 +5146,7 @@
         <v>27.14285714285714</v>
       </c>
       <c r="B20" t="n">
-        <v>-368.52</v>
+        <v>2593.08</v>
       </c>
       <c r="D20" t="n">
         <v>2.25371e-07</v>
@@ -5196,7 +5196,7 @@
         <v>28.57142857142857</v>
       </c>
       <c r="B21" t="n">
-        <v>-379.8200000000002</v>
+        <v>2555.902</v>
       </c>
       <c r="D21" t="n">
         <v>2.26332e-07</v>
@@ -5246,7 +5246,7 @@
         <v>30</v>
       </c>
       <c r="B22" t="n">
-        <v>-353.6400000000003</v>
+        <v>2546.351</v>
       </c>
       <c r="D22" t="n">
         <v>2.27732e-07</v>
@@ -5442,7 +5442,7 @@
         <v>1.5</v>
       </c>
       <c r="B2" t="n">
-        <v>-2912.600000000002</v>
+        <v>29789.774</v>
       </c>
       <c r="D2" t="n">
         <v>1.32072e-08</v>
@@ -5492,7 +5492,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="n">
-        <v>-2718.200000000001</v>
+        <v>26771.408</v>
       </c>
       <c r="D3" t="n">
         <v>1.55996e-08</v>
@@ -5542,7 +5542,7 @@
         <v>4.5</v>
       </c>
       <c r="B4" t="n">
-        <v>-2677.599999999999</v>
+        <v>25920.575</v>
       </c>
       <c r="D4" t="n">
         <v>1.64421e-08</v>
@@ -5592,7 +5592,7 @@
         <v>6</v>
       </c>
       <c r="B5" t="n">
-        <v>-2665.600000000002</v>
+        <v>25441.851</v>
       </c>
       <c r="D5" t="n">
         <v>1.69735e-08</v>
@@ -5642,7 +5642,7 @@
         <v>7.5</v>
       </c>
       <c r="B6" t="n">
-        <v>-2695.099999999999</v>
+        <v>25040.895</v>
       </c>
       <c r="D6" t="n">
         <v>1.74184e-08</v>
@@ -5692,7 +5692,7 @@
         <v>9</v>
       </c>
       <c r="B7" t="n">
-        <v>-2688.900000000001</v>
+        <v>24678.185</v>
       </c>
       <c r="D7" t="n">
         <v>1.78152e-08</v>
@@ -5742,7 +5742,7 @@
         <v>10.5</v>
       </c>
       <c r="B8" t="n">
-        <v>-2689.600000000002</v>
+        <v>24327.646</v>
       </c>
       <c r="D8" t="n">
         <v>1.81812e-08</v>
@@ -5792,7 +5792,7 @@
         <v>12</v>
       </c>
       <c r="B9" t="n">
-        <v>-2663.900000000001</v>
+        <v>24010.532</v>
       </c>
       <c r="D9" t="n">
         <v>1.85606e-08</v>
@@ -5842,7 +5842,7 @@
         <v>13.5</v>
       </c>
       <c r="B10" t="n">
-        <v>-2681.299999999999</v>
+        <v>23694.74</v>
       </c>
       <c r="D10" t="n">
         <v>1.88953e-08</v>
@@ -5892,7 +5892,7 @@
         <v>15</v>
       </c>
       <c r="B11" t="n">
-        <v>-2660.700000000001</v>
+        <v>23404.509</v>
       </c>
       <c r="D11" t="n">
         <v>1.92428e-08</v>
@@ -6088,7 +6088,7 @@
         <v>1.428571428571429</v>
       </c>
       <c r="B2" t="n">
-        <v>-758.0999999999999</v>
+        <v>3322.365</v>
       </c>
       <c r="D2" t="n">
         <v>1.78228e-07</v>
@@ -6138,7 +6138,7 @@
         <v>2.857142857142857</v>
       </c>
       <c r="B3" t="n">
-        <v>-712.6700000000001</v>
+        <v>3111.638</v>
       </c>
       <c r="D3" t="n">
         <v>1.87857e-07</v>
@@ -6188,7 +6188,7 @@
         <v>4.285714285714286</v>
       </c>
       <c r="B4" t="n">
-        <v>-702.6100000000001</v>
+        <v>3042.006</v>
       </c>
       <c r="D4" t="n">
         <v>1.91062e-07</v>
@@ -6238,7 +6238,7 @@
         <v>5.714285714285714</v>
       </c>
       <c r="B5" t="n">
-        <v>-688.3299999999999</v>
+        <v>3004.488</v>
       </c>
       <c r="D5" t="n">
         <v>1.93204e-07</v>
@@ -6288,7 +6288,7 @@
         <v>7.142857142857143</v>
       </c>
       <c r="B6" t="n">
-        <v>-682.8699999999999</v>
+        <v>2967.235</v>
       </c>
       <c r="D6" t="n">
         <v>1.94892e-07</v>
@@ -6338,7 +6338,7 @@
         <v>8.571428571428571</v>
       </c>
       <c r="B7" t="n">
-        <v>-669.9400000000001</v>
+        <v>2931.648</v>
       </c>
       <c r="D7" t="n">
         <v>1.96906e-07</v>
@@ -6388,7 +6388,7 @@
         <v>10</v>
       </c>
       <c r="B8" t="n">
-        <v>-664.0700000000002</v>
+        <v>2899.958</v>
       </c>
       <c r="D8" t="n">
         <v>1.9842e-07</v>
@@ -6438,7 +6438,7 @@
         <v>11.42857142857143</v>
       </c>
       <c r="B9" t="n">
-        <v>-657.4099999999999</v>
+        <v>2868.943</v>
       </c>
       <c r="D9" t="n">
         <v>1.99958e-07</v>
@@ -6488,7 +6488,7 @@
         <v>12.85714285714286</v>
       </c>
       <c r="B10" t="n">
-        <v>-647.9000000000001</v>
+        <v>2838.5</v>
       </c>
       <c r="D10" t="n">
         <v>2.01527e-07</v>
@@ -6538,7 +6538,7 @@
         <v>14.28571428571429</v>
       </c>
       <c r="B11" t="n">
-        <v>-643.7400000000002</v>
+        <v>2812.453</v>
       </c>
       <c r="D11" t="n">
         <v>2.02732e-07</v>
@@ -6588,7 +6588,7 @@
         <v>15.71428571428572</v>
       </c>
       <c r="B12" t="n">
-        <v>-646.8200000000002</v>
+        <v>2771.025</v>
       </c>
       <c r="D12" t="n">
         <v>2.04309e-07</v>
@@ -6638,7 +6638,7 @@
         <v>17.14285714285714</v>
       </c>
       <c r="B13" t="n">
-        <v>-643.23</v>
+        <v>2744.331</v>
       </c>
       <c r="D13" t="n">
         <v>2.0556e-07</v>
@@ -6688,7 +6688,7 @@
         <v>18.57142857142857</v>
       </c>
       <c r="B14" t="n">
-        <v>-623.8000000000002</v>
+        <v>2736.308</v>
       </c>
       <c r="D14" t="n">
         <v>2.06697e-07</v>
@@ -6738,7 +6738,7 @@
         <v>20</v>
       </c>
       <c r="B15" t="n">
-        <v>-618.7000000000003</v>
+        <v>2711.123</v>
       </c>
       <c r="D15" t="n">
         <v>2.0799e-07</v>
@@ -6788,7 +6788,7 @@
         <v>21.42857142857143</v>
       </c>
       <c r="B16" t="n">
-        <v>-610.1700000000001</v>
+        <v>2681.612</v>
       </c>
       <c r="D16" t="n">
         <v>2.09486e-07</v>
@@ -6838,7 +6838,7 @@
         <v>22.85714285714286</v>
       </c>
       <c r="B17" t="n">
-        <v>-598.5599999999999</v>
+        <v>2660.27</v>
       </c>
       <c r="D17" t="n">
         <v>2.10877e-07</v>
@@ -6888,7 +6888,7 @@
         <v>24.28571428571428</v>
       </c>
       <c r="B18" t="n">
-        <v>-613.0899999999997</v>
+        <v>2617.769</v>
       </c>
       <c r="D18" t="n">
         <v>2.12058e-07</v>
@@ -6938,7 +6938,7 @@
         <v>25.71428571428572</v>
       </c>
       <c r="B19" t="n">
-        <v>-594.2599999999998</v>
+        <v>2609.157</v>
       </c>
       <c r="D19" t="n">
         <v>2.13129e-07</v>
@@ -6988,7 +6988,7 @@
         <v>27.14285714285714</v>
       </c>
       <c r="B20" t="n">
-        <v>-582.8000000000002</v>
+        <v>2587.246</v>
       </c>
       <c r="D20" t="n">
         <v>2.14538e-07</v>
@@ -7038,7 +7038,7 @@
         <v>28.57142857142857</v>
       </c>
       <c r="B21" t="n">
-        <v>-577.4700000000003</v>
+        <v>2559.778</v>
       </c>
       <c r="D21" t="n">
         <v>2.1588e-07</v>
@@ -7088,7 +7088,7 @@
         <v>30</v>
       </c>
       <c r="B22" t="n">
-        <v>-572.5799999999999</v>
+        <v>2535.847</v>
       </c>
       <c r="D22" t="n">
         <v>2.17096e-07</v>
@@ -7284,7 +7284,7 @@
         <v>1.5</v>
       </c>
       <c r="B2" t="n">
-        <v>-2141.299999999999</v>
+        <v>21355.602</v>
       </c>
       <c r="D2" t="n">
         <v>2.19312e-08</v>
@@ -7334,7 +7334,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="n">
-        <v>-2049</v>
+        <v>19995.383</v>
       </c>
       <c r="D3" t="n">
         <v>2.3848e-08</v>
@@ -7384,7 +7384,7 @@
         <v>4.5</v>
       </c>
       <c r="B4" t="n">
-        <v>-2006</v>
+        <v>19535.205</v>
       </c>
       <c r="D4" t="n">
         <v>2.45918e-08</v>
@@ -7434,7 +7434,7 @@
         <v>6</v>
       </c>
       <c r="B5" t="n">
-        <v>-1995.799999999999</v>
+        <v>19229.25</v>
       </c>
       <c r="D5" t="n">
         <v>2.50677e-08</v>
@@ -7484,7 +7484,7 @@
         <v>7.5</v>
       </c>
       <c r="B6" t="n">
-        <v>-1985</v>
+        <v>18966.987</v>
       </c>
       <c r="D6" t="n">
         <v>2.54918e-08</v>
@@ -7534,7 +7534,7 @@
         <v>9</v>
       </c>
       <c r="B7" t="n">
-        <v>-1968.5</v>
+        <v>18716.335</v>
       </c>
       <c r="D7" t="n">
         <v>2.59352e-08</v>
@@ -7584,7 +7584,7 @@
         <v>10.5</v>
       </c>
       <c r="B8" t="n">
-        <v>-1958.599999999999</v>
+        <v>18490.21</v>
       </c>
       <c r="D8" t="n">
         <v>2.6343e-08</v>
@@ -7634,7 +7634,7 @@
         <v>12</v>
       </c>
       <c r="B9" t="n">
-        <v>-1927.5</v>
+        <v>18273.95</v>
       </c>
       <c r="D9" t="n">
         <v>2.67788e-08</v>
@@ -7684,7 +7684,7 @@
         <v>13.5</v>
       </c>
       <c r="B10" t="n">
-        <v>-1911.800000000003</v>
+        <v>18051.387</v>
       </c>
       <c r="D10" t="n">
         <v>2.72089e-08</v>
@@ -7734,7 +7734,7 @@
         <v>15</v>
       </c>
       <c r="B11" t="n">
-        <v>-1900.5</v>
+        <v>17846.934</v>
       </c>
       <c r="D11" t="n">
         <v>2.76149e-08</v>
@@ -7930,7 +7930,7 @@
         <v>1.428571428571429</v>
       </c>
       <c r="B2" t="n">
-        <v>-689.3400000000001</v>
+        <v>3325.154</v>
       </c>
       <c r="D2" t="n">
         <v>1.81236e-07</v>
@@ -7980,7 +7980,7 @@
         <v>2.857142857142857</v>
       </c>
       <c r="B3" t="n">
-        <v>-622.9000000000001</v>
+        <v>3141.792</v>
       </c>
       <c r="D3" t="n">
         <v>1.9048e-07</v>
@@ -8030,7 +8030,7 @@
         <v>4.285714285714286</v>
       </c>
       <c r="B4" t="n">
-        <v>-637.5699999999997</v>
+        <v>3060.812</v>
       </c>
       <c r="D4" t="n">
         <v>1.93226e-07</v>
@@ -8080,7 +8080,7 @@
         <v>5.714285714285714</v>
       </c>
       <c r="B5" t="n">
-        <v>-610.0599999999999</v>
+        <v>3034.613</v>
       </c>
       <c r="D5" t="n">
         <v>1.95508e-07</v>
@@ -8130,7 +8130,7 @@
         <v>7.142857142857143</v>
       </c>
       <c r="B6" t="n">
-        <v>-620.27</v>
+        <v>2976.087</v>
       </c>
       <c r="D6" t="n">
         <v>1.97471e-07</v>
@@ -8180,7 +8180,7 @@
         <v>8.571428571428571</v>
       </c>
       <c r="B7" t="n">
-        <v>-617.1799999999998</v>
+        <v>2940.544</v>
       </c>
       <c r="D7" t="n">
         <v>1.99153e-07</v>
@@ -8230,7 +8230,7 @@
         <v>10</v>
       </c>
       <c r="B8" t="n">
-        <v>-605.4100000000003</v>
+        <v>2907.828</v>
       </c>
       <c r="D8" t="n">
         <v>2.01033e-07</v>
@@ -8280,7 +8280,7 @@
         <v>11.42857142857143</v>
       </c>
       <c r="B9" t="n">
-        <v>-625.48</v>
+        <v>2858.686</v>
       </c>
       <c r="D9" t="n">
         <v>2.02102e-07</v>
@@ -8330,7 +8330,7 @@
         <v>12.85714285714286</v>
       </c>
       <c r="B10" t="n">
-        <v>-607.4200000000001</v>
+        <v>2846.17</v>
       </c>
       <c r="D10" t="n">
         <v>2.03372e-07</v>
@@ -8380,7 +8380,7 @@
         <v>14.28571428571429</v>
       </c>
       <c r="B11" t="n">
-        <v>-607.5099999999998</v>
+        <v>2799.328</v>
       </c>
       <c r="D11" t="n">
         <v>2.05532e-07</v>
@@ -8430,7 +8430,7 @@
         <v>15.71428571428572</v>
       </c>
       <c r="B12" t="n">
-        <v>-580.0799999999999</v>
+        <v>2787.206</v>
       </c>
       <c r="D12" t="n">
         <v>2.07182e-07</v>
@@ -8480,7 +8480,7 @@
         <v>17.14285714285714</v>
       </c>
       <c r="B13" t="n">
-        <v>-573.3999999999996</v>
+        <v>2764.489</v>
       </c>
       <c r="D13" t="n">
         <v>2.08491e-07</v>
@@ -8530,7 +8530,7 @@
         <v>18.57142857142857</v>
       </c>
       <c r="B14" t="n">
-        <v>-562.2199999999998</v>
+        <v>2735.817</v>
       </c>
       <c r="D14" t="n">
         <v>2.10226e-07</v>
@@ -8580,7 +8580,7 @@
         <v>20</v>
       </c>
       <c r="B15" t="n">
-        <v>-555.21</v>
+        <v>2707</v>
       </c>
       <c r="D15" t="n">
         <v>2.11741e-07</v>
@@ -8630,7 +8630,7 @@
         <v>21.42857142857143</v>
       </c>
       <c r="B16" t="n">
-        <v>-546.6100000000001</v>
+        <v>2678.878</v>
       </c>
       <c r="D16" t="n">
         <v>2.13262e-07</v>
@@ -8680,7 +8680,7 @@
         <v>22.85714285714286</v>
       </c>
       <c r="B17" t="n">
-        <v>-557.5999999999999</v>
+        <v>2633.819</v>
       </c>
       <c r="D17" t="n">
         <v>2.1475e-07</v>
@@ -8730,7 +8730,7 @@
         <v>24.28571428571428</v>
       </c>
       <c r="B18" t="n">
-        <v>-540.46</v>
+        <v>2620.086</v>
       </c>
       <c r="D18" t="n">
         <v>2.1609e-07</v>
@@ -8780,7 +8780,7 @@
         <v>25.71428571428572</v>
       </c>
       <c r="B19" t="n">
-        <v>-529.46</v>
+        <v>2592.122</v>
       </c>
       <c r="D19" t="n">
         <v>2.1782e-07</v>
@@ -8830,7 +8830,7 @@
         <v>27.14285714285714</v>
       </c>
       <c r="B20" t="n">
-        <v>-533.9000000000001</v>
+        <v>2552.539</v>
       </c>
       <c r="D20" t="n">
         <v>2.19358e-07</v>
@@ -8880,7 +8880,7 @@
         <v>28.57142857142857</v>
       </c>
       <c r="B21" t="n">
-        <v>-510.9400000000001</v>
+        <v>2541.159</v>
       </c>
       <c r="D21" t="n">
         <v>2.20969e-07</v>
@@ -8930,7 +8930,7 @@
         <v>30</v>
       </c>
       <c r="B22" t="n">
-        <v>-520.3700000000003</v>
+        <v>2502.932</v>
       </c>
       <c r="D22" t="n">
         <v>2.22296e-07</v>
@@ -9126,7 +9126,7 @@
         <v>1.5</v>
       </c>
       <c r="B2" t="n">
-        <v>-7685.355</v>
+        <v>1.840000000000003</v>
       </c>
       <c r="D2" t="n">
         <v>9.7505e-08</v>
@@ -9176,7 +9176,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="n">
-        <v>-6655.179999999999</v>
+        <v>1.292999999999978</v>
       </c>
       <c r="D3" t="n">
         <v>1.14436e-07</v>
@@ -9226,7 +9226,7 @@
         <v>4.5</v>
       </c>
       <c r="B4" t="n">
-        <v>-6413.009999999999</v>
+        <v>0</v>
       </c>
       <c r="D4" t="n">
         <v>1.19016e-07</v>
@@ -9276,7 +9276,7 @@
         <v>6</v>
       </c>
       <c r="B5" t="n">
-        <v>-870.4200000000001</v>
+        <v>5421.400000000001</v>
       </c>
       <c r="D5" t="n">
         <v>1.21355e-07</v>
@@ -9326,7 +9326,7 @@
         <v>7.5</v>
       </c>
       <c r="B6" t="n">
-        <v>-864.4000000000005</v>
+        <v>5335.116</v>
       </c>
       <c r="D6" t="n">
         <v>1.23201e-07</v>
@@ -9376,7 +9376,7 @@
         <v>9</v>
       </c>
       <c r="B7" t="n">
-        <v>-858.6799999999994</v>
+        <v>5266.168000000001</v>
       </c>
       <c r="D7" t="n">
         <v>1.24738e-07</v>
@@ -9426,7 +9426,7 @@
         <v>10.5</v>
       </c>
       <c r="B8" t="n">
-        <v>-839.7600000000002</v>
+        <v>5199.491</v>
       </c>
       <c r="D8" t="n">
         <v>1.26549e-07</v>
@@ -9476,7 +9476,7 @@
         <v>12</v>
       </c>
       <c r="B9" t="n">
-        <v>-828.3000000000002</v>
+        <v>5135.626</v>
       </c>
       <c r="D9" t="n">
         <v>1.28225e-07</v>
@@ -9526,7 +9526,7 @@
         <v>13.5</v>
       </c>
       <c r="B10" t="n">
-        <v>-834.3899999999994</v>
+        <v>5074.596</v>
       </c>
       <c r="D10" t="n">
         <v>1.29444e-07</v>
@@ -9576,7 +9576,7 @@
         <v>15</v>
       </c>
       <c r="B11" t="n">
-        <v>-823.4700000000003</v>
+        <v>5012.176</v>
       </c>
       <c r="D11" t="n">
         <v>1.3106e-07</v>

</xml_diff>

<commit_message>
added to deepta bid data excel sheet
</commit_message>
<xml_diff>
--- a/BioSensorAnalysisSrcCode/EIS_Analysis/Austin_EIS/MegaExcel/Processed Chips for PCAI1ia/Chip 21.xlsx
+++ b/BioSensorAnalysisSrcCode/EIS_Analysis/Austin_EIS/MegaExcel/Processed Chips for PCAI1ia/Chip 21.xlsx
@@ -438,7 +438,7 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Rct-d</t>
+          <t>delta Rct-d</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -564,6 +564,9 @@
       <c r="B2" t="n">
         <v>3413.305</v>
       </c>
+      <c r="C2" t="n">
+        <v>3705.781582992509</v>
+      </c>
       <c r="D2" t="n">
         <v>1.84241e-07</v>
       </c>
@@ -614,6 +617,9 @@
       <c r="B3" t="n">
         <v>3306.557</v>
       </c>
+      <c r="C3" t="n">
+        <v>3596.875521990378</v>
+      </c>
       <c r="D3" t="n">
         <v>1.89606e-07</v>
       </c>
@@ -664,6 +670,9 @@
       <c r="B4" t="n">
         <v>3231.904</v>
       </c>
+      <c r="C4" t="n">
+        <v>3521.527944144097</v>
+      </c>
       <c r="D4" t="n">
         <v>1.92888e-07</v>
       </c>
@@ -714,6 +723,9 @@
       <c r="B5" t="n">
         <v>3169.252</v>
       </c>
+      <c r="C5" t="n">
+        <v>3460.849069286025</v>
+      </c>
       <c r="D5" t="n">
         <v>1.96208e-07</v>
       </c>
@@ -764,6 +776,9 @@
       <c r="B6" t="n">
         <v>3112.06</v>
       </c>
+      <c r="C6" t="n">
+        <v>3402.561588564839</v>
+      </c>
       <c r="D6" t="n">
         <v>1.98503e-07</v>
       </c>
@@ -814,6 +829,9 @@
       <c r="B7" t="n">
         <v>3058.458</v>
       </c>
+      <c r="C7" t="n">
+        <v>3353.906615492061</v>
+      </c>
       <c r="D7" t="n">
         <v>2.00804e-07</v>
       </c>
@@ -864,6 +882,9 @@
       <c r="B8" t="n">
         <v>3000.47</v>
       </c>
+      <c r="C8" t="n">
+        <v>3301.803960481059</v>
+      </c>
       <c r="D8" t="n">
         <v>2.02918e-07</v>
       </c>
@@ -914,6 +935,9 @@
       <c r="B9" t="n">
         <v>2954.274</v>
       </c>
+      <c r="C9" t="n">
+        <v>3261.354513794582</v>
+      </c>
       <c r="D9" t="n">
         <v>2.04758e-07</v>
       </c>
@@ -964,6 +988,9 @@
       <c r="B10" t="n">
         <v>2919.242</v>
       </c>
+      <c r="C10" t="n">
+        <v>3222.528243017276</v>
+      </c>
       <c r="D10" t="n">
         <v>2.06513e-07</v>
       </c>
@@ -1013,6 +1040,9 @@
       </c>
       <c r="B11" t="n">
         <v>2899.646</v>
+      </c>
+      <c r="C11" t="n">
+        <v>3196.256838416664</v>
       </c>
       <c r="D11" t="n">
         <v>2.08089e-07</v>
@@ -1084,7 +1114,7 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Rct-d</t>
+          <t>delta Rct-d</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -1210,6 +1240,9 @@
       <c r="B2" t="n">
         <v>3248.999</v>
       </c>
+      <c r="C2" t="n">
+        <v>3548.586750022529</v>
+      </c>
       <c r="D2" t="n">
         <v>1.88742e-07</v>
       </c>
@@ -1260,6 +1293,9 @@
       <c r="B3" t="n">
         <v>3097.392</v>
       </c>
+      <c r="C3" t="n">
+        <v>3393.368475201361</v>
+      </c>
       <c r="D3" t="n">
         <v>1.94412e-07</v>
       </c>
@@ -1310,6 +1346,9 @@
       <c r="B4" t="n">
         <v>3064.714</v>
       </c>
+      <c r="C4" t="n">
+        <v>3347.518943184852</v>
+      </c>
       <c r="D4" t="n">
         <v>1.96919e-07</v>
       </c>
@@ -1360,6 +1399,9 @@
       <c r="B5" t="n">
         <v>3009.657</v>
       </c>
+      <c r="C5" t="n">
+        <v>3305.924419102164</v>
+      </c>
       <c r="D5" t="n">
         <v>1.98783e-07</v>
       </c>
@@ -1410,6 +1452,9 @@
       <c r="B6" t="n">
         <v>2957.534</v>
       </c>
+      <c r="C6" t="n">
+        <v>3262.624882560889</v>
+      </c>
       <c r="D6" t="n">
         <v>2.0035e-07</v>
       </c>
@@ -1460,6 +1505,9 @@
       <c r="B7" t="n">
         <v>2943.712</v>
       </c>
+      <c r="C7" t="n">
+        <v>3238.402733392615</v>
+      </c>
       <c r="D7" t="n">
         <v>2.02176e-07</v>
       </c>
@@ -1510,6 +1558,9 @@
       <c r="B8" t="n">
         <v>2911.219</v>
       </c>
+      <c r="C8" t="n">
+        <v>3206.810911233661</v>
+      </c>
       <c r="D8" t="n">
         <v>2.03803e-07</v>
       </c>
@@ -1560,6 +1611,9 @@
       <c r="B9" t="n">
         <v>2880.446</v>
       </c>
+      <c r="C9" t="n">
+        <v>3175.008438643334</v>
+      </c>
       <c r="D9" t="n">
         <v>2.05322e-07</v>
       </c>
@@ -1610,6 +1664,9 @@
       <c r="B10" t="n">
         <v>2852.948</v>
       </c>
+      <c r="C10" t="n">
+        <v>3150.513995253195</v>
+      </c>
       <c r="D10" t="n">
         <v>2.07006e-07</v>
       </c>
@@ -1660,6 +1717,9 @@
       <c r="B11" t="n">
         <v>2828.632</v>
       </c>
+      <c r="C11" t="n">
+        <v>3121.949193174544</v>
+      </c>
       <c r="D11" t="n">
         <v>2.08414e-07</v>
       </c>
@@ -1710,6 +1770,9 @@
       <c r="B12" t="n">
         <v>2797.849</v>
       </c>
+      <c r="C12" t="n">
+        <v>3092.841849043207</v>
+      </c>
       <c r="D12" t="n">
         <v>2.09889e-07</v>
       </c>
@@ -1760,6 +1823,9 @@
       <c r="B13" t="n">
         <v>2771.233</v>
       </c>
+      <c r="C13" t="n">
+        <v>3065.227073523505</v>
+      </c>
       <c r="D13" t="n">
         <v>2.11233e-07</v>
       </c>
@@ -1810,6 +1876,9 @@
       <c r="B14" t="n">
         <v>2747.889</v>
       </c>
+      <c r="C14" t="n">
+        <v>3040.965506931002</v>
+      </c>
       <c r="D14" t="n">
         <v>2.12644e-07</v>
       </c>
@@ -1860,6 +1929,9 @@
       <c r="B15" t="n">
         <v>2720.894</v>
       </c>
+      <c r="C15" t="n">
+        <v>3013.64217727477</v>
+      </c>
       <c r="D15" t="n">
         <v>2.14135e-07</v>
       </c>
@@ -1910,6 +1982,9 @@
       <c r="B16" t="n">
         <v>2697.365</v>
       </c>
+      <c r="C16" t="n">
+        <v>2989.976366977899</v>
+      </c>
       <c r="D16" t="n">
         <v>2.15492e-07</v>
       </c>
@@ -1960,6 +2035,9 @@
       <c r="B17" t="n">
         <v>2668.899</v>
       </c>
+      <c r="C17" t="n">
+        <v>2961.628340163529</v>
+      </c>
       <c r="D17" t="n">
         <v>2.16987e-07</v>
       </c>
@@ -2010,6 +2088,9 @@
       <c r="B18" t="n">
         <v>2644.901</v>
       </c>
+      <c r="C18" t="n">
+        <v>2936.03129800163</v>
+      </c>
       <c r="D18" t="n">
         <v>2.18403e-07</v>
       </c>
@@ -2060,6 +2141,9 @@
       <c r="B19" t="n">
         <v>2603.785</v>
       </c>
+      <c r="C19" t="n">
+        <v>2903.906072749533</v>
+      </c>
       <c r="D19" t="n">
         <v>2.19807e-07</v>
       </c>
@@ -2110,6 +2194,9 @@
       <c r="B20" t="n">
         <v>2591.371</v>
       </c>
+      <c r="C20" t="n">
+        <v>2884.962679319052</v>
+      </c>
       <c r="D20" t="n">
         <v>2.21247e-07</v>
       </c>
@@ -2160,6 +2247,9 @@
       <c r="B21" t="n">
         <v>2569.274</v>
       </c>
+      <c r="C21" t="n">
+        <v>2858.194917716988</v>
+      </c>
       <c r="D21" t="n">
         <v>2.22464e-07</v>
       </c>
@@ -2209,6 +2299,9 @@
       </c>
       <c r="B22" t="n">
         <v>2529.954</v>
+      </c>
+      <c r="C22" t="n">
+        <v>2828.208967482188</v>
       </c>
       <c r="D22" t="n">
         <v>2.24132e-07</v>
@@ -2280,7 +2373,7 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Rct-d</t>
+          <t>delta Rct-d</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -2406,6 +2499,9 @@
       <c r="B2" t="n">
         <v>3304.173</v>
       </c>
+      <c r="C2" t="n">
+        <v>3617.638513947961</v>
+      </c>
       <c r="D2" t="n">
         <v>1.87206e-07</v>
       </c>
@@ -2456,6 +2552,9 @@
       <c r="B3" t="n">
         <v>3121.984</v>
       </c>
+      <c r="C3" t="n">
+        <v>3418.678972156053</v>
+      </c>
       <c r="D3" t="n">
         <v>1.97114e-07</v>
       </c>
@@ -2506,6 +2605,9 @@
       <c r="B4" t="n">
         <v>3056.405</v>
       </c>
+      <c r="C4" t="n">
+        <v>3349.286450015036</v>
+      </c>
       <c r="D4" t="n">
         <v>2.00293e-07</v>
       </c>
@@ -2556,6 +2658,9 @@
       <c r="B5" t="n">
         <v>3037.554</v>
       </c>
+      <c r="C5" t="n">
+        <v>3314.45511250991</v>
+      </c>
       <c r="D5" t="n">
         <v>2.02227e-07</v>
       </c>
@@ -2606,6 +2711,9 @@
       <c r="B6" t="n">
         <v>2978.261</v>
       </c>
+      <c r="C6" t="n">
+        <v>3271.143678062786</v>
+      </c>
       <c r="D6" t="n">
         <v>2.03998e-07</v>
       </c>
@@ -2656,6 +2764,9 @@
       <c r="B7" t="n">
         <v>2959.788</v>
       </c>
+      <c r="C7" t="n">
+        <v>3242.753550935369</v>
+      </c>
       <c r="D7" t="n">
         <v>2.05772e-07</v>
       </c>
@@ -2706,6 +2817,9 @@
       <c r="B8" t="n">
         <v>2896.144</v>
       </c>
+      <c r="C8" t="n">
+        <v>3197.530824562</v>
+      </c>
       <c r="D8" t="n">
         <v>2.07111e-07</v>
       </c>
@@ -2756,6 +2870,9 @@
       <c r="B9" t="n">
         <v>2888.916</v>
       </c>
+      <c r="C9" t="n">
+        <v>3178.401365770566</v>
+      </c>
       <c r="D9" t="n">
         <v>2.08269e-07</v>
       </c>
@@ -2806,6 +2923,9 @@
       <c r="B10" t="n">
         <v>2858.486</v>
       </c>
+      <c r="C10" t="n">
+        <v>3151.851265917903</v>
+      </c>
       <c r="D10" t="n">
         <v>2.09535e-07</v>
       </c>
@@ -2856,6 +2976,9 @@
       <c r="B11" t="n">
         <v>2818.328</v>
       </c>
+      <c r="C11" t="n">
+        <v>3118.595611701044</v>
+      </c>
       <c r="D11" t="n">
         <v>2.10802e-07</v>
       </c>
@@ -2906,6 +3029,9 @@
       <c r="B12" t="n">
         <v>2803.71</v>
       </c>
+      <c r="C12" t="n">
+        <v>3099.990984607326</v>
+      </c>
       <c r="D12" t="n">
         <v>2.11994e-07</v>
       </c>
@@ -2956,6 +3082,9 @@
       <c r="B13" t="n">
         <v>2761.828</v>
       </c>
+      <c r="C13" t="n">
+        <v>3065.213845201413</v>
+      </c>
       <c r="D13" t="n">
         <v>2.13431e-07</v>
       </c>
@@ -3006,6 +3135,9 @@
       <c r="B14" t="n">
         <v>2751.992</v>
       </c>
+      <c r="C14" t="n">
+        <v>3041.991470148206</v>
+      </c>
       <c r="D14" t="n">
         <v>2.14758e-07</v>
       </c>
@@ -3056,6 +3188,9 @@
       <c r="B15" t="n">
         <v>2724.057</v>
       </c>
+      <c r="C15" t="n">
+        <v>3013.758567933961</v>
+      </c>
       <c r="D15" t="n">
         <v>2.15967e-07</v>
       </c>
@@ -3106,6 +3241,9 @@
       <c r="B16" t="n">
         <v>2712.438</v>
       </c>
+      <c r="C16" t="n">
+        <v>2993.29750291965</v>
+      </c>
       <c r="D16" t="n">
         <v>2.17439e-07</v>
       </c>
@@ -3156,6 +3294,9 @@
       <c r="B17" t="n">
         <v>2648.633</v>
       </c>
+      <c r="C17" t="n">
+        <v>2949.437375412275</v>
+      </c>
       <c r="D17" t="n">
         <v>2.18927e-07</v>
       </c>
@@ -3206,6 +3347,9 @@
       <c r="B18" t="n">
         <v>2635.999</v>
       </c>
+      <c r="C18" t="n">
+        <v>2928.86459690938</v>
+      </c>
       <c r="D18" t="n">
         <v>2.20174e-07</v>
       </c>
@@ -3256,6 +3400,9 @@
       <c r="B19" t="n">
         <v>2609.567</v>
       </c>
+      <c r="C19" t="n">
+        <v>2902.61908256478</v>
+      </c>
       <c r="D19" t="n">
         <v>2.21328e-07</v>
       </c>
@@ -3306,6 +3453,9 @@
       <c r="B20" t="n">
         <v>2582.512</v>
       </c>
+      <c r="C20" t="n">
+        <v>2876.03564247402</v>
+      </c>
       <c r="D20" t="n">
         <v>2.22747e-07</v>
       </c>
@@ -3356,6 +3506,9 @@
       <c r="B21" t="n">
         <v>2556.327</v>
       </c>
+      <c r="C21" t="n">
+        <v>2849.253397272075</v>
+      </c>
       <c r="D21" t="n">
         <v>2.24003e-07</v>
       </c>
@@ -3405,6 +3558,9 @@
       </c>
       <c r="B22" t="n">
         <v>2533.141</v>
+      </c>
+      <c r="C22" t="n">
+        <v>2825.573592770365</v>
       </c>
       <c r="D22" t="n">
         <v>2.24989e-07</v>
@@ -3476,7 +3632,7 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Rct-d</t>
+          <t>delta Rct-d</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -3951,6 +4107,9 @@
       </c>
       <c r="B9" t="n">
         <v>25183.032</v>
+      </c>
+      <c r="C9" t="n">
+        <v>14.05900507842058</v>
       </c>
       <c r="D9" t="n">
         <v>1.66744e-08</v>
@@ -4122,7 +4281,7 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Rct-d</t>
+          <t>delta Rct-d</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -4248,6 +4407,9 @@
       <c r="B2" t="n">
         <v>3321.554</v>
       </c>
+      <c r="C2" t="n">
+        <v>3623.895495047583</v>
+      </c>
       <c r="D2" t="n">
         <v>1.86118e-07</v>
       </c>
@@ -4298,6 +4460,9 @@
       <c r="B3" t="n">
         <v>3106.75</v>
       </c>
+      <c r="C3" t="n">
+        <v>3399.158274198141</v>
+      </c>
       <c r="D3" t="n">
         <v>1.97542e-07</v>
       </c>
@@ -4348,6 +4513,9 @@
       <c r="B4" t="n">
         <v>3042.389</v>
       </c>
+      <c r="C4" t="n">
+        <v>3331.220355672339</v>
+      </c>
       <c r="D4" t="n">
         <v>2.01286e-07</v>
       </c>
@@ -4398,6 +4566,9 @@
       <c r="B5" t="n">
         <v>3019.559</v>
       </c>
+      <c r="C5" t="n">
+        <v>3296.409968256175</v>
+      </c>
       <c r="D5" t="n">
         <v>2.036e-07</v>
       </c>
@@ -4448,6 +4619,9 @@
       <c r="B6" t="n">
         <v>2961.543</v>
       </c>
+      <c r="C6" t="n">
+        <v>3253.553499472222</v>
+      </c>
       <c r="D6" t="n">
         <v>2.05551e-07</v>
       </c>
@@ -4498,6 +4672,9 @@
       <c r="B7" t="n">
         <v>2942.584</v>
       </c>
+      <c r="C7" t="n">
+        <v>3224.452653954537</v>
+      </c>
       <c r="D7" t="n">
         <v>2.07554e-07</v>
       </c>
@@ -4548,6 +4725,9 @@
       <c r="B8" t="n">
         <v>2896.458</v>
       </c>
+      <c r="C8" t="n">
+        <v>3188.953281812711</v>
+      </c>
       <c r="D8" t="n">
         <v>2.10392e-07</v>
       </c>
@@ -4598,6 +4778,9 @@
       <c r="B9" t="n">
         <v>2867.432</v>
       </c>
+      <c r="C9" t="n">
+        <v>3157.296565413375</v>
+      </c>
       <c r="D9" t="n">
         <v>2.11914e-07</v>
       </c>
@@ -4648,6 +4831,9 @@
       <c r="B10" t="n">
         <v>2837.095</v>
       </c>
+      <c r="C10" t="n">
+        <v>3130.289419778871</v>
+      </c>
       <c r="D10" t="n">
         <v>2.13002e-07</v>
       </c>
@@ -4698,6 +4884,9 @@
       <c r="B11" t="n">
         <v>2812.008</v>
       </c>
+      <c r="C11" t="n">
+        <v>3103.437764191142</v>
+      </c>
       <c r="D11" t="n">
         <v>2.14599e-07</v>
       </c>
@@ -4748,6 +4937,9 @@
       <c r="B12" t="n">
         <v>2790.329</v>
       </c>
+      <c r="C12" t="n">
+        <v>3081.172605096426</v>
+      </c>
       <c r="D12" t="n">
         <v>2.15609e-07</v>
       </c>
@@ -4798,6 +4990,9 @@
       <c r="B13" t="n">
         <v>2766.869</v>
       </c>
+      <c r="C13" t="n">
+        <v>3054.056548180853</v>
+      </c>
       <c r="D13" t="n">
         <v>2.16844e-07</v>
       </c>
@@ -4848,6 +5043,9 @@
       <c r="B14" t="n">
         <v>2739.898</v>
       </c>
+      <c r="C14" t="n">
+        <v>3027.751634308126</v>
+      </c>
       <c r="D14" t="n">
         <v>2.18279e-07</v>
       </c>
@@ -4898,6 +5096,9 @@
       <c r="B15" t="n">
         <v>2715.872</v>
       </c>
+      <c r="C15" t="n">
+        <v>3005.808770667482</v>
+      </c>
       <c r="D15" t="n">
         <v>2.19196e-07</v>
       </c>
@@ -4948,6 +5149,9 @@
       <c r="B16" t="n">
         <v>2690.1</v>
       </c>
+      <c r="C16" t="n">
+        <v>2980.095194621601</v>
+      </c>
       <c r="D16" t="n">
         <v>2.20409e-07</v>
       </c>
@@ -4998,6 +5202,9 @@
       <c r="B17" t="n">
         <v>2669.379</v>
       </c>
+      <c r="C17" t="n">
+        <v>2954.535706711022</v>
+      </c>
       <c r="D17" t="n">
         <v>2.21682e-07</v>
       </c>
@@ -5048,6 +5255,9 @@
       <c r="B18" t="n">
         <v>2641.589</v>
       </c>
+      <c r="C18" t="n">
+        <v>2930.796794881062</v>
+      </c>
       <c r="D18" t="n">
         <v>2.22962e-07</v>
       </c>
@@ -5098,6 +5308,9 @@
       <c r="B19" t="n">
         <v>2606.438</v>
       </c>
+      <c r="C19" t="n">
+        <v>2901.536778522359</v>
+      </c>
       <c r="D19" t="n">
         <v>2.23933e-07</v>
       </c>
@@ -5148,6 +5361,9 @@
       <c r="B20" t="n">
         <v>2593.08</v>
       </c>
+      <c r="C20" t="n">
+        <v>2880.725951501829</v>
+      </c>
       <c r="D20" t="n">
         <v>2.25371e-07</v>
       </c>
@@ -5198,6 +5414,9 @@
       <c r="B21" t="n">
         <v>2555.902</v>
       </c>
+      <c r="C21" t="n">
+        <v>2848.778205815445</v>
+      </c>
       <c r="D21" t="n">
         <v>2.26332e-07</v>
       </c>
@@ -5247,6 +5466,9 @@
       </c>
       <c r="B22" t="n">
         <v>2546.351</v>
+      </c>
+      <c r="C22" t="n">
+        <v>2831.00210979433</v>
       </c>
       <c r="D22" t="n">
         <v>2.27732e-07</v>
@@ -5318,7 +5540,7 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Rct-d</t>
+          <t>delta Rct-d</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -5964,7 +6186,7 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Rct-d</t>
+          <t>delta Rct-d</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -6090,6 +6312,9 @@
       <c r="B2" t="n">
         <v>3322.365</v>
       </c>
+      <c r="C2" t="n">
+        <v>3650.82957047494</v>
+      </c>
       <c r="D2" t="n">
         <v>1.78228e-07</v>
       </c>
@@ -6140,6 +6365,9 @@
       <c r="B3" t="n">
         <v>3111.638</v>
       </c>
+      <c r="C3" t="n">
+        <v>3407.80629029734</v>
+      </c>
       <c r="D3" t="n">
         <v>1.87857e-07</v>
       </c>
@@ -6190,6 +6418,9 @@
       <c r="B4" t="n">
         <v>3042.006</v>
       </c>
+      <c r="C4" t="n">
+        <v>3338.49633367049</v>
+      </c>
       <c r="D4" t="n">
         <v>1.91062e-07</v>
       </c>
@@ -6240,6 +6471,9 @@
       <c r="B5" t="n">
         <v>3004.488</v>
       </c>
+      <c r="C5" t="n">
+        <v>3297.608195317027</v>
+      </c>
       <c r="D5" t="n">
         <v>1.93204e-07</v>
       </c>
@@ -6290,6 +6524,9 @@
       <c r="B6" t="n">
         <v>2967.235</v>
       </c>
+      <c r="C6" t="n">
+        <v>3261.150775920038</v>
+      </c>
       <c r="D6" t="n">
         <v>1.94892e-07</v>
       </c>
@@ -6340,6 +6577,9 @@
       <c r="B7" t="n">
         <v>2931.648</v>
       </c>
+      <c r="C7" t="n">
+        <v>3227.150281694132</v>
+      </c>
       <c r="D7" t="n">
         <v>1.96906e-07</v>
       </c>
@@ -6390,6 +6630,9 @@
       <c r="B8" t="n">
         <v>2899.958</v>
       </c>
+      <c r="C8" t="n">
+        <v>3194.324153581093</v>
+      </c>
       <c r="D8" t="n">
         <v>1.9842e-07</v>
       </c>
@@ -6440,6 +6683,9 @@
       <c r="B9" t="n">
         <v>2868.943</v>
       </c>
+      <c r="C9" t="n">
+        <v>3162.916373339117</v>
+      </c>
       <c r="D9" t="n">
         <v>1.99958e-07</v>
       </c>
@@ -6490,6 +6736,9 @@
       <c r="B10" t="n">
         <v>2838.5</v>
       </c>
+      <c r="C10" t="n">
+        <v>3134.406504013357</v>
+      </c>
       <c r="D10" t="n">
         <v>2.01527e-07</v>
       </c>
@@ -6540,6 +6789,9 @@
       <c r="B11" t="n">
         <v>2812.453</v>
       </c>
+      <c r="C11" t="n">
+        <v>3106.500043048217</v>
+      </c>
       <c r="D11" t="n">
         <v>2.02732e-07</v>
       </c>
@@ -6590,6 +6842,9 @@
       <c r="B12" t="n">
         <v>2771.025</v>
       </c>
+      <c r="C12" t="n">
+        <v>3070.899102276457</v>
+      </c>
       <c r="D12" t="n">
         <v>2.04309e-07</v>
       </c>
@@ -6640,6 +6895,9 @@
       <c r="B13" t="n">
         <v>2744.331</v>
       </c>
+      <c r="C13" t="n">
+        <v>3046.585549572324</v>
+      </c>
       <c r="D13" t="n">
         <v>2.0556e-07</v>
       </c>
@@ -6690,6 +6948,9 @@
       <c r="B14" t="n">
         <v>2736.308</v>
       </c>
+      <c r="C14" t="n">
+        <v>3025.904766034668</v>
+      </c>
       <c r="D14" t="n">
         <v>2.06697e-07</v>
       </c>
@@ -6740,6 +7001,9 @@
       <c r="B15" t="n">
         <v>2711.123</v>
       </c>
+      <c r="C15" t="n">
+        <v>3001.219302926584</v>
+      </c>
       <c r="D15" t="n">
         <v>2.0799e-07</v>
       </c>
@@ -6790,6 +7054,9 @@
       <c r="B16" t="n">
         <v>2681.612</v>
       </c>
+      <c r="C16" t="n">
+        <v>2975.634922521201</v>
+      </c>
       <c r="D16" t="n">
         <v>2.09486e-07</v>
       </c>
@@ -6840,6 +7107,9 @@
       <c r="B17" t="n">
         <v>2660.27</v>
       </c>
+      <c r="C17" t="n">
+        <v>2951.298267920116</v>
+      </c>
       <c r="D17" t="n">
         <v>2.10877e-07</v>
       </c>
@@ -6890,6 +7160,9 @@
       <c r="B18" t="n">
         <v>2617.769</v>
       </c>
+      <c r="C18" t="n">
+        <v>2920.537579861825</v>
+      </c>
       <c r="D18" t="n">
         <v>2.12058e-07</v>
       </c>
@@ -6940,6 +7213,9 @@
       <c r="B19" t="n">
         <v>2609.157</v>
       </c>
+      <c r="C19" t="n">
+        <v>2901.6142971371</v>
+      </c>
       <c r="D19" t="n">
         <v>2.13129e-07</v>
       </c>
@@ -6990,6 +7266,9 @@
       <c r="B20" t="n">
         <v>2587.246</v>
       </c>
+      <c r="C20" t="n">
+        <v>2874.331699071025</v>
+      </c>
       <c r="D20" t="n">
         <v>2.14538e-07</v>
       </c>
@@ -7040,6 +7319,9 @@
       <c r="B21" t="n">
         <v>2559.778</v>
       </c>
+      <c r="C21" t="n">
+        <v>2850.137979121015</v>
+      </c>
       <c r="D21" t="n">
         <v>2.1588e-07</v>
       </c>
@@ -7089,6 +7371,9 @@
       </c>
       <c r="B22" t="n">
         <v>2535.847</v>
+      </c>
+      <c r="C22" t="n">
+        <v>2825.269874185038</v>
       </c>
       <c r="D22" t="n">
         <v>2.17096e-07</v>
@@ -7160,7 +7445,7 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Rct-d</t>
+          <t>delta Rct-d</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -7386,6 +7671,9 @@
       <c r="B4" t="n">
         <v>19535.205</v>
       </c>
+      <c r="C4" t="n">
+        <v>33.3011248279415</v>
+      </c>
       <c r="D4" t="n">
         <v>2.45918e-08</v>
       </c>
@@ -7685,6 +7973,9 @@
       </c>
       <c r="B10" t="n">
         <v>18051.387</v>
+      </c>
+      <c r="C10" t="n">
+        <v>11.59040584074107</v>
       </c>
       <c r="D10" t="n">
         <v>2.72089e-08</v>
@@ -7806,7 +8097,7 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Rct-d</t>
+          <t>delta Rct-d</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -7932,6 +8223,9 @@
       <c r="B2" t="n">
         <v>3325.154</v>
       </c>
+      <c r="C2" t="n">
+        <v>3630.726008721113</v>
+      </c>
       <c r="D2" t="n">
         <v>1.81236e-07</v>
       </c>
@@ -7982,6 +8276,9 @@
       <c r="B3" t="n">
         <v>3141.792</v>
       </c>
+      <c r="C3" t="n">
+        <v>3422.511115955506</v>
+      </c>
       <c r="D3" t="n">
         <v>1.9048e-07</v>
       </c>
@@ -8032,6 +8329,9 @@
       <c r="B4" t="n">
         <v>3060.812</v>
       </c>
+      <c r="C4" t="n">
+        <v>3351.096234653782</v>
+      </c>
       <c r="D4" t="n">
         <v>1.93226e-07</v>
       </c>
@@ -8082,6 +8382,9 @@
       <c r="B5" t="n">
         <v>3034.613</v>
       </c>
+      <c r="C5" t="n">
+        <v>3316.089935460038</v>
+      </c>
       <c r="D5" t="n">
         <v>1.95508e-07</v>
       </c>
@@ -8132,6 +8435,9 @@
       <c r="B6" t="n">
         <v>2976.087</v>
       </c>
+      <c r="C6" t="n">
+        <v>3270.613190918845</v>
+      </c>
       <c r="D6" t="n">
         <v>1.97471e-07</v>
       </c>
@@ -8182,6 +8488,9 @@
       <c r="B7" t="n">
         <v>2940.544</v>
       </c>
+      <c r="C7" t="n">
+        <v>3233.286901548908</v>
+      </c>
       <c r="D7" t="n">
         <v>1.99153e-07</v>
       </c>
@@ -8232,6 +8541,9 @@
       <c r="B8" t="n">
         <v>2907.828</v>
       </c>
+      <c r="C8" t="n">
+        <v>3197.462404060361</v>
+      </c>
       <c r="D8" t="n">
         <v>2.01033e-07</v>
       </c>
@@ -8282,6 +8594,9 @@
       <c r="B9" t="n">
         <v>2858.686</v>
       </c>
+      <c r="C9" t="n">
+        <v>3159.784101077867</v>
+      </c>
       <c r="D9" t="n">
         <v>2.02102e-07</v>
       </c>
@@ -8332,6 +8647,9 @@
       <c r="B10" t="n">
         <v>2846.17</v>
       </c>
+      <c r="C10" t="n">
+        <v>3136.358904322622</v>
+      </c>
       <c r="D10" t="n">
         <v>2.03372e-07</v>
       </c>
@@ -8382,6 +8700,9 @@
       <c r="B11" t="n">
         <v>2799.328</v>
       </c>
+      <c r="C11" t="n">
+        <v>3102.544920355321</v>
+      </c>
       <c r="D11" t="n">
         <v>2.05532e-07</v>
       </c>
@@ -8432,6 +8753,9 @@
       <c r="B12" t="n">
         <v>2787.206</v>
       </c>
+      <c r="C12" t="n">
+        <v>3081.418551896954</v>
+      </c>
       <c r="D12" t="n">
         <v>2.07182e-07</v>
       </c>
@@ -8482,6 +8806,9 @@
       <c r="B13" t="n">
         <v>2764.489</v>
       </c>
+      <c r="C13" t="n">
+        <v>3054.279845068714</v>
+      </c>
       <c r="D13" t="n">
         <v>2.08491e-07</v>
       </c>
@@ -8532,6 +8859,9 @@
       <c r="B14" t="n">
         <v>2735.817</v>
       </c>
+      <c r="C14" t="n">
+        <v>3024.075233880629</v>
+      </c>
       <c r="D14" t="n">
         <v>2.10226e-07</v>
       </c>
@@ -8582,6 +8912,9 @@
       <c r="B15" t="n">
         <v>2707</v>
       </c>
+      <c r="C15" t="n">
+        <v>2995.846099839061</v>
+      </c>
       <c r="D15" t="n">
         <v>2.11741e-07</v>
       </c>
@@ -8632,6 +8965,9 @@
       <c r="B16" t="n">
         <v>2678.878</v>
       </c>
+      <c r="C16" t="n">
+        <v>2968.215587582626</v>
+      </c>
       <c r="D16" t="n">
         <v>2.13262e-07</v>
       </c>
@@ -8682,6 +9018,9 @@
       <c r="B17" t="n">
         <v>2633.819</v>
       </c>
+      <c r="C17" t="n">
+        <v>2932.894652037672</v>
+      </c>
       <c r="D17" t="n">
         <v>2.1475e-07</v>
       </c>
@@ -8732,6 +9071,9 @@
       <c r="B18" t="n">
         <v>2620.086</v>
       </c>
+      <c r="C18" t="n">
+        <v>2911.194669997487</v>
+      </c>
       <c r="D18" t="n">
         <v>2.1609e-07</v>
       </c>
@@ -8782,6 +9124,9 @@
       <c r="B19" t="n">
         <v>2592.122</v>
       </c>
+      <c r="C19" t="n">
+        <v>2882.923897820968</v>
+      </c>
       <c r="D19" t="n">
         <v>2.1782e-07</v>
       </c>
@@ -8832,6 +9177,9 @@
       <c r="B20" t="n">
         <v>2552.539</v>
       </c>
+      <c r="C20" t="n">
+        <v>2845.928313409928</v>
+      </c>
       <c r="D20" t="n">
         <v>2.19358e-07</v>
       </c>
@@ -8882,6 +9230,9 @@
       <c r="B21" t="n">
         <v>2541.159</v>
       </c>
+      <c r="C21" t="n">
+        <v>2826.707504808937</v>
+      </c>
       <c r="D21" t="n">
         <v>2.20969e-07</v>
       </c>
@@ -8931,6 +9282,9 @@
       </c>
       <c r="B22" t="n">
         <v>2502.932</v>
+      </c>
+      <c r="C22" t="n">
+        <v>2793.370445717521</v>
       </c>
       <c r="D22" t="n">
         <v>2.22296e-07</v>
@@ -9002,7 +9356,7 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Rct-d</t>
+          <t>delta Rct-d</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -9278,6 +9632,9 @@
       <c r="B5" t="n">
         <v>5421.400000000001</v>
       </c>
+      <c r="C5" t="n">
+        <v>5643.658179915051</v>
+      </c>
       <c r="D5" t="n">
         <v>1.21355e-07</v>
       </c>
@@ -9328,6 +9685,9 @@
       <c r="B6" t="n">
         <v>5335.116</v>
       </c>
+      <c r="C6" t="n">
+        <v>5557.267393916522</v>
+      </c>
       <c r="D6" t="n">
         <v>1.23201e-07</v>
       </c>
@@ -9378,6 +9738,9 @@
       <c r="B7" t="n">
         <v>5266.168000000001</v>
       </c>
+      <c r="C7" t="n">
+        <v>5481.168039354905</v>
+      </c>
       <c r="D7" t="n">
         <v>1.24738e-07</v>
       </c>
@@ -9428,6 +9791,9 @@
       <c r="B8" t="n">
         <v>5199.491</v>
       </c>
+      <c r="C8" t="n">
+        <v>5410.207537072618</v>
+      </c>
       <c r="D8" t="n">
         <v>1.26549e-07</v>
       </c>
@@ -9478,6 +9844,9 @@
       <c r="B9" t="n">
         <v>5135.626</v>
       </c>
+      <c r="C9" t="n">
+        <v>5348.861747908688</v>
+      </c>
       <c r="D9" t="n">
         <v>1.28225e-07</v>
       </c>
@@ -9528,6 +9897,9 @@
       <c r="B10" t="n">
         <v>5074.596</v>
       </c>
+      <c r="C10" t="n">
+        <v>5292.93248541252</v>
+      </c>
       <c r="D10" t="n">
         <v>1.29444e-07</v>
       </c>
@@ -9577,6 +9949,9 @@
       </c>
       <c r="B11" t="n">
         <v>5012.176</v>
+      </c>
+      <c r="C11" t="n">
+        <v>5226.635561220613</v>
       </c>
       <c r="D11" t="n">
         <v>1.3106e-07</v>

</xml_diff>

<commit_message>
im at my witts end
</commit_message>
<xml_diff>
--- a/BioSensorAnalysisSrcCode/EIS_Analysis/Austin_EIS/MegaExcel/Processed Chips for PCAI1ia/Chip 21.xlsx
+++ b/BioSensorAnalysisSrcCode/EIS_Analysis/Austin_EIS/MegaExcel/Processed Chips for PCAI1ia/Chip 21.xlsx
@@ -565,7 +565,7 @@
         <v>3413.305</v>
       </c>
       <c r="C2" t="n">
-        <v>3705.781582992509</v>
+        <v>17385.90666108369</v>
       </c>
       <c r="D2" t="n">
         <v>1.84241e-07</v>
@@ -598,10 +598,7 @@
         <v>-25925.97725441957</v>
       </c>
       <c r="Y2" t="n">
-        <v>3.973360418002409e-09</v>
-      </c>
-      <c r="Z2" t="n">
-        <v>4338.281983477777</v>
+        <v>-13024.54837611532</v>
       </c>
       <c r="AA2" t="n">
         <v>1.000000000002033e-08</v>
@@ -618,7 +615,7 @@
         <v>3306.557</v>
       </c>
       <c r="C3" t="n">
-        <v>3596.875521990378</v>
+        <v>18236.33397966523</v>
       </c>
       <c r="D3" t="n">
         <v>1.89606e-07</v>
@@ -651,10 +648,7 @@
         <v>-27402.84736786969</v>
       </c>
       <c r="Y3" t="n">
-        <v>1.897271783591817e-18</v>
-      </c>
-      <c r="Z3" t="n">
-        <v>4211.914002274965</v>
+        <v>-14016.89659339496</v>
       </c>
       <c r="AA3" t="n">
         <v>1e-08</v>
@@ -671,7 +665,7 @@
         <v>3231.904</v>
       </c>
       <c r="C4" t="n">
-        <v>3521.527944144097</v>
+        <v>18151.49333681268</v>
       </c>
       <c r="D4" t="n">
         <v>1.92888e-07</v>
@@ -704,10 +698,7 @@
         <v>-27984.20086789379</v>
       </c>
       <c r="Y4" t="n">
-        <v>1.274334709434572e-10</v>
-      </c>
-      <c r="Z4" t="n">
-        <v>4123.658205090058</v>
+        <v>-14014.76224746521</v>
       </c>
       <c r="AA4" t="n">
         <v>1.000000000000405e-08</v>
@@ -724,7 +715,7 @@
         <v>3169.252</v>
       </c>
       <c r="C5" t="n">
-        <v>3460.849069286025</v>
+        <v>18413.9760440465</v>
       </c>
       <c r="D5" t="n">
         <v>1.96208e-07</v>
@@ -757,10 +748,7 @@
         <v>-29046.99463667542</v>
       </c>
       <c r="Y5" t="n">
-        <v>1.579012405788227e-10</v>
-      </c>
-      <c r="Z5" t="n">
-        <v>4045.209555784623</v>
+        <v>-14359.95996855919</v>
       </c>
       <c r="AA5" t="n">
         <v>1.00000000000001e-08</v>
@@ -777,7 +765,7 @@
         <v>3112.06</v>
       </c>
       <c r="C6" t="n">
-        <v>3402.561588564839</v>
+        <v>18409.28380957767</v>
       </c>
       <c r="D6" t="n">
         <v>1.98503e-07</v>
@@ -810,10 +798,7 @@
         <v>-29058.63871125671</v>
       </c>
       <c r="Y6" t="n">
-        <v>4.911906337866607e-10</v>
-      </c>
-      <c r="Z6" t="n">
-        <v>3976.629059890452</v>
+        <v>-14414.64122354775</v>
       </c>
       <c r="AA6" t="n">
         <v>1.000000000000073e-08</v>
@@ -830,7 +815,7 @@
         <v>3058.458</v>
       </c>
       <c r="C7" t="n">
-        <v>3353.906615492061</v>
+        <v>18774.46624093795</v>
       </c>
       <c r="D7" t="n">
         <v>2.00804e-07</v>
@@ -863,10 +848,7 @@
         <v>-29264.9409855333</v>
       </c>
       <c r="Y7" t="n">
-        <v>1.123012009317532e-16</v>
-      </c>
-      <c r="Z7" t="n">
-        <v>3915.936364038092</v>
+        <v>-14840.93949501779</v>
       </c>
       <c r="AA7" t="n">
         <v>1e-08</v>
@@ -883,7 +865,7 @@
         <v>3000.47</v>
       </c>
       <c r="C8" t="n">
-        <v>3301.803960481059</v>
+        <v>18748.8361745695</v>
       </c>
       <c r="D8" t="n">
         <v>2.02918e-07</v>
@@ -916,10 +898,7 @@
         <v>-27659.99456902865</v>
       </c>
       <c r="Y8" t="n">
-        <v>5.529700177760481e-12</v>
-      </c>
-      <c r="Z8" t="n">
-        <v>3860.964985101534</v>
+        <v>-14866.19754393462</v>
       </c>
       <c r="AA8" t="n">
         <v>1.000000000000038e-08</v>
@@ -936,7 +915,7 @@
         <v>2954.274</v>
       </c>
       <c r="C9" t="n">
-        <v>3261.354513794582</v>
+        <v>18763.2790086604</v>
       </c>
       <c r="D9" t="n">
         <v>2.04758e-07</v>
@@ -969,10 +948,7 @@
         <v>-27949.07001255509</v>
       </c>
       <c r="Y9" t="n">
-        <v>3.952318134702614e-09</v>
-      </c>
-      <c r="Z9" t="n">
-        <v>3810.555620282222</v>
+        <v>-14927.28124176743</v>
       </c>
       <c r="AA9" t="n">
         <v>1.000000000014565e-08</v>
@@ -989,7 +965,7 @@
         <v>2919.242</v>
       </c>
       <c r="C10" t="n">
-        <v>3222.528243017276</v>
+        <v>19085.12773867075</v>
       </c>
       <c r="D10" t="n">
         <v>2.06513e-07</v>
@@ -1022,10 +998,7 @@
         <v>-28364.1585730412</v>
       </c>
       <c r="Y10" t="n">
-        <v>8.695782116767691e-09</v>
-      </c>
-      <c r="Z10" t="n">
-        <v>3764.259433155244</v>
+        <v>-15295.88305682766</v>
       </c>
       <c r="AA10" t="n">
         <v>1.000000000000013e-08</v>
@@ -1042,7 +1015,7 @@
         <v>2899.646</v>
       </c>
       <c r="C11" t="n">
-        <v>3196.256838416664</v>
+        <v>20019.41225721822</v>
       </c>
       <c r="D11" t="n">
         <v>2.08089e-07</v>
@@ -1075,10 +1048,7 @@
         <v>-30286.63477810142</v>
       </c>
       <c r="Y11" t="n">
-        <v>7.399923275621092e-09</v>
-      </c>
-      <c r="Z11" t="n">
-        <v>3722.293840317449</v>
+        <v>-16278.27365810443</v>
       </c>
       <c r="AA11" t="n">
         <v>1.000000000000328e-08</v>
@@ -1241,7 +1211,7 @@
         <v>3248.999</v>
       </c>
       <c r="C2" t="n">
-        <v>3548.586750022529</v>
+        <v>20233.71034351494</v>
       </c>
       <c r="D2" t="n">
         <v>1.88742e-07</v>
@@ -1274,10 +1244,7 @@
         <v>-28805.24954287466</v>
       </c>
       <c r="Y2" t="n">
-        <v>3.461751648758845e-09</v>
-      </c>
-      <c r="Z2" t="n">
-        <v>4126.568694892875</v>
+        <v>-16059.54448609244</v>
       </c>
       <c r="AA2" t="n">
         <v>1.000000000000682e-08</v>
@@ -1294,7 +1261,7 @@
         <v>3097.392</v>
       </c>
       <c r="C3" t="n">
-        <v>3393.368475201361</v>
+        <v>20458.53186345361</v>
       </c>
       <c r="D3" t="n">
         <v>1.94412e-07</v>
@@ -1327,10 +1294,7 @@
         <v>-26594.52615563833</v>
       </c>
       <c r="Y3" t="n">
-        <v>1.945267163618647e-08</v>
-      </c>
-      <c r="Z3" t="n">
-        <v>3984.43311368162</v>
+        <v>-16431.9858712189</v>
       </c>
       <c r="AA3" t="n">
         <v>1.000000000000073e-08</v>
@@ -1347,7 +1311,7 @@
         <v>3064.714</v>
       </c>
       <c r="C4" t="n">
-        <v>3347.518943184852</v>
+        <v>20559.94845170144</v>
       </c>
       <c r="D4" t="n">
         <v>1.96919e-07</v>
@@ -1380,10 +1344,7 @@
         <v>-27815.87381972411</v>
       </c>
       <c r="Y4" t="n">
-        <v>9.744149832265997e-15</v>
-      </c>
-      <c r="Z4" t="n">
-        <v>3924.695747861717</v>
+        <v>-16592.61926955419</v>
       </c>
       <c r="AA4" t="n">
         <v>1.000000000000394e-08</v>
@@ -1400,7 +1361,7 @@
         <v>3009.657</v>
       </c>
       <c r="C5" t="n">
-        <v>3305.924419102164</v>
+        <v>19990.76783117134</v>
       </c>
       <c r="D5" t="n">
         <v>1.98783e-07</v>
@@ -1433,10 +1394,7 @@
         <v>-26194.98924499944</v>
       </c>
       <c r="Y5" t="n">
-        <v>2.041724315974994e-15</v>
-      </c>
-      <c r="Z5" t="n">
-        <v>3877.998216129423</v>
+        <v>-16062.15535368631</v>
       </c>
       <c r="AA5" t="n">
         <v>1e-08</v>
@@ -1453,7 +1411,7 @@
         <v>2957.534</v>
       </c>
       <c r="C6" t="n">
-        <v>3262.624882560889</v>
+        <v>20774.94545658191</v>
       </c>
       <c r="D6" t="n">
         <v>2.0035e-07</v>
@@ -1486,10 +1444,7 @@
         <v>-24734.36023161278</v>
       </c>
       <c r="Y6" t="n">
-        <v>2.64856299099321e-10</v>
-      </c>
-      <c r="Z6" t="n">
-        <v>3835.907573896849</v>
+        <v>-16891.07830277646</v>
       </c>
       <c r="AA6" t="n">
         <v>1.000000000000014e-08</v>
@@ -1506,7 +1461,7 @@
         <v>2943.712</v>
       </c>
       <c r="C7" t="n">
-        <v>3238.402733392615</v>
+        <v>20770.76431823789</v>
       </c>
       <c r="D7" t="n">
         <v>2.02176e-07</v>
@@ -1539,10 +1494,7 @@
         <v>-26162.31709657338</v>
       </c>
       <c r="Y7" t="n">
-        <v>3.845840421510457e-10</v>
-      </c>
-      <c r="Z7" t="n">
-        <v>3796.855465673337</v>
+        <v>-16927.1999272504</v>
       </c>
       <c r="AA7" t="n">
         <v>1.000000000000006e-08</v>
@@ -1559,7 +1511,7 @@
         <v>2911.219</v>
       </c>
       <c r="C8" t="n">
-        <v>3206.810911233661</v>
+        <v>20812.36840858139</v>
       </c>
       <c r="D8" t="n">
         <v>2.03803e-07</v>
@@ -1592,10 +1544,7 @@
         <v>-26167.61583122996</v>
       </c>
       <c r="Y8" t="n">
-        <v>9.518381345387516e-11</v>
-      </c>
-      <c r="Z8" t="n">
-        <v>3757.938164876658</v>
+        <v>-17006.14820232087</v>
       </c>
       <c r="AA8" t="n">
         <v>1.000000000000125e-08</v>
@@ -1612,7 +1561,7 @@
         <v>2880.446</v>
       </c>
       <c r="C9" t="n">
-        <v>3175.008438643334</v>
+        <v>21477.90066053313</v>
       </c>
       <c r="D9" t="n">
         <v>2.05322e-07</v>
@@ -1645,10 +1594,7 @@
         <v>-26000.87059454789</v>
       </c>
       <c r="Y9" t="n">
-        <v>8.962322664060081e-11</v>
-      </c>
-      <c r="Z9" t="n">
-        <v>3720.957971118632</v>
+        <v>-17711.00550074706</v>
       </c>
       <c r="AA9" t="n">
         <v>1e-08</v>
@@ -1665,7 +1611,7 @@
         <v>2852.948</v>
       </c>
       <c r="C10" t="n">
-        <v>3150.513995253195</v>
+        <v>20878.77623298187</v>
       </c>
       <c r="D10" t="n">
         <v>2.07006e-07</v>
@@ -1698,10 +1644,7 @@
         <v>-26168.49190365453</v>
       </c>
       <c r="Y10" t="n">
-        <v>1.490559670089616e-10</v>
-      </c>
-      <c r="Z10" t="n">
-        <v>3684.621667345081</v>
+        <v>-17143.72525920299</v>
       </c>
       <c r="AA10" t="n">
         <v>1.000000000003612e-08</v>
@@ -1718,7 +1661,7 @@
         <v>2828.632</v>
       </c>
       <c r="C11" t="n">
-        <v>3121.949193174544</v>
+        <v>21073.57946398586</v>
       </c>
       <c r="D11" t="n">
         <v>2.08414e-07</v>
@@ -1751,10 +1694,7 @@
         <v>-26289.53935116196</v>
       </c>
       <c r="Y11" t="n">
-        <v>4.437929537938406e-09</v>
-      </c>
-      <c r="Z11" t="n">
-        <v>3650.464634807239</v>
+        <v>-17371.95556644195</v>
       </c>
       <c r="AA11" t="n">
         <v>1.000000000000007e-08</v>
@@ -1771,7 +1711,7 @@
         <v>2797.849</v>
       </c>
       <c r="C12" t="n">
-        <v>3092.841849043207</v>
+        <v>20892.40055776931</v>
       </c>
       <c r="D12" t="n">
         <v>2.09889e-07</v>
@@ -1804,10 +1744,7 @@
         <v>-26240.54747800111</v>
       </c>
       <c r="Y12" t="n">
-        <v>2.383232571510424e-10</v>
-      </c>
-      <c r="Z12" t="n">
-        <v>3617.155723543447</v>
+        <v>-17221.90251755224</v>
       </c>
       <c r="AA12" t="n">
         <v>1.000000000001773e-08</v>
@@ -1824,7 +1761,7 @@
         <v>2771.233</v>
       </c>
       <c r="C13" t="n">
-        <v>3065.227073523505</v>
+        <v>20913.68319622014</v>
       </c>
       <c r="D13" t="n">
         <v>2.11233e-07</v>
@@ -1857,10 +1794,7 @@
         <v>-26122.0567214235</v>
       </c>
       <c r="Y13" t="n">
-        <v>4.014741715271358e-13</v>
-      </c>
-      <c r="Z13" t="n">
-        <v>3582.32258116732</v>
+        <v>-17273.07216696975</v>
       </c>
       <c r="AA13" t="n">
         <v>1.000000000000027e-08</v>
@@ -1877,7 +1811,7 @@
         <v>2747.889</v>
       </c>
       <c r="C14" t="n">
-        <v>3040.965506931002</v>
+        <v>21081.80882396756</v>
       </c>
       <c r="D14" t="n">
         <v>2.12644e-07</v>
@@ -1910,10 +1844,7 @@
         <v>-26249.61645178953</v>
       </c>
       <c r="Y14" t="n">
-        <v>1.888537158384933e-12</v>
-      </c>
-      <c r="Z14" t="n">
-        <v>3549.319981128023</v>
+        <v>-17474.55831436993</v>
       </c>
       <c r="AA14" t="n">
         <v>1.000000000000761e-08</v>
@@ -1930,7 +1861,7 @@
         <v>2720.894</v>
       </c>
       <c r="C15" t="n">
-        <v>3013.64217727477</v>
+        <v>21648.75145788236</v>
       </c>
       <c r="D15" t="n">
         <v>2.14135e-07</v>
@@ -1963,10 +1894,7 @@
         <v>-26350.97202279682</v>
       </c>
       <c r="Y15" t="n">
-        <v>1.326908466148628e-09</v>
-      </c>
-      <c r="Z15" t="n">
-        <v>3516.682615553374</v>
+        <v>-18078.24652090655</v>
       </c>
       <c r="AA15" t="n">
         <v>1.000000000015281e-08</v>
@@ -1983,7 +1911,7 @@
         <v>2697.365</v>
       </c>
       <c r="C16" t="n">
-        <v>2989.976366977899</v>
+        <v>21025.19329692206</v>
       </c>
       <c r="D16" t="n">
         <v>2.15492e-07</v>
@@ -2016,10 +1944,7 @@
         <v>-26514.20003327129</v>
       </c>
       <c r="Y16" t="n">
-        <v>2.361418140254665e-09</v>
-      </c>
-      <c r="Z16" t="n">
-        <v>3483.903390530033</v>
+        <v>-17480.57280043867</v>
       </c>
       <c r="AA16" t="n">
         <v>1.000000000023654e-08</v>
@@ -2036,7 +1961,7 @@
         <v>2668.899</v>
       </c>
       <c r="C17" t="n">
-        <v>2961.628340163529</v>
+        <v>21366.72869563878</v>
       </c>
       <c r="D17" t="n">
         <v>2.16987e-07</v>
@@ -2069,10 +1994,7 @@
         <v>-26560.82693334683</v>
       </c>
       <c r="Y17" t="n">
-        <v>2.435386738540102e-09</v>
-      </c>
-      <c r="Z17" t="n">
-        <v>3450.868737054808</v>
+        <v>-17857.30103852316</v>
       </c>
       <c r="AA17" t="n">
         <v>1.000000000015642e-08</v>
@@ -2089,7 +2011,7 @@
         <v>2644.901</v>
       </c>
       <c r="C18" t="n">
-        <v>2936.03129800163</v>
+        <v>21501.49872404988</v>
       </c>
       <c r="D18" t="n">
         <v>2.18403e-07</v>
@@ -2122,10 +2044,7 @@
         <v>-26574.96493488604</v>
       </c>
       <c r="Y18" t="n">
-        <v>2.737982188141498e-09</v>
-      </c>
-      <c r="Z18" t="n">
-        <v>3418.952274950283</v>
+        <v>-18023.53037472664</v>
       </c>
       <c r="AA18" t="n">
         <v>1.000000000016111e-08</v>
@@ -2142,7 +2061,7 @@
         <v>2603.785</v>
       </c>
       <c r="C19" t="n">
-        <v>2903.906072749533</v>
+        <v>21587.94096813227</v>
       </c>
       <c r="D19" t="n">
         <v>2.19807e-07</v>
@@ -2175,10 +2094,7 @@
         <v>-25251.2601737917</v>
       </c>
       <c r="Y19" t="n">
-        <v>1.084371702312922e-10</v>
-      </c>
-      <c r="Z19" t="n">
-        <v>3386.141736488252</v>
+        <v>-18141.23011223017</v>
       </c>
       <c r="AA19" t="n">
         <v>1.000000000001499e-08</v>
@@ -2195,7 +2111,7 @@
         <v>2591.371</v>
       </c>
       <c r="C20" t="n">
-        <v>2884.962679319052</v>
+        <v>21600.34408187487</v>
       </c>
       <c r="D20" t="n">
         <v>2.21247e-07</v>
@@ -2228,10 +2144,7 @@
         <v>-26666.73359235622</v>
       </c>
       <c r="Y20" t="n">
-        <v>2.691471049114605e-10</v>
-      </c>
-      <c r="Z20" t="n">
-        <v>3353.553789033743</v>
+        <v>-18184.92688372917</v>
       </c>
       <c r="AA20" t="n">
         <v>1.000000000000395e-08</v>
@@ -2248,7 +2161,7 @@
         <v>2569.274</v>
       </c>
       <c r="C21" t="n">
-        <v>2858.194917716988</v>
+        <v>22166.70262344149</v>
       </c>
       <c r="D21" t="n">
         <v>2.22464e-07</v>
@@ -2281,10 +2194,7 @@
         <v>-26660.41809050335</v>
       </c>
       <c r="Y21" t="n">
-        <v>2.87682995133163e-09</v>
-      </c>
-      <c r="Z21" t="n">
-        <v>3321.892580425197</v>
+        <v>-18782.64461125029</v>
       </c>
       <c r="AA21" t="n">
         <v>1.000000000063688e-08</v>
@@ -2301,7 +2211,7 @@
         <v>2529.954</v>
       </c>
       <c r="C22" t="n">
-        <v>2828.208967482188</v>
+        <v>22213.13291204726</v>
       </c>
       <c r="D22" t="n">
         <v>2.24132e-07</v>
@@ -2334,10 +2244,7 @@
         <v>-25628.79036655436</v>
       </c>
       <c r="Y22" t="n">
-        <v>1.176717711878263e-10</v>
-      </c>
-      <c r="Z22" t="n">
-        <v>3290.260175203482</v>
+        <v>-18863.96513993586</v>
       </c>
       <c r="AA22" t="n">
         <v>1.000000000002077e-08</v>
@@ -2500,7 +2407,7 @@
         <v>3304.173</v>
       </c>
       <c r="C2" t="n">
-        <v>3617.638513947961</v>
+        <v>17806.55787171127</v>
       </c>
       <c r="D2" t="n">
         <v>1.87206e-07</v>
@@ -2533,10 +2440,7 @@
         <v>-24495.06033497604</v>
       </c>
       <c r="Y2" t="n">
-        <v>9.372481880738808e-09</v>
-      </c>
-      <c r="Z2" t="n">
-        <v>4196.134374984057</v>
+        <v>-13535.21066825889</v>
       </c>
       <c r="AA2" t="n">
         <v>1.000000000000242e-08</v>
@@ -2553,7 +2457,7 @@
         <v>3121.984</v>
       </c>
       <c r="C3" t="n">
-        <v>3418.678972156053</v>
+        <v>18616.03386501097</v>
       </c>
       <c r="D3" t="n">
         <v>1.97114e-07</v>
@@ -2586,10 +2490,7 @@
         <v>-26459.89008797356</v>
       </c>
       <c r="Y3" t="n">
-        <v>1.008242152951607e-09</v>
-      </c>
-      <c r="Z3" t="n">
-        <v>4001.223256966525</v>
+        <v>-14591.14731956164</v>
       </c>
       <c r="AA3" t="n">
         <v>1e-08</v>
@@ -2606,7 +2507,7 @@
         <v>3056.405</v>
       </c>
       <c r="C4" t="n">
-        <v>3349.286450015036</v>
+        <v>18918.38737533531</v>
       </c>
       <c r="D4" t="n">
         <v>2.00293e-07</v>
@@ -2639,10 +2540,7 @@
         <v>-26910.56761976944</v>
       </c>
       <c r="Y4" t="n">
-        <v>1.569572573701757e-10</v>
-      </c>
-      <c r="Z4" t="n">
-        <v>3927.541019956939</v>
+        <v>-14973.79283383203</v>
       </c>
       <c r="AA4" t="n">
         <v>1.000000000000016e-08</v>
@@ -2659,7 +2557,7 @@
         <v>3037.554</v>
       </c>
       <c r="C5" t="n">
-        <v>3314.45511250991</v>
+        <v>18581.01166301137</v>
       </c>
       <c r="D5" t="n">
         <v>2.02227e-07</v>
@@ -2692,10 +2590,7 @@
         <v>-29195.63144525173</v>
       </c>
       <c r="Y5" t="n">
-        <v>5.336967142759836e-10</v>
-      </c>
-      <c r="Z5" t="n">
-        <v>3877.104852299329</v>
+        <v>-14680.56679585464</v>
       </c>
       <c r="AA5" t="n">
         <v>1.000000000000285e-08</v>
@@ -2712,7 +2607,7 @@
         <v>2978.261</v>
       </c>
       <c r="C6" t="n">
-        <v>3271.143678062786</v>
+        <v>18451.80430279524</v>
       </c>
       <c r="D6" t="n">
         <v>2.03998e-07</v>
@@ -2745,10 +2640,7 @@
         <v>-27475.48268528328</v>
       </c>
       <c r="Y6" t="n">
-        <v>5.254567269568468e-09</v>
-      </c>
-      <c r="Z6" t="n">
-        <v>3829.970003896831</v>
+        <v>-14592.93313919188</v>
       </c>
       <c r="AA6" t="n">
         <v>1.000000000000448e-08</v>
@@ -2765,7 +2657,7 @@
         <v>2959.788</v>
       </c>
       <c r="C7" t="n">
-        <v>3242.753550935369</v>
+        <v>19277.10453787626</v>
       </c>
       <c r="D7" t="n">
         <v>2.05772e-07</v>
@@ -2798,10 +2690,7 @@
         <v>-29552.57746903169</v>
       </c>
       <c r="Y7" t="n">
-        <v>5.172261010524144e-18</v>
-      </c>
-      <c r="Z7" t="n">
-        <v>3785.515982341406</v>
+        <v>-15470.14101628375</v>
       </c>
       <c r="AA7" t="n">
         <v>1e-08</v>
@@ -2818,7 +2707,7 @@
         <v>2896.144</v>
       </c>
       <c r="C8" t="n">
-        <v>3197.530824562</v>
+        <v>18940.09506535078</v>
       </c>
       <c r="D8" t="n">
         <v>2.07111e-07</v>
@@ -2851,10 +2740,7 @@
         <v>-26156.50274033273</v>
       </c>
       <c r="Y8" t="n">
-        <v>1.199142879722051e-08</v>
-      </c>
-      <c r="Z8" t="n">
-        <v>3748.021297279653</v>
+        <v>-15162.92833519332</v>
       </c>
       <c r="AA8" t="n">
         <v>1.000000000000031e-08</v>
@@ -2871,7 +2757,7 @@
         <v>2888.916</v>
       </c>
       <c r="C9" t="n">
-        <v>3178.401365770566</v>
+        <v>19497.50652095514</v>
       </c>
       <c r="D9" t="n">
         <v>2.08269e-07</v>
@@ -2904,10 +2790,7 @@
         <v>-28122.51402882813</v>
       </c>
       <c r="Y9" t="n">
-        <v>1.637636171640223e-10</v>
-      </c>
-      <c r="Z9" t="n">
-        <v>3715.869776117712</v>
+        <v>-15755.96204506431</v>
       </c>
       <c r="AA9" t="n">
         <v>1.000000000000328e-08</v>
@@ -2924,7 +2807,7 @@
         <v>2858.486</v>
       </c>
       <c r="C10" t="n">
-        <v>3151.851265917903</v>
+        <v>18925.42843486792</v>
       </c>
       <c r="D10" t="n">
         <v>2.09535e-07</v>
@@ -2957,10 +2840,7 @@
         <v>-28110.58107177476</v>
       </c>
       <c r="Y10" t="n">
-        <v>3.136585321634133e-10</v>
-      </c>
-      <c r="Z10" t="n">
-        <v>3684.196568731055</v>
+        <v>-15207.42631571441</v>
       </c>
       <c r="AA10" t="n">
         <v>1.000000000002126e-08</v>
@@ -2977,7 +2857,7 @@
         <v>2818.328</v>
       </c>
       <c r="C11" t="n">
-        <v>3118.595611701044</v>
+        <v>19257.26839971999</v>
       </c>
       <c r="D11" t="n">
         <v>2.10802e-07</v>
@@ -3010,10 +2890,7 @@
         <v>-26730.66167624396</v>
       </c>
       <c r="Y11" t="n">
-        <v>5.822225911921077e-10</v>
-      </c>
-      <c r="Z11" t="n">
-        <v>3651.20362987053</v>
+        <v>-15574.09919881867</v>
       </c>
       <c r="AA11" t="n">
         <v>1.000000000000367e-08</v>
@@ -3030,7 +2907,7 @@
         <v>2803.71</v>
       </c>
       <c r="C12" t="n">
-        <v>3099.990984607326</v>
+        <v>19157.76587076979</v>
       </c>
       <c r="D12" t="n">
         <v>2.11994e-07</v>
@@ -3063,10 +2940,7 @@
         <v>-28254.60890465227</v>
       </c>
       <c r="Y12" t="n">
-        <v>2.341753663240482e-10</v>
-      </c>
-      <c r="Z12" t="n">
-        <v>3616.918719992228</v>
+        <v>-15502.98251064955</v>
       </c>
       <c r="AA12" t="n">
         <v>1.000000000000736e-08</v>
@@ -3083,7 +2957,7 @@
         <v>2761.828</v>
       </c>
       <c r="C13" t="n">
-        <v>3065.213845201413</v>
+        <v>20011.42453218765</v>
       </c>
       <c r="D13" t="n">
         <v>2.13431e-07</v>
@@ -3116,10 +2990,7 @@
         <v>-26870.43207501114</v>
       </c>
       <c r="Y13" t="n">
-        <v>9.977220009734805e-09</v>
-      </c>
-      <c r="Z13" t="n">
-        <v>3581.519667313898</v>
+        <v>-16399.55097607947</v>
       </c>
       <c r="AA13" t="n">
         <v>1.000000000006445e-08</v>
@@ -3136,7 +3007,7 @@
         <v>2751.992</v>
       </c>
       <c r="C14" t="n">
-        <v>3041.991470148206</v>
+        <v>19942.70173437285</v>
       </c>
       <c r="D14" t="n">
         <v>2.14758e-07</v>
@@ -3169,10 +3040,7 @@
         <v>-28865.08604200661</v>
       </c>
       <c r="Y14" t="n">
-        <v>1.846181921349008e-10</v>
-      </c>
-      <c r="Z14" t="n">
-        <v>3545.4081768414</v>
+        <v>-16362.99011010424</v>
       </c>
       <c r="AA14" t="n">
         <v>1.000000000002417e-08</v>
@@ -3189,7 +3057,7 @@
         <v>2724.057</v>
       </c>
       <c r="C15" t="n">
-        <v>3013.758567933961</v>
+        <v>20063.76937320794</v>
       </c>
       <c r="D15" t="n">
         <v>2.15967e-07</v>
@@ -3222,10 +3090,7 @@
         <v>-28999.21012447367</v>
       </c>
       <c r="Y15" t="n">
-        <v>7.274745846453659e-17</v>
-      </c>
-      <c r="Z15" t="n">
-        <v>3509.33830096486</v>
+        <v>-16515.77705853782</v>
       </c>
       <c r="AA15" t="n">
         <v>1e-08</v>
@@ -3242,7 +3107,7 @@
         <v>2712.438</v>
       </c>
       <c r="C16" t="n">
-        <v>2993.29750291965</v>
+        <v>20518.24405402767</v>
       </c>
       <c r="D16" t="n">
         <v>2.17439e-07</v>
@@ -3275,10 +3140,7 @@
         <v>-31332.51856013672</v>
       </c>
       <c r="Y16" t="n">
-        <v>6.987080395847131e-11</v>
-      </c>
-      <c r="Z16" t="n">
-        <v>3473.240372442296</v>
+        <v>-17009.75975822243</v>
       </c>
       <c r="AA16" t="n">
         <v>1.000000000000087e-08</v>
@@ -3295,7 +3157,7 @@
         <v>2648.633</v>
       </c>
       <c r="C17" t="n">
-        <v>2949.437375412275</v>
+        <v>20362.43794771805</v>
       </c>
       <c r="D17" t="n">
         <v>2.18927e-07</v>
@@ -3328,10 +3190,7 @@
         <v>-27488.91959558622</v>
       </c>
       <c r="Y17" t="n">
-        <v>3.287138289903484e-11</v>
-      </c>
-      <c r="Z17" t="n">
-        <v>3437.571463798545</v>
+        <v>-16886.28018551526</v>
       </c>
       <c r="AA17" t="n">
         <v>1.000000000001291e-08</v>
@@ -3348,7 +3207,7 @@
         <v>2635.999</v>
       </c>
       <c r="C18" t="n">
-        <v>2928.86459690938</v>
+        <v>20484.37092938511</v>
       </c>
       <c r="D18" t="n">
         <v>2.20174e-07</v>
@@ -3381,10 +3240,7 @@
         <v>-29291.80914406236</v>
       </c>
       <c r="Y18" t="n">
-        <v>2.418275026610593e-10</v>
-      </c>
-      <c r="Z18" t="n">
-        <v>3402.6790027316</v>
+        <v>-17039.8451448916</v>
       </c>
       <c r="AA18" t="n">
         <v>1.00000000000023e-08</v>
@@ -3401,7 +3257,7 @@
         <v>2609.567</v>
       </c>
       <c r="C19" t="n">
-        <v>2902.61908256478</v>
+        <v>20837.53464307007</v>
       </c>
       <c r="D19" t="n">
         <v>2.21328e-07</v>
@@ -3434,10 +3290,7 @@
         <v>-29172.39393842236</v>
       </c>
       <c r="Y19" t="n">
-        <v>2.771806947516841e-10</v>
-      </c>
-      <c r="Z19" t="n">
-        <v>3368.694983689623</v>
+        <v>-17424.42406160838</v>
       </c>
       <c r="AA19" t="n">
         <v>1.000000000000171e-08</v>
@@ -3454,7 +3307,7 @@
         <v>2582.512</v>
       </c>
       <c r="C20" t="n">
-        <v>2876.03564247402</v>
+        <v>20915.72837511411</v>
       </c>
       <c r="D20" t="n">
         <v>2.22747e-07</v>
@@ -3487,10 +3340,7 @@
         <v>-29428.38938475875</v>
       </c>
       <c r="Y20" t="n">
-        <v>2.072852205262699e-10</v>
-      </c>
-      <c r="Z20" t="n">
-        <v>3335.453195006065</v>
+        <v>-17537.1813823277</v>
       </c>
       <c r="AA20" t="n">
         <v>1.000000000000288e-08</v>
@@ -3507,7 +3357,7 @@
         <v>2556.327</v>
       </c>
       <c r="C21" t="n">
-        <v>2849.253397272075</v>
+        <v>20957.71961972298</v>
       </c>
       <c r="D21" t="n">
         <v>2.24003e-07</v>
@@ -3540,10 +3390,7 @@
         <v>-29591.87863106111</v>
       </c>
       <c r="Y21" t="n">
-        <v>2.092233388533273e-10</v>
-      </c>
-      <c r="Z21" t="n">
-        <v>3302.771891228992</v>
+        <v>-17609.33822145547</v>
       </c>
       <c r="AA21" t="n">
         <v>1.000000000000298e-08</v>
@@ -3560,7 +3407,7 @@
         <v>2533.141</v>
       </c>
       <c r="C22" t="n">
-        <v>2825.573592770365</v>
+        <v>20772.27288051934</v>
       </c>
       <c r="D22" t="n">
         <v>2.24989e-07</v>
@@ -3593,10 +3440,7 @@
         <v>-29268.61044251429</v>
       </c>
       <c r="Y22" t="n">
-        <v>3.390292703957733e-10</v>
-      </c>
-      <c r="Z22" t="n">
-        <v>3271.052418534506</v>
+        <v>-17447.50183943682</v>
       </c>
       <c r="AA22" t="n">
         <v>1.00000000000001e-08</v>
@@ -3758,6 +3602,9 @@
       <c r="B2" t="n">
         <v>33526.17</v>
       </c>
+      <c r="C2" t="n">
+        <v>36967.09216734418</v>
+      </c>
       <c r="D2" t="n">
         <v>1.07149e-08</v>
       </c>
@@ -3789,10 +3636,7 @@
         <v>-43677.778780635</v>
       </c>
       <c r="Y2" t="n">
-        <v>2883.489211920488</v>
-      </c>
-      <c r="Z2" t="n">
-        <v>2080.703758691029</v>
+        <v>-816.2323885033766</v>
       </c>
       <c r="AA2" t="n">
         <v>2.191155442269083e-06</v>
@@ -3808,6 +3652,9 @@
       <c r="B3" t="n">
         <v>28322.376</v>
       </c>
+      <c r="C3" t="n">
+        <v>31264.20508501418</v>
+      </c>
       <c r="D3" t="n">
         <v>1.37638e-08</v>
       </c>
@@ -3839,10 +3686,7 @@
         <v>-46447.82712472187</v>
       </c>
       <c r="Y3" t="n">
-        <v>1950.814450412289</v>
-      </c>
-      <c r="Z3" t="n">
-        <v>1764.10020359153</v>
+        <v>-772.3761901199396</v>
       </c>
       <c r="AA3" t="n">
         <v>1.764139868533671e-06</v>
@@ -3858,6 +3702,9 @@
       <c r="B4" t="n">
         <v>27190.091</v>
       </c>
+      <c r="C4" t="n">
+        <v>30027.90448843535</v>
+      </c>
       <c r="D4" t="n">
         <v>1.46789e-08</v>
       </c>
@@ -3889,10 +3736,7 @@
         <v>-47352.15425404939</v>
       </c>
       <c r="Y4" t="n">
-        <v>2015.383294903022</v>
-      </c>
-      <c r="Z4" t="n">
-        <v>1825.196364559226</v>
+        <v>-753.3597451355909</v>
       </c>
       <c r="AA4" t="n">
         <v>1.414664423208874e-06</v>
@@ -3908,6 +3752,9 @@
       <c r="B5" t="n">
         <v>26657.818</v>
       </c>
+      <c r="C5" t="n">
+        <v>29528.13501808441</v>
+      </c>
       <c r="D5" t="n">
         <v>1.51748e-08</v>
       </c>
@@ -3939,10 +3786,7 @@
         <v>-48044.55278719714</v>
       </c>
       <c r="Y5" t="n">
-        <v>2019.360931709148</v>
-      </c>
-      <c r="Z5" t="n">
-        <v>1829.841161391234</v>
+        <v>-788.0291703879302</v>
       </c>
       <c r="AA5" t="n">
         <v>1.405679274327418e-06</v>
@@ -3958,6 +3802,9 @@
       <c r="B6" t="n">
         <v>26254.083</v>
       </c>
+      <c r="C6" t="n">
+        <v>29071.04481278188</v>
+      </c>
       <c r="D6" t="n">
         <v>1.5568e-08</v>
       </c>
@@ -3989,10 +3836,7 @@
         <v>-48301.49317769516</v>
       </c>
       <c r="Y6" t="n">
-        <v>2013.376304596488</v>
-      </c>
-      <c r="Z6" t="n">
-        <v>1825.085703212622</v>
+        <v>-766.1338762235791</v>
       </c>
       <c r="AA6" t="n">
         <v>1.661507495215767e-06</v>
@@ -4008,6 +3852,9 @@
       <c r="B7" t="n">
         <v>25885.734</v>
       </c>
+      <c r="C7" t="n">
+        <v>28687.23037229063</v>
+      </c>
       <c r="D7" t="n">
         <v>1.59554e-08</v>
       </c>
@@ -4039,10 +3886,7 @@
         <v>-48536.4509105106</v>
       </c>
       <c r="Y7" t="n">
-        <v>2010.272054506718</v>
-      </c>
-      <c r="Z7" t="n">
-        <v>1822.911231973246</v>
+        <v>-765.5822543115682</v>
       </c>
       <c r="AA7" t="n">
         <v>1.654722408470943e-06</v>
@@ -4058,6 +3902,9 @@
       <c r="B8" t="n">
         <v>25521.475</v>
       </c>
+      <c r="C8" t="n">
+        <v>28431.4120189409</v>
+      </c>
       <c r="D8" t="n">
         <v>1.6328e-08</v>
       </c>
@@ -4089,10 +3936,7 @@
         <v>-48625.74946949843</v>
       </c>
       <c r="Y8" t="n">
-        <v>2006.865871564456</v>
-      </c>
-      <c r="Z8" t="n">
-        <v>1820.427341985811</v>
+        <v>-831.1814468109988</v>
       </c>
       <c r="AA8" t="n">
         <v>1.652679632918364e-06</v>
@@ -4109,7 +3953,7 @@
         <v>25183.032</v>
       </c>
       <c r="C9" t="n">
-        <v>14.05900507842058</v>
+        <v>28025.72455602025</v>
       </c>
       <c r="D9" t="n">
         <v>1.66744e-08</v>
@@ -4142,10 +3986,7 @@
         <v>-48529.13810753277</v>
       </c>
       <c r="Y9" t="n">
-        <v>2048.121562254793</v>
-      </c>
-      <c r="Z9" t="n">
-        <v>1859.966738194793</v>
+        <v>-796.9802640888392</v>
       </c>
       <c r="AA9" t="n">
         <v>1.610289555534342e-06</v>
@@ -4161,6 +4002,9 @@
       <c r="B10" t="n">
         <v>24857.975</v>
       </c>
+      <c r="C10" t="n">
+        <v>27739.47746344164</v>
+      </c>
       <c r="D10" t="n">
         <v>1.70294e-08</v>
       </c>
@@ -4192,10 +4036,7 @@
         <v>-48484.0635360629</v>
       </c>
       <c r="Y10" t="n">
-        <v>2056.781931524606</v>
-      </c>
-      <c r="Z10" t="n">
-        <v>1868.963630238603</v>
+        <v>-825.6994883514053</v>
       </c>
       <c r="AA10" t="n">
         <v>1.596751668275329e-06</v>
@@ -4211,6 +4052,9 @@
       <c r="B11" t="n">
         <v>24538.509</v>
       </c>
+      <c r="C11" t="n">
+        <v>27306.28815965744</v>
+      </c>
       <c r="D11" t="n">
         <v>1.73844e-08</v>
       </c>
@@ -4242,10 +4086,7 @@
         <v>-48283.0499287217</v>
       </c>
       <c r="Y11" t="n">
-        <v>2014.642061059314</v>
-      </c>
-      <c r="Z11" t="n">
-        <v>1829.866113799269</v>
+        <v>-753.2580909594344</v>
       </c>
       <c r="AA11" t="n">
         <v>1.626963053200119e-06</v>
@@ -4408,7 +4249,7 @@
         <v>3321.554</v>
       </c>
       <c r="C2" t="n">
-        <v>3623.895495047583</v>
+        <v>18174.83840942915</v>
       </c>
       <c r="D2" t="n">
         <v>1.86118e-07</v>
@@ -4441,10 +4282,7 @@
         <v>-24183.13325951939</v>
       </c>
       <c r="Y2" t="n">
-        <v>8.18558636998039e-09</v>
-      </c>
-      <c r="Z2" t="n">
-        <v>4197.135296207487</v>
+        <v>-13882.90644844266</v>
       </c>
       <c r="AA2" t="n">
         <v>1.000000000003627e-08</v>
@@ -4461,7 +4299,7 @@
         <v>3106.75</v>
       </c>
       <c r="C3" t="n">
-        <v>3399.158274198141</v>
+        <v>18103.12098074183</v>
       </c>
       <c r="D3" t="n">
         <v>1.97542e-07</v>
@@ -4494,10 +4332,7 @@
         <v>-25132.25704839991</v>
       </c>
       <c r="Y3" t="n">
-        <v>2.855706839303508e-09</v>
-      </c>
-      <c r="Z3" t="n">
-        <v>3982.710374021114</v>
+        <v>-14079.1906986449</v>
       </c>
       <c r="AA3" t="n">
         <v>1.000000000000005e-08</v>
@@ -4514,7 +4349,7 @@
         <v>3042.389</v>
       </c>
       <c r="C4" t="n">
-        <v>3331.220355672339</v>
+        <v>18097.21444582372</v>
       </c>
       <c r="D4" t="n">
         <v>2.01286e-07</v>
@@ -4547,10 +4382,7 @@
         <v>-25921.32667909566</v>
       </c>
       <c r="Y4" t="n">
-        <v>1.061910452679619e-11</v>
-      </c>
-      <c r="Z4" t="n">
-        <v>3908.154320430063</v>
+        <v>-14158.69584433965</v>
       </c>
       <c r="AA4" t="n">
         <v>1e-08</v>
@@ -4567,7 +4399,7 @@
         <v>3019.559</v>
       </c>
       <c r="C5" t="n">
-        <v>3296.409968256175</v>
+        <v>18285.40839061189</v>
       </c>
       <c r="D5" t="n">
         <v>2.036e-07</v>
@@ -4600,10 +4432,7 @@
         <v>-28240.68808179591</v>
       </c>
       <c r="Y5" t="n">
-        <v>2.392805453571923e-09</v>
-      </c>
-      <c r="Z5" t="n">
-        <v>3856.895157992336</v>
+        <v>-14402.64375928205</v>
       </c>
       <c r="AA5" t="n">
         <v>1.000000000000218e-08</v>
@@ -4620,7 +4449,7 @@
         <v>2961.543</v>
       </c>
       <c r="C6" t="n">
-        <v>3253.553499472222</v>
+        <v>17951.11200315564</v>
       </c>
       <c r="D6" t="n">
         <v>2.05551e-07</v>
@@ -4653,10 +4482,7 @@
         <v>-26753.21345103956</v>
       </c>
       <c r="Y6" t="n">
-        <v>9.456756740009373e-11</v>
-      </c>
-      <c r="Z6" t="n">
-        <v>3811.837128442961</v>
+        <v>-14109.43952438269</v>
       </c>
       <c r="AA6" t="n">
         <v>1.000000000000069e-08</v>
@@ -4673,7 +4499,7 @@
         <v>2942.584</v>
       </c>
       <c r="C7" t="n">
-        <v>3224.452653954537</v>
+        <v>18586.0327635418</v>
       </c>
       <c r="D7" t="n">
         <v>2.07554e-07</v>
@@ -4706,10 +4532,7 @@
         <v>-29115.47264585606</v>
       </c>
       <c r="Y7" t="n">
-        <v>125.0389400380478</v>
-      </c>
-      <c r="Z7" t="n">
-        <v>4016.786618265003</v>
+        <v>-14796.59609022763</v>
       </c>
       <c r="AA7" t="n">
         <v>1.911798595083981e-08</v>
@@ -4726,7 +4549,7 @@
         <v>2896.458</v>
       </c>
       <c r="C8" t="n">
-        <v>3188.953281812711</v>
+        <v>17776.45140767347</v>
       </c>
       <c r="D8" t="n">
         <v>2.10392e-07</v>
@@ -4759,10 +4582,7 @@
         <v>-28394.39105021164</v>
       </c>
       <c r="Y8" t="n">
-        <v>2.063089794802132e-08</v>
-      </c>
-      <c r="Z8" t="n">
-        <v>3730.626176126394</v>
+        <v>-14031.81730826824</v>
       </c>
       <c r="AA8" t="n">
         <v>1.000000000000704e-08</v>
@@ -4779,7 +4599,7 @@
         <v>2867.432</v>
       </c>
       <c r="C9" t="n">
-        <v>3157.296565413375</v>
+        <v>17581.05389711935</v>
       </c>
       <c r="D9" t="n">
         <v>2.11914e-07</v>
@@ -4812,10 +4632,7 @@
         <v>-28548.42548320814</v>
       </c>
       <c r="Y9" t="n">
-        <v>1.630872492385224e-10</v>
-      </c>
-      <c r="Z9" t="n">
-        <v>3694.783648524833</v>
+        <v>-13868.35429667352</v>
       </c>
       <c r="AA9" t="n">
         <v>1.00000000000811e-08</v>
@@ -4832,7 +4649,7 @@
         <v>2837.095</v>
       </c>
       <c r="C10" t="n">
-        <v>3130.289419778871</v>
+        <v>18304.68667064222</v>
       </c>
       <c r="D10" t="n">
         <v>2.13002e-07</v>
@@ -4865,10 +4682,7 @@
         <v>-28674.71482569155</v>
       </c>
       <c r="Y10" t="n">
-        <v>3.259689340340592e-10</v>
-      </c>
-      <c r="Z10" t="n">
-        <v>3661.15466635551</v>
+        <v>-14629.21574080399</v>
       </c>
       <c r="AA10" t="n">
         <v>1.000000000000035e-08</v>
@@ -4885,7 +4699,7 @@
         <v>2812.008</v>
       </c>
       <c r="C11" t="n">
-        <v>3103.437764191142</v>
+        <v>18139.72608498709</v>
       </c>
       <c r="D11" t="n">
         <v>2.14599e-07</v>
@@ -4918,10 +4732,7 @@
         <v>-28898.50286554719</v>
       </c>
       <c r="Y11" t="n">
-        <v>2.584869732792946e-10</v>
-      </c>
-      <c r="Z11" t="n">
-        <v>3628.426219168407</v>
+        <v>-14496.30558013267</v>
       </c>
       <c r="AA11" t="n">
         <v>1.000000000000108e-08</v>
@@ -4938,7 +4749,7 @@
         <v>2790.329</v>
       </c>
       <c r="C12" t="n">
-        <v>3081.172605096426</v>
+        <v>18313.42932698556</v>
       </c>
       <c r="D12" t="n">
         <v>2.15609e-07</v>
@@ -4971,10 +4782,7 @@
         <v>-29319.53796829532</v>
       </c>
       <c r="Y12" t="n">
-        <v>1.514289416406875e-10</v>
-      </c>
-      <c r="Z12" t="n">
-        <v>3596.877893152952</v>
+        <v>-14697.95143155157</v>
       </c>
       <c r="AA12" t="n">
         <v>1.00000000000106e-08</v>
@@ -4991,7 +4799,7 @@
         <v>2766.869</v>
       </c>
       <c r="C13" t="n">
-        <v>3054.056548180853</v>
+        <v>18515.39358344079</v>
       </c>
       <c r="D13" t="n">
         <v>2.16844e-07</v>
@@ -5024,10 +4832,7 @@
         <v>-29404.16599194265</v>
       </c>
       <c r="Y13" t="n">
-        <v>1.120530536052821e-08</v>
-      </c>
-      <c r="Z13" t="n">
-        <v>3565.168694081408</v>
+        <v>-14931.47402642812</v>
       </c>
       <c r="AA13" t="n">
         <v>1.000000000000027e-08</v>
@@ -5044,7 +4849,7 @@
         <v>2739.898</v>
       </c>
       <c r="C14" t="n">
-        <v>3027.751634308126</v>
+        <v>18412.31764435051</v>
       </c>
       <c r="D14" t="n">
         <v>2.18279e-07</v>
@@ -5077,10 +4882,7 @@
         <v>-29709.0951033068</v>
       </c>
       <c r="Y14" t="n">
-        <v>9.505757559990949e-09</v>
-      </c>
-      <c r="Z14" t="n">
-        <v>3534.132273106329</v>
+        <v>-14859.04802795805</v>
       </c>
       <c r="AA14" t="n">
         <v>1.000000000000331e-08</v>
@@ -5097,7 +4899,7 @@
         <v>2715.872</v>
       </c>
       <c r="C15" t="n">
-        <v>3005.808770667482</v>
+        <v>18371.74321303145</v>
       </c>
       <c r="D15" t="n">
         <v>2.19196e-07</v>
@@ -5130,10 +4932,7 @@
         <v>-29577.41319756097</v>
       </c>
       <c r="Y15" t="n">
-        <v>4.405966353261179e-12</v>
-      </c>
-      <c r="Z15" t="n">
-        <v>3503.030557362109</v>
+        <v>-14842.03771639043</v>
       </c>
       <c r="AA15" t="n">
         <v>1.000000000005382e-08</v>
@@ -5150,7 +4949,7 @@
         <v>2690.1</v>
       </c>
       <c r="C16" t="n">
-        <v>2980.095194621601</v>
+        <v>18415.6229306647</v>
       </c>
       <c r="D16" t="n">
         <v>2.20409e-07</v>
@@ -5183,10 +4982,7 @@
         <v>-29628.45510555273</v>
       </c>
       <c r="Y16" t="n">
-        <v>8.707214415280754e-10</v>
-      </c>
-      <c r="Z16" t="n">
-        <v>3472.204119141927</v>
+        <v>-14914.04648096412</v>
       </c>
       <c r="AA16" t="n">
         <v>1e-08</v>
@@ -5203,7 +4999,7 @@
         <v>2669.379</v>
       </c>
       <c r="C17" t="n">
-        <v>2954.535706711022</v>
+        <v>18936.14954346593</v>
       </c>
       <c r="D17" t="n">
         <v>2.21682e-07</v>
@@ -5236,10 +5032,7 @@
         <v>-30028.57892337986</v>
       </c>
       <c r="Y17" t="n">
-        <v>1.390207030577781e-09</v>
-      </c>
-      <c r="Z17" t="n">
-        <v>3441.373366417077</v>
+        <v>-15470.61176119759</v>
       </c>
       <c r="AA17" t="n">
         <v>1.00000000001704e-08</v>
@@ -5256,7 +5049,7 @@
         <v>2641.589</v>
       </c>
       <c r="C18" t="n">
-        <v>2930.796794881062</v>
+        <v>18761.09597691229</v>
       </c>
       <c r="D18" t="n">
         <v>2.22962e-07</v>
@@ -5289,10 +5082,7 @@
         <v>-30211.57208073499</v>
       </c>
       <c r="Y18" t="n">
-        <v>1.154298452146454e-11</v>
-      </c>
-      <c r="Z18" t="n">
-        <v>3410.426010644573</v>
+        <v>-15322.81822464216</v>
       </c>
       <c r="AA18" t="n">
         <v>1.000000000000535e-08</v>
@@ -5309,7 +5099,7 @@
         <v>2606.438</v>
       </c>
       <c r="C19" t="n">
-        <v>2901.536778522359</v>
+        <v>19287.49797700406</v>
       </c>
       <c r="D19" t="n">
         <v>2.23933e-07</v>
@@ -5342,10 +5132,7 @@
         <v>-28412.79198105791</v>
       </c>
       <c r="Y19" t="n">
-        <v>2.517315629913945e-09</v>
-      </c>
-      <c r="Z19" t="n">
-        <v>3380.128435820616</v>
+        <v>-15880.81107592259</v>
       </c>
       <c r="AA19" t="n">
         <v>1.000000000089883e-08</v>
@@ -5362,7 +5149,7 @@
         <v>2593.08</v>
       </c>
       <c r="C20" t="n">
-        <v>2880.725951501829</v>
+        <v>18917.29831138294</v>
       </c>
       <c r="D20" t="n">
         <v>2.25371e-07</v>
@@ -5395,10 +5182,7 @@
         <v>-30467.94887651073</v>
       </c>
       <c r="Y20" t="n">
-        <v>2.5093519068961e-11</v>
-      </c>
-      <c r="Z20" t="n">
-        <v>3348.381877410202</v>
+        <v>-15537.04911191654</v>
       </c>
       <c r="AA20" t="n">
         <v>1.00000000000073e-08</v>
@@ -5415,7 +5199,7 @@
         <v>2555.902</v>
       </c>
       <c r="C21" t="n">
-        <v>2848.778205815445</v>
+        <v>19667.83645257719</v>
       </c>
       <c r="D21" t="n">
         <v>2.26332e-07</v>
@@ -5448,10 +5232,7 @@
         <v>-28565.88371232273</v>
       </c>
       <c r="Y21" t="n">
-        <v>1.449632556628533e-11</v>
-      </c>
-      <c r="Z21" t="n">
-        <v>3316.26452106183</v>
+        <v>-16321.72691395519</v>
       </c>
       <c r="AA21" t="n">
         <v>1.000000000000639e-08</v>
@@ -5468,7 +5249,7 @@
         <v>2546.351</v>
       </c>
       <c r="C22" t="n">
-        <v>2831.00210979433</v>
+        <v>19742.31910497937</v>
       </c>
       <c r="D22" t="n">
         <v>2.27732e-07</v>
@@ -5501,10 +5282,7 @@
         <v>-31006.39486152134</v>
       </c>
       <c r="Y22" t="n">
-        <v>1.409007508995995e-11</v>
-      </c>
-      <c r="Z22" t="n">
-        <v>3284.11934365875</v>
+        <v>-16428.68713186582</v>
       </c>
       <c r="AA22" t="n">
         <v>1.000000000000556e-08</v>
@@ -5666,6 +5444,9 @@
       <c r="B2" t="n">
         <v>29789.774</v>
       </c>
+      <c r="C2" t="n">
+        <v>33327.71262074241</v>
+      </c>
       <c r="D2" t="n">
         <v>1.32072e-08</v>
       </c>
@@ -5697,10 +5478,7 @@
         <v>-45240.3889864725</v>
       </c>
       <c r="Y2" t="n">
-        <v>1956.981062621956</v>
-      </c>
-      <c r="Z2" t="n">
-        <v>1768.128452230034</v>
+        <v>-924.5168181810222</v>
       </c>
       <c r="AA2" t="n">
         <v>1.571690957730544e-06</v>
@@ -5716,6 +5494,9 @@
       <c r="B3" t="n">
         <v>26771.408</v>
       </c>
+      <c r="C3" t="n">
+        <v>30165.0717318478</v>
+      </c>
       <c r="D3" t="n">
         <v>1.55996e-08</v>
       </c>
@@ -5747,10 +5528,7 @@
         <v>-45857.04613273493</v>
       </c>
       <c r="Y3" t="n">
-        <v>1979.249072103158</v>
-      </c>
-      <c r="Z3" t="n">
-        <v>1792.33888738741</v>
+        <v>-956.6068246394989</v>
       </c>
       <c r="AA3" t="n">
         <v>1.450875310280992e-06</v>
@@ -5766,6 +5544,9 @@
       <c r="B4" t="n">
         <v>25920.575</v>
       </c>
+      <c r="C4" t="n">
+        <v>29228.62355226164</v>
+      </c>
       <c r="D4" t="n">
         <v>1.64421e-08</v>
       </c>
@@ -5797,10 +5578,7 @@
         <v>-45986.20733642069</v>
       </c>
       <c r="Y4" t="n">
-        <v>2019.450788730009</v>
-      </c>
-      <c r="Z4" t="n">
-        <v>1831.238120154344</v>
+        <v>-917.4575299026928</v>
       </c>
       <c r="AA4" t="n">
         <v>1.408136428363595e-06</v>
@@ -5816,6 +5594,9 @@
       <c r="B5" t="n">
         <v>25441.851</v>
       </c>
+      <c r="C5" t="n">
+        <v>28872.02318999152</v>
+      </c>
       <c r="D5" t="n">
         <v>1.69735e-08</v>
       </c>
@@ -5847,10 +5628,7 @@
         <v>-46019.63413940557</v>
       </c>
       <c r="Y5" t="n">
-        <v>2032.692439338152</v>
-      </c>
-      <c r="Z5" t="n">
-        <v>1844.767937746745</v>
+        <v>-1006.114289155465</v>
       </c>
       <c r="AA5" t="n">
         <v>1.642772286163007e-06</v>
@@ -5866,6 +5644,9 @@
       <c r="B6" t="n">
         <v>25040.895</v>
       </c>
+      <c r="C6" t="n">
+        <v>28401.05929905374</v>
+      </c>
       <c r="D6" t="n">
         <v>1.74184e-08</v>
       </c>
@@ -5897,10 +5678,7 @@
         <v>-45443.82219027122</v>
       </c>
       <c r="Y6" t="n">
-        <v>2037.839430945596</v>
-      </c>
-      <c r="Z6" t="n">
-        <v>1850.520666925785</v>
+        <v>-945.6094405018739</v>
       </c>
       <c r="AA6" t="n">
         <v>1.631187797574851e-06</v>
@@ -5916,6 +5694,9 @@
       <c r="B7" t="n">
         <v>24678.185</v>
       </c>
+      <c r="C7" t="n">
+        <v>28186.0616362541</v>
+      </c>
       <c r="D7" t="n">
         <v>1.78152e-08</v>
       </c>
@@ -5947,10 +5728,7 @@
         <v>-45181.24346535742</v>
       </c>
       <c r="Y7" t="n">
-        <v>2089.150040683206</v>
-      </c>
-      <c r="Z7" t="n">
-        <v>1900.018103241254</v>
+        <v>-1039.795124461414</v>
       </c>
       <c r="AA7" t="n">
         <v>1.324157460973251e-06</v>
@@ -5966,6 +5744,9 @@
       <c r="B8" t="n">
         <v>24327.646</v>
       </c>
+      <c r="C8" t="n">
+        <v>27838.37221448872</v>
+      </c>
       <c r="D8" t="n">
         <v>1.81812e-08</v>
       </c>
@@ -5997,10 +5778,7 @@
         <v>-44667.20504721891</v>
       </c>
       <c r="Y8" t="n">
-        <v>2055.020950709662</v>
-      </c>
-      <c r="Z8" t="n">
-        <v>1868.58676095677</v>
+        <v>-1041.441389868525</v>
       </c>
       <c r="AA8" t="n">
         <v>1.60057361096518e-06</v>
@@ -6016,6 +5794,9 @@
       <c r="B9" t="n">
         <v>24010.532</v>
       </c>
+      <c r="C9" t="n">
+        <v>27579.06123718683</v>
+      </c>
       <c r="D9" t="n">
         <v>1.85606e-08</v>
       </c>
@@ -6047,10 +5828,7 @@
         <v>-44748.72817072683</v>
       </c>
       <c r="Y9" t="n">
-        <v>2053.697762144098</v>
-      </c>
-      <c r="Z9" t="n">
-        <v>1868.2901992821</v>
+        <v>-1084.195988369804</v>
       </c>
       <c r="AA9" t="n">
         <v>1.595567646677031e-06</v>
@@ -6066,6 +5844,9 @@
       <c r="B10" t="n">
         <v>23694.74</v>
       </c>
+      <c r="C10" t="n">
+        <v>27233.05123336418</v>
+      </c>
       <c r="D10" t="n">
         <v>1.88953e-08</v>
       </c>
@@ -6097,10 +5878,7 @@
         <v>-44007.99359489807</v>
       </c>
       <c r="Y10" t="n">
-        <v>2069.231919864614</v>
-      </c>
-      <c r="Z10" t="n">
-        <v>1884.084555784315</v>
+        <v>-1059.857980212515</v>
       </c>
       <c r="AA10" t="n">
         <v>1.574361891415273e-06</v>
@@ -6116,6 +5894,9 @@
       <c r="B11" t="n">
         <v>23404.509</v>
       </c>
+      <c r="C11" t="n">
+        <v>26905.73337588082</v>
+      </c>
       <c r="D11" t="n">
         <v>1.92428e-08</v>
       </c>
@@ -6147,10 +5928,7 @@
         <v>-43836.83812154708</v>
       </c>
       <c r="Y11" t="n">
-        <v>2065.449527872279</v>
-      </c>
-      <c r="Z11" t="n">
-        <v>1881.401289827784</v>
+        <v>-1048.117402880951</v>
       </c>
       <c r="AA11" t="n">
         <v>1.571495531452732e-06</v>
@@ -6313,7 +6091,7 @@
         <v>3322.365</v>
       </c>
       <c r="C2" t="n">
-        <v>3650.82957047494</v>
+        <v>21882.83107702006</v>
       </c>
       <c r="D2" t="n">
         <v>1.78228e-07</v>
@@ -6346,10 +6124,7 @@
         <v>-23177.17443704293</v>
       </c>
       <c r="Y2" t="n">
-        <v>8.893462476884348e-10</v>
-      </c>
-      <c r="Z2" t="n">
-        <v>4228.089117988718</v>
+        <v>-17485.45935755949</v>
       </c>
       <c r="AA2" t="n">
         <v>1.000000000000006e-08</v>
@@ -6366,7 +6141,7 @@
         <v>3111.638</v>
       </c>
       <c r="C3" t="n">
-        <v>3407.80629029734</v>
+        <v>23304.00698293357</v>
       </c>
       <c r="D3" t="n">
         <v>1.87857e-07</v>
@@ -6399,10 +6174,7 @@
         <v>-22620.91124627536</v>
       </c>
       <c r="Y3" t="n">
-        <v>3.064630490463671e-09</v>
-      </c>
-      <c r="Z3" t="n">
-        <v>3995.00470750756</v>
+        <v>-19173.73886167778</v>
       </c>
       <c r="AA3" t="n">
         <v>1.000000000000431e-08</v>
@@ -6419,7 +6191,7 @@
         <v>3042.006</v>
       </c>
       <c r="C4" t="n">
-        <v>3338.49633367049</v>
+        <v>22709.43293993048</v>
       </c>
       <c r="D4" t="n">
         <v>1.91062e-07</v>
@@ -6452,10 +6224,7 @@
         <v>-22344.30760975299</v>
       </c>
       <c r="Y4" t="n">
-        <v>1.437133177459935e-09</v>
-      </c>
-      <c r="Z4" t="n">
-        <v>3919.7152960145</v>
+        <v>-18654.38836496458</v>
       </c>
       <c r="AA4" t="n">
         <v>1.000000000000007e-08</v>
@@ -6472,7 +6241,7 @@
         <v>3004.488</v>
       </c>
       <c r="C5" t="n">
-        <v>3297.608195317027</v>
+        <v>21905.785843766</v>
       </c>
       <c r="D5" t="n">
         <v>1.93204e-07</v>
@@ -6505,10 +6274,7 @@
         <v>-22318.02970931322</v>
       </c>
       <c r="Y5" t="n">
-        <v>8.525199959196454e-09</v>
-      </c>
-      <c r="Z5" t="n">
-        <v>3869.999130203362</v>
+        <v>-17896.08293850533</v>
       </c>
       <c r="AA5" t="n">
         <v>1.000000000000002e-08</v>
@@ -6525,7 +6291,7 @@
         <v>2967.235</v>
       </c>
       <c r="C6" t="n">
-        <v>3261.150775920038</v>
+        <v>23166.01071295244</v>
       </c>
       <c r="D6" t="n">
         <v>1.94892e-07</v>
@@ -6558,10 +6324,7 @@
         <v>-22244.56552976538</v>
       </c>
       <c r="Y6" t="n">
-        <v>108.5492817197652</v>
-      </c>
-      <c r="Z6" t="n">
-        <v>4157.638945999423</v>
+        <v>-19206.16325523783</v>
       </c>
       <c r="AA6" t="n">
         <v>1.540680380679318e-08</v>
@@ -6578,7 +6341,7 @@
         <v>2931.648</v>
       </c>
       <c r="C7" t="n">
-        <v>3227.150281694132</v>
+        <v>23149.10676072998</v>
       </c>
       <c r="D7" t="n">
         <v>1.96906e-07</v>
@@ -6611,10 +6374,7 @@
         <v>-22361.41772853267</v>
       </c>
       <c r="Y7" t="n">
-        <v>3.161141659038213e-10</v>
-      </c>
-      <c r="Z7" t="n">
-        <v>3783.196584692455</v>
+        <v>-19235.98678336375</v>
       </c>
       <c r="AA7" t="n">
         <v>1.000000000002135e-08</v>
@@ -6631,7 +6391,7 @@
         <v>2899.958</v>
       </c>
       <c r="C8" t="n">
-        <v>3194.324153581093</v>
+        <v>22437.696518278</v>
       </c>
       <c r="D8" t="n">
         <v>1.9842e-07</v>
@@ -6664,10 +6424,7 @@
         <v>-22260.46846365806</v>
       </c>
       <c r="Y8" t="n">
-        <v>7.603127593450079e-10</v>
-      </c>
-      <c r="Z8" t="n">
-        <v>3742.39318797351</v>
+        <v>-18557.02217627203</v>
       </c>
       <c r="AA8" t="n">
         <v>1.000000000000009e-08</v>
@@ -6684,7 +6441,7 @@
         <v>2868.943</v>
       </c>
       <c r="C9" t="n">
-        <v>3162.916373339117</v>
+        <v>23263.91756812149</v>
       </c>
       <c r="D9" t="n">
         <v>1.99958e-07</v>
@@ -6717,10 +6474,7 @@
         <v>-22222.79574531389</v>
       </c>
       <c r="Y9" t="n">
-        <v>1.521868844776335e-10</v>
-      </c>
-      <c r="Z9" t="n">
-        <v>3703.725698002615</v>
+        <v>-19425.61221051296</v>
       </c>
       <c r="AA9" t="n">
         <v>1.000000000000382e-08</v>
@@ -6737,7 +6491,7 @@
         <v>2838.5</v>
       </c>
       <c r="C10" t="n">
-        <v>3134.406504013357</v>
+        <v>23020.28907006311</v>
       </c>
       <c r="D10" t="n">
         <v>2.01527e-07</v>
@@ -6770,10 +6524,7 @@
         <v>-22321.13870224415</v>
       </c>
       <c r="Y10" t="n">
-        <v>1.914373975216812e-11</v>
-      </c>
-      <c r="Z10" t="n">
-        <v>3666.83455351343</v>
+        <v>-19217.89608233833</v>
       </c>
       <c r="AA10" t="n">
         <v>1e-08</v>
@@ -6790,7 +6541,7 @@
         <v>2812.453</v>
       </c>
       <c r="C11" t="n">
-        <v>3106.500043048217</v>
+        <v>22979.73155508696</v>
       </c>
       <c r="D11" t="n">
         <v>2.02732e-07</v>
@@ -6823,10 +6574,7 @@
         <v>-22237.74262316509</v>
       </c>
       <c r="Y11" t="n">
-        <v>1.537612853485187e-09</v>
-      </c>
-      <c r="Z11" t="n">
-        <v>3631.830470287303</v>
+        <v>-19207.76768152517</v>
       </c>
       <c r="AA11" t="n">
         <v>1e-08</v>
@@ -6843,7 +6591,7 @@
         <v>2771.025</v>
       </c>
       <c r="C12" t="n">
-        <v>3070.899102276457</v>
+        <v>22795.52636169256</v>
       </c>
       <c r="D12" t="n">
         <v>2.04309e-07</v>
@@ -6876,10 +6624,7 @@
         <v>-21469.97362443178</v>
       </c>
       <c r="Y12" t="n">
-        <v>2.59594962930328e-10</v>
-      </c>
-      <c r="Z12" t="n">
-        <v>3597.710134803611</v>
+        <v>-19058.57239403903</v>
       </c>
       <c r="AA12" t="n">
         <v>1.000000000000025e-08</v>
@@ -6896,7 +6641,7 @@
         <v>2744.331</v>
       </c>
       <c r="C13" t="n">
-        <v>3046.585549572324</v>
+        <v>22874.38243035931</v>
       </c>
       <c r="D13" t="n">
         <v>2.0556e-07</v>
@@ -6929,10 +6674,7 @@
         <v>-21355.93043890158</v>
       </c>
       <c r="Y13" t="n">
-        <v>2.201600607771591e-09</v>
-      </c>
-      <c r="Z13" t="n">
-        <v>3565.162528323268</v>
+        <v>-19167.54941299073</v>
       </c>
       <c r="AA13" t="n">
         <v>1.000000000004395e-08</v>
@@ -6949,7 +6691,7 @@
         <v>2736.308</v>
       </c>
       <c r="C14" t="n">
-        <v>3025.904766034668</v>
+        <v>23574.84239008972</v>
       </c>
       <c r="D14" t="n">
         <v>2.06697e-07</v>
@@ -6982,10 +6724,7 @@
         <v>-22274.28733436464</v>
       </c>
       <c r="Y14" t="n">
-        <v>9.726162347189987e-10</v>
-      </c>
-      <c r="Z14" t="n">
-        <v>3533.235419048723</v>
+        <v>-19900.16492248893</v>
       </c>
       <c r="AA14" t="n">
         <v>1.000000000000054e-08</v>
@@ -7002,7 +6741,7 @@
         <v>2711.123</v>
       </c>
       <c r="C15" t="n">
-        <v>3001.219302926584</v>
+        <v>23964.83447880792</v>
       </c>
       <c r="D15" t="n">
         <v>2.0799e-07</v>
@@ -7035,10 +6774,7 @@
         <v>-22305.63043253864</v>
       </c>
       <c r="Y15" t="n">
-        <v>2.388420229840544e-13</v>
-      </c>
-      <c r="Z15" t="n">
-        <v>3502.544657250044</v>
+        <v>-20323.04658907605</v>
       </c>
       <c r="AA15" t="n">
         <v>1.00000000000016e-08</v>
@@ -7055,7 +6791,7 @@
         <v>2681.612</v>
       </c>
       <c r="C16" t="n">
-        <v>2975.634922521201</v>
+        <v>22668.46326878448</v>
       </c>
       <c r="D16" t="n">
         <v>2.09486e-07</v>
@@ -7088,10 +6824,7 @@
         <v>-22446.19013596027</v>
       </c>
       <c r="Y16" t="n">
-        <v>2.934456815630635e-13</v>
-      </c>
-      <c r="Z16" t="n">
-        <v>3470.791470776857</v>
+        <v>-19053.80287434614</v>
       </c>
       <c r="AA16" t="n">
         <v>1e-08</v>
@@ -7108,7 +6841,7 @@
         <v>2660.27</v>
       </c>
       <c r="C17" t="n">
-        <v>2951.298267920116</v>
+        <v>23764.58488279068</v>
       </c>
       <c r="D17" t="n">
         <v>2.10877e-07</v>
@@ -7141,10 +6874,7 @@
         <v>-22596.09049655399</v>
       </c>
       <c r="Y17" t="n">
-        <v>4.093997846238827e-11</v>
-      </c>
-      <c r="Z17" t="n">
-        <v>3439.868900978634</v>
+        <v>-20188.20251899966</v>
       </c>
       <c r="AA17" t="n">
         <v>1.000000000000001e-08</v>
@@ -7161,7 +6891,7 @@
         <v>2617.769</v>
       </c>
       <c r="C18" t="n">
-        <v>2920.537579861825</v>
+        <v>23832.87791817626</v>
       </c>
       <c r="D18" t="n">
         <v>2.12058e-07</v>
@@ -7194,10 +6924,7 @@
         <v>-21479.22854676919</v>
       </c>
       <c r="Y18" t="n">
-        <v>3.318572629114995e-10</v>
-      </c>
-      <c r="Z18" t="n">
-        <v>3407.362653459402</v>
+        <v>-20285.01675445477</v>
       </c>
       <c r="AA18" t="n">
         <v>1.000000000000108e-08</v>
@@ -7214,7 +6941,7 @@
         <v>2609.157</v>
       </c>
       <c r="C19" t="n">
-        <v>2901.6142971371</v>
+        <v>23859.29548521081</v>
       </c>
       <c r="D19" t="n">
         <v>2.13129e-07</v>
@@ -7247,10 +6974,7 @@
         <v>-22438.99957906457</v>
       </c>
       <c r="Y19" t="n">
-        <v>3.254157878042292e-10</v>
-      </c>
-      <c r="Z19" t="n">
-        <v>3376.308599464076</v>
+        <v>-20338.40856103564</v>
       </c>
       <c r="AA19" t="n">
         <v>1.000000000000126e-08</v>
@@ -7267,7 +6991,7 @@
         <v>2587.246</v>
       </c>
       <c r="C20" t="n">
-        <v>2874.331699071025</v>
+        <v>24451.9489637303</v>
       </c>
       <c r="D20" t="n">
         <v>2.14538e-07</v>
@@ -7300,10 +7024,7 @@
         <v>-22600.62203483048</v>
       </c>
       <c r="Y20" t="n">
-        <v>4.211313836099983e-10</v>
-      </c>
-      <c r="Z20" t="n">
-        <v>3343.295576878203</v>
+        <v>-20967.13911240837</v>
       </c>
       <c r="AA20" t="n">
         <v>1.000000000000235e-08</v>
@@ -7320,7 +7041,7 @@
         <v>2559.778</v>
       </c>
       <c r="C21" t="n">
-        <v>2850.137979121015</v>
+        <v>23901.71429163749</v>
       </c>
       <c r="D21" t="n">
         <v>2.1588e-07</v>
@@ -7353,10 +7074,7 @@
         <v>-22600.83675982003</v>
       </c>
       <c r="Y21" t="n">
-        <v>4.352747599166061e-10</v>
-      </c>
-      <c r="Z21" t="n">
-        <v>3311.167146405325</v>
+        <v>-20444.93452610614</v>
       </c>
       <c r="AA21" t="n">
         <v>1.000000000000249e-08</v>
@@ -7373,7 +7091,7 @@
         <v>2535.847</v>
       </c>
       <c r="C22" t="n">
-        <v>2825.269874185038</v>
+        <v>23638.60499697087</v>
       </c>
       <c r="D22" t="n">
         <v>2.17096e-07</v>
@@ -7406,10 +7124,7 @@
         <v>-22571.66848477024</v>
       </c>
       <c r="Y22" t="n">
-        <v>5.382503022771223e-10</v>
-      </c>
-      <c r="Z22" t="n">
-        <v>3279.976366698247</v>
+        <v>-20208.85125501974</v>
       </c>
       <c r="AA22" t="n">
         <v>1.000000000000328e-08</v>
@@ -7571,6 +7286,9 @@
       <c r="B2" t="n">
         <v>21355.602</v>
       </c>
+      <c r="C2" t="n">
+        <v>24310.35332797161</v>
+      </c>
       <c r="D2" t="n">
         <v>2.19312e-08</v>
       </c>
@@ -7602,10 +7320,7 @@
         <v>-49517.09064727029</v>
       </c>
       <c r="Y2" t="n">
-        <v>2129.258059778241</v>
-      </c>
-      <c r="Z2" t="n">
-        <v>1951.723150083427</v>
+        <v>-901.5598522225791</v>
       </c>
       <c r="AA2" t="n">
         <v>1.331561679608598e-06</v>
@@ -7621,6 +7336,9 @@
       <c r="B3" t="n">
         <v>19995.383</v>
       </c>
+      <c r="C3" t="n">
+        <v>22741.41292829712</v>
+      </c>
       <c r="D3" t="n">
         <v>2.3848e-08</v>
       </c>
@@ -7652,10 +7370,7 @@
         <v>-47690.15351683742</v>
       </c>
       <c r="Y3" t="n">
-        <v>1024.357689096387</v>
-      </c>
-      <c r="Z3" t="n">
-        <v>805.7256111545275</v>
+        <v>-836.6940407679376</v>
       </c>
       <c r="AA3" t="n">
         <v>5.084512325403472e-06</v>
@@ -7672,7 +7387,7 @@
         <v>19535.205</v>
       </c>
       <c r="C4" t="n">
-        <v>33.3011248279415</v>
+        <v>22311.9358369029</v>
       </c>
       <c r="D4" t="n">
         <v>2.45918e-08</v>
@@ -7705,10 +7420,7 @@
         <v>-47355.04958175466</v>
       </c>
       <c r="Y4" t="n">
-        <v>1024.280845988597</v>
-      </c>
-      <c r="Z4" t="n">
-        <v>805.6647883388291</v>
+        <v>-887.3995769490102</v>
       </c>
       <c r="AA4" t="n">
         <v>5.758943613172105e-07</v>
@@ -7724,6 +7436,9 @@
       <c r="B5" t="n">
         <v>19229.25</v>
       </c>
+      <c r="C5" t="n">
+        <v>21971.80860447977</v>
+      </c>
       <c r="D5" t="n">
         <v>2.50677e-08</v>
       </c>
@@ -7755,10 +7470,7 @@
         <v>-46602.83010421869</v>
       </c>
       <c r="Y5" t="n">
-        <v>1020.435705028042</v>
-      </c>
-      <c r="Z5" t="n">
-        <v>802.6869968887955</v>
+        <v>-879.4881439012697</v>
       </c>
       <c r="AA5" t="n">
         <v>5.815535215137008e-07</v>
@@ -7774,6 +7486,9 @@
       <c r="B6" t="n">
         <v>18966.987</v>
       </c>
+      <c r="C6" t="n">
+        <v>21646.29884215402</v>
+      </c>
       <c r="D6" t="n">
         <v>2.54918e-08</v>
       </c>
@@ -7805,10 +7520,7 @@
         <v>-46037.55812443314</v>
       </c>
       <c r="Y6" t="n">
-        <v>1018.750217461095</v>
-      </c>
-      <c r="Z6" t="n">
-        <v>801.3644191667836</v>
+        <v>-850.1123768140296</v>
       </c>
       <c r="AA6" t="n">
         <v>5.873364916621856e-07</v>
@@ -7824,6 +7536,9 @@
       <c r="B7" t="n">
         <v>18716.335</v>
       </c>
+      <c r="C7" t="n">
+        <v>21203.92089546782</v>
+      </c>
       <c r="D7" t="n">
         <v>2.59352e-08</v>
       </c>
@@ -7855,10 +7570,7 @@
         <v>-45732.5218983997</v>
       </c>
       <c r="Y7" t="n">
-        <v>1050.278977589443</v>
-      </c>
-      <c r="Z7" t="n">
-        <v>825.9004722203405</v>
+        <v>-736.5088603431268</v>
       </c>
       <c r="AA7" t="n">
         <v>6.083861780229042e-07</v>
@@ -7874,6 +7586,9 @@
       <c r="B8" t="n">
         <v>18490.21</v>
       </c>
+      <c r="C8" t="n">
+        <v>21188.06911028613</v>
+      </c>
       <c r="D8" t="n">
         <v>2.6343e-08</v>
       </c>
@@ -7905,10 +7620,7 @@
         <v>-45235.98649035033</v>
       </c>
       <c r="Y8" t="n">
-        <v>1034.012317430827</v>
-      </c>
-      <c r="Z8" t="n">
-        <v>813.2709220478805</v>
+        <v>-878.2427655348456</v>
       </c>
       <c r="AA8" t="n">
         <v>6.070105779354064e-07</v>
@@ -7924,6 +7636,9 @@
       <c r="B9" t="n">
         <v>18273.95</v>
       </c>
+      <c r="C9" t="n">
+        <v>20848.39441290161</v>
+      </c>
       <c r="D9" t="n">
         <v>2.67788e-08</v>
       </c>
@@ -7955,10 +7670,7 @@
         <v>-45376.59162594052</v>
       </c>
       <c r="Y9" t="n">
-        <v>1032.644189121561</v>
-      </c>
-      <c r="Z9" t="n">
-        <v>812.2355099879258</v>
+        <v>-820.697165913085</v>
       </c>
       <c r="AA9" t="n">
         <v>6.128409756477646e-07</v>
@@ -7975,7 +7687,7 @@
         <v>18051.387</v>
       </c>
       <c r="C10" t="n">
-        <v>11.59040584074107</v>
+        <v>20859.55767566495</v>
       </c>
       <c r="D10" t="n">
         <v>2.72089e-08</v>
@@ -8008,10 +7720,7 @@
         <v>-45061.15871900824</v>
       </c>
       <c r="Y10" t="n">
-        <v>1054.766489828831</v>
-      </c>
-      <c r="Z10" t="n">
-        <v>829.4637197581885</v>
+        <v>-974.5656399042509</v>
       </c>
       <c r="AA10" t="n">
         <v>6.296471027099854e-07</v>
@@ -8027,6 +7736,9 @@
       <c r="B11" t="n">
         <v>17846.934</v>
       </c>
+      <c r="C11" t="n">
+        <v>20596.7865654321</v>
+      </c>
       <c r="D11" t="n">
         <v>2.76149e-08</v>
       </c>
@@ -8058,10 +7770,7 @@
         <v>-44681.57681083908</v>
       </c>
       <c r="Y11" t="n">
-        <v>1039.18120141719</v>
-      </c>
-      <c r="Z11" t="n">
-        <v>817.3672774843495</v>
+        <v>-945.0894185892012</v>
       </c>
       <c r="AA11" t="n">
         <v>6.282777388457208e-07</v>
@@ -8224,7 +7933,7 @@
         <v>3325.154</v>
       </c>
       <c r="C2" t="n">
-        <v>3630.726008721113</v>
+        <v>22338.41667036461</v>
       </c>
       <c r="D2" t="n">
         <v>1.81236e-07</v>
@@ -8257,10 +7966,7 @@
         <v>-25240.86560628705</v>
       </c>
       <c r="Y2" t="n">
-        <v>6.270757693317334e-11</v>
-      </c>
-      <c r="Z2" t="n">
-        <v>4205.884890064634</v>
+        <v>-18010.7886179743</v>
       </c>
       <c r="AA2" t="n">
         <v>1.000000000000227e-08</v>
@@ -8277,7 +7983,7 @@
         <v>3141.792</v>
       </c>
       <c r="C3" t="n">
-        <v>3422.511115955506</v>
+        <v>22074.72994442551</v>
       </c>
       <c r="D3" t="n">
         <v>1.9048e-07</v>
@@ -8310,10 +8016,7 @@
         <v>-25918.45067978542</v>
       </c>
       <c r="Y3" t="n">
-        <v>1.366125040588221e-09</v>
-      </c>
-      <c r="Z3" t="n">
-        <v>4006.036155422891</v>
+        <v>-17985.85448697049</v>
       </c>
       <c r="AA3" t="n">
         <v>1.000000000001866e-08</v>
@@ -8330,7 +8033,7 @@
         <v>3060.812</v>
       </c>
       <c r="C4" t="n">
-        <v>3351.096234653782</v>
+        <v>22130.26395784057</v>
       </c>
       <c r="D4" t="n">
         <v>1.93226e-07</v>
@@ -8363,10 +8066,7 @@
         <v>-24256.1941018422</v>
       </c>
       <c r="Y4" t="n">
-        <v>1.090156318120623e-10</v>
-      </c>
-      <c r="Z4" t="n">
-        <v>3935.821912233584</v>
+        <v>-18109.11039232884</v>
       </c>
       <c r="AA4" t="n">
         <v>1.00000000000013e-08</v>
@@ -8383,7 +8083,7 @@
         <v>3034.613</v>
       </c>
       <c r="C5" t="n">
-        <v>3316.089935460038</v>
+        <v>21722.29175471588</v>
       </c>
       <c r="D5" t="n">
         <v>1.95508e-07</v>
@@ -8416,10 +8116,7 @@
         <v>-25357.76128331328</v>
       </c>
       <c r="Y5" t="n">
-        <v>1.062312420446039e-09</v>
-      </c>
-      <c r="Z5" t="n">
-        <v>3883.031795920439</v>
+        <v>-17751.04407209818</v>
       </c>
       <c r="AA5" t="n">
         <v>1.000000000003094e-08</v>
@@ -8436,7 +8133,7 @@
         <v>2976.087</v>
       </c>
       <c r="C6" t="n">
-        <v>3270.613190918845</v>
+        <v>22307.84934380135</v>
       </c>
       <c r="D6" t="n">
         <v>1.97471e-07</v>
@@ -8469,10 +8166,7 @@
         <v>-24112.9860223846</v>
       </c>
       <c r="Y6" t="n">
-        <v>8.118152899628944e-10</v>
-      </c>
-      <c r="Z6" t="n">
-        <v>3835.022553553898</v>
+        <v>-18387.40079505501</v>
       </c>
       <c r="AA6" t="n">
         <v>1.000000000085918e-08</v>
@@ -8489,7 +8183,7 @@
         <v>2940.544</v>
       </c>
       <c r="C7" t="n">
-        <v>3233.286901548908</v>
+        <v>22617.29035669901</v>
       </c>
       <c r="D7" t="n">
         <v>1.99153e-07</v>
@@ -8522,10 +8216,7 @@
         <v>-23880.97846679137</v>
       </c>
       <c r="Y7" t="n">
-        <v>5.527629492869572e-09</v>
-      </c>
-      <c r="Z7" t="n">
-        <v>3789.242727888626</v>
+        <v>-18738.98268711635</v>
       </c>
       <c r="AA7" t="n">
         <v>1.000000000001076e-08</v>
@@ -8542,7 +8233,7 @@
         <v>2907.828</v>
       </c>
       <c r="C8" t="n">
-        <v>3197.462404060361</v>
+        <v>22304.82026443247</v>
       </c>
       <c r="D8" t="n">
         <v>2.01033e-07</v>
@@ -8575,10 +8266,7 @@
         <v>-23942.89984628868</v>
       </c>
       <c r="Y8" t="n">
-        <v>1.841086815799093e-18</v>
-      </c>
-      <c r="Z8" t="n">
-        <v>3746.924357180184</v>
+        <v>-18467.05848532115</v>
       </c>
       <c r="AA8" t="n">
         <v>1e-08</v>
@@ -8595,7 +8283,7 @@
         <v>2858.686</v>
       </c>
       <c r="C9" t="n">
-        <v>3159.784101077867</v>
+        <v>22544.47686629575</v>
       </c>
       <c r="D9" t="n">
         <v>2.02102e-07</v>
@@ -8628,10 +8316,7 @@
         <v>-22608.23938092466</v>
       </c>
       <c r="Y9" t="n">
-        <v>5.253107119837181e-09</v>
-      </c>
-      <c r="Z9" t="n">
-        <v>3707.706541242992</v>
+        <v>-18737.49211091574</v>
       </c>
       <c r="AA9" t="n">
         <v>1.000000000000546e-08</v>
@@ -8648,7 +8333,7 @@
         <v>2846.17</v>
       </c>
       <c r="C10" t="n">
-        <v>3136.358904322622</v>
+        <v>22658.22965194684</v>
       </c>
       <c r="D10" t="n">
         <v>2.03372e-07</v>
@@ -8681,10 +8366,7 @@
         <v>-23554.23940132603</v>
       </c>
       <c r="Y10" t="n">
-        <v>1.065173126294553e-09</v>
-      </c>
-      <c r="Z10" t="n">
-        <v>3671.700118648755</v>
+        <v>-18883.64396315628</v>
       </c>
       <c r="AA10" t="n">
         <v>1.000000000003668e-08</v>
@@ -8701,7 +8383,7 @@
         <v>2799.328</v>
       </c>
       <c r="C11" t="n">
-        <v>3102.544920355321</v>
+        <v>21907.7716915847</v>
       </c>
       <c r="D11" t="n">
         <v>2.05532e-07</v>
@@ -8734,10 +8416,7 @@
         <v>-22608.79222095496</v>
       </c>
       <c r="Y11" t="n">
-        <v>1.443028795686406e-11</v>
-      </c>
-      <c r="Z11" t="n">
-        <v>3636.999587679381</v>
+        <v>-18170.61474990889</v>
       </c>
       <c r="AA11" t="n">
         <v>1e-08</v>
@@ -8754,7 +8433,7 @@
         <v>2787.206</v>
       </c>
       <c r="C12" t="n">
-        <v>3081.418551896954</v>
+        <v>22065.75044260388</v>
       </c>
       <c r="D12" t="n">
         <v>2.07182e-07</v>
@@ -8787,10 +8466,7 @@
         <v>-23927.93281765433</v>
       </c>
       <c r="Y12" t="n">
-        <v>6.340449691658653e-09</v>
-      </c>
-      <c r="Z12" t="n">
-        <v>3601.486744222801</v>
+        <v>-18366.76525758787</v>
       </c>
       <c r="AA12" t="n">
         <v>1.000000000000003e-08</v>
@@ -8807,7 +8483,7 @@
         <v>2764.489</v>
       </c>
       <c r="C13" t="n">
-        <v>3054.279845068714</v>
+        <v>22162.85092856931</v>
       </c>
       <c r="D13" t="n">
         <v>2.08491e-07</v>
@@ -8840,10 +8516,7 @@
         <v>-23877.65084057717</v>
       </c>
       <c r="Y13" t="n">
-        <v>2.483823806000081e-09</v>
-      </c>
-      <c r="Z13" t="n">
-        <v>3567.391755983299</v>
+        <v>-18495.12837106384</v>
       </c>
       <c r="AA13" t="n">
         <v>1.00000000000465e-08</v>
@@ -8860,7 +8533,7 @@
         <v>2735.817</v>
       </c>
       <c r="C14" t="n">
-        <v>3024.075233880629</v>
+        <v>22085.30104383794</v>
       </c>
       <c r="D14" t="n">
         <v>2.10226e-07</v>
@@ -8893,10 +8566,7 @@
         <v>-24035.14571194406</v>
       </c>
       <c r="Y14" t="n">
-        <v>8.260371997464482e-10</v>
-      </c>
-      <c r="Z14" t="n">
-        <v>3530.136990515655</v>
+        <v>-18455.09117227094</v>
       </c>
       <c r="AA14" t="n">
         <v>1.00000000000052e-08</v>
@@ -8913,7 +8583,7 @@
         <v>2707</v>
       </c>
       <c r="C15" t="n">
-        <v>2995.846099839061</v>
+        <v>22474.37285338949</v>
       </c>
       <c r="D15" t="n">
         <v>2.11741e-07</v>
@@ -8946,10 +8616,7 @@
         <v>-24077.96734353064</v>
       </c>
       <c r="Y15" t="n">
-        <v>1.045967857513008e-08</v>
-      </c>
-      <c r="Z15" t="n">
-        <v>3494.753960988774</v>
+        <v>-18881.64817775163</v>
       </c>
       <c r="AA15" t="n">
         <v>1.000000000000096e-08</v>
@@ -8966,7 +8633,7 @@
         <v>2678.878</v>
       </c>
       <c r="C16" t="n">
-        <v>2968.215587582626</v>
+        <v>22364.30219117351</v>
       </c>
       <c r="D16" t="n">
         <v>2.13262e-07</v>
@@ -8999,10 +8666,7 @@
         <v>-24198.23749121563</v>
       </c>
       <c r="Y16" t="n">
-        <v>1.948108843070904e-11</v>
-      </c>
-      <c r="Z16" t="n">
-        <v>3458.818557263857</v>
+        <v>-18804.96558876591</v>
       </c>
       <c r="AA16" t="n">
         <v>1e-08</v>
@@ -9019,7 +8683,7 @@
         <v>2633.819</v>
       </c>
       <c r="C17" t="n">
-        <v>2932.894652037672</v>
+        <v>22376.08278100589</v>
       </c>
       <c r="D17" t="n">
         <v>2.1475e-07</v>
@@ -9052,10 +8716,7 @@
         <v>-23037.61815999198</v>
       </c>
       <c r="Y17" t="n">
-        <v>1.043567252003006e-10</v>
-      </c>
-      <c r="Z17" t="n">
-        <v>3422.892343149957</v>
+        <v>-18850.99068901324</v>
       </c>
       <c r="AA17" t="n">
         <v>1.000000000000179e-08</v>
@@ -9072,7 +8733,7 @@
         <v>2620.086</v>
       </c>
       <c r="C18" t="n">
-        <v>2911.194669997487</v>
+        <v>22972.14432512193</v>
       </c>
       <c r="D18" t="n">
         <v>2.1609e-07</v>
@@ -9105,10 +8766,7 @@
         <v>-24101.99252541294</v>
       </c>
       <c r="Y18" t="n">
-        <v>9.423737355848379e-10</v>
-      </c>
-      <c r="Z18" t="n">
-        <v>3386.592759906148</v>
+        <v>-19482.38783517939</v>
       </c>
       <c r="AA18" t="n">
         <v>1.000000000013627e-08</v>
@@ -9125,7 +8783,7 @@
         <v>2592.122</v>
       </c>
       <c r="C19" t="n">
-        <v>2882.923897820968</v>
+        <v>22693.72339483428</v>
       </c>
       <c r="D19" t="n">
         <v>2.1782e-07</v>
@@ -9158,10 +8816,7 @@
         <v>-24210.42648286345</v>
       </c>
       <c r="Y19" t="n">
-        <v>7.560569546736046e-10</v>
-      </c>
-      <c r="Z19" t="n">
-        <v>3350.73296563084</v>
+        <v>-19239.0611533708</v>
       </c>
       <c r="AA19" t="n">
         <v>1.000000000000281e-08</v>
@@ -9178,7 +8833,7 @@
         <v>2552.539</v>
       </c>
       <c r="C20" t="n">
-        <v>2845.928313409928</v>
+        <v>23219.88969473338</v>
       </c>
       <c r="D20" t="n">
         <v>2.19358e-07</v>
@@ -9211,10 +8866,7 @@
         <v>-23325.0883676794</v>
       </c>
       <c r="Y20" t="n">
-        <v>8.443247870371154e-10</v>
-      </c>
-      <c r="Z20" t="n">
-        <v>3315.237452897345</v>
+        <v>-19803.73628549997</v>
       </c>
       <c r="AA20" t="n">
         <v>1.00000000000028e-08</v>
@@ -9231,7 +8883,7 @@
         <v>2541.159</v>
       </c>
       <c r="C21" t="n">
-        <v>2826.707504808937</v>
+        <v>22811.1870061072</v>
       </c>
       <c r="D21" t="n">
         <v>2.20969e-07</v>
@@ -9264,10 +8916,7 @@
         <v>-24580.98805300962</v>
       </c>
       <c r="Y21" t="n">
-        <v>1.059451165241389e-09</v>
-      </c>
-      <c r="Z21" t="n">
-        <v>3280.066896952231</v>
+        <v>-19427.59015570354</v>
       </c>
       <c r="AA21" t="n">
         <v>1.000000000000019e-08</v>
@@ -9284,7 +8933,7 @@
         <v>2502.932</v>
       </c>
       <c r="C22" t="n">
-        <v>2793.370445717521</v>
+        <v>23037.95154138989</v>
       </c>
       <c r="D22" t="n">
         <v>2.22296e-07</v>
@@ -9317,10 +8966,7 @@
         <v>-23311.86417902619</v>
       </c>
       <c r="Y22" t="n">
-        <v>5.943266053885061e-11</v>
-      </c>
-      <c r="Z22" t="n">
-        <v>3244.75084351878</v>
+        <v>-19685.82416935624</v>
       </c>
       <c r="AA22" t="n">
         <v>1.000000000000284e-08</v>
@@ -9482,6 +9128,9 @@
       <c r="B2" t="n">
         <v>1.840000000000003</v>
       </c>
+      <c r="C2" t="n">
+        <v>15284.19921817283</v>
+      </c>
       <c r="D2" t="n">
         <v>9.7505e-08</v>
       </c>
@@ -9513,10 +9162,7 @@
         <v>1473.924585948794</v>
       </c>
       <c r="Y2" t="n">
-        <v>1401.196004579856</v>
-      </c>
-      <c r="Z2" t="n">
-        <v>1631.18191604417</v>
+        <v>-7289.556985469727</v>
       </c>
       <c r="AA2" t="n">
         <v>1.051011123548062e-06</v>
@@ -9532,6 +9178,9 @@
       <c r="B3" t="n">
         <v>1.292999999999978</v>
       </c>
+      <c r="C3" t="n">
+        <v>17266.57697535981</v>
+      </c>
       <c r="D3" t="n">
         <v>1.14436e-07</v>
       </c>
@@ -9563,10 +9212,7 @@
         <v>1422.856753080394</v>
       </c>
       <c r="Y3" t="n">
-        <v>1347.116838125768</v>
-      </c>
-      <c r="Z3" t="n">
-        <v>1908.251136774144</v>
+        <v>-10321.73835520386</v>
       </c>
       <c r="AA3" t="n">
         <v>1.08770333002106e-06</v>
@@ -9582,6 +9228,9 @@
       <c r="B4" t="n">
         <v>0</v>
       </c>
+      <c r="C4" t="n">
+        <v>17393.87234931476</v>
+      </c>
       <c r="D4" t="n">
         <v>1.19016e-07</v>
       </c>
@@ -9613,10 +9262,7 @@
         <v>1403.472960239763</v>
       </c>
       <c r="Y4" t="n">
-        <v>1332.669021893373</v>
-      </c>
-      <c r="Z4" t="n">
-        <v>1978.149661239184</v>
+        <v>-10691.7340515778</v>
       </c>
       <c r="AA4" t="n">
         <v>4.270518337465608e-07</v>
@@ -9633,7 +9279,7 @@
         <v>5421.400000000001</v>
       </c>
       <c r="C5" t="n">
-        <v>5643.658179915051</v>
+        <v>17282.75154256652</v>
       </c>
       <c r="D5" t="n">
         <v>1.21355e-07</v>
@@ -9666,10 +9312,7 @@
         <v>-32709.54889527945</v>
       </c>
       <c r="Y5" t="n">
-        <v>1326.417365955968</v>
-      </c>
-      <c r="Z5" t="n">
-        <v>1998.175729126543</v>
+        <v>-10698.80942292155</v>
       </c>
       <c r="AA5" t="n">
         <v>6.826957621136403e-07</v>
@@ -9686,7 +9329,7 @@
         <v>5335.116</v>
       </c>
       <c r="C6" t="n">
-        <v>5557.267393916522</v>
+        <v>18003.69914817091</v>
       </c>
       <c r="D6" t="n">
         <v>1.23201e-07</v>
@@ -9719,10 +9362,7 @@
         <v>-32337.57892839805</v>
       </c>
       <c r="Y6" t="n">
-        <v>1320.827331146576</v>
-      </c>
-      <c r="Z6" t="n">
-        <v>2033.248541069018</v>
+        <v>-11520.09538121229</v>
       </c>
       <c r="AA6" t="n">
         <v>7.760050573478072e-07</v>
@@ -9739,7 +9379,7 @@
         <v>5266.168000000001</v>
       </c>
       <c r="C7" t="n">
-        <v>5481.168039354905</v>
+        <v>18320.41261935746</v>
       </c>
       <c r="D7" t="n">
         <v>1.24738e-07</v>
@@ -9772,10 +9412,7 @@
         <v>-32085.27061135535</v>
       </c>
       <c r="Y7" t="n">
-        <v>1315.908761296211</v>
-      </c>
-      <c r="Z7" t="n">
-        <v>2022.189329838532</v>
+        <v>-11918.21283957857</v>
       </c>
       <c r="AA7" t="n">
         <v>7.749964132148386e-07</v>
@@ -9792,7 +9429,7 @@
         <v>5199.491</v>
       </c>
       <c r="C8" t="n">
-        <v>5410.207537072618</v>
+        <v>17942.87306599994</v>
       </c>
       <c r="D8" t="n">
         <v>1.26549e-07</v>
@@ -9825,10 +9462,7 @@
         <v>-32163.55918792906</v>
       </c>
       <c r="Y8" t="n">
-        <v>1307.59177113655</v>
-      </c>
-      <c r="Z8" t="n">
-        <v>2080.286576406515</v>
+        <v>-11618.05657575635</v>
       </c>
       <c r="AA8" t="n">
         <v>6.154688151701993e-07</v>
@@ -9845,7 +9479,7 @@
         <v>5135.626</v>
       </c>
       <c r="C9" t="n">
-        <v>5348.861747908688</v>
+        <v>17907.96873703426</v>
       </c>
       <c r="D9" t="n">
         <v>1.28225e-07</v>
@@ -9878,10 +9512,7 @@
         <v>-32317.31811041562</v>
       </c>
       <c r="Y9" t="n">
-        <v>1280.492410046041</v>
-      </c>
-      <c r="Z9" t="n">
-        <v>2085.27265334374</v>
+        <v>-11657.46385907079</v>
       </c>
       <c r="AA9" t="n">
         <v>3.492951438614063e-07</v>
@@ -9898,7 +9529,7 @@
         <v>5074.596</v>
       </c>
       <c r="C10" t="n">
-        <v>5292.93248541252</v>
+        <v>17590.24873468074</v>
       </c>
       <c r="D10" t="n">
         <v>1.29444e-07</v>
@@ -9931,10 +9562,7 @@
         <v>-31493.67015169379</v>
       </c>
       <c r="Y10" t="n">
-        <v>1274.975530408735</v>
-      </c>
-      <c r="Z10" t="n">
-        <v>2094.781360184912</v>
+        <v>-11392.91138391374</v>
       </c>
       <c r="AA10" t="n">
         <v>3.42099152654186e-07</v>
@@ -9951,7 +9579,7 @@
         <v>5012.176</v>
       </c>
       <c r="C11" t="n">
-        <v>5226.635561220613</v>
+        <v>17699.02881553981</v>
       </c>
       <c r="D11" t="n">
         <v>1.3106e-07</v>
@@ -9984,10 +9612,7 @@
         <v>-31522.51990936588</v>
       </c>
       <c r="Y11" t="n">
-        <v>1268.580589533905</v>
-      </c>
-      <c r="Z11" t="n">
-        <v>2113.911687240773</v>
+        <v>-11573.73122852622</v>
       </c>
       <c r="AA11" t="n">
         <v>3.320901754157028e-07</v>

</xml_diff>